<commit_message>
updated to latest component metrics
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JoshuaJohnstone\LTG Dropbox\Joshua Johnstone\RwoD Research\Team A\Experiments\Small somatic mutations\CODECseq\20250507 Component level metrics\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cameron Fraser\LTG Dropbox\Cameron Fraser\RwoD Research\Team A\Experiments\Small somatic mutations\CODECseq\20250507 Component level metrics\Archive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABA1F321-ABF3-4899-B848-4A10EB48D57B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D6160E8-4676-47D9-BB20-5C8A4A086C83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="component_metrics" sheetId="1" r:id="rId1"/>
@@ -1203,9 +1203,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="8"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1591,19 +1590,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
   <dimension ref="A1:K84"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="35.140625" customWidth="1"/>
-    <col min="2" max="2" width="82.140625" customWidth="1"/>
-    <col min="3" max="4" width="35.28515625" customWidth="1"/>
+    <col min="1" max="1" width="35.1796875" customWidth="1"/>
+    <col min="2" max="2" width="82.1796875" customWidth="1"/>
+    <col min="3" max="4" width="35.26953125" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" customWidth="1"/>
-    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="12.81640625" customWidth="1"/>
+    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="54" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>41</v>
       </c>
@@ -1638,7 +1637,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>45</v>
       </c>
@@ -1667,7 +1666,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>46</v>
       </c>
@@ -1702,7 +1701,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>47</v>
       </c>
@@ -1731,7 +1730,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>59</v>
       </c>
@@ -1760,7 +1759,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>58</v>
       </c>
@@ -1795,7 +1794,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>60</v>
       </c>
@@ -1824,7 +1823,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>61</v>
       </c>
@@ -1859,7 +1858,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -1894,7 +1893,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -1929,7 +1928,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -1964,7 +1963,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -1999,7 +1998,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>128</v>
       </c>
@@ -2034,7 +2033,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>129</v>
       </c>
@@ -2069,7 +2068,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>124</v>
       </c>
@@ -2104,7 +2103,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>125</v>
       </c>
@@ -2139,7 +2138,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>126</v>
       </c>
@@ -2174,7 +2173,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>127</v>
       </c>
@@ -2209,7 +2208,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>114</v>
       </c>
@@ -2244,7 +2243,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>115</v>
       </c>
@@ -2279,7 +2278,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>92</v>
       </c>
@@ -2314,7 +2313,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>93</v>
       </c>
@@ -2349,7 +2348,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>94</v>
       </c>
@@ -2384,7 +2383,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>95</v>
       </c>
@@ -2419,7 +2418,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>96</v>
       </c>
@@ -2454,7 +2453,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>97</v>
       </c>
@@ -2489,7 +2488,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>98</v>
       </c>
@@ -2524,7 +2523,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>99</v>
       </c>
@@ -2559,7 +2558,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>101</v>
       </c>
@@ -2594,7 +2593,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>156</v>
       </c>
@@ -2629,7 +2628,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>155</v>
       </c>
@@ -2664,7 +2663,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>154</v>
       </c>
@@ -2699,7 +2698,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>33</v>
       </c>
@@ -2734,7 +2733,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>6</v>
       </c>
@@ -2769,7 +2768,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>7</v>
       </c>
@@ -2804,7 +2803,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -2839,7 +2838,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>9</v>
       </c>
@@ -2874,7 +2873,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>10</v>
       </c>
@@ -2909,7 +2908,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>80</v>
       </c>
@@ -2944,7 +2943,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>28</v>
       </c>
@@ -2973,7 +2972,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>36</v>
       </c>
@@ -3008,7 +3007,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>44</v>
       </c>
@@ -3043,7 +3042,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>53</v>
       </c>
@@ -3072,7 +3071,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>48</v>
       </c>
@@ -3107,7 +3106,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>49</v>
       </c>
@@ -3142,7 +3141,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>50</v>
       </c>
@@ -3171,7 +3170,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>29</v>
       </c>
@@ -3206,7 +3205,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>30</v>
       </c>
@@ -3241,7 +3240,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>118</v>
       </c>
@@ -3276,7 +3275,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>119</v>
       </c>
@@ -3311,7 +3310,7 @@
         <v>196</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>120</v>
       </c>
@@ -3346,7 +3345,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>121</v>
       </c>
@@ -3381,7 +3380,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>122</v>
       </c>
@@ -3416,7 +3415,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>123</v>
       </c>
@@ -3451,7 +3450,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>117</v>
       </c>
@@ -3486,7 +3485,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>130</v>
       </c>
@@ -3521,7 +3520,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>131</v>
       </c>
@@ -3556,7 +3555,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>132</v>
       </c>
@@ -3591,7 +3590,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>133</v>
       </c>
@@ -3626,7 +3625,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>134</v>
       </c>
@@ -3661,7 +3660,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>135</v>
       </c>
@@ -3696,7 +3695,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>136</v>
       </c>
@@ -3731,7 +3730,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>137</v>
       </c>
@@ -3766,7 +3765,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>138</v>
       </c>
@@ -3801,7 +3800,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>139</v>
       </c>
@@ -3836,7 +3835,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>140</v>
       </c>
@@ -3871,7 +3870,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>82</v>
       </c>
@@ -3906,7 +3905,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>149</v>
       </c>
@@ -3941,7 +3940,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>83</v>
       </c>
@@ -3976,7 +3975,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>84</v>
       </c>
@@ -4011,7 +4010,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>87</v>
       </c>
@@ -4046,7 +4045,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>86</v>
       </c>
@@ -4081,7 +4080,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>88</v>
       </c>
@@ -4116,7 +4115,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>171</v>
       </c>
@@ -4151,7 +4150,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>153</v>
       </c>
@@ -4186,7 +4185,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>159</v>
       </c>
@@ -4221,7 +4220,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>158</v>
       </c>
@@ -4256,7 +4255,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>160</v>
       </c>
@@ -4291,7 +4290,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>21</v>
       </c>
@@ -4326,7 +4325,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>19</v>
       </c>
@@ -4361,7 +4360,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>13</v>
       </c>
@@ -4389,10 +4388,8 @@
       <c r="I81" t="b">
         <v>1</v>
       </c>
-      <c r="J81" s="1"/>
-      <c r="K81" s="1"/>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>18</v>
       </c>
@@ -4427,7 +4424,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>24</v>
       </c>
@@ -4462,7 +4459,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>64</v>
       </c>

</xml_diff>

<commit_message>
Metrics report integrated into pipeline
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cameron Fraser\LTG Dropbox\Cameron Fraser\RwoD Research\Team A\Experiments\Small somatic mutations\CODECseq\20250507 Component level metrics\Archive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D6160E8-4676-47D9-BB20-5C8A4A086C83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65479668-8895-4392-9CCA-4A4ABA70422F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
-    <sheet name="component_metrics" sheetId="1" r:id="rId1"/>
+    <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">component_metrics!$A$1:$K$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$82</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>

<commit_message>
Fixed regexes for metrics report
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Cameron Fraser\LTG Dropbox\Cameron Fraser\RwoD Research\Team A\Experiments\Small somatic mutations\CODECseq\20250507 Component level metrics\Archive\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65479668-8895-4392-9CCA-4A4ABA70422F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1408767-860D-45CF-8725-A86A6022184B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -530,24 +530,12 @@
     <t>Percentage of raw reads filtered by length threshold</t>
   </si>
   <si>
-    <t>r"^\d+ \+ \d+ mapped \(([\d.]+)%\s*:"</t>
-  </si>
-  <si>
-    <t>r"^S\d+_lib\s+\S+\s+\S+\s+\S+\s+\S+\s+\S+\s+\S+\s+([\d.]+)"</t>
-  </si>
-  <si>
     <t>Fraction of mapped reads that are marked as duplicates</t>
   </si>
   <si>
     <t>r"^S\d+_combined_mask\.bed\t\d+\t([\d.]+)%"</t>
   </si>
   <si>
-    <t>r"Pairs written \(passing filters\):\s+[\d,]+ \(([\d\.]+)%\)"</t>
-  </si>
-  <si>
-    <t>r"^\d+ \+ \d+ properly paired \(([\d\.]+)%"</t>
-  </si>
-  <si>
     <t>Percentage of reads lost from creation of DSC (beyond expected halving)</t>
   </si>
   <si>
@@ -557,9 +545,6 @@
     <t>r"^S\d+\t\d+\t\d+\t([0-9.]+)$"</t>
   </si>
   <si>
-    <t>r'"percent_reads_lost"\s*:\s*([0-9.]+)'</t>
-  </si>
-  <si>
     <t>file_pattern</t>
   </si>
   <si>
@@ -680,12 +665,6 @@
     <t>_demux_metrics_gini.json</t>
   </si>
   <si>
-    <t>r"^Pairs that were too short:.*\(([\d.]+)%\)"</t>
-  </si>
-  <si>
-    <t>r"^([0-9]+)\t"</t>
-  </si>
-  <si>
     <t>reads_filtered_length</t>
   </si>
   <si>
@@ -720,6 +699,27 @@
   </si>
   <si>
     <t>Percentage of genome with 1. MS depth &gt; half MS depth theshold and 2. EX duplex depth &gt; 0</t>
+  </si>
+  <si>
+    <t>^Pairs that were too short:\s+\d+\s+\((?P&lt;percent&gt;[\d.]+)%\)$</t>
+  </si>
+  <si>
+    <t>^\d+ \+ 0 mapped \((?P&lt;percent&gt;[\d.]+)% : N/A\)$</t>
+  </si>
+  <si>
+    <t>^(\S+\t){8}(?P&lt;value&gt;[\d.]+)</t>
+  </si>
+  <si>
+    <t>^(?P&lt;value&gt;\d+)\b</t>
+  </si>
+  <si>
+    <t>^Pairs discarded as untrimmed:\s+(?P&lt;value&gt;\d+)\s+\([\d.]+%\)$</t>
+  </si>
+  <si>
+    <t>^\d+ \+ 0 properly paired \((?P&lt;percent&gt;[\d.]+)% : N/A\)$</t>
+  </si>
+  <si>
+    <t>percent_reads_lost</t>
   </si>
 </sst>
 </file>
@@ -1599,7 +1599,7 @@
     <col min="8" max="8" width="9" customWidth="1"/>
     <col min="9" max="9" width="12.81640625" customWidth="1"/>
     <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="54" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="58.7265625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
@@ -1631,10 +1631,10 @@
         <v>40</v>
       </c>
       <c r="J1" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="K1" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
@@ -1957,10 +1957,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="K11" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
@@ -1992,10 +1992,10 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="K12" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
@@ -2027,10 +2027,10 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="K13" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
@@ -2062,10 +2062,10 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="K14" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
@@ -2097,10 +2097,10 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="K15" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
@@ -2132,10 +2132,10 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="K16" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
@@ -2167,10 +2167,10 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="K17" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
@@ -2202,10 +2202,10 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="K18" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
@@ -2237,10 +2237,10 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="K19" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">
@@ -2272,10 +2272,10 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="K20" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
@@ -2307,10 +2307,10 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="K21" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.35">
@@ -2342,10 +2342,10 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="K22" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.35">
@@ -2377,10 +2377,10 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="K23" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
@@ -2412,10 +2412,10 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="K24" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
@@ -2447,10 +2447,10 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="K25" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
@@ -2482,10 +2482,10 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="K26" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
@@ -2517,10 +2517,10 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
       <c r="K27" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.35">
@@ -2552,10 +2552,10 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="K28" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.35">
@@ -2587,10 +2587,10 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="K29" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
@@ -2622,10 +2622,10 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="K30" t="s">
-        <v>164</v>
+        <v>222</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.35">
@@ -2633,7 +2633,7 @@
         <v>155</v>
       </c>
       <c r="B31" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C31" t="s">
         <v>74</v>
@@ -2657,10 +2657,10 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="K31" t="s">
-        <v>165</v>
+        <v>223</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
@@ -2692,10 +2692,10 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="K32" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
@@ -2727,10 +2727,10 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="K33" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.35">
@@ -2762,10 +2762,10 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="K34" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.35">
@@ -2797,10 +2797,10 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="K35" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.35">
@@ -2832,10 +2832,10 @@
         <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="K36" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.35">
@@ -2867,10 +2867,10 @@
         <v>1</v>
       </c>
       <c r="J37" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="K37" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.35">
@@ -2902,10 +2902,10 @@
         <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="K38" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.35">
@@ -2937,10 +2937,10 @@
         <v>1</v>
       </c>
       <c r="J39" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="K39" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.35">
@@ -3269,10 +3269,10 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="K49" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.35">
@@ -3304,10 +3304,10 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="K50" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.35">
@@ -3339,10 +3339,10 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="K51" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.35">
@@ -3374,10 +3374,10 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="K52" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.35">
@@ -3409,10 +3409,10 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="K53" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.35">
@@ -3444,10 +3444,10 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="K54" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.35">
@@ -3479,10 +3479,10 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="K55" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.35">
@@ -3514,10 +3514,10 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="K56" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.35">
@@ -3549,10 +3549,10 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="K57" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.35">
@@ -3584,10 +3584,10 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
+        <v>185</v>
+      </c>
+      <c r="K58" t="s">
         <v>190</v>
-      </c>
-      <c r="K58" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.35">
@@ -3619,10 +3619,10 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="K59" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.35">
@@ -3654,10 +3654,10 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="K60" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.35">
@@ -3689,10 +3689,10 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="K61" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.35">
@@ -3724,10 +3724,10 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="K62" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.35">
@@ -3759,10 +3759,10 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="K63" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.35">
@@ -3794,10 +3794,10 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="K64" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.35">
@@ -3829,10 +3829,10 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="K65" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.35">
@@ -3864,10 +3864,10 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="K66" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.35">
@@ -3899,10 +3899,10 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="K67" t="s">
-        <v>168</v>
+        <v>225</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.35">
@@ -3934,10 +3934,10 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="K68" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.35">
@@ -3969,10 +3969,10 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="K69" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.35">
@@ -4004,10 +4004,10 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="K70" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.35">
@@ -4039,10 +4039,10 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="K71" t="s">
-        <v>164</v>
+        <v>222</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.35">
@@ -4074,10 +4074,10 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="K72" t="s">
-        <v>169</v>
+        <v>226</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.35">
@@ -4109,18 +4109,18 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="K73" t="s">
-        <v>215</v>
+        <v>224</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B74" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="C74" t="s">
         <v>75</v>
@@ -4144,10 +4144,10 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>219</v>
+        <v>212</v>
       </c>
       <c r="K74" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.35">
@@ -4179,10 +4179,10 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
       <c r="K75" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.35">
@@ -4214,10 +4214,10 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="K76" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.35">
@@ -4249,10 +4249,10 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>223</v>
+        <v>216</v>
       </c>
       <c r="K77" t="s">
-        <v>222</v>
+        <v>215</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.35">
@@ -4284,10 +4284,10 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="K78" t="s">
-        <v>224</v>
+        <v>217</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.35">
@@ -4319,10 +4319,10 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
       <c r="K79" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.35">
@@ -4354,7 +4354,7 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="K80" t="s">
         <v>19</v>
@@ -4418,10 +4418,10 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="K82" t="s">
-        <v>225</v>
+        <v>218</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.35">
@@ -4453,10 +4453,10 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="K83" t="s">
-        <v>173</v>
+        <v>227</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.35">
@@ -4464,7 +4464,7 @@
         <v>64</v>
       </c>
       <c r="B84" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="C84" t="s">
         <v>79</v>
@@ -4488,7 +4488,7 @@
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="K84" t="s">
         <v>64</v>

</xml_diff>

<commit_message>
Updated file names and patterns for refactored metrics script files
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1408767-860D-45CF-8725-A86A6022184B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3797D472-92A5-48D4-BCED-2AAA9CA3A574}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -524,27 +524,18 @@
     <t>Mean duplex depth of final DSC passed to variant calling</t>
   </si>
   <si>
-    <t>Percentage of reads that are unique</t>
-  </si>
-  <si>
     <t>Percentage of raw reads filtered by length threshold</t>
   </si>
   <si>
     <t>Fraction of mapped reads that are marked as duplicates</t>
   </si>
   <si>
-    <t>r"^S\d+_combined_mask\.bed\t\d+\t([\d.]+)%"</t>
-  </si>
-  <si>
     <t>Percentage of reads lost from creation of DSC (beyond expected halving)</t>
   </si>
   <si>
     <t>ex_reads_lost_call_dsc</t>
   </si>
   <si>
-    <t>r"^S\d+\t\d+\t\d+\t([0-9.]+)$"</t>
-  </si>
-  <si>
     <t>file_pattern</t>
   </si>
   <si>
@@ -557,9 +548,6 @@
     <t>_insert_metrics.txt</t>
   </si>
   <si>
-    <t>_duplication_metrics.txt</t>
-  </si>
-  <si>
     <t>_softclipping_metrics.json</t>
   </si>
   <si>
@@ -587,9 +575,6 @@
     <t>_insert_size_metrics.txt</t>
   </si>
   <si>
-    <t>_mask_metrics.txt</t>
-  </si>
-  <si>
     <t>_r1_fastqc_raw_metrics_summary.json</t>
   </si>
   <si>
@@ -695,9 +680,6 @@
     <t>ex_dsc_coverage_wholegenome</t>
   </si>
   <si>
-    <t>dsc_coverage_metrics.json</t>
-  </si>
-  <si>
     <t>Percentage of genome with 1. MS depth &gt; half MS depth theshold and 2. EX duplex depth &gt; 0</t>
   </si>
   <si>
@@ -720,6 +702,24 @@
   </si>
   <si>
     <t>percent_reads_lost</t>
+  </si>
+  <si>
+    <t>_mask_metrics.json</t>
+  </si>
+  <si>
+    <t>mask_files.combined_mask.percentage_of_ref_genome</t>
+  </si>
+  <si>
+    <t>pct_unique_reads</t>
+  </si>
+  <si>
+    <t>_duplication_metrics.json</t>
+  </si>
+  <si>
+    <t>_dsc_coverage_metrics.json</t>
+  </si>
+  <si>
+    <t>Percentage of reads that are unique following initial alignment</t>
   </si>
 </sst>
 </file>
@@ -1590,19 +1590,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
   <dimension ref="A1:K84"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.1796875" customWidth="1"/>
-    <col min="2" max="2" width="82.1796875" customWidth="1"/>
-    <col min="3" max="4" width="35.26953125" customWidth="1"/>
+    <col min="1" max="1" width="35.140625" customWidth="1"/>
+    <col min="2" max="2" width="82.140625" customWidth="1"/>
+    <col min="3" max="4" width="35.28515625" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.81640625" customWidth="1"/>
-    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="58.7265625" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="58.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>41</v>
       </c>
@@ -1631,13 +1631,13 @@
         <v>40</v>
       </c>
       <c r="J1" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="K1" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>45</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>46</v>
       </c>
@@ -1701,7 +1701,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>47</v>
       </c>
@@ -1730,7 +1730,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>59</v>
       </c>
@@ -1759,7 +1759,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>58</v>
       </c>
@@ -1794,7 +1794,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>60</v>
       </c>
@@ -1823,7 +1823,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>61</v>
       </c>
@@ -1858,7 +1858,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>31</v>
       </c>
@@ -1893,7 +1893,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>32</v>
       </c>
@@ -1928,7 +1928,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -1957,13 +1957,13 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="K11" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -1992,13 +1992,13 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="K12" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>128</v>
       </c>
@@ -2027,13 +2027,13 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="K13" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>129</v>
       </c>
@@ -2062,13 +2062,13 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="K14" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>124</v>
       </c>
@@ -2097,13 +2097,13 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="K15" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>125</v>
       </c>
@@ -2132,13 +2132,13 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="K16" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>126</v>
       </c>
@@ -2167,13 +2167,13 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="K17" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>127</v>
       </c>
@@ -2202,13 +2202,13 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="K18" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>114</v>
       </c>
@@ -2237,13 +2237,13 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="K19" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>115</v>
       </c>
@@ -2272,13 +2272,13 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="K20" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>92</v>
       </c>
@@ -2307,13 +2307,13 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="K21" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>93</v>
       </c>
@@ -2342,13 +2342,13 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="K22" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>94</v>
       </c>
@@ -2377,13 +2377,13 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="K23" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>95</v>
       </c>
@@ -2412,13 +2412,13 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="K24" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>96</v>
       </c>
@@ -2447,13 +2447,13 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="K25" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>97</v>
       </c>
@@ -2482,13 +2482,13 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="K26" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>98</v>
       </c>
@@ -2517,13 +2517,13 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="K27" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>99</v>
       </c>
@@ -2552,18 +2552,18 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="K28" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>101</v>
       </c>
       <c r="B29" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C29" t="s">
         <v>73</v>
@@ -2587,13 +2587,13 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="K29" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>156</v>
       </c>
@@ -2622,18 +2622,18 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="K30" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>155</v>
       </c>
       <c r="B31" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C31" t="s">
         <v>74</v>
@@ -2657,13 +2657,13 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="K31" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>154</v>
       </c>
@@ -2692,13 +2692,13 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="K32" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>33</v>
       </c>
@@ -2727,13 +2727,13 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="K33" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>6</v>
       </c>
@@ -2762,13 +2762,13 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="K34" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>7</v>
       </c>
@@ -2797,13 +2797,13 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="K35" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -2832,13 +2832,13 @@
         <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="K36" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>9</v>
       </c>
@@ -2867,13 +2867,13 @@
         <v>1</v>
       </c>
       <c r="J37" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="K37" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>10</v>
       </c>
@@ -2902,13 +2902,13 @@
         <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="K38" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>80</v>
       </c>
@@ -2937,13 +2937,13 @@
         <v>1</v>
       </c>
       <c r="J39" t="s">
-        <v>183</v>
+        <v>222</v>
       </c>
       <c r="K39" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>28</v>
       </c>
@@ -2972,7 +2972,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>36</v>
       </c>
@@ -3007,7 +3007,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>44</v>
       </c>
@@ -3042,7 +3042,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>53</v>
       </c>
@@ -3071,7 +3071,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>48</v>
       </c>
@@ -3106,7 +3106,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>49</v>
       </c>
@@ -3141,7 +3141,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>50</v>
       </c>
@@ -3170,7 +3170,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>29</v>
       </c>
@@ -3205,7 +3205,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>30</v>
       </c>
@@ -3240,7 +3240,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>118</v>
       </c>
@@ -3269,13 +3269,13 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="K49" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>119</v>
       </c>
@@ -3304,13 +3304,13 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="K50" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>120</v>
       </c>
@@ -3339,13 +3339,13 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="K51" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>121</v>
       </c>
@@ -3374,13 +3374,13 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="K52" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>122</v>
       </c>
@@ -3409,13 +3409,13 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="K53" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>123</v>
       </c>
@@ -3444,13 +3444,13 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="K54" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>117</v>
       </c>
@@ -3479,13 +3479,13 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="K55" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>130</v>
       </c>
@@ -3514,13 +3514,13 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="K56" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>131</v>
       </c>
@@ -3549,13 +3549,13 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
       <c r="K57" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>132</v>
       </c>
@@ -3584,13 +3584,13 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
+        <v>180</v>
+      </c>
+      <c r="K58" t="s">
         <v>185</v>
       </c>
-      <c r="K58" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>133</v>
       </c>
@@ -3619,13 +3619,13 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="K59" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>134</v>
       </c>
@@ -3654,13 +3654,13 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="K60" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>135</v>
       </c>
@@ -3689,13 +3689,13 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="K61" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>136</v>
       </c>
@@ -3724,13 +3724,13 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="K62" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>137</v>
       </c>
@@ -3759,13 +3759,13 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="K63" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>138</v>
       </c>
@@ -3794,13 +3794,13 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="K64" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>139</v>
       </c>
@@ -3829,13 +3829,13 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
       <c r="K65" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>140</v>
       </c>
@@ -3864,13 +3864,13 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="K66" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>82</v>
       </c>
@@ -3899,13 +3899,13 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
       <c r="K67" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>149</v>
       </c>
@@ -3934,13 +3934,13 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="K68" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>83</v>
       </c>
@@ -3969,13 +3969,13 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="K69" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>84</v>
       </c>
@@ -4004,13 +4004,13 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="K70" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>87</v>
       </c>
@@ -4039,13 +4039,13 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="K71" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>86</v>
       </c>
@@ -4074,13 +4074,13 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="K72" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>88</v>
       </c>
@@ -4109,18 +4109,18 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="K73" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B74" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C74" t="s">
         <v>75</v>
@@ -4144,18 +4144,18 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="K74" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>153</v>
       </c>
       <c r="B75" t="s">
-        <v>162</v>
+        <v>227</v>
       </c>
       <c r="C75" t="s">
         <v>75</v>
@@ -4179,13 +4179,13 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>173</v>
+        <v>225</v>
       </c>
       <c r="K75" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>159</v>
       </c>
@@ -4214,13 +4214,13 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="K76" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>158</v>
       </c>
@@ -4249,13 +4249,13 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="K77" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>160</v>
       </c>
@@ -4284,13 +4284,13 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="K78" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>21</v>
       </c>
@@ -4319,13 +4319,13 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="K79" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>19</v>
       </c>
@@ -4354,13 +4354,13 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="K80" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>13</v>
       </c>
@@ -4389,7 +4389,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>18</v>
       </c>
@@ -4418,13 +4418,13 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="K82" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>24</v>
       </c>
@@ -4453,18 +4453,18 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
       <c r="K83" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>64</v>
       </c>
       <c r="B84" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="C84" t="s">
         <v>79</v>
@@ -4488,7 +4488,7 @@
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="K84" t="s">
         <v>64</v>

</xml_diff>

<commit_message>
Added test to test that regexes used to get metrics are correct
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAFF3DBA-4AB2-44CF-913D-4685D7CD0B13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A2AFF04-293E-4DCF-8D4A-F141DB3AD0F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -686,15 +686,9 @@
     <t>^\d+ \+ 0 mapped \((?P&lt;percent&gt;[\d.]+)% : N/A\)$</t>
   </si>
   <si>
-    <t>^(\S+\t){8}(?P&lt;value&gt;[\d.]+)</t>
-  </si>
-  <si>
     <t>^(?P&lt;value&gt;\d+)\b</t>
   </si>
   <si>
-    <t>^Pairs discarded as untrimmed:\s+(?P&lt;value&gt;\d+)\s+\([\d.]+%\)$</t>
-  </si>
-  <si>
     <t>^\d+ \+ 0 properly paired \((?P&lt;percent&gt;[\d.]+)% : N/A\)$</t>
   </si>
   <si>
@@ -720,6 +714,12 @@
   </si>
   <si>
     <t>_filtered_fq_metrics.txt</t>
+  </si>
+  <si>
+    <t>^(\S+\t){9}(?P&lt;value&gt;[\d.]+)</t>
+  </si>
+  <si>
+    <t>^Pairs discarded as untrimmed:\s+\d+\s+\((?P&lt;value&gt;[\d.]+)%\)</t>
   </si>
 </sst>
 </file>
@@ -2587,7 +2587,7 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="K29" t="s">
         <v>214</v>
@@ -2660,7 +2660,7 @@
         <v>176</v>
       </c>
       <c r="K31" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
@@ -2695,7 +2695,7 @@
         <v>177</v>
       </c>
       <c r="K32" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
@@ -2937,10 +2937,10 @@
         <v>1</v>
       </c>
       <c r="J39" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="K39" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.35">
@@ -3884,16 +3884,16 @@
         <v>85</v>
       </c>
       <c r="E67">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="F67">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="G67">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="H67">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="I67" t="b">
         <v>1</v>
@@ -3902,7 +3902,7 @@
         <v>182</v>
       </c>
       <c r="K67" t="s">
-        <v>218</v>
+        <v>227</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.35">
@@ -4077,7 +4077,7 @@
         <v>168</v>
       </c>
       <c r="K72" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.35">
@@ -4094,16 +4094,16 @@
         <v>34</v>
       </c>
       <c r="E73">
-        <v>50</v>
+        <v>125</v>
       </c>
       <c r="F73">
-        <v>300</v>
+        <v>175</v>
       </c>
       <c r="G73">
-        <v>100</v>
+        <v>140</v>
       </c>
       <c r="H73">
-        <v>200</v>
+        <v>160</v>
       </c>
       <c r="I73" t="b">
         <v>1</v>
@@ -4112,7 +4112,7 @@
         <v>169</v>
       </c>
       <c r="K73" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.35">
@@ -4155,7 +4155,7 @@
         <v>153</v>
       </c>
       <c r="B75" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C75" t="s">
         <v>75</v>
@@ -4179,10 +4179,10 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="K75" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.35">
@@ -4284,7 +4284,7 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="K78" t="s">
         <v>211</v>
@@ -4354,7 +4354,7 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="K80" t="s">
         <v>19</v>
@@ -4418,7 +4418,7 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="K82" t="s">
         <v>212</v>
@@ -4456,7 +4456,7 @@
         <v>183</v>
       </c>
       <c r="K83" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.35">
@@ -4488,7 +4488,7 @@
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="K84" t="s">
         <v>64</v>

</xml_diff>

<commit_message>
1. Added tests for metrics report 2. Fixed errors in metrics spreadshseets found by tests
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A2AFF04-293E-4DCF-8D4A-F141DB3AD0F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C119EBD-7D38-40CA-BC31-F4B4E1C7AE68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -4386,7 +4386,7 @@
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="I81" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Updated component and system metrics. Improved consistency of stage variable
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{24710D4D-D1A1-45A5-B30F-FF52FAE45155}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0414BF8-3B8C-4ED6-916B-B08A196C6C66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -260,9 +260,6 @@
     <t>Mask regions</t>
   </si>
   <si>
-    <t>EX Call somatic variants</t>
-  </si>
-  <si>
     <t>NA</t>
   </si>
   <si>
@@ -720,6 +717,9 @@
   </si>
   <si>
     <t>Distinct band at aprox 290 and sometimes 480 bp, with no smears. 1 = pass 0 = fail.</t>
+  </si>
+  <si>
+    <t>EX call somatic variants</t>
   </si>
 </sst>
 </file>
@@ -1631,10 +1631,10 @@
         <v>39</v>
       </c>
       <c r="J1" t="s">
+        <v>161</v>
+      </c>
+      <c r="K1" t="s">
         <v>162</v>
-      </c>
-      <c r="K1" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
@@ -1660,10 +1660,10 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
@@ -1695,10 +1695,10 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
@@ -1706,7 +1706,7 @@
         <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C4" t="s">
         <v>61</v>
@@ -1730,10 +1730,10 @@
         <v>0</v>
       </c>
       <c r="J4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
@@ -1759,10 +1759,10 @@
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
@@ -1794,10 +1794,10 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
@@ -1823,10 +1823,10 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K7" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
@@ -1858,10 +1858,10 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
@@ -1869,7 +1869,7 @@
         <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C9" t="s">
         <v>63</v>
@@ -1893,10 +1893,10 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
@@ -1904,7 +1904,7 @@
         <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C10" t="s">
         <v>63</v>
@@ -1928,10 +1928,10 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
@@ -1939,7 +1939,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C11" t="s">
         <v>67</v>
@@ -1963,10 +1963,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K11" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
@@ -1974,7 +1974,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C12" t="s">
         <v>67</v>
@@ -1998,18 +1998,18 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K12" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B13" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C13" t="s">
         <v>64</v>
@@ -2033,18 +2033,18 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K13" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B14" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C14" t="s">
         <v>64</v>
@@ -2068,18 +2068,18 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K14" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B15" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C15" t="s">
         <v>67</v>
@@ -2103,18 +2103,18 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K15" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B16" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C16" t="s">
         <v>67</v>
@@ -2138,18 +2138,18 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K16" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B17" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C17" t="s">
         <v>67</v>
@@ -2173,18 +2173,18 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K17" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B18" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C18" t="s">
         <v>67</v>
@@ -2208,18 +2208,18 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K18" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B19" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C19" t="s">
         <v>64</v>
@@ -2243,18 +2243,18 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K19" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
+        <v>110</v>
+      </c>
+      <c r="B20" t="s">
         <v>111</v>
-      </c>
-      <c r="B20" t="s">
-        <v>112</v>
       </c>
       <c r="C20" t="s">
         <v>64</v>
@@ -2278,18 +2278,18 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K20" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B21" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C21" t="s">
         <v>64</v>
@@ -2313,18 +2313,18 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K21" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B22" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C22" t="s">
         <v>64</v>
@@ -2348,18 +2348,18 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="K22" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B23" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C23" t="s">
         <v>64</v>
@@ -2383,18 +2383,18 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K23" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B24" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C24" t="s">
         <v>64</v>
@@ -2418,18 +2418,18 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="K24" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B25" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C25" t="s">
         <v>64</v>
@@ -2453,18 +2453,18 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K25" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B26" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C26" t="s">
         <v>64</v>
@@ -2488,18 +2488,18 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="K26" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B27" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C27" t="s">
         <v>64</v>
@@ -2523,18 +2523,18 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K27" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B28" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C28" t="s">
         <v>64</v>
@@ -2558,18 +2558,18 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="K28" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B29" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C29" t="s">
         <v>69</v>
@@ -2593,18 +2593,18 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="K29" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B30" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C30" t="s">
         <v>70</v>
@@ -2628,18 +2628,18 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="K30" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B31" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C31" t="s">
         <v>70</v>
@@ -2663,18 +2663,18 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K31" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B32" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C32" t="s">
         <v>70</v>
@@ -2698,10 +2698,10 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="K32" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
@@ -2709,7 +2709,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C33" t="s">
         <v>72</v>
@@ -2733,10 +2733,10 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="K33" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.35">
@@ -2744,7 +2744,7 @@
         <v>6</v>
       </c>
       <c r="B34" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C34" t="s">
         <v>72</v>
@@ -2768,10 +2768,10 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="K34" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.35">
@@ -2779,7 +2779,7 @@
         <v>7</v>
       </c>
       <c r="B35" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C35" t="s">
         <v>72</v>
@@ -2803,10 +2803,10 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="K35" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.35">
@@ -2814,7 +2814,7 @@
         <v>8</v>
       </c>
       <c r="B36" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C36" t="s">
         <v>72</v>
@@ -2838,10 +2838,10 @@
         <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="K36" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.35">
@@ -2849,7 +2849,7 @@
         <v>9</v>
       </c>
       <c r="B37" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C37" t="s">
         <v>72</v>
@@ -2873,10 +2873,10 @@
         <v>1</v>
       </c>
       <c r="J37" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="K37" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.35">
@@ -2884,7 +2884,7 @@
         <v>10</v>
       </c>
       <c r="B38" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C38" t="s">
         <v>72</v>
@@ -2908,15 +2908,15 @@
         <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="K38" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B39" t="s">
         <v>4</v>
@@ -2943,10 +2943,10 @@
         <v>1</v>
       </c>
       <c r="J39" t="s">
+        <v>214</v>
+      </c>
+      <c r="K39" t="s">
         <v>215</v>
-      </c>
-      <c r="K39" t="s">
-        <v>216</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.35">
@@ -2972,10 +2972,10 @@
         <v>0</v>
       </c>
       <c r="J40" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K40" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.35">
@@ -3007,10 +3007,10 @@
         <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K41" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.35">
@@ -3018,7 +3018,7 @@
         <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C42" t="s">
         <v>62</v>
@@ -3042,10 +3042,10 @@
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K42" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.35">
@@ -3071,10 +3071,10 @@
         <v>0</v>
       </c>
       <c r="J43" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K43" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.35">
@@ -3106,10 +3106,10 @@
         <v>0</v>
       </c>
       <c r="J44" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K44" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.35">
@@ -3117,7 +3117,7 @@
         <v>48</v>
       </c>
       <c r="B45" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C45" t="s">
         <v>62</v>
@@ -3141,10 +3141,10 @@
         <v>0</v>
       </c>
       <c r="J45" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K45" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.35">
@@ -3152,7 +3152,7 @@
         <v>49</v>
       </c>
       <c r="B46" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C46" t="s">
         <v>62</v>
@@ -3176,10 +3176,10 @@
         <v>0</v>
       </c>
       <c r="J46" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K46" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.35">
@@ -3211,10 +3211,10 @@
         <v>0</v>
       </c>
       <c r="J47" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K47" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.35">
@@ -3246,24 +3246,24 @@
         <v>0</v>
       </c>
       <c r="J48" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="K48" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B49" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C49" t="s">
         <v>66</v>
       </c>
       <c r="D49" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E49">
         <v>35</v>
@@ -3281,24 +3281,24 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K49" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B50" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C50" t="s">
         <v>66</v>
       </c>
       <c r="D50" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E50">
         <v>35</v>
@@ -3316,24 +3316,24 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="K50" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B51" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C51" t="s">
         <v>66</v>
       </c>
       <c r="D51" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E51">
         <v>30</v>
@@ -3351,24 +3351,24 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K51" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B52" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C52" t="s">
         <v>66</v>
       </c>
       <c r="D52" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E52">
         <v>30</v>
@@ -3386,15 +3386,15 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="K52" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B53" t="s">
         <v>15</v>
@@ -3403,7 +3403,7 @@
         <v>66</v>
       </c>
       <c r="D53" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E53">
         <v>0</v>
@@ -3421,15 +3421,15 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K53" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B54" t="s">
         <v>15</v>
@@ -3438,7 +3438,7 @@
         <v>66</v>
       </c>
       <c r="D54" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E54">
         <v>0</v>
@@ -3456,24 +3456,24 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="K54" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B55" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C55" t="s">
         <v>66</v>
       </c>
       <c r="D55" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E55">
         <v>150</v>
@@ -3491,24 +3491,24 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K55" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B56" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C56" t="s">
         <v>66</v>
       </c>
       <c r="D56" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E56">
         <v>150</v>
@@ -3526,24 +3526,24 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="K56" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B57" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C57" t="s">
         <v>66</v>
       </c>
       <c r="D57" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E57">
         <v>2850</v>
@@ -3561,24 +3561,24 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="K57" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B58" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C58" t="s">
         <v>66</v>
       </c>
       <c r="D58" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E58">
         <v>2850</v>
@@ -3596,18 +3596,18 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="K58" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B59" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C59" t="s">
         <v>66</v>
@@ -3631,18 +3631,18 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="K59" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B60" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C60" t="s">
         <v>66</v>
@@ -3666,18 +3666,18 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K60" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B61" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C61" t="s">
         <v>66</v>
@@ -3701,18 +3701,18 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="K61" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B62" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C62" t="s">
         <v>66</v>
@@ -3736,18 +3736,18 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K62" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B63" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C63" t="s">
         <v>66</v>
@@ -3771,18 +3771,18 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="K63" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B64" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C64" t="s">
         <v>66</v>
@@ -3806,18 +3806,18 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K64" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B65" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C65" t="s">
         <v>66</v>
@@ -3841,18 +3841,18 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="K65" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="B66" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C66" t="s">
         <v>66</v>
@@ -3876,24 +3876,24 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K66" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B67" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C67" t="s">
         <v>68</v>
       </c>
       <c r="D67" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E67">
         <v>0</v>
@@ -3911,24 +3911,24 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="K67" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
+        <v>144</v>
+      </c>
+      <c r="B68" t="s">
         <v>145</v>
-      </c>
-      <c r="B68" t="s">
-        <v>146</v>
       </c>
       <c r="C68" t="s">
         <v>68</v>
       </c>
       <c r="D68" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E68">
         <v>0</v>
@@ -3946,18 +3946,18 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K68" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B69" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C69" t="s">
         <v>68</v>
@@ -3981,18 +3981,18 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="K69" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B70" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C70" t="s">
         <v>68</v>
@@ -4016,18 +4016,18 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="K70" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B71" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C71" t="s">
         <v>65</v>
@@ -4051,18 +4051,18 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K71" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B72" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C72" t="s">
         <v>65</v>
@@ -4086,18 +4086,18 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K72" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B73" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C73" t="s">
         <v>65</v>
@@ -4121,18 +4121,18 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K73" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B74" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C74" t="s">
         <v>71</v>
@@ -4156,18 +4156,18 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
+        <v>201</v>
+      </c>
+      <c r="K74" t="s">
         <v>202</v>
-      </c>
-      <c r="K74" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B75" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C75" t="s">
         <v>71</v>
@@ -4191,15 +4191,15 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="K75" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B76" t="s">
         <v>16</v>
@@ -4226,18 +4226,18 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="K76" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B77" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C77" t="s">
         <v>71</v>
@@ -4261,18 +4261,18 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="K77" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
+        <v>155</v>
+      </c>
+      <c r="B78" t="s">
         <v>156</v>
-      </c>
-      <c r="B78" t="s">
-        <v>157</v>
       </c>
       <c r="C78" t="s">
         <v>71</v>
@@ -4296,10 +4296,10 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="K78" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.35">
@@ -4331,10 +4331,10 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="K79" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.35">
@@ -4366,7 +4366,7 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="K80" t="s">
         <v>19</v>
@@ -4409,7 +4409,7 @@
         <v>17</v>
       </c>
       <c r="C82" t="s">
-        <v>74</v>
+        <v>227</v>
       </c>
       <c r="D82" t="s">
         <v>33</v>
@@ -4430,10 +4430,10 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="K82" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.35">
@@ -4444,10 +4444,10 @@
         <v>23</v>
       </c>
       <c r="C83" t="s">
-        <v>75</v>
+        <v>227</v>
       </c>
       <c r="D83" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E83">
         <v>0</v>
@@ -4465,10 +4465,10 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="K83" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.35">
@@ -4476,10 +4476,10 @@
         <v>60</v>
       </c>
       <c r="B84" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C84" t="s">
-        <v>75</v>
+        <v>227</v>
       </c>
       <c r="D84" t="s">
         <v>33</v>
@@ -4500,7 +4500,7 @@
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="K84" t="s">
         <v>60</v>

</xml_diff>

<commit_message>
Updated component level metrics
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0414BF8-3B8C-4ED6-916B-B08A196C6C66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5B4BAE2-AD2C-4FFE-8012-EBF3FBA2C751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$83</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="230">
   <si>
     <t>nn_lower</t>
   </si>
@@ -720,6 +720,12 @@
   </si>
   <si>
     <t>EX call somatic variants</t>
+  </si>
+  <si>
+    <t>ex_bases_trimmed</t>
+  </si>
+  <si>
+    <t>Percentage of bases lost during trimming</t>
   </si>
 </sst>
 </file>
@@ -1589,7 +1595,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K84"/>
+  <dimension ref="A1:K85"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.1796875" customWidth="1"/>
@@ -3954,10 +3960,10 @@
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>78</v>
+        <v>228</v>
       </c>
       <c r="B69" t="s">
-        <v>146</v>
+        <v>229</v>
       </c>
       <c r="C69" t="s">
         <v>68</v>
@@ -3966,33 +3972,27 @@
         <v>33</v>
       </c>
       <c r="E69">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F69">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="G69">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H69">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="I69" t="b">
-        <v>1</v>
-      </c>
-      <c r="J69" t="s">
-        <v>200</v>
-      </c>
-      <c r="K69" t="s">
-        <v>198</v>
+        <v>0</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B70" t="s">
-        <v>76</v>
+        <v>146</v>
       </c>
       <c r="C70" t="s">
         <v>68</v>
@@ -4004,13 +4004,13 @@
         <v>0</v>
       </c>
       <c r="F70">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="G70">
         <v>0</v>
       </c>
       <c r="H70">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="I70" t="b">
         <v>1</v>
@@ -4019,50 +4019,50 @@
         <v>200</v>
       </c>
       <c r="K70" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B71" t="s">
-        <v>97</v>
+        <v>76</v>
       </c>
       <c r="C71" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="D71" t="s">
         <v>33</v>
       </c>
       <c r="E71">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="F71">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="G71">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H71">
-        <v>100</v>
+        <v>7.5</v>
       </c>
       <c r="I71" t="b">
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>163</v>
+        <v>200</v>
       </c>
       <c r="K71" t="s">
-        <v>210</v>
+        <v>199</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B72" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C72" t="s">
         <v>65</v>
@@ -4071,13 +4071,13 @@
         <v>33</v>
       </c>
       <c r="E72">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="F72">
         <v>100</v>
       </c>
       <c r="G72">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="H72">
         <v>100</v>
@@ -4089,15 +4089,15 @@
         <v>163</v>
       </c>
       <c r="K72" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B73" t="s">
-        <v>147</v>
+        <v>98</v>
       </c>
       <c r="C73" t="s">
         <v>65</v>
@@ -4106,68 +4106,68 @@
         <v>33</v>
       </c>
       <c r="E73">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="F73">
-        <v>175</v>
+        <v>100</v>
       </c>
       <c r="G73">
-        <v>140</v>
+        <v>75</v>
       </c>
       <c r="H73">
-        <v>160</v>
+        <v>100</v>
       </c>
       <c r="I73" t="b">
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K73" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
+        <v>83</v>
+      </c>
+      <c r="B74" t="s">
+        <v>147</v>
+      </c>
+      <c r="C74" t="s">
+        <v>65</v>
+      </c>
+      <c r="D74" t="s">
+        <v>33</v>
+      </c>
+      <c r="E74">
+        <v>125</v>
+      </c>
+      <c r="F74">
+        <v>175</v>
+      </c>
+      <c r="G74">
+        <v>140</v>
+      </c>
+      <c r="H74">
         <v>160</v>
       </c>
-      <c r="B74" t="s">
-        <v>159</v>
-      </c>
-      <c r="C74" t="s">
-        <v>71</v>
-      </c>
-      <c r="D74" t="s">
-        <v>33</v>
-      </c>
-      <c r="E74">
-        <v>0</v>
-      </c>
-      <c r="F74">
-        <v>10</v>
-      </c>
-      <c r="G74">
-        <v>0</v>
-      </c>
-      <c r="H74">
-        <v>5</v>
-      </c>
       <c r="I74" t="b">
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>201</v>
+        <v>164</v>
       </c>
       <c r="K74" t="s">
-        <v>202</v>
+        <v>211</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>148</v>
+        <v>160</v>
       </c>
       <c r="B75" t="s">
-        <v>219</v>
+        <v>159</v>
       </c>
       <c r="C75" t="s">
         <v>71</v>
@@ -4176,33 +4176,33 @@
         <v>33</v>
       </c>
       <c r="E75">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="F75">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G75">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="H75">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="I75" t="b">
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>217</v>
+        <v>201</v>
       </c>
       <c r="K75" t="s">
-        <v>216</v>
+        <v>202</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="B76" t="s">
-        <v>16</v>
+        <v>219</v>
       </c>
       <c r="C76" t="s">
         <v>71</v>
@@ -4211,13 +4211,13 @@
         <v>33</v>
       </c>
       <c r="E76">
-        <v>99</v>
+        <v>60</v>
       </c>
       <c r="F76">
         <v>100</v>
       </c>
       <c r="G76">
-        <v>99.5</v>
+        <v>90</v>
       </c>
       <c r="H76">
         <v>100</v>
@@ -4226,18 +4226,18 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>205</v>
+        <v>217</v>
       </c>
       <c r="K76" t="s">
-        <v>203</v>
+        <v>216</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B77" t="s">
-        <v>152</v>
+        <v>16</v>
       </c>
       <c r="C77" t="s">
         <v>71</v>
@@ -4246,16 +4246,16 @@
         <v>33</v>
       </c>
       <c r="E77">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="F77">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="G77">
-        <v>0</v>
+        <v>99.5</v>
       </c>
       <c r="H77">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="I77" t="b">
         <v>1</v>
@@ -4264,15 +4264,15 @@
         <v>205</v>
       </c>
       <c r="K77" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B78" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
       <c r="C78" t="s">
         <v>71</v>
@@ -4281,33 +4281,33 @@
         <v>33</v>
       </c>
       <c r="E78">
-        <v>0.5</v>
-      </c>
-      <c r="F78" t="s">
+        <v>0</v>
+      </c>
+      <c r="F78">
+        <v>15</v>
+      </c>
+      <c r="G78">
+        <v>0</v>
+      </c>
+      <c r="H78">
         <v>5</v>
       </c>
-      <c r="G78">
-        <v>1</v>
-      </c>
-      <c r="H78" t="s">
-        <v>5</v>
-      </c>
       <c r="I78" t="b">
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>218</v>
+        <v>205</v>
       </c>
       <c r="K78" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>21</v>
+        <v>155</v>
       </c>
       <c r="B79" t="s">
-        <v>22</v>
+        <v>156</v>
       </c>
       <c r="C79" t="s">
         <v>71</v>
@@ -4316,33 +4316,33 @@
         <v>33</v>
       </c>
       <c r="E79">
-        <v>0</v>
-      </c>
-      <c r="F79">
-        <v>0</v>
+        <v>0.5</v>
+      </c>
+      <c r="F79" t="s">
+        <v>5</v>
       </c>
       <c r="G79">
-        <v>0</v>
-      </c>
-      <c r="H79">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H79" t="s">
+        <v>5</v>
       </c>
       <c r="I79" t="b">
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>165</v>
+        <v>218</v>
       </c>
       <c r="K79" t="s">
-        <v>188</v>
+        <v>206</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B80" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C80" t="s">
         <v>71</v>
@@ -4351,33 +4351,33 @@
         <v>33</v>
       </c>
       <c r="E80">
-        <v>14.5</v>
+        <v>0</v>
       </c>
       <c r="F80">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G80">
-        <v>26.1</v>
+        <v>0</v>
       </c>
       <c r="H80">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I80" t="b">
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>218</v>
+        <v>165</v>
       </c>
       <c r="K80" t="s">
-        <v>19</v>
+        <v>188</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="B81" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C81" t="s">
         <v>71</v>
@@ -4386,128 +4386,163 @@
         <v>33</v>
       </c>
       <c r="E81">
-        <v>5.0000000000000001E-4</v>
+        <v>14.5</v>
       </c>
       <c r="F81">
-        <v>8.0000000000000004E-4</v>
+        <v>100</v>
       </c>
       <c r="G81">
-        <v>2.0000000000000001E-4</v>
+        <v>26.1</v>
       </c>
       <c r="H81">
-        <v>5.0000000000000001E-4</v>
+        <v>100</v>
       </c>
       <c r="I81" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="J81" t="s">
+        <v>218</v>
+      </c>
+      <c r="K81" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="B82" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="C82" t="s">
-        <v>227</v>
+        <v>71</v>
       </c>
       <c r="D82" t="s">
         <v>33</v>
       </c>
       <c r="E82">
-        <v>5</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="F82">
-        <v>100</v>
+        <v>8.0000000000000004E-4</v>
       </c>
       <c r="G82">
-        <v>20</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="H82">
-        <v>100</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="I82" t="b">
-        <v>1</v>
-      </c>
-      <c r="J82" t="s">
-        <v>218</v>
-      </c>
-      <c r="K82" t="s">
-        <v>207</v>
+        <v>0</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="B83" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="C83" t="s">
         <v>227</v>
       </c>
       <c r="D83" t="s">
-        <v>80</v>
+        <v>33</v>
       </c>
       <c r="E83">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F83">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="G83">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H83">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="I83" t="b">
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>178</v>
+        <v>218</v>
       </c>
       <c r="K83" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="B84" t="s">
-        <v>208</v>
+        <v>23</v>
       </c>
       <c r="C84" t="s">
         <v>227</v>
       </c>
       <c r="D84" t="s">
-        <v>33</v>
+        <v>80</v>
       </c>
       <c r="E84">
+        <v>0</v>
+      </c>
+      <c r="F84">
+        <v>95</v>
+      </c>
+      <c r="G84">
+        <v>0</v>
+      </c>
+      <c r="H84">
+        <v>80</v>
+      </c>
+      <c r="I84" t="b">
+        <v>1</v>
+      </c>
+      <c r="J84" t="s">
+        <v>178</v>
+      </c>
+      <c r="K84" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A85" t="s">
+        <v>60</v>
+      </c>
+      <c r="B85" t="s">
+        <v>208</v>
+      </c>
+      <c r="C85" t="s">
+        <v>227</v>
+      </c>
+      <c r="D85" t="s">
+        <v>33</v>
+      </c>
+      <c r="E85">
         <v>90</v>
       </c>
-      <c r="F84">
+      <c r="F85">
         <v>100</v>
       </c>
-      <c r="G84">
+      <c r="G85">
         <v>95</v>
       </c>
-      <c r="H84">
+      <c r="H85">
         <v>100</v>
       </c>
-      <c r="I84" t="b">
-        <v>1</v>
-      </c>
-      <c r="J84" t="s">
+      <c r="I85" t="b">
+        <v>1</v>
+      </c>
+      <c r="J85" t="s">
         <v>218</v>
       </c>
-      <c r="K84" t="s">
+      <c r="K85" t="s">
         <v>60</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K82" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K83" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Replaced Fastp with Trimmomatic for ex fitlering. No longer filteres for number fo N bases
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5B4BAE2-AD2C-4FFE-8012-EBF3FBA2C751}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED623A10-5EDC-4950-81FD-7F5ABC31AF5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -4013,7 +4013,7 @@
         <v>10</v>
       </c>
       <c r="I70" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J70" t="s">
         <v>200</v>
@@ -4048,7 +4048,7 @@
         <v>7.5</v>
       </c>
       <c r="I71" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J71" t="s">
         <v>200</v>

</xml_diff>

<commit_message>
Component metrics for ex filtering now work (temporarily broke when we cahnged filtering tool)
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED623A10-5EDC-4950-81FD-7F5ABC31AF5D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B822DF5-F356-4206-9B6B-C14C4495FC75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -266,9 +266,6 @@
     <t>combined_mask_coverage</t>
   </si>
   <si>
-    <t>Percentage of reads that are lost during mean quality filtering</t>
-  </si>
-  <si>
     <t>ex_reads_lost_demux</t>
   </si>
   <si>
@@ -476,9 +473,6 @@
     <t>Gini coefficient of demultiplexed sample read count</t>
   </si>
   <si>
-    <t>Percentage of reads that are lost during length filtering</t>
-  </si>
-  <si>
     <t>Median insert size (start of R1 to end of R2) as determined by initial alignment (bp)</t>
   </si>
   <si>
@@ -632,15 +626,6 @@
     <t>_demux_metrics_gini.json</t>
   </si>
   <si>
-    <t>reads_filtered_length</t>
-  </si>
-  <si>
-    <t>reads_filtered_meanquality</t>
-  </si>
-  <si>
-    <t>_fastp_filter_summary_metrics.json</t>
-  </si>
-  <si>
     <t>_call_dsc_metrics.json</t>
   </si>
   <si>
@@ -726,6 +711,21 @@
   </si>
   <si>
     <t>Percentage of bases lost during trimming</t>
+  </si>
+  <si>
+    <t>Percentage of reads that retained after length filtering</t>
+  </si>
+  <si>
+    <t>Percentage of reads that are retained after mean quality filtering</t>
+  </si>
+  <si>
+    <t>(?m)^\s*Both Surviving Read Percent:\s*(?P&lt;value&gt;100(?:\.0+)?|(?:\d{1,2})(?:\.\d+)?)\s*$</t>
+  </si>
+  <si>
+    <t>_filter_length.txt</t>
+  </si>
+  <si>
+    <t>_filter_quality.txt</t>
   </si>
 </sst>
 </file>
@@ -1605,7 +1605,7 @@
     <col min="8" max="8" width="9" customWidth="1"/>
     <col min="9" max="9" width="12.81640625" customWidth="1"/>
     <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="58.7265625" customWidth="1"/>
+    <col min="11" max="11" width="76.81640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
@@ -1637,10 +1637,10 @@
         <v>39</v>
       </c>
       <c r="J1" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
@@ -1712,7 +1712,7 @@
         <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="C4" t="s">
         <v>61</v>
@@ -1875,7 +1875,7 @@
         <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C9" t="s">
         <v>63</v>
@@ -1910,7 +1910,7 @@
         <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C10" t="s">
         <v>63</v>
@@ -1945,7 +1945,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C11" t="s">
         <v>67</v>
@@ -1969,10 +1969,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="K11" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
@@ -1980,7 +1980,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C12" t="s">
         <v>67</v>
@@ -2004,18 +2004,18 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="K12" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B13" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C13" t="s">
         <v>64</v>
@@ -2039,18 +2039,18 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="K13" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B14" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C14" t="s">
         <v>64</v>
@@ -2074,18 +2074,18 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="K14" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B15" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C15" t="s">
         <v>67</v>
@@ -2109,18 +2109,18 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="K15" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B16" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C16" t="s">
         <v>67</v>
@@ -2144,18 +2144,18 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="K16" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B17" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C17" t="s">
         <v>67</v>
@@ -2179,18 +2179,18 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="K17" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B18" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C18" t="s">
         <v>67</v>
@@ -2214,18 +2214,18 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="K18" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B19" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C19" t="s">
         <v>64</v>
@@ -2249,18 +2249,18 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="K19" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
+        <v>109</v>
+      </c>
+      <c r="B20" t="s">
         <v>110</v>
-      </c>
-      <c r="B20" t="s">
-        <v>111</v>
       </c>
       <c r="C20" t="s">
         <v>64</v>
@@ -2284,18 +2284,18 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="K20" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B21" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C21" t="s">
         <v>64</v>
@@ -2319,18 +2319,18 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="K21" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B22" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C22" t="s">
         <v>64</v>
@@ -2354,18 +2354,18 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="K22" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B23" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C23" t="s">
         <v>64</v>
@@ -2389,18 +2389,18 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="K23" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B24" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C24" t="s">
         <v>64</v>
@@ -2424,18 +2424,18 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="K24" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B25" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C25" t="s">
         <v>64</v>
@@ -2459,18 +2459,18 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="K25" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B26" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C26" t="s">
         <v>64</v>
@@ -2494,18 +2494,18 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="K26" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B27" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C27" t="s">
         <v>64</v>
@@ -2529,18 +2529,18 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="K27" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B28" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C28" t="s">
         <v>64</v>
@@ -2564,18 +2564,18 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="K28" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B29" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C29" t="s">
         <v>69</v>
@@ -2599,18 +2599,18 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="K29" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="B30" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C30" t="s">
         <v>70</v>
@@ -2634,18 +2634,18 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="K30" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="B31" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C31" t="s">
         <v>70</v>
@@ -2669,18 +2669,18 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="K31" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="B32" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C32" t="s">
         <v>70</v>
@@ -2704,10 +2704,10 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="K32" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
@@ -2715,7 +2715,7 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C33" t="s">
         <v>72</v>
@@ -2739,10 +2739,10 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="K33" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.35">
@@ -2750,7 +2750,7 @@
         <v>6</v>
       </c>
       <c r="B34" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C34" t="s">
         <v>72</v>
@@ -2774,10 +2774,10 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="K34" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.35">
@@ -2785,7 +2785,7 @@
         <v>7</v>
       </c>
       <c r="B35" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C35" t="s">
         <v>72</v>
@@ -2809,10 +2809,10 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="K35" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.35">
@@ -2820,7 +2820,7 @@
         <v>8</v>
       </c>
       <c r="B36" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C36" t="s">
         <v>72</v>
@@ -2844,10 +2844,10 @@
         <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="K36" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.35">
@@ -2855,7 +2855,7 @@
         <v>9</v>
       </c>
       <c r="B37" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C37" t="s">
         <v>72</v>
@@ -2879,10 +2879,10 @@
         <v>1</v>
       </c>
       <c r="J37" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="K37" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.35">
@@ -2890,7 +2890,7 @@
         <v>10</v>
       </c>
       <c r="B38" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C38" t="s">
         <v>72</v>
@@ -2914,10 +2914,10 @@
         <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="K38" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.35">
@@ -2949,10 +2949,10 @@
         <v>1</v>
       </c>
       <c r="J39" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="K39" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.35">
@@ -3024,7 +3024,7 @@
         <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C42" t="s">
         <v>62</v>
@@ -3123,7 +3123,7 @@
         <v>48</v>
       </c>
       <c r="B45" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="C45" t="s">
         <v>62</v>
@@ -3158,7 +3158,7 @@
         <v>49</v>
       </c>
       <c r="B46" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="C46" t="s">
         <v>62</v>
@@ -3260,16 +3260,16 @@
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B49" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C49" t="s">
         <v>66</v>
       </c>
       <c r="D49" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E49">
         <v>35</v>
@@ -3287,24 +3287,24 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="K49" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B50" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C50" t="s">
         <v>66</v>
       </c>
       <c r="D50" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E50">
         <v>35</v>
@@ -3322,24 +3322,24 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="K50" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B51" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C51" t="s">
         <v>66</v>
       </c>
       <c r="D51" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E51">
         <v>30</v>
@@ -3357,24 +3357,24 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="K51" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B52" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C52" t="s">
         <v>66</v>
       </c>
       <c r="D52" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E52">
         <v>30</v>
@@ -3392,15 +3392,15 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="K52" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B53" t="s">
         <v>15</v>
@@ -3409,7 +3409,7 @@
         <v>66</v>
       </c>
       <c r="D53" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E53">
         <v>0</v>
@@ -3427,15 +3427,15 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="K53" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B54" t="s">
         <v>15</v>
@@ -3444,7 +3444,7 @@
         <v>66</v>
       </c>
       <c r="D54" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E54">
         <v>0</v>
@@ -3462,24 +3462,24 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="K54" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B55" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C55" t="s">
         <v>66</v>
       </c>
       <c r="D55" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E55">
         <v>150</v>
@@ -3497,24 +3497,24 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="K55" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B56" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C56" t="s">
         <v>66</v>
       </c>
       <c r="D56" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E56">
         <v>150</v>
@@ -3532,24 +3532,24 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="K56" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B57" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C57" t="s">
         <v>66</v>
       </c>
       <c r="D57" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E57">
         <v>2850</v>
@@ -3567,24 +3567,24 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="K57" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B58" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C58" t="s">
         <v>66</v>
       </c>
       <c r="D58" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E58">
         <v>2850</v>
@@ -3602,18 +3602,18 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="K58" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B59" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C59" t="s">
         <v>66</v>
@@ -3637,18 +3637,18 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="K59" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B60" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C60" t="s">
         <v>66</v>
@@ -3672,18 +3672,18 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="K60" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B61" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C61" t="s">
         <v>66</v>
@@ -3707,18 +3707,18 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="K61" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B62" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C62" t="s">
         <v>66</v>
@@ -3742,18 +3742,18 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="K62" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B63" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C63" t="s">
         <v>66</v>
@@ -3777,18 +3777,18 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="K63" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B64" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C64" t="s">
         <v>66</v>
@@ -3812,18 +3812,18 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="K64" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="B65" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C65" t="s">
         <v>66</v>
@@ -3847,18 +3847,18 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="K65" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B66" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C66" t="s">
         <v>66</v>
@@ -3882,24 +3882,24 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="K66" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B67" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C67" t="s">
         <v>68</v>
       </c>
       <c r="D67" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E67">
         <v>0</v>
@@ -3917,24 +3917,24 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="K67" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
+        <v>143</v>
+      </c>
+      <c r="B68" t="s">
         <v>144</v>
-      </c>
-      <c r="B68" t="s">
-        <v>145</v>
       </c>
       <c r="C68" t="s">
         <v>68</v>
       </c>
       <c r="D68" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E68">
         <v>0</v>
@@ -3952,18 +3952,18 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="K68" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="B69" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="C69" t="s">
         <v>68</v>
@@ -3989,10 +3989,10 @@
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B70" t="s">
-        <v>146</v>
+        <v>225</v>
       </c>
       <c r="C70" t="s">
         <v>68</v>
@@ -4001,33 +4001,33 @@
         <v>33</v>
       </c>
       <c r="E70">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F70">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="G70">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="H70">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="I70" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>200</v>
+        <v>228</v>
       </c>
       <c r="K70" t="s">
-        <v>198</v>
+        <v>227</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B71" t="s">
-        <v>76</v>
+        <v>226</v>
       </c>
       <c r="C71" t="s">
         <v>68</v>
@@ -4036,33 +4036,33 @@
         <v>33</v>
       </c>
       <c r="E71">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="F71">
-        <v>15</v>
+        <v>99</v>
       </c>
       <c r="G71">
-        <v>0</v>
+        <v>92.5</v>
       </c>
       <c r="H71">
-        <v>7.5</v>
+        <v>99</v>
       </c>
       <c r="I71" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>200</v>
+        <v>229</v>
       </c>
       <c r="K71" t="s">
-        <v>199</v>
+        <v>227</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B72" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C72" t="s">
         <v>65</v>
@@ -4086,18 +4086,18 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="K72" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B73" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C73" t="s">
         <v>65</v>
@@ -4121,18 +4121,18 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="K73" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B74" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="C74" t="s">
         <v>65</v>
@@ -4156,18 +4156,18 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="K74" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="B75" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C75" t="s">
         <v>71</v>
@@ -4191,18 +4191,18 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="K75" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B76" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="C76" t="s">
         <v>71</v>
@@ -4226,15 +4226,15 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="K76" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="B77" t="s">
         <v>16</v>
@@ -4261,18 +4261,18 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="K77" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="B78" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="C78" t="s">
         <v>71</v>
@@ -4296,18 +4296,18 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="K78" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="B79" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C79" t="s">
         <v>71</v>
@@ -4331,10 +4331,10 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="K79" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.35">
@@ -4366,10 +4366,10 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="K80" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.35">
@@ -4401,7 +4401,7 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="K81" t="s">
         <v>19</v>
@@ -4444,7 +4444,7 @@
         <v>17</v>
       </c>
       <c r="C83" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="D83" t="s">
         <v>33</v>
@@ -4465,10 +4465,10 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="K83" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.35">
@@ -4479,10 +4479,10 @@
         <v>23</v>
       </c>
       <c r="C84" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="D84" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E84">
         <v>0</v>
@@ -4500,10 +4500,10 @@
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="K84" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.35">
@@ -4511,10 +4511,10 @@
         <v>60</v>
       </c>
       <c r="B85" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C85" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
       <c r="D85" t="s">
         <v>33</v>
@@ -4535,7 +4535,7 @@
         <v>1</v>
       </c>
       <c r="J85" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="K85" t="s">
         <v>60</v>

</xml_diff>

<commit_message>
Added call_codec_consensus_metrics.txt metrics file and included in component metrics script
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B822DF5-F356-4206-9B6B-C14C4495FC75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8834BD05-6A2E-48B1-A06B-89C792DD01F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="523" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="232">
   <si>
     <t>nn_lower</t>
   </si>
@@ -726,6 +726,12 @@
   </si>
   <si>
     <t>_filter_quality.txt</t>
+  </si>
+  <si>
+    <t>^duplex_disagreement_rate\s+([0-9]*\.?[0-9]+)</t>
+  </si>
+  <si>
+    <t>_call_codec_consensus_metrics.txt</t>
   </si>
 </sst>
 </file>
@@ -1596,19 +1602,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
   <dimension ref="A1:K85"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.1796875" customWidth="1"/>
-    <col min="2" max="2" width="87.26953125" customWidth="1"/>
-    <col min="3" max="4" width="35.26953125" customWidth="1"/>
+    <col min="1" max="1" width="35.140625" customWidth="1"/>
+    <col min="2" max="2" width="87.28515625" customWidth="1"/>
+    <col min="3" max="4" width="35.28515625" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.81640625" customWidth="1"/>
-    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="76.81640625" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="76.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>40</v>
       </c>
@@ -1643,7 +1649,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>44</v>
       </c>
@@ -1672,7 +1678,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>45</v>
       </c>
@@ -1707,7 +1713,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>46</v>
       </c>
@@ -1742,7 +1748,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>55</v>
       </c>
@@ -1771,7 +1777,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>54</v>
       </c>
@@ -1806,7 +1812,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>56</v>
       </c>
@@ -1835,7 +1841,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>57</v>
       </c>
@@ -1870,7 +1876,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -1905,7 +1911,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>31</v>
       </c>
@@ -1940,7 +1946,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -1975,7 +1981,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -2010,7 +2016,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>122</v>
       </c>
@@ -2045,7 +2051,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>123</v>
       </c>
@@ -2080,7 +2086,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>118</v>
       </c>
@@ -2115,7 +2121,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>119</v>
       </c>
@@ -2150,7 +2156,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>120</v>
       </c>
@@ -2185,7 +2191,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>121</v>
       </c>
@@ -2220,7 +2226,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>108</v>
       </c>
@@ -2255,7 +2261,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>109</v>
       </c>
@@ -2290,7 +2296,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>86</v>
       </c>
@@ -2325,7 +2331,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>87</v>
       </c>
@@ -2360,7 +2366,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>88</v>
       </c>
@@ -2395,7 +2401,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>89</v>
       </c>
@@ -2430,7 +2436,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>90</v>
       </c>
@@ -2465,7 +2471,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>91</v>
       </c>
@@ -2500,7 +2506,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>92</v>
       </c>
@@ -2535,7 +2541,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>93</v>
       </c>
@@ -2570,7 +2576,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>95</v>
       </c>
@@ -2605,7 +2611,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>149</v>
       </c>
@@ -2640,7 +2646,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>148</v>
       </c>
@@ -2675,7 +2681,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>147</v>
       </c>
@@ -2710,7 +2716,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -2745,7 +2751,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>6</v>
       </c>
@@ -2780,7 +2786,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>7</v>
       </c>
@@ -2815,7 +2821,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -2850,7 +2856,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>9</v>
       </c>
@@ -2885,7 +2891,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>10</v>
       </c>
@@ -2920,7 +2926,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>75</v>
       </c>
@@ -2955,7 +2961,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>27</v>
       </c>
@@ -2984,7 +2990,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>35</v>
       </c>
@@ -3019,7 +3025,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>43</v>
       </c>
@@ -3054,7 +3060,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>52</v>
       </c>
@@ -3083,7 +3089,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>47</v>
       </c>
@@ -3118,7 +3124,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>48</v>
       </c>
@@ -3153,7 +3159,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>49</v>
       </c>
@@ -3188,7 +3194,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>28</v>
       </c>
@@ -3223,7 +3229,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>29</v>
       </c>
@@ -3258,7 +3264,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>112</v>
       </c>
@@ -3293,7 +3299,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>113</v>
       </c>
@@ -3328,7 +3334,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>114</v>
       </c>
@@ -3363,7 +3369,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>115</v>
       </c>
@@ -3398,7 +3404,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>116</v>
       </c>
@@ -3433,7 +3439,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>117</v>
       </c>
@@ -3468,7 +3474,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>111</v>
       </c>
@@ -3503,7 +3509,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>124</v>
       </c>
@@ -3538,7 +3544,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>125</v>
       </c>
@@ -3573,7 +3579,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>126</v>
       </c>
@@ -3608,7 +3614,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>127</v>
       </c>
@@ -3643,7 +3649,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>128</v>
       </c>
@@ -3678,7 +3684,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>129</v>
       </c>
@@ -3713,7 +3719,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>130</v>
       </c>
@@ -3748,7 +3754,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>131</v>
       </c>
@@ -3783,7 +3789,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>132</v>
       </c>
@@ -3818,7 +3824,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>133</v>
       </c>
@@ -3853,7 +3859,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>134</v>
       </c>
@@ -3888,7 +3894,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>76</v>
       </c>
@@ -3923,7 +3929,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>143</v>
       </c>
@@ -3958,7 +3964,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>223</v>
       </c>
@@ -3987,7 +3993,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>77</v>
       </c>
@@ -4022,7 +4028,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>78</v>
       </c>
@@ -4057,7 +4063,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>81</v>
       </c>
@@ -4092,7 +4098,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>80</v>
       </c>
@@ -4127,7 +4133,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>82</v>
       </c>
@@ -4162,7 +4168,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>158</v>
       </c>
@@ -4197,7 +4203,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>146</v>
       </c>
@@ -4232,7 +4238,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>152</v>
       </c>
@@ -4267,7 +4273,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>151</v>
       </c>
@@ -4302,7 +4308,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>153</v>
       </c>
@@ -4337,7 +4343,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>21</v>
       </c>
@@ -4372,7 +4378,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>19</v>
       </c>
@@ -4407,7 +4413,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>13</v>
       </c>
@@ -4433,10 +4439,16 @@
         <v>5.0000000000000001E-4</v>
       </c>
       <c r="I82" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
+        <v>1</v>
+      </c>
+      <c r="J82" t="s">
+        <v>231</v>
+      </c>
+      <c r="K82" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>18</v>
       </c>
@@ -4471,7 +4483,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>24</v>
       </c>
@@ -4506,7 +4518,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>60</v>
       </c>

</xml_diff>

<commit_message>
Added percent_reads_bases_lost.py and test. Deleted ex_fastp_filter_summary_metrics.py as no longer needed due to change to trimmomatic
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8834BD05-6A2E-48B1-A06B-89C792DD01F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CC9FD9A-11C8-45A7-B6A2-8ECC491DA1DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="232">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="234">
   <si>
     <t>nn_lower</t>
   </si>
@@ -732,6 +732,12 @@
   </si>
   <si>
     <t>_call_codec_consensus_metrics.txt</t>
+  </si>
+  <si>
+    <t>pct_bases_lost</t>
+  </si>
+  <si>
+    <t>_bases_trimmed.json</t>
   </si>
 </sst>
 </file>
@@ -3990,7 +3996,13 @@
         <v>15</v>
       </c>
       <c r="I69" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="J69" t="s">
+        <v>233</v>
+      </c>
+      <c r="K69" t="s">
+        <v>232</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Updated germline variant rate calc
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CC9FD9A-11C8-45A7-B6A2-8ECC491DA1DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{597BCD48-4B56-4398-A8D8-A0892FE3837F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -359,9 +359,6 @@
     <t>Peak in mean sequence quality across raw r2 reads (Phred score)</t>
   </si>
   <si>
-    <t>Lower quartile of IQR for base quality at each position in raw reads (Phred score)</t>
-  </si>
-  <si>
     <t>ms_raw_read_length_r1</t>
   </si>
   <si>
@@ -380,24 +377,12 @@
     <t>ex_lane_raw_per_sequence_quality_r2</t>
   </si>
   <si>
-    <t>ex_lane_raw_per_base_quality_r1</t>
-  </si>
-  <si>
-    <t>ex_lane_raw_per_quality_r2</t>
-  </si>
-  <si>
     <t>ex_lane_raw_per_tile_quality_r1</t>
   </si>
   <si>
     <t>ex_lane_raw_per_tile_quality_r2</t>
   </si>
   <si>
-    <t>ms_raw_per_base_quality_r1</t>
-  </si>
-  <si>
-    <t>ms_raw_per_base_quality_r2</t>
-  </si>
-  <si>
     <t>ms_raw_per_tile_quality_r1</t>
   </si>
   <si>
@@ -738,6 +723,21 @@
   </si>
   <si>
     <t>_bases_trimmed.json</t>
+  </si>
+  <si>
+    <t>ex_filtered_per_base_quality_r1</t>
+  </si>
+  <si>
+    <t>ex_filtered_per_base_quality_r2</t>
+  </si>
+  <si>
+    <t>ms_filtered_per_base_quality_r1</t>
+  </si>
+  <si>
+    <t>ms_filtered_per_base_quality_r2</t>
+  </si>
+  <si>
+    <t>Lower quartile of IQR for base quality at each position in filtered reads (Phred score)</t>
   </si>
 </sst>
 </file>
@@ -1649,10 +1649,10 @@
         <v>39</v>
       </c>
       <c r="J1" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="K1" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -1724,7 +1724,7 @@
         <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="C4" t="s">
         <v>61</v>
@@ -1957,7 +1957,7 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="C11" t="s">
         <v>67</v>
@@ -1981,10 +1981,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="K11" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1992,7 +1992,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="C12" t="s">
         <v>67</v>
@@ -2016,15 +2016,15 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="K12" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B13" t="s">
         <v>105</v>
@@ -2051,15 +2051,15 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="K13" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B14" t="s">
         <v>106</v>
@@ -2086,18 +2086,18 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="K14" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B15" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="C15" t="s">
         <v>67</v>
@@ -2106,33 +2106,33 @@
         <v>33</v>
       </c>
       <c r="E15">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F15">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="G15">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H15">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="I15" t="b">
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="K15" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B16" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="C16" t="s">
         <v>67</v>
@@ -2141,165 +2141,165 @@
         <v>33</v>
       </c>
       <c r="E16">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F16">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="G16">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H16">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="I16" t="b">
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="K16" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
       <c r="B17" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="C17" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D17" t="s">
         <v>33</v>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="F17">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="G17">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="H17">
-        <v>5</v>
+        <v>150</v>
       </c>
       <c r="I17" t="b">
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="K17" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>121</v>
+        <v>108</v>
       </c>
       <c r="B18" t="s">
-        <v>94</v>
+        <v>109</v>
       </c>
       <c r="C18" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D18" t="s">
         <v>33</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="F18">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="G18">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="H18">
-        <v>5</v>
+        <v>150</v>
       </c>
       <c r="I18" t="b">
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="K18" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>108</v>
+        <v>231</v>
       </c>
       <c r="B19" t="s">
-        <v>110</v>
+        <v>233</v>
       </c>
       <c r="C19" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D19" t="s">
         <v>33</v>
       </c>
       <c r="E19">
-        <v>150</v>
+        <v>30</v>
       </c>
       <c r="F19">
-        <v>150</v>
+        <v>40</v>
       </c>
       <c r="G19">
-        <v>150</v>
+        <v>35</v>
       </c>
       <c r="H19">
-        <v>150</v>
+        <v>40</v>
       </c>
       <c r="I19" t="b">
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="K19" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>109</v>
+        <v>232</v>
       </c>
       <c r="B20" t="s">
-        <v>110</v>
+        <v>233</v>
       </c>
       <c r="C20" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="D20" t="s">
         <v>33</v>
       </c>
       <c r="E20">
-        <v>150</v>
+        <v>30</v>
       </c>
       <c r="F20">
-        <v>150</v>
+        <v>40</v>
       </c>
       <c r="G20">
-        <v>150</v>
+        <v>35</v>
       </c>
       <c r="H20">
-        <v>150</v>
+        <v>40</v>
       </c>
       <c r="I20" t="b">
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="K20" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -2307,7 +2307,7 @@
         <v>86</v>
       </c>
       <c r="B21" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C21" t="s">
         <v>64</v>
@@ -2331,10 +2331,10 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="K21" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -2342,7 +2342,7 @@
         <v>87</v>
       </c>
       <c r="B22" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C22" t="s">
         <v>64</v>
@@ -2366,10 +2366,10 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="K22" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -2377,7 +2377,7 @@
         <v>88</v>
       </c>
       <c r="B23" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C23" t="s">
         <v>64</v>
@@ -2401,10 +2401,10 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="K23" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -2412,7 +2412,7 @@
         <v>89</v>
       </c>
       <c r="B24" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C24" t="s">
         <v>64</v>
@@ -2436,10 +2436,10 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="K24" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -2447,7 +2447,7 @@
         <v>90</v>
       </c>
       <c r="B25" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C25" t="s">
         <v>64</v>
@@ -2471,10 +2471,10 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="K25" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -2482,7 +2482,7 @@
         <v>91</v>
       </c>
       <c r="B26" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C26" t="s">
         <v>64</v>
@@ -2506,10 +2506,10 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="K26" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -2517,7 +2517,7 @@
         <v>92</v>
       </c>
       <c r="B27" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C27" t="s">
         <v>64</v>
@@ -2541,10 +2541,10 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="K27" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -2552,7 +2552,7 @@
         <v>93</v>
       </c>
       <c r="B28" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C28" t="s">
         <v>64</v>
@@ -2576,10 +2576,10 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
       <c r="K28" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -2587,7 +2587,7 @@
         <v>95</v>
       </c>
       <c r="B29" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="C29" t="s">
         <v>69</v>
@@ -2611,18 +2611,18 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="K29" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="B30" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="C30" t="s">
         <v>70</v>
@@ -2646,18 +2646,18 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
       <c r="K30" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="B31" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="C31" t="s">
         <v>70</v>
@@ -2681,15 +2681,15 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
       <c r="K31" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="B32" t="s">
         <v>98</v>
@@ -2716,10 +2716,10 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
       <c r="K32" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -2751,10 +2751,10 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="K33" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -2786,10 +2786,10 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="K34" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -2821,10 +2821,10 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="K35" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -2856,10 +2856,10 @@
         <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="K36" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
@@ -2891,10 +2891,10 @@
         <v>1</v>
       </c>
       <c r="J37" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="K37" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
@@ -2926,10 +2926,10 @@
         <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
       <c r="K38" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
@@ -2961,10 +2961,10 @@
         <v>1</v>
       </c>
       <c r="J39" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="K39" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
@@ -3036,7 +3036,7 @@
         <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="C42" t="s">
         <v>62</v>
@@ -3135,7 +3135,7 @@
         <v>48</v>
       </c>
       <c r="B45" t="s">
-        <v>220</v>
+        <v>215</v>
       </c>
       <c r="C45" t="s">
         <v>62</v>
@@ -3170,7 +3170,7 @@
         <v>49</v>
       </c>
       <c r="B46" t="s">
-        <v>221</v>
+        <v>216</v>
       </c>
       <c r="C46" t="s">
         <v>62</v>
@@ -3272,7 +3272,7 @@
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B49" t="s">
         <v>105</v>
@@ -3299,15 +3299,15 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="K49" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B50" t="s">
         <v>106</v>
@@ -3334,18 +3334,18 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="K50" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B51" t="s">
-        <v>107</v>
+        <v>15</v>
       </c>
       <c r="C51" t="s">
         <v>66</v>
@@ -3354,33 +3354,33 @@
         <v>79</v>
       </c>
       <c r="E51">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F51">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="G51">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H51">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="I51" t="b">
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="K51" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B52" t="s">
-        <v>107</v>
+        <v>15</v>
       </c>
       <c r="C52" t="s">
         <v>66</v>
@@ -3389,33 +3389,33 @@
         <v>79</v>
       </c>
       <c r="E52">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F52">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="G52">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H52">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="I52" t="b">
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="K52" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>116</v>
+        <v>110</v>
       </c>
       <c r="B53" t="s">
-        <v>15</v>
+        <v>109</v>
       </c>
       <c r="C53" t="s">
         <v>66</v>
@@ -3424,33 +3424,33 @@
         <v>79</v>
       </c>
       <c r="E53">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="F53">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="G53">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="H53">
-        <v>5</v>
+        <v>150</v>
       </c>
       <c r="I53" t="b">
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="K53" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B54" t="s">
-        <v>15</v>
+        <v>109</v>
       </c>
       <c r="C54" t="s">
         <v>66</v>
@@ -3459,33 +3459,33 @@
         <v>79</v>
       </c>
       <c r="E54">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="F54">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="G54">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="H54">
-        <v>5</v>
+        <v>150</v>
       </c>
       <c r="I54" t="b">
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
       <c r="K54" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="B55" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C55" t="s">
         <v>66</v>
@@ -3494,33 +3494,33 @@
         <v>79</v>
       </c>
       <c r="E55">
-        <v>150</v>
-      </c>
-      <c r="F55">
-        <v>150</v>
+        <v>2850</v>
+      </c>
+      <c r="F55" t="s">
+        <v>5</v>
       </c>
       <c r="G55">
-        <v>150</v>
-      </c>
-      <c r="H55">
-        <v>150</v>
+        <v>3000</v>
+      </c>
+      <c r="H55" t="s">
+        <v>5</v>
       </c>
       <c r="I55" t="b">
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
       <c r="K55" t="s">
-        <v>181</v>
+        <v>172</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B56" t="s">
-        <v>110</v>
+        <v>130</v>
       </c>
       <c r="C56" t="s">
         <v>66</v>
@@ -3529,103 +3529,103 @@
         <v>79</v>
       </c>
       <c r="E56">
-        <v>150</v>
-      </c>
-      <c r="F56">
-        <v>150</v>
+        <v>2850</v>
+      </c>
+      <c r="F56" t="s">
+        <v>5</v>
       </c>
       <c r="G56">
-        <v>150</v>
-      </c>
-      <c r="H56">
-        <v>150</v>
+        <v>3000</v>
+      </c>
+      <c r="H56" t="s">
+        <v>5</v>
       </c>
       <c r="I56" t="b">
         <v>1</v>
       </c>
       <c r="J56" t="s">
+        <v>167</v>
+      </c>
+      <c r="K56" t="s">
         <v>172</v>
-      </c>
-      <c r="K56" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>125</v>
+        <v>229</v>
       </c>
       <c r="B57" t="s">
-        <v>135</v>
+        <v>233</v>
       </c>
       <c r="C57" t="s">
         <v>66</v>
       </c>
       <c r="D57" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="E57">
-        <v>2850</v>
-      </c>
-      <c r="F57" t="s">
-        <v>5</v>
+        <v>30</v>
+      </c>
+      <c r="F57">
+        <v>40</v>
       </c>
       <c r="G57">
-        <v>3000</v>
-      </c>
-      <c r="H57" t="s">
-        <v>5</v>
+        <v>35</v>
+      </c>
+      <c r="H57">
+        <v>40</v>
       </c>
       <c r="I57" t="b">
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="K57" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>126</v>
+        <v>230</v>
       </c>
       <c r="B58" t="s">
-        <v>135</v>
+        <v>233</v>
       </c>
       <c r="C58" t="s">
         <v>66</v>
       </c>
       <c r="D58" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="E58">
-        <v>2850</v>
-      </c>
-      <c r="F58" t="s">
-        <v>5</v>
+        <v>30</v>
+      </c>
+      <c r="F58">
+        <v>40</v>
       </c>
       <c r="G58">
-        <v>3000</v>
-      </c>
-      <c r="H58" t="s">
-        <v>5</v>
+        <v>35</v>
+      </c>
+      <c r="H58">
+        <v>40</v>
       </c>
       <c r="I58" t="b">
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="K58" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B59" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C59" t="s">
         <v>66</v>
@@ -3649,18 +3649,18 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="K59" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="B60" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="C60" t="s">
         <v>66</v>
@@ -3684,18 +3684,18 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="K60" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B61" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C61" t="s">
         <v>66</v>
@@ -3719,18 +3719,18 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="K61" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B62" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="C62" t="s">
         <v>66</v>
@@ -3754,18 +3754,18 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="K62" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B63" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C63" t="s">
         <v>66</v>
@@ -3789,18 +3789,18 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="K63" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B64" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="C64" t="s">
         <v>66</v>
@@ -3824,18 +3824,18 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="K64" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="B65" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C65" t="s">
         <v>66</v>
@@ -3859,18 +3859,18 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
       <c r="K65" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B66" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="C66" t="s">
         <v>66</v>
@@ -3894,10 +3894,10 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
       <c r="K66" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
@@ -3929,18 +3929,18 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="K67" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="B68" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="C68" t="s">
         <v>68</v>
@@ -3964,18 +3964,18 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
       <c r="K68" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>223</v>
+        <v>218</v>
       </c>
       <c r="B69" t="s">
-        <v>224</v>
+        <v>219</v>
       </c>
       <c r="C69" t="s">
         <v>68</v>
@@ -3999,10 +3999,10 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>233</v>
+        <v>228</v>
       </c>
       <c r="K69" t="s">
-        <v>232</v>
+        <v>227</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
@@ -4010,7 +4010,7 @@
         <v>77</v>
       </c>
       <c r="B70" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="C70" t="s">
         <v>68</v>
@@ -4034,10 +4034,10 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>228</v>
+        <v>223</v>
       </c>
       <c r="K70" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
@@ -4045,7 +4045,7 @@
         <v>78</v>
       </c>
       <c r="B71" t="s">
-        <v>226</v>
+        <v>221</v>
       </c>
       <c r="C71" t="s">
         <v>68</v>
@@ -4069,10 +4069,10 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>229</v>
+        <v>224</v>
       </c>
       <c r="K71" t="s">
-        <v>227</v>
+        <v>222</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
@@ -4104,10 +4104,10 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="K72" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
@@ -4139,10 +4139,10 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="K73" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
@@ -4150,7 +4150,7 @@
         <v>82</v>
       </c>
       <c r="B74" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="C74" t="s">
         <v>65</v>
@@ -4174,18 +4174,18 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="K74" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B75" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="C75" t="s">
         <v>71</v>
@@ -4209,18 +4209,18 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="K75" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B76" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="C76" t="s">
         <v>71</v>
@@ -4244,15 +4244,15 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="K76" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="B77" t="s">
         <v>16</v>
@@ -4279,18 +4279,18 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="K77" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B78" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="C78" t="s">
         <v>71</v>
@@ -4314,18 +4314,18 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="K78" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="B79" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="C79" t="s">
         <v>71</v>
@@ -4349,10 +4349,10 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="K79" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
@@ -4384,10 +4384,10 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="K80" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
@@ -4419,7 +4419,7 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="K81" t="s">
         <v>19</v>
@@ -4454,10 +4454,10 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>231</v>
+        <v>226</v>
       </c>
       <c r="K82" t="s">
-        <v>230</v>
+        <v>225</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
@@ -4468,7 +4468,7 @@
         <v>17</v>
       </c>
       <c r="C83" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="D83" t="s">
         <v>33</v>
@@ -4489,10 +4489,10 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="K83" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
@@ -4503,7 +4503,7 @@
         <v>23</v>
       </c>
       <c r="C84" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="D84" t="s">
         <v>79</v>
@@ -4524,10 +4524,10 @@
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="K84" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
@@ -4535,10 +4535,10 @@
         <v>60</v>
       </c>
       <c r="B85" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="C85" t="s">
-        <v>222</v>
+        <v>217</v>
       </c>
       <c r="D85" t="s">
         <v>33</v>
@@ -4559,7 +4559,7 @@
         <v>1</v>
       </c>
       <c r="J85" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
       <c r="K85" t="s">
         <v>60</v>

</xml_diff>

<commit_message>
Added component metric for zero length ex redas after trimming
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{597BCD48-4B56-4398-A8D8-A0892FE3837F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48CEC0F6-FB25-4D9B-8854-69DBAF544F08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$84</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="527" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="236">
   <si>
     <t>nn_lower</t>
   </si>
@@ -738,6 +738,12 @@
   </si>
   <si>
     <t>Lower quartile of IQR for base quality at each position in filtered reads (Phred score)</t>
+  </si>
+  <si>
+    <t>ex_zero_length</t>
+  </si>
+  <si>
+    <t>Reads with a length of zero after trimming (e.g. blank ligation)</t>
   </si>
 </sst>
 </file>
@@ -1607,20 +1613,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K85"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K86"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="35.140625" customWidth="1"/>
-    <col min="2" max="2" width="87.28515625" customWidth="1"/>
-    <col min="3" max="4" width="35.28515625" customWidth="1"/>
+    <col min="1" max="1" width="35.1796875" customWidth="1"/>
+    <col min="2" max="2" width="87.26953125" customWidth="1"/>
+    <col min="3" max="4" width="35.26953125" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" customWidth="1"/>
-    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="76.85546875" customWidth="1"/>
+    <col min="9" max="9" width="12.81640625" customWidth="1"/>
+    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="76.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>40</v>
       </c>
@@ -1655,7 +1661,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>44</v>
       </c>
@@ -1684,7 +1690,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>45</v>
       </c>
@@ -1719,7 +1725,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>46</v>
       </c>
@@ -1754,7 +1760,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>55</v>
       </c>
@@ -1783,7 +1789,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>54</v>
       </c>
@@ -1818,7 +1824,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>56</v>
       </c>
@@ -1847,7 +1853,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>57</v>
       </c>
@@ -1882,7 +1888,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -1917,7 +1923,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>31</v>
       </c>
@@ -1952,7 +1958,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -1987,7 +1993,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -2022,7 +2028,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>117</v>
       </c>
@@ -2057,7 +2063,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>118</v>
       </c>
@@ -2092,7 +2098,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>115</v>
       </c>
@@ -2127,7 +2133,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>116</v>
       </c>
@@ -2162,7 +2168,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>107</v>
       </c>
@@ -2197,7 +2203,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>108</v>
       </c>
@@ -2232,7 +2238,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>231</v>
       </c>
@@ -2267,7 +2273,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>232</v>
       </c>
@@ -2302,7 +2308,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>86</v>
       </c>
@@ -2337,7 +2343,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>87</v>
       </c>
@@ -2372,7 +2378,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>88</v>
       </c>
@@ -2407,7 +2413,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>89</v>
       </c>
@@ -2442,7 +2448,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>90</v>
       </c>
@@ -2477,7 +2483,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>91</v>
       </c>
@@ -2512,7 +2518,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>92</v>
       </c>
@@ -2547,7 +2553,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>93</v>
       </c>
@@ -2582,7 +2588,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>95</v>
       </c>
@@ -2617,7 +2623,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>144</v>
       </c>
@@ -2652,7 +2658,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>143</v>
       </c>
@@ -2687,7 +2693,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>142</v>
       </c>
@@ -2722,7 +2728,7 @@
         <v>201</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -2757,7 +2763,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>6</v>
       </c>
@@ -2792,7 +2798,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>7</v>
       </c>
@@ -2827,7 +2833,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -2862,7 +2868,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>9</v>
       </c>
@@ -2897,7 +2903,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>10</v>
       </c>
@@ -2932,7 +2938,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>75</v>
       </c>
@@ -2967,7 +2973,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>27</v>
       </c>
@@ -2996,7 +3002,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>35</v>
       </c>
@@ -3031,7 +3037,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>43</v>
       </c>
@@ -3066,7 +3072,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>52</v>
       </c>
@@ -3095,7 +3101,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>47</v>
       </c>
@@ -3130,7 +3136,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>48</v>
       </c>
@@ -3165,7 +3171,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>49</v>
       </c>
@@ -3200,7 +3206,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>28</v>
       </c>
@@ -3235,7 +3241,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>29</v>
       </c>
@@ -3270,7 +3276,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>111</v>
       </c>
@@ -3305,7 +3311,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>112</v>
       </c>
@@ -3340,7 +3346,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>113</v>
       </c>
@@ -3375,7 +3381,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>114</v>
       </c>
@@ -3410,7 +3416,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>110</v>
       </c>
@@ -3445,7 +3451,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>119</v>
       </c>
@@ -3480,7 +3486,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>120</v>
       </c>
@@ -3515,7 +3521,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>121</v>
       </c>
@@ -3550,7 +3556,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>229</v>
       </c>
@@ -3585,7 +3591,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>230</v>
       </c>
@@ -3620,7 +3626,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>122</v>
       </c>
@@ -3655,7 +3661,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>123</v>
       </c>
@@ -3690,7 +3696,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>124</v>
       </c>
@@ -3725,7 +3731,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>125</v>
       </c>
@@ -3760,7 +3766,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>126</v>
       </c>
@@ -3795,7 +3801,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>127</v>
       </c>
@@ -3830,7 +3836,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>128</v>
       </c>
@@ -3865,7 +3871,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>129</v>
       </c>
@@ -3900,7 +3906,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>76</v>
       </c>
@@ -3935,7 +3941,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>138</v>
       </c>
@@ -3970,7 +3976,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>218</v>
       </c>
@@ -4005,12 +4011,12 @@
         <v>227</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>77</v>
+        <v>234</v>
       </c>
       <c r="B70" t="s">
-        <v>220</v>
+        <v>235</v>
       </c>
       <c r="C70" t="s">
         <v>68</v>
@@ -4019,33 +4025,27 @@
         <v>33</v>
       </c>
       <c r="E70">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F70">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="G70">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="H70">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="I70" t="b">
-        <v>1</v>
-      </c>
-      <c r="J70" t="s">
-        <v>223</v>
-      </c>
-      <c r="K70" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B71" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C71" t="s">
         <v>68</v>
@@ -4054,13 +4054,13 @@
         <v>33</v>
       </c>
       <c r="E71">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="F71">
         <v>99</v>
       </c>
       <c r="G71">
-        <v>92.5</v>
+        <v>90</v>
       </c>
       <c r="H71">
         <v>99</v>
@@ -4069,53 +4069,53 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="K71" t="s">
         <v>222</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
+        <v>78</v>
+      </c>
+      <c r="B72" t="s">
+        <v>221</v>
+      </c>
+      <c r="C72" t="s">
+        <v>68</v>
+      </c>
+      <c r="D72" t="s">
+        <v>33</v>
+      </c>
+      <c r="E72">
+        <v>85</v>
+      </c>
+      <c r="F72">
+        <v>99</v>
+      </c>
+      <c r="G72">
+        <v>92.5</v>
+      </c>
+      <c r="H72">
+        <v>99</v>
+      </c>
+      <c r="I72" t="b">
+        <v>1</v>
+      </c>
+      <c r="J72" t="s">
+        <v>224</v>
+      </c>
+      <c r="K72" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A73" t="s">
         <v>81</v>
       </c>
-      <c r="B72" t="s">
+      <c r="B73" t="s">
         <v>96</v>
-      </c>
-      <c r="C72" t="s">
-        <v>65</v>
-      </c>
-      <c r="D72" t="s">
-        <v>33</v>
-      </c>
-      <c r="E72">
-        <v>90</v>
-      </c>
-      <c r="F72">
-        <v>100</v>
-      </c>
-      <c r="G72">
-        <v>95</v>
-      </c>
-      <c r="H72">
-        <v>100</v>
-      </c>
-      <c r="I72" t="b">
-        <v>1</v>
-      </c>
-      <c r="J72" t="s">
-        <v>156</v>
-      </c>
-      <c r="K72" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>80</v>
-      </c>
-      <c r="B73" t="s">
-        <v>97</v>
       </c>
       <c r="C73" t="s">
         <v>65</v>
@@ -4124,13 +4124,13 @@
         <v>33</v>
       </c>
       <c r="E73">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="F73">
         <v>100</v>
       </c>
       <c r="G73">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="H73">
         <v>100</v>
@@ -4142,15 +4142,15 @@
         <v>156</v>
       </c>
       <c r="K73" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B74" t="s">
-        <v>140</v>
+        <v>97</v>
       </c>
       <c r="C74" t="s">
         <v>65</v>
@@ -4159,68 +4159,68 @@
         <v>33</v>
       </c>
       <c r="E74">
+        <v>50</v>
+      </c>
+      <c r="F74">
+        <v>100</v>
+      </c>
+      <c r="G74">
+        <v>75</v>
+      </c>
+      <c r="H74">
+        <v>100</v>
+      </c>
+      <c r="I74" t="b">
+        <v>1</v>
+      </c>
+      <c r="J74" t="s">
+        <v>156</v>
+      </c>
+      <c r="K74" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A75" t="s">
+        <v>82</v>
+      </c>
+      <c r="B75" t="s">
+        <v>140</v>
+      </c>
+      <c r="C75" t="s">
+        <v>65</v>
+      </c>
+      <c r="D75" t="s">
+        <v>33</v>
+      </c>
+      <c r="E75">
         <v>125</v>
       </c>
-      <c r="F74">
+      <c r="F75">
         <v>175</v>
       </c>
-      <c r="G74">
+      <c r="G75">
         <v>140</v>
       </c>
-      <c r="H74">
+      <c r="H75">
         <v>160</v>
       </c>
-      <c r="I74" t="b">
-        <v>1</v>
-      </c>
-      <c r="J74" t="s">
+      <c r="I75" t="b">
+        <v>1</v>
+      </c>
+      <c r="J75" t="s">
         <v>157</v>
       </c>
-      <c r="K74" t="s">
+      <c r="K75" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A76" t="s">
         <v>153</v>
       </c>
-      <c r="B75" t="s">
+      <c r="B76" t="s">
         <v>152</v>
-      </c>
-      <c r="C75" t="s">
-        <v>71</v>
-      </c>
-      <c r="D75" t="s">
-        <v>33</v>
-      </c>
-      <c r="E75">
-        <v>0</v>
-      </c>
-      <c r="F75">
-        <v>10</v>
-      </c>
-      <c r="G75">
-        <v>0</v>
-      </c>
-      <c r="H75">
-        <v>5</v>
-      </c>
-      <c r="I75" t="b">
-        <v>1</v>
-      </c>
-      <c r="J75" t="s">
-        <v>191</v>
-      </c>
-      <c r="K75" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>141</v>
-      </c>
-      <c r="B76" t="s">
-        <v>209</v>
       </c>
       <c r="C76" t="s">
         <v>71</v>
@@ -4229,33 +4229,33 @@
         <v>33</v>
       </c>
       <c r="E76">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="F76">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G76">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="H76">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="I76" t="b">
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>207</v>
+        <v>191</v>
       </c>
       <c r="K76" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="B77" t="s">
-        <v>16</v>
+        <v>209</v>
       </c>
       <c r="C77" t="s">
         <v>71</v>
@@ -4264,13 +4264,13 @@
         <v>33</v>
       </c>
       <c r="E77">
-        <v>99</v>
+        <v>60</v>
       </c>
       <c r="F77">
         <v>100</v>
       </c>
       <c r="G77">
-        <v>99.5</v>
+        <v>90</v>
       </c>
       <c r="H77">
         <v>100</v>
@@ -4279,18 +4279,18 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>195</v>
+        <v>207</v>
       </c>
       <c r="K77" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B78" t="s">
-        <v>145</v>
+        <v>16</v>
       </c>
       <c r="C78" t="s">
         <v>71</v>
@@ -4299,16 +4299,16 @@
         <v>33</v>
       </c>
       <c r="E78">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="F78">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="G78">
-        <v>0</v>
+        <v>99.5</v>
       </c>
       <c r="H78">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="I78" t="b">
         <v>1</v>
@@ -4317,15 +4317,15 @@
         <v>195</v>
       </c>
       <c r="K78" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B79" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="C79" t="s">
         <v>71</v>
@@ -4334,33 +4334,33 @@
         <v>33</v>
       </c>
       <c r="E79">
-        <v>0.5</v>
-      </c>
-      <c r="F79" t="s">
+        <v>0</v>
+      </c>
+      <c r="F79">
+        <v>15</v>
+      </c>
+      <c r="G79">
+        <v>0</v>
+      </c>
+      <c r="H79">
         <v>5</v>
       </c>
-      <c r="G79">
-        <v>1</v>
-      </c>
-      <c r="H79" t="s">
-        <v>5</v>
-      </c>
       <c r="I79" t="b">
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>208</v>
+        <v>195</v>
       </c>
       <c r="K79" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>21</v>
+        <v>148</v>
       </c>
       <c r="B80" t="s">
-        <v>22</v>
+        <v>149</v>
       </c>
       <c r="C80" t="s">
         <v>71</v>
@@ -4369,33 +4369,33 @@
         <v>33</v>
       </c>
       <c r="E80">
-        <v>0</v>
-      </c>
-      <c r="F80">
-        <v>0</v>
+        <v>0.5</v>
+      </c>
+      <c r="F80" t="s">
+        <v>5</v>
       </c>
       <c r="G80">
-        <v>0</v>
-      </c>
-      <c r="H80">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H80" t="s">
+        <v>5</v>
       </c>
       <c r="I80" t="b">
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>158</v>
+        <v>208</v>
       </c>
       <c r="K80" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B81" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C81" t="s">
         <v>71</v>
@@ -4404,33 +4404,33 @@
         <v>33</v>
       </c>
       <c r="E81">
-        <v>14.5</v>
+        <v>0</v>
       </c>
       <c r="F81">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G81">
-        <v>26.1</v>
+        <v>0</v>
       </c>
       <c r="H81">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I81" t="b">
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>208</v>
+        <v>158</v>
       </c>
       <c r="K81" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
-        <v>13</v>
-      </c>
       <c r="B82" t="s">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="C82" t="s">
         <v>71</v>
@@ -4439,134 +4439,169 @@
         <v>33</v>
       </c>
       <c r="E82">
+        <v>14.5</v>
+      </c>
+      <c r="F82">
+        <v>100</v>
+      </c>
+      <c r="G82">
+        <v>26.1</v>
+      </c>
+      <c r="H82">
+        <v>100</v>
+      </c>
+      <c r="I82" t="b">
+        <v>1</v>
+      </c>
+      <c r="J82" t="s">
+        <v>208</v>
+      </c>
+      <c r="K82" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
+        <v>13</v>
+      </c>
+      <c r="B83" t="s">
+        <v>14</v>
+      </c>
+      <c r="C83" t="s">
+        <v>71</v>
+      </c>
+      <c r="D83" t="s">
+        <v>33</v>
+      </c>
+      <c r="E83">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="F82">
+      <c r="F83">
         <v>8.0000000000000004E-4</v>
       </c>
-      <c r="G82">
+      <c r="G83">
         <v>2.0000000000000001E-4</v>
       </c>
-      <c r="H82">
+      <c r="H83">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="I82" t="b">
-        <v>1</v>
-      </c>
-      <c r="J82" t="s">
+      <c r="I83" t="b">
+        <v>1</v>
+      </c>
+      <c r="J83" t="s">
         <v>226</v>
       </c>
-      <c r="K82" t="s">
+      <c r="K83" t="s">
         <v>225</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A84" t="s">
         <v>18</v>
       </c>
-      <c r="B83" t="s">
+      <c r="B84" t="s">
         <v>17</v>
-      </c>
-      <c r="C83" t="s">
-        <v>217</v>
-      </c>
-      <c r="D83" t="s">
-        <v>33</v>
-      </c>
-      <c r="E83">
-        <v>5</v>
-      </c>
-      <c r="F83">
-        <v>100</v>
-      </c>
-      <c r="G83">
-        <v>20</v>
-      </c>
-      <c r="H83">
-        <v>100</v>
-      </c>
-      <c r="I83" t="b">
-        <v>1</v>
-      </c>
-      <c r="J83" t="s">
-        <v>208</v>
-      </c>
-      <c r="K83" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>24</v>
-      </c>
-      <c r="B84" t="s">
-        <v>23</v>
       </c>
       <c r="C84" t="s">
         <v>217</v>
       </c>
       <c r="D84" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="E84">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F84">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="G84">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H84">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="I84" t="b">
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>171</v>
+        <v>208</v>
       </c>
       <c r="K84" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
       <c r="B85" t="s">
-        <v>198</v>
+        <v>23</v>
       </c>
       <c r="C85" t="s">
         <v>217</v>
       </c>
       <c r="D85" t="s">
-        <v>33</v>
+        <v>79</v>
       </c>
       <c r="E85">
+        <v>0</v>
+      </c>
+      <c r="F85">
+        <v>95</v>
+      </c>
+      <c r="G85">
+        <v>0</v>
+      </c>
+      <c r="H85">
+        <v>80</v>
+      </c>
+      <c r="I85" t="b">
+        <v>1</v>
+      </c>
+      <c r="J85" t="s">
+        <v>171</v>
+      </c>
+      <c r="K85" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A86" t="s">
+        <v>60</v>
+      </c>
+      <c r="B86" t="s">
+        <v>198</v>
+      </c>
+      <c r="C86" t="s">
+        <v>217</v>
+      </c>
+      <c r="D86" t="s">
+        <v>33</v>
+      </c>
+      <c r="E86">
         <v>90</v>
       </c>
-      <c r="F85">
+      <c r="F86">
         <v>100</v>
       </c>
-      <c r="G85">
+      <c r="G86">
         <v>95</v>
       </c>
-      <c r="H85">
+      <c r="H86">
         <v>100</v>
       </c>
-      <c r="I85" t="b">
-        <v>1</v>
-      </c>
-      <c r="J85" t="s">
+      <c r="I86" t="b">
+        <v>1</v>
+      </c>
+      <c r="J86" t="s">
         <v>208</v>
       </c>
-      <c r="K85" t="s">
+      <c r="K86" t="s">
         <v>60</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K83" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K84" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Added metric definitions to ex_dsc_coverage_metrics.py
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48CEC0F6-FB25-4D9B-8854-69DBAF544F08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{246DBD04-7EE6-47A7-8A4B-9845865B77B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -632,9 +632,6 @@
     <t>ex_dsc_coverage_wholegenome</t>
   </si>
   <si>
-    <t>Percentage of genome with 1. MS depth &gt; half MS depth theshold and 2. EX duplex depth &gt; 0</t>
-  </si>
-  <si>
     <t>^Pairs that were too short:\s+\d+\s+\((?P&lt;percent&gt;[\d.]+)%\)$</t>
   </si>
   <si>
@@ -744,6 +741,9 @@
   </si>
   <si>
     <t>Reads with a length of zero after trimming (e.g. blank ligation)</t>
+  </si>
+  <si>
+    <t>Percentage of all sequenced bases with 1. MS depth &gt; half MS depth theshold and 2. EX duplex depth &gt; 0</t>
   </si>
 </sst>
 </file>
@@ -1614,19 +1614,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
   <dimension ref="A1:K86"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.1796875" customWidth="1"/>
-    <col min="2" max="2" width="87.26953125" customWidth="1"/>
-    <col min="3" max="4" width="35.26953125" customWidth="1"/>
+    <col min="1" max="1" width="35.140625" customWidth="1"/>
+    <col min="2" max="2" width="87.28515625" customWidth="1"/>
+    <col min="3" max="4" width="35.28515625" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.81640625" customWidth="1"/>
-    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="76.81640625" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="76.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>40</v>
       </c>
@@ -1661,7 +1661,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>44</v>
       </c>
@@ -1690,7 +1690,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>45</v>
       </c>
@@ -1725,12 +1725,12 @@
         <v>74</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C4" t="s">
         <v>61</v>
@@ -1760,7 +1760,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>55</v>
       </c>
@@ -1789,7 +1789,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>54</v>
       </c>
@@ -1824,7 +1824,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>56</v>
       </c>
@@ -1853,7 +1853,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>57</v>
       </c>
@@ -1888,7 +1888,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>30</v>
       </c>
@@ -1923,7 +1923,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>31</v>
       </c>
@@ -1958,7 +1958,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -1993,7 +1993,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -2028,7 +2028,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>117</v>
       </c>
@@ -2063,7 +2063,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>118</v>
       </c>
@@ -2098,7 +2098,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>115</v>
       </c>
@@ -2133,7 +2133,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>116</v>
       </c>
@@ -2168,7 +2168,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>107</v>
       </c>
@@ -2203,7 +2203,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>108</v>
       </c>
@@ -2238,12 +2238,12 @@
         <v>176</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B19" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C19" t="s">
         <v>67</v>
@@ -2273,12 +2273,12 @@
         <v>174</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>231</v>
+      </c>
+      <c r="B20" t="s">
         <v>232</v>
-      </c>
-      <c r="B20" t="s">
-        <v>233</v>
       </c>
       <c r="C20" t="s">
         <v>67</v>
@@ -2308,7 +2308,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>86</v>
       </c>
@@ -2343,7 +2343,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>87</v>
       </c>
@@ -2378,7 +2378,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>88</v>
       </c>
@@ -2413,7 +2413,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>89</v>
       </c>
@@ -2448,7 +2448,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>90</v>
       </c>
@@ -2483,7 +2483,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>91</v>
       </c>
@@ -2518,7 +2518,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>92</v>
       </c>
@@ -2553,7 +2553,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>93</v>
       </c>
@@ -2588,7 +2588,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>95</v>
       </c>
@@ -2617,13 +2617,13 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="K29" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>144</v>
       </c>
@@ -2655,10 +2655,10 @@
         <v>163</v>
       </c>
       <c r="K30" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>143</v>
       </c>
@@ -2690,10 +2690,10 @@
         <v>164</v>
       </c>
       <c r="K31" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>142</v>
       </c>
@@ -2725,10 +2725,10 @@
         <v>165</v>
       </c>
       <c r="K32" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -2763,7 +2763,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>6</v>
       </c>
@@ -2798,7 +2798,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>7</v>
       </c>
@@ -2833,7 +2833,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>8</v>
       </c>
@@ -2868,7 +2868,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>9</v>
       </c>
@@ -2903,7 +2903,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>10</v>
       </c>
@@ -2938,7 +2938,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>75</v>
       </c>
@@ -2967,13 +2967,13 @@
         <v>1</v>
       </c>
       <c r="J39" t="s">
+        <v>203</v>
+      </c>
+      <c r="K39" t="s">
         <v>204</v>
       </c>
-      <c r="K39" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>27</v>
       </c>
@@ -3002,7 +3002,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>35</v>
       </c>
@@ -3037,12 +3037,12 @@
         <v>74</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C42" t="s">
         <v>62</v>
@@ -3072,7 +3072,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>52</v>
       </c>
@@ -3101,7 +3101,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>47</v>
       </c>
@@ -3136,12 +3136,12 @@
         <v>74</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>48</v>
       </c>
       <c r="B45" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C45" t="s">
         <v>62</v>
@@ -3171,12 +3171,12 @@
         <v>74</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>49</v>
       </c>
       <c r="B46" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C46" t="s">
         <v>62</v>
@@ -3206,7 +3206,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>28</v>
       </c>
@@ -3241,7 +3241,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>29</v>
       </c>
@@ -3276,7 +3276,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>111</v>
       </c>
@@ -3311,7 +3311,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>112</v>
       </c>
@@ -3346,7 +3346,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>113</v>
       </c>
@@ -3381,7 +3381,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>114</v>
       </c>
@@ -3416,7 +3416,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>110</v>
       </c>
@@ -3451,7 +3451,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>119</v>
       </c>
@@ -3486,7 +3486,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>120</v>
       </c>
@@ -3521,7 +3521,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>121</v>
       </c>
@@ -3556,12 +3556,12 @@
         <v>172</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B57" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C57" t="s">
         <v>66</v>
@@ -3591,12 +3591,12 @@
         <v>174</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B58" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C58" t="s">
         <v>66</v>
@@ -3626,7 +3626,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>122</v>
       </c>
@@ -3661,7 +3661,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>123</v>
       </c>
@@ -3696,7 +3696,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>124</v>
       </c>
@@ -3731,7 +3731,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>125</v>
       </c>
@@ -3766,7 +3766,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>126</v>
       </c>
@@ -3801,7 +3801,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>127</v>
       </c>
@@ -3836,7 +3836,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>128</v>
       </c>
@@ -3871,7 +3871,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>129</v>
       </c>
@@ -3906,7 +3906,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>76</v>
       </c>
@@ -3938,10 +3938,10 @@
         <v>170</v>
       </c>
       <c r="K67" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>138</v>
       </c>
@@ -3976,12 +3976,12 @@
         <v>189</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>217</v>
+      </c>
+      <c r="B69" t="s">
         <v>218</v>
-      </c>
-      <c r="B69" t="s">
-        <v>219</v>
       </c>
       <c r="C69" t="s">
         <v>68</v>
@@ -4005,18 +4005,18 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="K69" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>233</v>
+      </c>
+      <c r="B70" t="s">
         <v>234</v>
-      </c>
-      <c r="B70" t="s">
-        <v>235</v>
       </c>
       <c r="C70" t="s">
         <v>68</v>
@@ -4040,12 +4040,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>77</v>
       </c>
       <c r="B71" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C71" t="s">
         <v>68</v>
@@ -4069,18 +4069,18 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="K71" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>78</v>
       </c>
       <c r="B72" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C72" t="s">
         <v>68</v>
@@ -4104,13 +4104,13 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="K72" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>81</v>
       </c>
@@ -4142,10 +4142,10 @@
         <v>156</v>
       </c>
       <c r="K73" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>80</v>
       </c>
@@ -4177,10 +4177,10 @@
         <v>156</v>
       </c>
       <c r="K74" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>82</v>
       </c>
@@ -4212,10 +4212,10 @@
         <v>157</v>
       </c>
       <c r="K75" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>153</v>
       </c>
@@ -4250,12 +4250,12 @@
         <v>192</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>141</v>
       </c>
       <c r="B77" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C77" t="s">
         <v>71</v>
@@ -4279,13 +4279,13 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K77" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>147</v>
       </c>
@@ -4320,7 +4320,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>146</v>
       </c>
@@ -4355,7 +4355,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>148</v>
       </c>
@@ -4384,13 +4384,13 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="K80" t="s">
         <v>196</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>21</v>
       </c>
@@ -4425,7 +4425,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>19</v>
       </c>
@@ -4454,13 +4454,13 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="K82" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>13</v>
       </c>
@@ -4489,13 +4489,13 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="K83" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>18</v>
       </c>
@@ -4503,7 +4503,7 @@
         <v>17</v>
       </c>
       <c r="C84" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D84" t="s">
         <v>33</v>
@@ -4524,13 +4524,13 @@
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="K84" t="s">
         <v>197</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>24</v>
       </c>
@@ -4538,7 +4538,7 @@
         <v>23</v>
       </c>
       <c r="C85" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D85" t="s">
         <v>79</v>
@@ -4562,18 +4562,18 @@
         <v>171</v>
       </c>
       <c r="K85" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.35">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>60</v>
       </c>
       <c r="B86" t="s">
-        <v>198</v>
+        <v>235</v>
       </c>
       <c r="C86" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="D86" t="s">
         <v>33</v>
@@ -4594,7 +4594,7 @@
         <v>1</v>
       </c>
       <c r="J86" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="K86" t="s">
         <v>60</v>

</xml_diff>

<commit_message>
Moved memory and thread allocation into config
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{246DBD04-7EE6-47A7-8A4B-9845865B77B6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4581BEA1-8E85-456F-9A7A-AB4B33563959}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -632,9 +632,6 @@
     <t>ex_dsc_coverage_wholegenome</t>
   </si>
   <si>
-    <t>^Pairs that were too short:\s+\d+\s+\((?P&lt;percent&gt;[\d.]+)%\)$</t>
-  </si>
-  <si>
     <t>^\d+ \+ 0 mapped \((?P&lt;percent&gt;[\d.]+)% : N/A\)$</t>
   </si>
   <si>
@@ -744,6 +741,9 @@
   </si>
   <si>
     <t>Percentage of all sequenced bases with 1. MS depth &gt; half MS depth theshold and 2. EX duplex depth &gt; 0</t>
+  </si>
+  <si>
+    <t>^Pairs that were too short:\s+[\d,]+\s+\((?P&lt;percent&gt;[\d.]+)%\)\s*$</t>
   </si>
 </sst>
 </file>
@@ -1227,8 +1227,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1730,7 +1731,7 @@
         <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C4" t="s">
         <v>61</v>
@@ -2240,10 +2241,10 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B19" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C19" t="s">
         <v>67</v>
@@ -2275,10 +2276,10 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>230</v>
+      </c>
+      <c r="B20" t="s">
         <v>231</v>
-      </c>
-      <c r="B20" t="s">
-        <v>232</v>
       </c>
       <c r="C20" t="s">
         <v>67</v>
@@ -2617,10 +2618,10 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>209</v>
-      </c>
-      <c r="K29" t="s">
-        <v>198</v>
+        <v>208</v>
+      </c>
+      <c r="K29" s="1" t="s">
+        <v>235</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -2655,7 +2656,7 @@
         <v>163</v>
       </c>
       <c r="K30" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -2690,7 +2691,7 @@
         <v>164</v>
       </c>
       <c r="K31" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
@@ -2725,7 +2726,7 @@
         <v>165</v>
       </c>
       <c r="K32" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -2967,10 +2968,10 @@
         <v>1</v>
       </c>
       <c r="J39" t="s">
+        <v>202</v>
+      </c>
+      <c r="K39" t="s">
         <v>203</v>
-      </c>
-      <c r="K39" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
@@ -3042,7 +3043,7 @@
         <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C42" t="s">
         <v>62</v>
@@ -3141,7 +3142,7 @@
         <v>48</v>
       </c>
       <c r="B45" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C45" t="s">
         <v>62</v>
@@ -3176,7 +3177,7 @@
         <v>49</v>
       </c>
       <c r="B46" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C46" t="s">
         <v>62</v>
@@ -3558,10 +3559,10 @@
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B57" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C57" t="s">
         <v>66</v>
@@ -3593,10 +3594,10 @@
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B58" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C58" t="s">
         <v>66</v>
@@ -3938,7 +3939,7 @@
         <v>170</v>
       </c>
       <c r="K67" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
@@ -3978,10 +3979,10 @@
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>216</v>
+      </c>
+      <c r="B69" t="s">
         <v>217</v>
-      </c>
-      <c r="B69" t="s">
-        <v>218</v>
       </c>
       <c r="C69" t="s">
         <v>68</v>
@@ -4005,18 +4006,18 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="K69" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>232</v>
+      </c>
+      <c r="B70" t="s">
         <v>233</v>
-      </c>
-      <c r="B70" t="s">
-        <v>234</v>
       </c>
       <c r="C70" t="s">
         <v>68</v>
@@ -4045,7 +4046,7 @@
         <v>77</v>
       </c>
       <c r="B71" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C71" t="s">
         <v>68</v>
@@ -4069,10 +4070,10 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="K71" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
@@ -4080,7 +4081,7 @@
         <v>78</v>
       </c>
       <c r="B72" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C72" t="s">
         <v>68</v>
@@ -4104,10 +4105,10 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="K72" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
@@ -4142,7 +4143,7 @@
         <v>156</v>
       </c>
       <c r="K73" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
@@ -4177,7 +4178,7 @@
         <v>156</v>
       </c>
       <c r="K74" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
@@ -4212,7 +4213,7 @@
         <v>157</v>
       </c>
       <c r="K75" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
@@ -4255,7 +4256,7 @@
         <v>141</v>
       </c>
       <c r="B77" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C77" t="s">
         <v>71</v>
@@ -4279,10 +4280,10 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="K77" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
@@ -4384,7 +4385,7 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K80" t="s">
         <v>196</v>
@@ -4454,7 +4455,7 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K82" t="s">
         <v>19</v>
@@ -4489,10 +4490,10 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="K83" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
@@ -4503,7 +4504,7 @@
         <v>17</v>
       </c>
       <c r="C84" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D84" t="s">
         <v>33</v>
@@ -4524,7 +4525,7 @@
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K84" t="s">
         <v>197</v>
@@ -4538,7 +4539,7 @@
         <v>23</v>
       </c>
       <c r="C85" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D85" t="s">
         <v>79</v>
@@ -4562,7 +4563,7 @@
         <v>171</v>
       </c>
       <c r="K85" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
@@ -4570,10 +4571,10 @@
         <v>60</v>
       </c>
       <c r="B86" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C86" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D86" t="s">
         <v>33</v>
@@ -4594,7 +4595,7 @@
         <v>1</v>
       </c>
       <c r="J86" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K86" t="s">
         <v>60</v>

</xml_diff>

<commit_message>
Removex extra columns from sample metadata
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4581BEA1-8E85-456F-9A7A-AB4B33563959}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{386C84DA-2C0B-4F51-BD8E-4F1FAD0C2E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -494,9 +494,6 @@
     <t>Fraction of mapped reads that are marked as duplicates</t>
   </si>
   <si>
-    <t>Percentage of reads lost from creation of DSC (beyond expected halving)</t>
-  </si>
-  <si>
     <t>ex_reads_lost_call_dsc</t>
   </si>
   <si>
@@ -744,6 +741,9 @@
   </si>
   <si>
     <t>^Pairs that were too short:\s+[\d,]+\s+\((?P&lt;percent&gt;[\d.]+)%\)\s*$</t>
+  </si>
+  <si>
+    <t>Percentage of reads lost from creation of DSC</t>
   </si>
 </sst>
 </file>
@@ -1656,10 +1656,10 @@
         <v>39</v>
       </c>
       <c r="J1" t="s">
+        <v>153</v>
+      </c>
+      <c r="K1" t="s">
         <v>154</v>
-      </c>
-      <c r="K1" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -1731,7 +1731,7 @@
         <v>46</v>
       </c>
       <c r="B4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C4" t="s">
         <v>61</v>
@@ -1988,10 +1988,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K11" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -2023,10 +2023,10 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K12" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -2058,10 +2058,10 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K13" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -2093,10 +2093,10 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K14" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -2128,10 +2128,10 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K15" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -2163,10 +2163,10 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K16" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -2198,10 +2198,10 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K17" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -2233,18 +2233,18 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K18" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B19" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C19" t="s">
         <v>67</v>
@@ -2268,18 +2268,18 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K19" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>229</v>
+      </c>
+      <c r="B20" t="s">
         <v>230</v>
-      </c>
-      <c r="B20" t="s">
-        <v>231</v>
       </c>
       <c r="C20" t="s">
         <v>67</v>
@@ -2303,10 +2303,10 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K20" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -2338,10 +2338,10 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K21" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -2373,10 +2373,10 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K22" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -2408,10 +2408,10 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K23" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -2443,10 +2443,10 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K24" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -2478,10 +2478,10 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K25" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -2513,10 +2513,10 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K26" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -2548,10 +2548,10 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K27" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -2583,10 +2583,10 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K28" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -2618,10 +2618,10 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -2653,10 +2653,10 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K30" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -2688,10 +2688,10 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K31" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
@@ -2723,10 +2723,10 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K32" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -2758,10 +2758,10 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="K33" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -2793,10 +2793,10 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="K34" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -2828,10 +2828,10 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="K35" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -2863,10 +2863,10 @@
         <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="K36" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
@@ -2898,10 +2898,10 @@
         <v>1</v>
       </c>
       <c r="J37" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="K37" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
@@ -2933,10 +2933,10 @@
         <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="K38" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
@@ -2968,10 +2968,10 @@
         <v>1</v>
       </c>
       <c r="J39" t="s">
+        <v>201</v>
+      </c>
+      <c r="K39" t="s">
         <v>202</v>
-      </c>
-      <c r="K39" t="s">
-        <v>203</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
@@ -3043,7 +3043,7 @@
         <v>43</v>
       </c>
       <c r="B42" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C42" t="s">
         <v>62</v>
@@ -3142,7 +3142,7 @@
         <v>48</v>
       </c>
       <c r="B45" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C45" t="s">
         <v>62</v>
@@ -3177,7 +3177,7 @@
         <v>49</v>
       </c>
       <c r="B46" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C46" t="s">
         <v>62</v>
@@ -3306,10 +3306,10 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="K49" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3341,10 +3341,10 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K50" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
@@ -3376,10 +3376,10 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="K51" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
@@ -3411,10 +3411,10 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K52" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
@@ -3446,10 +3446,10 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="K53" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
@@ -3481,10 +3481,10 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K54" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
@@ -3516,10 +3516,10 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="K55" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
@@ -3551,18 +3551,18 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K56" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B57" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C57" t="s">
         <v>66</v>
@@ -3586,18 +3586,18 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K57" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B58" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C58" t="s">
         <v>66</v>
@@ -3621,10 +3621,10 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K58" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
@@ -3656,10 +3656,10 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K59" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
@@ -3691,10 +3691,10 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K60" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
@@ -3726,10 +3726,10 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K61" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
@@ -3761,10 +3761,10 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K62" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
@@ -3796,10 +3796,10 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K63" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
@@ -3831,10 +3831,10 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K64" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
@@ -3866,10 +3866,10 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="K65" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
@@ -3901,10 +3901,10 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="K66" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
@@ -3936,10 +3936,10 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="K67" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
@@ -3971,18 +3971,18 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="K68" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>215</v>
+      </c>
+      <c r="B69" t="s">
         <v>216</v>
-      </c>
-      <c r="B69" t="s">
-        <v>217</v>
       </c>
       <c r="C69" t="s">
         <v>68</v>
@@ -4006,18 +4006,18 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="K69" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>231</v>
+      </c>
+      <c r="B70" t="s">
         <v>232</v>
-      </c>
-      <c r="B70" t="s">
-        <v>233</v>
       </c>
       <c r="C70" t="s">
         <v>68</v>
@@ -4046,7 +4046,7 @@
         <v>77</v>
       </c>
       <c r="B71" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C71" t="s">
         <v>68</v>
@@ -4070,10 +4070,10 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="K71" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
@@ -4081,7 +4081,7 @@
         <v>78</v>
       </c>
       <c r="B72" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C72" t="s">
         <v>68</v>
@@ -4105,10 +4105,10 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="K72" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
@@ -4140,10 +4140,10 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="K73" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
@@ -4175,10 +4175,10 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="K74" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
@@ -4210,18 +4210,18 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K75" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B76" t="s">
-        <v>152</v>
+        <v>235</v>
       </c>
       <c r="C76" t="s">
         <v>71</v>
@@ -4230,25 +4230,25 @@
         <v>33</v>
       </c>
       <c r="E76">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F76">
-        <v>10</v>
+        <v>55</v>
       </c>
       <c r="G76">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H76">
-        <v>5</v>
+        <v>52.5</v>
       </c>
       <c r="I76" t="b">
         <v>1</v>
       </c>
       <c r="J76" t="s">
+        <v>190</v>
+      </c>
+      <c r="K76" t="s">
         <v>191</v>
-      </c>
-      <c r="K76" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
@@ -4256,7 +4256,7 @@
         <v>141</v>
       </c>
       <c r="B77" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C77" t="s">
         <v>71</v>
@@ -4280,10 +4280,10 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="K77" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
@@ -4315,10 +4315,10 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="K78" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
@@ -4350,10 +4350,10 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="K79" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
@@ -4385,10 +4385,10 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="K80" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
@@ -4420,10 +4420,10 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K81" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
@@ -4455,7 +4455,7 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="K82" t="s">
         <v>19</v>
@@ -4490,10 +4490,10 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="K83" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
@@ -4504,7 +4504,7 @@
         <v>17</v>
       </c>
       <c r="C84" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D84" t="s">
         <v>33</v>
@@ -4525,10 +4525,10 @@
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="K84" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
@@ -4539,7 +4539,7 @@
         <v>23</v>
       </c>
       <c r="C85" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D85" t="s">
         <v>79</v>
@@ -4560,10 +4560,10 @@
         <v>1</v>
       </c>
       <c r="J85" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="K85" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
@@ -4571,10 +4571,10 @@
         <v>60</v>
       </c>
       <c r="B86" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C86" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="D86" t="s">
         <v>33</v>
@@ -4595,7 +4595,7 @@
         <v>1</v>
       </c>
       <c r="J86" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="K86" t="s">
         <v>60</v>

</xml_diff>

<commit_message>
Rescoped ex_total_read_loss to post-demux to end
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{386C84DA-2C0B-4F51-BD8E-4F1FAD0C2E3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C43745-A865-4EAD-A173-B47558A97236}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -4542,7 +4542,7 @@
         <v>214</v>
       </c>
       <c r="D85" t="s">
-        <v>79</v>
+        <v>33</v>
       </c>
       <c r="E85">
         <v>0</v>

</xml_diff>

<commit_message>
Created ex_demux_counts_and_gini.py, added disclaimer for ex_reads_lost_demux metric
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29C43745-A865-4EAD-A173-B47558A97236}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75CD41AF-3E45-4B8B-A392-6DDC523A23E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -161,9 +161,6 @@
     <t>Name</t>
   </si>
   <si>
-    <t>Quantity of DNA (ng) required to run assay &amp; QCs</t>
-  </si>
-  <si>
     <t>Variability in DNA extraction yield (normalised interquartile range). UL of 95% CI must meet target.</t>
   </si>
   <si>
@@ -212,9 +209,6 @@
     <t>ms_ligated_DNA_yield_variability</t>
   </si>
   <si>
-    <t>Quantity of DNA (ng) after adaptor ligation</t>
-  </si>
-  <si>
     <t>Variability in DNA quantity post adaptor ligation (normalised interquartile range). UL of 95% CI must meet target.</t>
   </si>
   <si>
@@ -287,9 +281,6 @@
     <t>ex_insert_size_initial_alignment</t>
   </si>
   <si>
-    <t>Percentage of reads that are lost during demultiplexing</t>
-  </si>
-  <si>
     <t>Mean length of the largest peak on the tape station report prior to sequencing</t>
   </si>
   <si>
@@ -545,9 +536,6 @@
     <t>_r2_fastqc_filter_metrics_summary.json</t>
   </si>
   <si>
-    <t>_demux_metrics.txt</t>
-  </si>
-  <si>
     <t>_total_read_loss.json</t>
   </si>
   <si>
@@ -605,9 +593,6 @@
     <t>gini_coefficient</t>
   </si>
   <si>
-    <t>_demux_metrics_gini.json</t>
-  </si>
-  <si>
     <t>_call_dsc_metrics.json</t>
   </si>
   <si>
@@ -665,9 +650,6 @@
     <t>^(\S+\t){9}(?P&lt;value&gt;[\d.]+)</t>
   </si>
   <si>
-    <t>^Pairs discarded as untrimmed:\s+\d+\s+\((?P&lt;value&gt;[\d.]+)%\)</t>
-  </si>
-  <si>
     <t>Percentage of fragments that fall within the expected size range on gel elextrophoresis (10,000-50,000 bp)</t>
   </si>
   <si>
@@ -744,6 +726,24 @@
   </si>
   <si>
     <t>Percentage of reads lost from creation of DSC</t>
+  </si>
+  <si>
+    <t>Quantity of DNA (ng) after adaptor ligation (ng/uL concentration x ul sample remaining after Qubit)</t>
+  </si>
+  <si>
+    <t>Quantity of DNA (ng) after enzymatic fragmentation (ng/uL concentration x ul sample remaining after Qubit)</t>
+  </si>
+  <si>
+    <t>Quantity of DNA (ng) required to run assay &amp; QCs (ng/uL concentration x ul sample remaining after Qubit)</t>
+  </si>
+  <si>
+    <t>_demux_counts_and_gini.json</t>
+  </si>
+  <si>
+    <t>pct_reads_lost_demux</t>
+  </si>
+  <si>
+    <t>Percentage of reads that are lost during demultiplexing (applicable only when all samples in lane are demuxed)</t>
   </si>
 </sst>
 </file>
@@ -1618,7 +1618,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" customWidth="1"/>
-    <col min="2" max="2" width="87.28515625" customWidth="1"/>
+    <col min="2" max="2" width="96.85546875" customWidth="1"/>
     <col min="3" max="4" width="35.28515625" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
@@ -1656,21 +1656,21 @@
         <v>39</v>
       </c>
       <c r="J1" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="K1" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B2" t="s">
-        <v>41</v>
+        <v>232</v>
       </c>
       <c r="C2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D2" t="s">
         <v>33</v>
@@ -1685,21 +1685,21 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D3" t="s">
         <v>34</v>
@@ -1720,21 +1720,21 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B4" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
       <c r="C4" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="D4" t="s">
         <v>33</v>
@@ -1755,21 +1755,21 @@
         <v>0</v>
       </c>
       <c r="J4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K4" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B5" t="s">
-        <v>50</v>
+        <v>231</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D5" t="s">
         <v>33</v>
@@ -1784,21 +1784,21 @@
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K5" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C6" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D6" t="s">
         <v>34</v>
@@ -1819,21 +1819,21 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K6" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B7" t="s">
-        <v>58</v>
+        <v>230</v>
       </c>
       <c r="C7" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D7" t="s">
         <v>33</v>
@@ -1848,21 +1848,21 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>56</v>
+      </c>
+      <c r="B8" t="s">
         <v>57</v>
       </c>
-      <c r="B8" t="s">
-        <v>59</v>
-      </c>
       <c r="C8" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D8" t="s">
         <v>34</v>
@@ -1883,10 +1883,10 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K8" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -1894,10 +1894,10 @@
         <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="C9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D9" t="s">
         <v>33</v>
@@ -1918,10 +1918,10 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K9" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -1929,10 +1929,10 @@
         <v>31</v>
       </c>
       <c r="B10" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="C10" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="D10" t="s">
         <v>33</v>
@@ -1953,10 +1953,10 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K10" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -1964,10 +1964,10 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C11" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D11" t="s">
         <v>33</v>
@@ -1988,10 +1988,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="K11" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1999,10 +1999,10 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D12" t="s">
         <v>33</v>
@@ -2023,21 +2023,21 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="K12" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B13" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C13" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D13" t="s">
         <v>33</v>
@@ -2058,21 +2058,21 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="K13" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B14" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C14" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D14" t="s">
         <v>33</v>
@@ -2093,21 +2093,21 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="K14" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B15" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C15" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D15" t="s">
         <v>33</v>
@@ -2128,21 +2128,21 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="K15" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B16" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C16" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D16" t="s">
         <v>33</v>
@@ -2163,21 +2163,21 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="K16" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B17" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C17" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D17" t="s">
         <v>33</v>
@@ -2198,21 +2198,21 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="K17" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B18" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C18" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D18" t="s">
         <v>33</v>
@@ -2233,21 +2233,21 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="K18" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="B19" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="C19" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D19" t="s">
         <v>33</v>
@@ -2268,21 +2268,21 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="K19" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="B20" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="C20" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="D20" t="s">
         <v>33</v>
@@ -2303,21 +2303,21 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="K20" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B21" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C21" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D21" t="s">
         <v>33</v>
@@ -2338,21 +2338,21 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="K21" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B22" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C22" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D22" t="s">
         <v>33</v>
@@ -2373,21 +2373,21 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="K22" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B23" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C23" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D23" t="s">
         <v>33</v>
@@ -2408,21 +2408,21 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="K23" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B24" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C24" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D24" t="s">
         <v>33</v>
@@ -2443,21 +2443,21 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="K24" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B25" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C25" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D25" t="s">
         <v>33</v>
@@ -2478,21 +2478,21 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="K25" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B26" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C26" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D26" t="s">
         <v>33</v>
@@ -2513,21 +2513,21 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="K26" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B27" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C27" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D27" t="s">
         <v>33</v>
@@ -2548,21 +2548,21 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="K27" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="B28" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C28" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D28" t="s">
         <v>33</v>
@@ -2583,21 +2583,21 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="K28" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="B29" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="C29" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="D29" t="s">
         <v>33</v>
@@ -2618,21 +2618,21 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="B30" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="C30" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D30" t="s">
         <v>33</v>
@@ -2653,21 +2653,21 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="K30" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B31" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C31" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D31" t="s">
         <v>33</v>
@@ -2688,21 +2688,21 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="K31" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="B32" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C32" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D32" t="s">
         <v>33</v>
@@ -2723,10 +2723,10 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="K32" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -2734,10 +2734,10 @@
         <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="C33" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D33" t="s">
         <v>33</v>
@@ -2758,10 +2758,10 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="K33" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -2769,10 +2769,10 @@
         <v>6</v>
       </c>
       <c r="B34" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C34" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D34" t="s">
         <v>33</v>
@@ -2793,10 +2793,10 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="K34" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -2804,10 +2804,10 @@
         <v>7</v>
       </c>
       <c r="B35" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C35" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D35" t="s">
         <v>33</v>
@@ -2828,10 +2828,10 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="K35" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -2839,10 +2839,10 @@
         <v>8</v>
       </c>
       <c r="B36" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C36" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D36" t="s">
         <v>33</v>
@@ -2863,10 +2863,10 @@
         <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="K36" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
@@ -2874,10 +2874,10 @@
         <v>9</v>
       </c>
       <c r="B37" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C37" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D37" t="s">
         <v>33</v>
@@ -2898,10 +2898,10 @@
         <v>1</v>
       </c>
       <c r="J37" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="K37" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
@@ -2909,10 +2909,10 @@
         <v>10</v>
       </c>
       <c r="B38" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C38" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="D38" t="s">
         <v>33</v>
@@ -2933,21 +2933,21 @@
         <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="K38" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B39" t="s">
         <v>4</v>
       </c>
       <c r="C39" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D39" t="s">
         <v>33</v>
@@ -2968,10 +2968,10 @@
         <v>1</v>
       </c>
       <c r="J39" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="K39" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
@@ -2979,10 +2979,10 @@
         <v>27</v>
       </c>
       <c r="B40" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C40" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D40" t="s">
         <v>33</v>
@@ -2997,10 +2997,10 @@
         <v>0</v>
       </c>
       <c r="J40" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K40" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
@@ -3008,10 +3008,10 @@
         <v>35</v>
       </c>
       <c r="B41" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C41" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D41" t="s">
         <v>34</v>
@@ -3032,21 +3032,21 @@
         <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K41" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B42" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
       <c r="C42" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D42" t="s">
         <v>33</v>
@@ -3067,21 +3067,21 @@
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K42" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>51</v>
+      </c>
+      <c r="B43" t="s">
         <v>52</v>
       </c>
-      <c r="B43" t="s">
-        <v>53</v>
-      </c>
       <c r="C43" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D43" t="s">
         <v>33</v>
@@ -3096,21 +3096,21 @@
         <v>0</v>
       </c>
       <c r="J43" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K43" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B44" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C44" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D44" t="s">
         <v>34</v>
@@ -3131,21 +3131,21 @@
         <v>0</v>
       </c>
       <c r="J44" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K44" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B45" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
       <c r="C45" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D45" t="s">
         <v>33</v>
@@ -3166,21 +3166,21 @@
         <v>0</v>
       </c>
       <c r="J45" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K45" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B46" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
       <c r="C46" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D46" t="s">
         <v>33</v>
@@ -3201,10 +3201,10 @@
         <v>0</v>
       </c>
       <c r="J46" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K46" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
@@ -3215,7 +3215,7 @@
         <v>25</v>
       </c>
       <c r="C47" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D47" t="s">
         <v>33</v>
@@ -3236,10 +3236,10 @@
         <v>0</v>
       </c>
       <c r="J47" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K47" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
@@ -3250,7 +3250,7 @@
         <v>26</v>
       </c>
       <c r="C48" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="D48" t="s">
         <v>33</v>
@@ -3271,24 +3271,24 @@
         <v>0</v>
       </c>
       <c r="J48" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="K48" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B49" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C49" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D49" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E49">
         <v>35</v>
@@ -3306,24 +3306,24 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="K49" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B50" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C50" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D50" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E50">
         <v>35</v>
@@ -3341,24 +3341,24 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="K50" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B51" t="s">
         <v>15</v>
       </c>
       <c r="C51" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D51" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E51">
         <v>0</v>
@@ -3376,24 +3376,24 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="K51" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B52" t="s">
         <v>15</v>
       </c>
       <c r="C52" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D52" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E52">
         <v>0</v>
@@ -3411,24 +3411,24 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="K52" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B53" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C53" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D53" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E53">
         <v>150</v>
@@ -3446,24 +3446,24 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="K53" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B54" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C54" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D54" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E54">
         <v>150</v>
@@ -3481,24 +3481,24 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="K54" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B55" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C55" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D55" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E55">
         <v>2850</v>
@@ -3516,24 +3516,24 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="K55" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B56" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C56" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D56" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E56">
         <v>2850</v>
@@ -3551,21 +3551,21 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="K56" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="B57" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="C57" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D57" t="s">
         <v>33</v>
@@ -3586,21 +3586,21 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="K57" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="B58" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="C58" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D58" t="s">
         <v>33</v>
@@ -3621,21 +3621,21 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="K58" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="B59" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C59" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D59" t="s">
         <v>33</v>
@@ -3656,21 +3656,21 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="K59" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="B60" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="C60" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D60" t="s">
         <v>33</v>
@@ -3691,21 +3691,21 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="K60" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="B61" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C61" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D61" t="s">
         <v>33</v>
@@ -3726,21 +3726,21 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="K61" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="B62" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C62" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D62" t="s">
         <v>33</v>
@@ -3761,21 +3761,21 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="K62" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B63" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C63" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D63" t="s">
         <v>33</v>
@@ -3796,21 +3796,21 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="K63" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="B64" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="C64" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D64" t="s">
         <v>33</v>
@@ -3831,21 +3831,21 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="K64" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="B65" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C65" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D65" t="s">
         <v>33</v>
@@ -3866,21 +3866,21 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="K65" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B66" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="C66" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="D66" t="s">
         <v>33</v>
@@ -3901,24 +3901,24 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="K66" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B67" t="s">
-        <v>83</v>
+        <v>235</v>
       </c>
       <c r="C67" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D67" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E67">
         <v>0</v>
@@ -3936,24 +3936,24 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>169</v>
+        <v>233</v>
       </c>
       <c r="K67" t="s">
-        <v>209</v>
+        <v>234</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B68" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C68" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D68" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="E68">
         <v>0</v>
@@ -3971,21 +3971,21 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>189</v>
+        <v>233</v>
       </c>
       <c r="K68" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
       <c r="B69" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
       <c r="C69" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D69" t="s">
         <v>33</v>
@@ -4006,21 +4006,21 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="K69" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B70" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="C70" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D70" t="s">
         <v>33</v>
@@ -4043,13 +4043,13 @@
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B71" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="C71" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D71" t="s">
         <v>33</v>
@@ -4070,21 +4070,21 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="K71" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B72" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="C72" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D72" t="s">
         <v>33</v>
@@ -4105,21 +4105,21 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="K72" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B73" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C73" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D73" t="s">
         <v>33</v>
@@ -4140,21 +4140,21 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K73" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B74" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C74" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D74" t="s">
         <v>33</v>
@@ -4175,21 +4175,21 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K74" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B75" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C75" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="D75" t="s">
         <v>33</v>
@@ -4210,21 +4210,21 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="K75" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B76" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="C76" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D76" t="s">
         <v>33</v>
@@ -4245,21 +4245,21 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="K76" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B77" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="C77" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D77" t="s">
         <v>33</v>
@@ -4280,21 +4280,21 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="K77" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="B78" t="s">
         <v>16</v>
       </c>
       <c r="C78" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D78" t="s">
         <v>33</v>
@@ -4315,21 +4315,21 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="K78" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="B79" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C79" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D79" t="s">
         <v>33</v>
@@ -4350,21 +4350,21 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="K79" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="B80" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C80" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D80" t="s">
         <v>33</v>
@@ -4385,10 +4385,10 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="K80" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
@@ -4399,7 +4399,7 @@
         <v>22</v>
       </c>
       <c r="C81" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D81" t="s">
         <v>33</v>
@@ -4420,10 +4420,10 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="K81" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
@@ -4434,7 +4434,7 @@
         <v>20</v>
       </c>
       <c r="C82" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D82" t="s">
         <v>33</v>
@@ -4455,7 +4455,7 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="K82" t="s">
         <v>19</v>
@@ -4469,7 +4469,7 @@
         <v>14</v>
       </c>
       <c r="C83" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D83" t="s">
         <v>33</v>
@@ -4490,10 +4490,10 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="K83" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
@@ -4504,7 +4504,7 @@
         <v>17</v>
       </c>
       <c r="C84" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="D84" t="s">
         <v>33</v>
@@ -4525,10 +4525,10 @@
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="K84" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
@@ -4539,7 +4539,7 @@
         <v>23</v>
       </c>
       <c r="C85" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="D85" t="s">
         <v>33</v>
@@ -4560,21 +4560,21 @@
         <v>1</v>
       </c>
       <c r="J85" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="K85" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B86" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="C86" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
       <c r="D86" t="s">
         <v>33</v>
@@ -4595,10 +4595,10 @@
         <v>1</v>
       </c>
       <c r="J86" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="K86" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Split count_reads_and_bases into two scripts, only counting bases for trimming rule
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75CD41AF-3E45-4B8B-A392-6DDC523A23E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F407ABD-2D3A-4821-B754-BF9C3E6BF815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -692,9 +692,6 @@
     <t>_call_codec_consensus_metrics.txt</t>
   </si>
   <si>
-    <t>pct_bases_lost</t>
-  </si>
-  <si>
     <t>_bases_trimmed.json</t>
   </si>
   <si>
@@ -744,6 +741,9 @@
   </si>
   <si>
     <t>Percentage of reads that are lost during demultiplexing (applicable only when all samples in lane are demuxed)</t>
+  </si>
+  <si>
+    <t>percent_bases_trimmed</t>
   </si>
 </sst>
 </file>
@@ -1667,7 +1667,7 @@
         <v>43</v>
       </c>
       <c r="B2" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C2" t="s">
         <v>59</v>
@@ -1766,7 +1766,7 @@
         <v>54</v>
       </c>
       <c r="B5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C5" t="s">
         <v>61</v>
@@ -1830,7 +1830,7 @@
         <v>55</v>
       </c>
       <c r="B7" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C7" t="s">
         <v>61</v>
@@ -2241,10 +2241,10 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B19" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C19" t="s">
         <v>65</v>
@@ -2276,10 +2276,10 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>222</v>
+      </c>
+      <c r="B20" t="s">
         <v>223</v>
-      </c>
-      <c r="B20" t="s">
-        <v>224</v>
       </c>
       <c r="C20" t="s">
         <v>65</v>
@@ -2621,7 +2621,7 @@
         <v>202</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -3559,10 +3559,10 @@
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B57" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C57" t="s">
         <v>64</v>
@@ -3594,10 +3594,10 @@
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B58" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C58" t="s">
         <v>64</v>
@@ -3912,7 +3912,7 @@
         <v>74</v>
       </c>
       <c r="B67" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="C67" t="s">
         <v>66</v>
@@ -3936,10 +3936,10 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
+        <v>232</v>
+      </c>
+      <c r="K67" t="s">
         <v>233</v>
-      </c>
-      <c r="K67" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
@@ -3971,7 +3971,7 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="K68" t="s">
         <v>184</v>
@@ -4006,18 +4006,18 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="K69" t="s">
-        <v>218</v>
+        <v>235</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>224</v>
+      </c>
+      <c r="B70" t="s">
         <v>225</v>
-      </c>
-      <c r="B70" t="s">
-        <v>226</v>
       </c>
       <c r="C70" t="s">
         <v>66</v>
@@ -4221,7 +4221,7 @@
         <v>149</v>
       </c>
       <c r="B76" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C76" t="s">
         <v>69</v>
@@ -4571,7 +4571,7 @@
         <v>58</v>
       </c>
       <c r="B86" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C86" t="s">
         <v>208</v>

</xml_diff>

<commit_message>
Added ex_trimmed_read_length_metrics.py and test
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F407ABD-2D3A-4821-B754-BF9C3E6BF815}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{689DB35F-E1E0-4556-B2A9-01B2D8E4A3EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="238">
   <si>
     <t>nn_lower</t>
   </si>
@@ -710,9 +710,6 @@
     <t>Lower quartile of IQR for base quality at each position in filtered reads (Phred score)</t>
   </si>
   <si>
-    <t>ex_zero_length</t>
-  </si>
-  <si>
     <t>Reads with a length of zero after trimming (e.g. blank ligation)</t>
   </si>
   <si>
@@ -744,6 +741,15 @@
   </si>
   <si>
     <t>percent_bases_trimmed</t>
+  </si>
+  <si>
+    <t>_trimmed_read_length_metrics.json</t>
+  </si>
+  <si>
+    <t>percent_zero_length</t>
+  </si>
+  <si>
+    <t>ex_zero_length_reads</t>
   </si>
 </sst>
 </file>
@@ -1667,7 +1673,7 @@
         <v>43</v>
       </c>
       <c r="B2" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C2" t="s">
         <v>59</v>
@@ -1766,7 +1772,7 @@
         <v>54</v>
       </c>
       <c r="B5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C5" t="s">
         <v>61</v>
@@ -1830,7 +1836,7 @@
         <v>55</v>
       </c>
       <c r="B7" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C7" t="s">
         <v>61</v>
@@ -2621,7 +2627,7 @@
         <v>202</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -3912,7 +3918,7 @@
         <v>74</v>
       </c>
       <c r="B67" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C67" t="s">
         <v>66</v>
@@ -3936,10 +3942,10 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
+        <v>231</v>
+      </c>
+      <c r="K67" t="s">
         <v>232</v>
-      </c>
-      <c r="K67" t="s">
-        <v>233</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
@@ -3971,7 +3977,7 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="K68" t="s">
         <v>184</v>
@@ -4009,15 +4015,15 @@
         <v>218</v>
       </c>
       <c r="K69" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>237</v>
+      </c>
+      <c r="B70" t="s">
         <v>224</v>
-      </c>
-      <c r="B70" t="s">
-        <v>225</v>
       </c>
       <c r="C70" t="s">
         <v>66</v>
@@ -4038,7 +4044,13 @@
         <v>10</v>
       </c>
       <c r="I70" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="J70" t="s">
+        <v>235</v>
+      </c>
+      <c r="K70" t="s">
+        <v>236</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
@@ -4221,7 +4233,7 @@
         <v>149</v>
       </c>
       <c r="B76" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C76" t="s">
         <v>69</v>
@@ -4571,7 +4583,7 @@
         <v>58</v>
       </c>
       <c r="B86" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C86" t="s">
         <v>208</v>

</xml_diff>

<commit_message>
Added ex_percent_eligible_N_bases.py and test
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{689DB35F-E1E0-4556-B2A9-01B2D8E4A3EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECED9E71-3C51-427C-A85F-85388243B45C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$85</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="533" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="242">
   <si>
     <t>nn_lower</t>
   </si>
@@ -89,9 +89,6 @@
     <t>Percentage of reads which successfully aligned during DSC realignment</t>
   </si>
   <si>
-    <t>Percentage of genome eligible for variant calling (duplex depth &gt; 0 &amp; unmasked)</t>
-  </si>
-  <si>
     <t>ex_variant_call_eligible</t>
   </si>
   <si>
@@ -750,6 +747,21 @@
   </si>
   <si>
     <t>ex_zero_length_reads</t>
+  </si>
+  <si>
+    <t>ex_N_bases_variant_call_eligible</t>
+  </si>
+  <si>
+    <t>Percentage of N bases in bases eligible for variant calling (duplex depth &gt; 0, unmasked, QUAL &gt; min_base_quality)</t>
+  </si>
+  <si>
+    <t>Percentage of genome eligible for variant calling (duplex depth &gt; 0, unmasked, QUAL &gt; min_base_quality)</t>
+  </si>
+  <si>
+    <t>_percent_eligible_N_bases.json</t>
+  </si>
+  <si>
+    <t>post_consensus_percent_N</t>
   </si>
 </sst>
 </file>
@@ -1620,11 +1632,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K86"/>
+  <dimension ref="A1:K87"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" customWidth="1"/>
-    <col min="2" max="2" width="96.85546875" customWidth="1"/>
+    <col min="2" max="2" width="103.140625" customWidth="1"/>
     <col min="3" max="4" width="35.28515625" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
@@ -1635,16 +1647,16 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" t="s">
         <v>36</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>37</v>
-      </c>
-      <c r="D1" t="s">
-        <v>38</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -1659,27 +1671,27 @@
         <v>3</v>
       </c>
       <c r="I1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="J1" t="s">
+        <v>149</v>
+      </c>
+      <c r="K1" t="s">
         <v>150</v>
-      </c>
-      <c r="K1" t="s">
-        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B2" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="C2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E2">
         <v>2500</v>
@@ -1691,24 +1703,24 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1726,24 +1738,24 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E4">
         <v>90</v>
@@ -1761,24 +1773,24 @@
         <v>0</v>
       </c>
       <c r="J4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C5" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E5">
         <v>90</v>
@@ -1790,24 +1802,24 @@
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K5" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1825,24 +1837,24 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C7" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D7" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E7">
         <v>45</v>
@@ -1854,24 +1866,24 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K7" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>55</v>
+      </c>
+      <c r="B8" t="s">
         <v>56</v>
       </c>
-      <c r="B8" t="s">
-        <v>57</v>
-      </c>
       <c r="C8" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -1889,24 +1901,24 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K8" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D9" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E9">
         <v>280</v>
@@ -1924,24 +1936,24 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E10">
         <v>95</v>
@@ -1959,10 +1971,10 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -1970,13 +1982,13 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C11" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D11" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E11">
         <v>200</v>
@@ -1994,10 +2006,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -2005,13 +2017,13 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C12" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D12" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E12">
         <v>200</v>
@@ -2029,24 +2041,24 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="K12" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B13" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C13" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E13">
         <v>35</v>
@@ -2064,24 +2076,24 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K13" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B14" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C14" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D14" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E14">
         <v>35</v>
@@ -2099,24 +2111,24 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="K14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B15" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C15" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D15" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -2134,24 +2146,24 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K15" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B16" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C16" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D16" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -2169,24 +2181,24 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="K16" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B17" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C17" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D17" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E17">
         <v>150</v>
@@ -2204,24 +2216,24 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K17" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>104</v>
+      </c>
+      <c r="B18" t="s">
         <v>105</v>
       </c>
-      <c r="B18" t="s">
-        <v>106</v>
-      </c>
       <c r="C18" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D18" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E18">
         <v>150</v>
@@ -2239,24 +2251,24 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="K18" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B19" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C19" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D19" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E19">
         <v>30</v>
@@ -2274,24 +2286,24 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K19" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>221</v>
+      </c>
+      <c r="B20" t="s">
         <v>222</v>
       </c>
-      <c r="B20" t="s">
-        <v>223</v>
-      </c>
       <c r="C20" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D20" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E20">
         <v>30</v>
@@ -2309,24 +2321,24 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K20" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B21" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C21" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D21" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -2344,24 +2356,24 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K21" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B22" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C22" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D22" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -2379,24 +2391,24 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K22" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B23" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D23" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -2414,24 +2426,24 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K23" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B24" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D24" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -2449,24 +2461,24 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K24" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B25" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C25" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D25" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -2484,24 +2496,24 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K25" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B26" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C26" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D26" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E26">
         <v>0</v>
@@ -2519,24 +2531,24 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K26" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B27" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C27" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -2554,24 +2566,24 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K27" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B28" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C28" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D28" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -2589,24 +2601,24 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K28" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B29" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C29" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D29" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -2624,24 +2636,24 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="B30" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C30" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D30" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E30">
         <v>90</v>
@@ -2659,24 +2671,24 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K30" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B31" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C31" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D31" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -2694,24 +2706,24 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K31" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="B32" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C32" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D32" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E32">
         <v>125</v>
@@ -2729,24 +2741,24 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K32" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B33" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C33" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D33" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E33">
         <v>1.2999999999999999E-3</v>
@@ -2764,10 +2776,10 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K33" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -2775,13 +2787,13 @@
         <v>6</v>
       </c>
       <c r="B34" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C34" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D34" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E34">
         <v>4</v>
@@ -2799,10 +2811,10 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K34" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -2810,13 +2822,13 @@
         <v>7</v>
       </c>
       <c r="B35" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C35" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D35" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E35">
         <v>0.5</v>
@@ -2834,10 +2846,10 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K35" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -2845,13 +2857,13 @@
         <v>8</v>
       </c>
       <c r="B36" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C36" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D36" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E36">
         <v>0</v>
@@ -2869,10 +2881,10 @@
         <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K36" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
@@ -2880,13 +2892,13 @@
         <v>9</v>
       </c>
       <c r="B37" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C37" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D37" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E37">
         <v>1.9</v>
@@ -2904,10 +2916,10 @@
         <v>1</v>
       </c>
       <c r="J37" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K37" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
@@ -2915,13 +2927,13 @@
         <v>10</v>
       </c>
       <c r="B38" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C38" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D38" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E38">
         <v>1.2</v>
@@ -2939,24 +2951,24 @@
         <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K38" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B39" t="s">
         <v>4</v>
       </c>
       <c r="C39" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D39" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E39">
         <v>70</v>
@@ -2974,24 +2986,24 @@
         <v>1</v>
       </c>
       <c r="J39" t="s">
+        <v>195</v>
+      </c>
+      <c r="K39" t="s">
         <v>196</v>
-      </c>
-      <c r="K39" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B40" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C40" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D40" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E40">
         <v>75</v>
@@ -3003,24 +3015,24 @@
         <v>0</v>
       </c>
       <c r="J40" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K40" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B41" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C41" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D41" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E41">
         <v>0</v>
@@ -3038,24 +3050,24 @@
         <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K41" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C42" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D42" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E42">
         <v>80</v>
@@ -3073,24 +3085,24 @@
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K42" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>50</v>
+      </c>
+      <c r="B43" t="s">
         <v>51</v>
       </c>
-      <c r="B43" t="s">
-        <v>52</v>
-      </c>
       <c r="C43" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D43" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E43">
         <v>4.3</v>
@@ -3102,24 +3114,24 @@
         <v>0</v>
       </c>
       <c r="J43" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K43" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B44" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C44" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D44" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E44">
         <v>0</v>
@@ -3137,24 +3149,24 @@
         <v>0</v>
       </c>
       <c r="J44" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K44" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B45" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C45" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D45" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E45">
         <v>80</v>
@@ -3172,24 +3184,24 @@
         <v>0</v>
       </c>
       <c r="J45" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K45" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B46" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C46" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D46" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E46">
         <v>1</v>
@@ -3207,24 +3219,24 @@
         <v>0</v>
       </c>
       <c r="J46" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K46" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B47" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C47" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D47" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E47">
         <v>544</v>
@@ -3242,24 +3254,24 @@
         <v>0</v>
       </c>
       <c r="J47" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K47" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B48" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C48" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D48" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E48">
         <v>98</v>
@@ -3277,24 +3289,24 @@
         <v>0</v>
       </c>
       <c r="J48" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="K48" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B49" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C49" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D49" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E49">
         <v>35</v>
@@ -3312,24 +3324,24 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K49" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B50" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C50" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D50" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E50">
         <v>35</v>
@@ -3347,24 +3359,24 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K50" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="B51" t="s">
         <v>15</v>
       </c>
       <c r="C51" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D51" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E51">
         <v>0</v>
@@ -3382,24 +3394,24 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K51" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B52" t="s">
         <v>15</v>
       </c>
       <c r="C52" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D52" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E52">
         <v>0</v>
@@ -3417,24 +3429,24 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K52" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B53" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C53" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D53" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E53">
         <v>150</v>
@@ -3452,24 +3464,24 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K53" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B54" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C54" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D54" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E54">
         <v>150</v>
@@ -3487,24 +3499,24 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K54" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B55" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C55" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D55" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E55">
         <v>2850</v>
@@ -3522,24 +3534,24 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K55" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B56" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C56" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D56" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E56">
         <v>2850</v>
@@ -3557,24 +3569,24 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K56" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B57" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C57" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D57" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E57">
         <v>30</v>
@@ -3592,24 +3604,24 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K57" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B58" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="C58" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D58" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E58">
         <v>30</v>
@@ -3627,24 +3639,24 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K58" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B59" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C59" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D59" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E59">
         <v>0</v>
@@ -3662,24 +3674,24 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K59" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B60" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C60" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D60" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E60">
         <v>0</v>
@@ -3697,24 +3709,24 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K60" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B61" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C61" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D61" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E61">
         <v>0</v>
@@ -3732,24 +3744,24 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K61" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B62" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C62" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D62" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E62">
         <v>0</v>
@@ -3767,24 +3779,24 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K62" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B63" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C63" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D63" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E63">
         <v>0</v>
@@ -3802,24 +3814,24 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K63" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B64" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C64" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D64" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E64">
         <v>0</v>
@@ -3837,24 +3849,24 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K64" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B65" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C65" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D65" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E65">
         <v>0</v>
@@ -3872,24 +3884,24 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K65" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B66" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C66" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D66" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E66">
         <v>0</v>
@@ -3907,24 +3919,24 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K66" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B67" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C67" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D67" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E67">
         <v>0</v>
@@ -3942,24 +3954,24 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
+        <v>230</v>
+      </c>
+      <c r="K67" t="s">
         <v>231</v>
-      </c>
-      <c r="K67" t="s">
-        <v>232</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>134</v>
+      </c>
+      <c r="B68" t="s">
         <v>135</v>
       </c>
-      <c r="B68" t="s">
-        <v>136</v>
-      </c>
       <c r="C68" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D68" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E68">
         <v>0</v>
@@ -3977,24 +3989,24 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="K68" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
+        <v>208</v>
+      </c>
+      <c r="B69" t="s">
         <v>209</v>
       </c>
-      <c r="B69" t="s">
-        <v>210</v>
-      </c>
       <c r="C69" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D69" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E69">
         <v>1</v>
@@ -4012,24 +4024,24 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="K69" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B70" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C70" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D70" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E70">
         <v>0</v>
@@ -4047,24 +4059,24 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
+        <v>234</v>
+      </c>
+      <c r="K70" t="s">
         <v>235</v>
-      </c>
-      <c r="K70" t="s">
-        <v>236</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B71" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C71" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D71" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E71">
         <v>80</v>
@@ -4082,24 +4094,24 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="K71" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B72" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C72" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D72" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E72">
         <v>85</v>
@@ -4117,24 +4129,24 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="K72" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B73" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C73" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D73" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E73">
         <v>90</v>
@@ -4152,24 +4164,24 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K73" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B74" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C74" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D74" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E74">
         <v>50</v>
@@ -4187,24 +4199,24 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="K74" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B75" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C75" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D75" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E75">
         <v>125</v>
@@ -4222,24 +4234,24 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="K75" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B76" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C76" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D76" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E76">
         <v>50</v>
@@ -4257,24 +4269,24 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
+        <v>184</v>
+      </c>
+      <c r="K76" t="s">
         <v>185</v>
-      </c>
-      <c r="K76" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="B77" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C77" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D77" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E77">
         <v>60</v>
@@ -4292,24 +4304,24 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="K77" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B78" t="s">
         <v>16</v>
       </c>
       <c r="C78" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D78" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E78">
         <v>99</v>
@@ -4327,24 +4339,24 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K78" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B79" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C79" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D79" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E79">
         <v>0</v>
@@ -4362,24 +4374,24 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K79" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>144</v>
+      </c>
+      <c r="B80" t="s">
         <v>145</v>
       </c>
-      <c r="B80" t="s">
-        <v>146</v>
-      </c>
       <c r="C80" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D80" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E80">
         <v>0.5</v>
@@ -4397,24 +4409,24 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K80" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
+        <v>20</v>
+      </c>
+      <c r="B81" t="s">
         <v>21</v>
       </c>
-      <c r="B81" t="s">
-        <v>22</v>
-      </c>
       <c r="C81" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D81" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E81">
         <v>0</v>
@@ -4432,24 +4444,24 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K81" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>18</v>
+      </c>
+      <c r="B82" t="s">
         <v>19</v>
       </c>
-      <c r="B82" t="s">
-        <v>20</v>
-      </c>
       <c r="C82" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D82" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E82">
         <v>14.5</v>
@@ -4467,10 +4479,10 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K82" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
@@ -4481,10 +4493,10 @@
         <v>14</v>
       </c>
       <c r="C83" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D83" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E83">
         <v>5.0000000000000001E-4</v>
@@ -4502,119 +4514,154 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="K83" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>18</v>
+        <v>237</v>
       </c>
       <c r="B84" t="s">
-        <v>17</v>
+        <v>238</v>
       </c>
       <c r="C84" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D84" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E84">
-        <v>5</v>
+        <v>0.05</v>
       </c>
       <c r="F84">
-        <v>100</v>
+        <v>0.08</v>
       </c>
       <c r="G84">
-        <v>20</v>
+        <v>0.02</v>
       </c>
       <c r="H84">
-        <v>100</v>
+        <v>0.05</v>
       </c>
       <c r="I84" t="b">
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>200</v>
+        <v>240</v>
       </c>
       <c r="K84" t="s">
-        <v>191</v>
+        <v>241</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="B85" t="s">
-        <v>23</v>
+        <v>239</v>
       </c>
       <c r="C85" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D85" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E85">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F85">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="G85">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H85">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="I85" t="b">
         <v>1</v>
       </c>
       <c r="J85" t="s">
-        <v>166</v>
+        <v>199</v>
       </c>
       <c r="K85" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>58</v>
+        <v>23</v>
       </c>
       <c r="B86" t="s">
-        <v>225</v>
+        <v>22</v>
       </c>
       <c r="C86" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="D86" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E86">
+        <v>0</v>
+      </c>
+      <c r="F86">
+        <v>95</v>
+      </c>
+      <c r="G86">
+        <v>0</v>
+      </c>
+      <c r="H86">
+        <v>80</v>
+      </c>
+      <c r="I86" t="b">
+        <v>1</v>
+      </c>
+      <c r="J86" t="s">
+        <v>165</v>
+      </c>
+      <c r="K86" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>57</v>
+      </c>
+      <c r="B87" t="s">
+        <v>224</v>
+      </c>
+      <c r="C87" t="s">
+        <v>207</v>
+      </c>
+      <c r="D87" t="s">
+        <v>32</v>
+      </c>
+      <c r="E87">
         <v>90</v>
       </c>
-      <c r="F86">
+      <c r="F87">
         <v>100</v>
       </c>
-      <c r="G86">
+      <c r="G87">
         <v>95</v>
       </c>
-      <c r="H86">
+      <c r="H87">
         <v>100</v>
       </c>
-      <c r="I86" t="b">
-        <v>1</v>
-      </c>
-      <c r="J86" t="s">
-        <v>200</v>
-      </c>
-      <c r="K86" t="s">
-        <v>58</v>
+      <c r="I87" t="b">
+        <v>1</v>
+      </c>
+      <c r="J87" t="s">
+        <v>199</v>
+      </c>
+      <c r="K87" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K84" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K85" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Added ms_duplication_metrics.py and test
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ECED9E71-3C51-427C-A85F-85388243B45C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD63228E-1168-4040-AA7F-2F9E59B95B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -515,9 +515,6 @@
     <t>_alignment_stats.txt</t>
   </si>
   <si>
-    <t>_markdup_metrics.txt</t>
-  </si>
-  <si>
     <t>_insert_size_metrics.txt</t>
   </si>
   <si>
@@ -644,9 +641,6 @@
     <t>_filtered_fq_metrics.txt</t>
   </si>
   <si>
-    <t>^(\S+\t){9}(?P&lt;value&gt;[\d.]+)</t>
-  </si>
-  <si>
     <t>Percentage of fragments that fall within the expected size range on gel elextrophoresis (10,000-50,000 bp)</t>
   </si>
   <si>
@@ -762,6 +756,12 @@
   </si>
   <si>
     <t>post_consensus_percent_N</t>
+  </si>
+  <si>
+    <t>duplication_rate</t>
+  </si>
+  <si>
+    <t>_duplication_metrics_ms.json</t>
   </si>
 </sst>
 </file>
@@ -1685,7 +1685,7 @@
         <v>42</v>
       </c>
       <c r="B2" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C2" t="s">
         <v>58</v>
@@ -1749,7 +1749,7 @@
         <v>44</v>
       </c>
       <c r="B4" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C4" t="s">
         <v>58</v>
@@ -1784,7 +1784,7 @@
         <v>53</v>
       </c>
       <c r="B5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C5" t="s">
         <v>60</v>
@@ -1848,7 +1848,7 @@
         <v>54</v>
       </c>
       <c r="B7" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="C7" t="s">
         <v>60</v>
@@ -2009,7 +2009,7 @@
         <v>154</v>
       </c>
       <c r="K11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -2044,7 +2044,7 @@
         <v>155</v>
       </c>
       <c r="K12" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -2079,7 +2079,7 @@
         <v>154</v>
       </c>
       <c r="K13" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -2114,7 +2114,7 @@
         <v>155</v>
       </c>
       <c r="K14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -2149,7 +2149,7 @@
         <v>154</v>
       </c>
       <c r="K15" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -2184,7 +2184,7 @@
         <v>155</v>
       </c>
       <c r="K16" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -2219,7 +2219,7 @@
         <v>154</v>
       </c>
       <c r="K17" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -2254,15 +2254,15 @@
         <v>155</v>
       </c>
       <c r="K18" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
+        <v>218</v>
+      </c>
+      <c r="B19" t="s">
         <v>220</v>
-      </c>
-      <c r="B19" t="s">
-        <v>222</v>
       </c>
       <c r="C19" t="s">
         <v>64</v>
@@ -2289,15 +2289,15 @@
         <v>156</v>
       </c>
       <c r="K19" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B20" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C20" t="s">
         <v>64</v>
@@ -2324,7 +2324,7 @@
         <v>157</v>
       </c>
       <c r="K20" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -2359,7 +2359,7 @@
         <v>156</v>
       </c>
       <c r="K21" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -2394,7 +2394,7 @@
         <v>157</v>
       </c>
       <c r="K22" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -2429,7 +2429,7 @@
         <v>156</v>
       </c>
       <c r="K23" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -2464,7 +2464,7 @@
         <v>157</v>
       </c>
       <c r="K24" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -2499,7 +2499,7 @@
         <v>156</v>
       </c>
       <c r="K25" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -2534,7 +2534,7 @@
         <v>157</v>
       </c>
       <c r="K26" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -2569,7 +2569,7 @@
         <v>156</v>
       </c>
       <c r="K27" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -2604,7 +2604,7 @@
         <v>157</v>
       </c>
       <c r="K28" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -2636,10 +2636,10 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -2674,7 +2674,7 @@
         <v>158</v>
       </c>
       <c r="K30" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
@@ -2706,10 +2706,10 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>159</v>
+        <v>241</v>
       </c>
       <c r="K31" t="s">
-        <v>202</v>
+        <v>240</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
@@ -2741,10 +2741,10 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K32" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -2776,10 +2776,10 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K33" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -2811,10 +2811,10 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K34" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -2846,10 +2846,10 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K35" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -2881,10 +2881,10 @@
         <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K36" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
@@ -2916,10 +2916,10 @@
         <v>1</v>
       </c>
       <c r="J37" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K37" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
@@ -2951,10 +2951,10 @@
         <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K38" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
@@ -2986,10 +2986,10 @@
         <v>1</v>
       </c>
       <c r="J39" t="s">
+        <v>194</v>
+      </c>
+      <c r="K39" t="s">
         <v>195</v>
-      </c>
-      <c r="K39" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
@@ -3061,7 +3061,7 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C42" t="s">
         <v>59</v>
@@ -3160,7 +3160,7 @@
         <v>46</v>
       </c>
       <c r="B45" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C45" t="s">
         <v>59</v>
@@ -3195,7 +3195,7 @@
         <v>47</v>
       </c>
       <c r="B46" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="C46" t="s">
         <v>59</v>
@@ -3324,10 +3324,10 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K49" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3359,10 +3359,10 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K50" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
@@ -3394,10 +3394,10 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K51" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
@@ -3429,10 +3429,10 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K52" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
@@ -3464,10 +3464,10 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K53" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
@@ -3499,10 +3499,10 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K54" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
@@ -3534,10 +3534,10 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K55" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
@@ -3569,18 +3569,18 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="K56" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B57" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C57" t="s">
         <v>63</v>
@@ -3604,18 +3604,18 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K57" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B58" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C58" t="s">
         <v>63</v>
@@ -3639,10 +3639,10 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K58" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
@@ -3674,10 +3674,10 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K59" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
@@ -3709,10 +3709,10 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K60" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
@@ -3744,10 +3744,10 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K61" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
@@ -3779,10 +3779,10 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K62" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
@@ -3814,10 +3814,10 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K63" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
@@ -3849,10 +3849,10 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K64" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
@@ -3884,10 +3884,10 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="K65" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
@@ -3919,10 +3919,10 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K66" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
@@ -3930,7 +3930,7 @@
         <v>73</v>
       </c>
       <c r="B67" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="C67" t="s">
         <v>65</v>
@@ -3954,10 +3954,10 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="K67" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
@@ -3989,18 +3989,18 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="K68" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B69" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C69" t="s">
         <v>65</v>
@@ -4024,18 +4024,18 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="K69" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B70" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="C70" t="s">
         <v>65</v>
@@ -4059,10 +4059,10 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="K70" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
@@ -4070,7 +4070,7 @@
         <v>74</v>
       </c>
       <c r="B71" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C71" t="s">
         <v>65</v>
@@ -4094,10 +4094,10 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="K71" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
@@ -4105,7 +4105,7 @@
         <v>75</v>
       </c>
       <c r="B72" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C72" t="s">
         <v>65</v>
@@ -4129,10 +4129,10 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="K72" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
@@ -4167,7 +4167,7 @@
         <v>151</v>
       </c>
       <c r="K73" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
@@ -4202,7 +4202,7 @@
         <v>151</v>
       </c>
       <c r="K74" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
@@ -4237,7 +4237,7 @@
         <v>152</v>
       </c>
       <c r="K75" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
@@ -4245,7 +4245,7 @@
         <v>148</v>
       </c>
       <c r="B76" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C76" t="s">
         <v>68</v>
@@ -4269,10 +4269,10 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
+        <v>183</v>
+      </c>
+      <c r="K76" t="s">
         <v>184</v>
-      </c>
-      <c r="K76" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
@@ -4280,7 +4280,7 @@
         <v>137</v>
       </c>
       <c r="B77" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C77" t="s">
         <v>68</v>
@@ -4304,10 +4304,10 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="K77" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
@@ -4339,10 +4339,10 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="K78" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
@@ -4374,10 +4374,10 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="K79" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
@@ -4409,10 +4409,10 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="K80" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
@@ -4447,7 +4447,7 @@
         <v>153</v>
       </c>
       <c r="K81" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
@@ -4479,7 +4479,7 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="K82" t="s">
         <v>18</v>
@@ -4514,21 +4514,21 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="K83" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B84" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="C84" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D84" t="s">
         <v>32</v>
@@ -4549,10 +4549,10 @@
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="K84" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
@@ -4560,10 +4560,10 @@
         <v>17</v>
       </c>
       <c r="B85" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C85" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D85" t="s">
         <v>32</v>
@@ -4584,10 +4584,10 @@
         <v>1</v>
       </c>
       <c r="J85" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="K85" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
@@ -4598,7 +4598,7 @@
         <v>22</v>
       </c>
       <c r="C86" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D86" t="s">
         <v>32</v>
@@ -4619,10 +4619,10 @@
         <v>1</v>
       </c>
       <c r="J86" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="K86" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.25">
@@ -4630,10 +4630,10 @@
         <v>57</v>
       </c>
       <c r="B87" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C87" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D87" t="s">
         <v>32</v>
@@ -4654,7 +4654,7 @@
         <v>1</v>
       </c>
       <c r="J87" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="K87" t="s">
         <v>57</v>

</xml_diff>

<commit_message>
1. Fixed calculation of per_tile_sequence_quality 2. Added definitions to fastqc_summary.json files 3. Updated fastqc metric definitions in component_level_metrics.csv 4. Fixed misc comments
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CD63228E-1168-4040-AA7F-2F9E59B95B2A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A59C136B-3E56-4A94-BFF2-93114394CF16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="241">
   <si>
     <t>nn_lower</t>
   </si>
@@ -83,9 +83,6 @@
     <t>Rate at which Watson and Crick complementary bases disagree (total R1R2 disagreements divided by total duplex bases for each sample)</t>
   </si>
   <si>
-    <t>Percent of flow cell tiles where mean quality score is &lt;Q36</t>
-  </si>
-  <si>
     <t>Percentage of reads which successfully aligned during DSC realignment</t>
   </si>
   <si>
@@ -308,9 +305,6 @@
     <t>ms_filtered_per_base_N_content_r2</t>
   </si>
   <si>
-    <t>Percentage of flow cell tiles where mean quality score is &lt;Q36</t>
-  </si>
-  <si>
     <t>ms_reads_filtered_length</t>
   </si>
   <si>
@@ -341,12 +335,6 @@
     <t>Ratio of called heterozygous variants to called homozygous variants</t>
   </si>
   <si>
-    <t>Peak in mean sequence quality across raw r1 reads (Phred score)</t>
-  </si>
-  <si>
-    <t>Peak in mean sequence quality across raw r2 reads (Phred score)</t>
-  </si>
-  <si>
     <t>ms_raw_read_length_r1</t>
   </si>
   <si>
@@ -431,9 +419,6 @@
     <t>Percentage difference in the proportion of A/T or C/G at each position in filtered reads</t>
   </si>
   <si>
-    <t>Percentage of bases recorded as N at any one position in filtered reads</t>
-  </si>
-  <si>
     <t>Percentage of filtered sequences made up by any one identical sequence</t>
   </si>
   <si>
@@ -698,9 +683,6 @@
     <t>ms_filtered_per_base_quality_r2</t>
   </si>
   <si>
-    <t>Lower quartile of IQR for base quality at each position in filtered reads (Phred score)</t>
-  </si>
-  <si>
     <t>Reads with a length of zero after trimming (e.g. blank ligation)</t>
   </si>
   <si>
@@ -762,6 +744,21 @@
   </si>
   <si>
     <t>_duplication_metrics_ms.json</t>
+  </si>
+  <si>
+    <t>Percentage of flow cell tiles where mean quality score at any read position is &gt;=5 less than the global mean quality for that position</t>
+  </si>
+  <si>
+    <t>Peak in distribution of mean sequence quality across raw r1 reads (Phred score)</t>
+  </si>
+  <si>
+    <t>Peak in distribution of mean sequence quality across raw r2 reads (Phred score)</t>
+  </si>
+  <si>
+    <t>Maximum percentage of bases recorded as N at any one position in filtered reads</t>
+  </si>
+  <si>
+    <t>Minimum IQR lower quartile for base quality at any position in reads (Phred score)</t>
   </si>
 </sst>
 </file>
@@ -1647,16 +1644,16 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" t="s">
         <v>35</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>36</v>
-      </c>
-      <c r="D1" t="s">
-        <v>37</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -1671,27 +1668,27 @@
         <v>3</v>
       </c>
       <c r="I1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="J1" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="K1" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B2" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="C2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E2">
         <v>2500</v>
@@ -1703,24 +1700,24 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K2" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1738,24 +1735,24 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K3" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
-        <v>201</v>
+        <v>196</v>
       </c>
       <c r="C4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E4">
         <v>90</v>
@@ -1773,24 +1770,24 @@
         <v>0</v>
       </c>
       <c r="J4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B5" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="C5" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E5">
         <v>90</v>
@@ -1802,24 +1799,24 @@
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K5" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C6" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1837,24 +1834,24 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K6" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B7" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="C7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E7">
         <v>45</v>
@@ -1866,24 +1863,24 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K7" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>54</v>
+      </c>
+      <c r="B8" t="s">
         <v>55</v>
       </c>
-      <c r="B8" t="s">
-        <v>56</v>
-      </c>
       <c r="C8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D8" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -1901,24 +1898,24 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K8" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C9" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D9" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E9">
         <v>280</v>
@@ -1936,24 +1933,24 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C10" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E10">
         <v>95</v>
@@ -1971,10 +1968,10 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -1982,13 +1979,13 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C11" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D11" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E11">
         <v>200</v>
@@ -2006,10 +2003,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="K11" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -2017,13 +2014,13 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="C12" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D12" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E12">
         <v>200</v>
@@ -2041,24 +2038,24 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="K12" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="B13" t="s">
-        <v>101</v>
+        <v>237</v>
       </c>
       <c r="C13" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D13" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E13">
         <v>35</v>
@@ -2076,24 +2073,24 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="K13" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="B14" t="s">
-        <v>102</v>
+        <v>238</v>
       </c>
       <c r="C14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D14" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E14">
         <v>35</v>
@@ -2111,24 +2108,24 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="K14" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
       <c r="B15" t="s">
-        <v>90</v>
+        <v>236</v>
       </c>
       <c r="C15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D15" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -2146,24 +2143,24 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="K15" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B16" t="s">
-        <v>90</v>
+        <v>236</v>
       </c>
       <c r="C16" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D16" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -2181,24 +2178,24 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="K16" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="B17" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C17" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D17" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E17">
         <v>150</v>
@@ -2216,24 +2213,24 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="K17" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="B18" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C18" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D18" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E18">
         <v>150</v>
@@ -2251,24 +2248,24 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="K18" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>218</v>
+        <v>213</v>
       </c>
       <c r="B19" t="s">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="C19" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D19" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E19">
         <v>30</v>
@@ -2286,24 +2283,24 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="K19" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>219</v>
+        <v>214</v>
       </c>
       <c r="B20" t="s">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="C20" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D20" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E20">
         <v>30</v>
@@ -2321,24 +2318,24 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="K20" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B21" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="C21" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D21" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -2356,24 +2353,24 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="K21" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B22" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="C22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D22" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -2391,24 +2388,24 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="K22" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B23" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C23" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D23" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -2426,24 +2423,24 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="K23" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B24" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C24" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D24" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -2461,24 +2458,24 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="K24" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B25" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D25" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -2496,24 +2493,24 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="K25" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B26" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C26" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D26" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E26">
         <v>0</v>
@@ -2531,24 +2528,24 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="K26" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B27" t="s">
-        <v>131</v>
+        <v>239</v>
       </c>
       <c r="C27" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D27" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -2566,24 +2563,24 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="K27" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B28" t="s">
-        <v>131</v>
+        <v>239</v>
       </c>
       <c r="C28" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D28" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -2601,24 +2598,24 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="K28" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B29" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="C29" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D29" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -2636,24 +2633,24 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>200</v>
+        <v>195</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B30" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="C30" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D30" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E30">
         <v>90</v>
@@ -2671,24 +2668,24 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="K30" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="B31" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="C31" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D31" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -2706,24 +2703,24 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="K31" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B32" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C32" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D32" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E32">
         <v>125</v>
@@ -2741,24 +2738,24 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="K32" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B33" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C33" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D33" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E33">
         <v>1.2999999999999999E-3</v>
@@ -2776,10 +2773,10 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="K33" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -2787,13 +2784,13 @@
         <v>6</v>
       </c>
       <c r="B34" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C34" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D34" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E34">
         <v>4</v>
@@ -2811,10 +2808,10 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="K34" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -2822,13 +2819,13 @@
         <v>7</v>
       </c>
       <c r="B35" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C35" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D35" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E35">
         <v>0.5</v>
@@ -2846,10 +2843,10 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="K35" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -2857,13 +2854,13 @@
         <v>8</v>
       </c>
       <c r="B36" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C36" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D36" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E36">
         <v>0</v>
@@ -2881,10 +2878,10 @@
         <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="K36" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
@@ -2892,13 +2889,13 @@
         <v>9</v>
       </c>
       <c r="B37" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C37" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D37" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E37">
         <v>1.9</v>
@@ -2916,10 +2913,10 @@
         <v>1</v>
       </c>
       <c r="J37" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="K37" t="s">
-        <v>178</v>
+        <v>173</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
@@ -2927,13 +2924,13 @@
         <v>10</v>
       </c>
       <c r="B38" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C38" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D38" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E38">
         <v>1.2</v>
@@ -2951,24 +2948,24 @@
         <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>181</v>
+        <v>176</v>
       </c>
       <c r="K38" t="s">
-        <v>179</v>
+        <v>174</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B39" t="s">
         <v>4</v>
       </c>
       <c r="C39" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D39" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E39">
         <v>70</v>
@@ -2986,24 +2983,24 @@
         <v>1</v>
       </c>
       <c r="J39" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="K39" t="s">
-        <v>195</v>
+        <v>190</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B40" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C40" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D40" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E40">
         <v>75</v>
@@ -3015,24 +3012,24 @@
         <v>0</v>
       </c>
       <c r="J40" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K40" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B41" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C41" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D41" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E41">
         <v>0</v>
@@ -3050,24 +3047,24 @@
         <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K41" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B42" t="s">
-        <v>202</v>
+        <v>197</v>
       </c>
       <c r="C42" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D42" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E42">
         <v>80</v>
@@ -3085,24 +3082,24 @@
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K42" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
+        <v>49</v>
+      </c>
+      <c r="B43" t="s">
         <v>50</v>
       </c>
-      <c r="B43" t="s">
-        <v>51</v>
-      </c>
       <c r="C43" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D43" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E43">
         <v>4.3</v>
@@ -3114,24 +3111,24 @@
         <v>0</v>
       </c>
       <c r="J43" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K43" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B44" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C44" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D44" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E44">
         <v>0</v>
@@ -3149,24 +3146,24 @@
         <v>0</v>
       </c>
       <c r="J44" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K44" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B45" t="s">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="C45" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D45" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E45">
         <v>80</v>
@@ -3184,24 +3181,24 @@
         <v>0</v>
       </c>
       <c r="J45" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K45" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B46" t="s">
-        <v>204</v>
+        <v>199</v>
       </c>
       <c r="C46" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D46" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E46">
         <v>1</v>
@@ -3219,24 +3216,24 @@
         <v>0</v>
       </c>
       <c r="J46" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K46" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B47" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C47" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D47" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E47">
         <v>544</v>
@@ -3254,24 +3251,24 @@
         <v>0</v>
       </c>
       <c r="J47" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K47" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B48" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C48" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D48" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E48">
         <v>98</v>
@@ -3289,24 +3286,24 @@
         <v>0</v>
       </c>
       <c r="J48" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="K48" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="B49" t="s">
-        <v>101</v>
+        <v>237</v>
       </c>
       <c r="C49" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D49" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E49">
         <v>35</v>
@@ -3324,24 +3321,24 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="K49" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
     </row>
     <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
       <c r="B50" t="s">
-        <v>102</v>
+        <v>238</v>
       </c>
       <c r="C50" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D50" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E50">
         <v>35</v>
@@ -3359,24 +3356,24 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
+        <v>156</v>
+      </c>
+      <c r="K50" t="s">
         <v>161</v>
-      </c>
-      <c r="K50" t="s">
-        <v>166</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="B51" t="s">
-        <v>15</v>
+        <v>236</v>
       </c>
       <c r="C51" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D51" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E51">
         <v>0</v>
@@ -3394,24 +3391,24 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="K51" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
       <c r="B52" t="s">
-        <v>15</v>
+        <v>236</v>
       </c>
       <c r="C52" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D52" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E52">
         <v>0</v>
@@ -3429,24 +3426,24 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="K52" t="s">
-        <v>168</v>
+        <v>163</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="B53" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C53" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D53" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E53">
         <v>150</v>
@@ -3464,24 +3461,24 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="K53" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="B54" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C54" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D54" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E54">
         <v>150</v>
@@ -3499,24 +3496,24 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="K54" t="s">
-        <v>169</v>
+        <v>164</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B55" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C55" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D55" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E55">
         <v>2850</v>
@@ -3534,24 +3531,24 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
+        <v>155</v>
+      </c>
+      <c r="K55" t="s">
         <v>160</v>
-      </c>
-      <c r="K55" t="s">
-        <v>165</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="B56" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="C56" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D56" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E56">
         <v>2850</v>
@@ -3569,24 +3566,24 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="K56" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>216</v>
+        <v>211</v>
       </c>
       <c r="B57" t="s">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="C57" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D57" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E57">
         <v>30</v>
@@ -3604,24 +3601,24 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
+        <v>157</v>
+      </c>
+      <c r="K57" t="s">
         <v>162</v>
-      </c>
-      <c r="K57" t="s">
-        <v>167</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>217</v>
+        <v>212</v>
       </c>
       <c r="B58" t="s">
-        <v>220</v>
+        <v>240</v>
       </c>
       <c r="C58" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D58" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E58">
         <v>30</v>
@@ -3639,24 +3636,24 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="K58" t="s">
-        <v>167</v>
+        <v>162</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B59" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C59" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D59" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E59">
         <v>0</v>
@@ -3674,24 +3671,24 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="K59" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="B60" t="s">
-        <v>128</v>
+        <v>124</v>
       </c>
       <c r="C60" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D60" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E60">
         <v>0</v>
@@ -3709,24 +3706,24 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="K60" t="s">
-        <v>170</v>
+        <v>165</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B61" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C61" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D61" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E61">
         <v>0</v>
@@ -3744,24 +3741,24 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="K61" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="B62" t="s">
-        <v>129</v>
+        <v>125</v>
       </c>
       <c r="C62" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D62" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E62">
         <v>0</v>
@@ -3779,24 +3776,24 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="K62" t="s">
-        <v>171</v>
+        <v>166</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B63" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C63" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D63" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E63">
         <v>0</v>
@@ -3814,24 +3811,24 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="K63" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="B64" t="s">
-        <v>130</v>
+        <v>126</v>
       </c>
       <c r="C64" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D64" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E64">
         <v>0</v>
@@ -3849,24 +3846,24 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="K64" t="s">
-        <v>172</v>
+        <v>167</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="B65" t="s">
-        <v>131</v>
+        <v>239</v>
       </c>
       <c r="C65" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D65" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E65">
         <v>0</v>
@@ -3884,24 +3881,24 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="K65" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="B66" t="s">
-        <v>131</v>
+        <v>239</v>
       </c>
       <c r="C66" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D66" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E66">
         <v>0</v>
@@ -3919,24 +3916,24 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="K66" t="s">
-        <v>173</v>
+        <v>168</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B67" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="C67" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D67" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E67">
         <v>0</v>
@@ -3954,24 +3951,24 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="K67" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B68" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="C68" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D68" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E68">
         <v>0</v>
@@ -3989,24 +3986,24 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="K68" t="s">
-        <v>182</v>
+        <v>177</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>206</v>
+        <v>201</v>
       </c>
       <c r="B69" t="s">
-        <v>207</v>
+        <v>202</v>
       </c>
       <c r="C69" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D69" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E69">
         <v>1</v>
@@ -4024,24 +4021,24 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>215</v>
+        <v>210</v>
       </c>
       <c r="K69" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="B70" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
       <c r="C70" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D70" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E70">
         <v>0</v>
@@ -4059,24 +4056,24 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="K70" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B71" t="s">
-        <v>208</v>
+        <v>203</v>
       </c>
       <c r="C71" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D71" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E71">
         <v>80</v>
@@ -4094,24 +4091,24 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>211</v>
+        <v>206</v>
       </c>
       <c r="K71" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B72" t="s">
-        <v>209</v>
+        <v>204</v>
       </c>
       <c r="C72" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D72" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E72">
         <v>85</v>
@@ -4129,24 +4126,24 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>212</v>
+        <v>207</v>
       </c>
       <c r="K72" t="s">
-        <v>210</v>
+        <v>205</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B73" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C73" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D73" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E73">
         <v>90</v>
@@ -4164,24 +4161,24 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="K73" t="s">
-        <v>190</v>
+        <v>185</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B74" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C74" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D74" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E74">
         <v>50</v>
@@ -4199,24 +4196,24 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="K74" t="s">
-        <v>192</v>
+        <v>187</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B75" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="C75" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D75" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E75">
         <v>125</v>
@@ -4234,24 +4231,24 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="K75" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="B76" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="C76" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D76" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E76">
         <v>50</v>
@@ -4269,24 +4266,24 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>183</v>
+        <v>178</v>
       </c>
       <c r="K76" t="s">
-        <v>184</v>
+        <v>179</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B77" t="s">
-        <v>199</v>
+        <v>194</v>
       </c>
       <c r="C77" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D77" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E77">
         <v>60</v>
@@ -4304,24 +4301,24 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>197</v>
+        <v>192</v>
       </c>
       <c r="K77" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="B78" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C78" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D78" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E78">
         <v>99</v>
@@ -4339,24 +4336,24 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="K78" t="s">
-        <v>185</v>
+        <v>180</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="B79" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="C79" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D79" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E79">
         <v>0</v>
@@ -4374,24 +4371,24 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>187</v>
+        <v>182</v>
       </c>
       <c r="K79" t="s">
-        <v>186</v>
+        <v>181</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B80" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="C80" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D80" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E80">
         <v>0.5</v>
@@ -4409,24 +4406,24 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="K80" t="s">
-        <v>188</v>
+        <v>183</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
+        <v>19</v>
+      </c>
+      <c r="B81" t="s">
         <v>20</v>
       </c>
-      <c r="B81" t="s">
-        <v>21</v>
-      </c>
       <c r="C81" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D81" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E81">
         <v>0</v>
@@ -4444,24 +4441,24 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="K81" t="s">
-        <v>174</v>
+        <v>169</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
+        <v>17</v>
+      </c>
+      <c r="B82" t="s">
         <v>18</v>
       </c>
-      <c r="B82" t="s">
-        <v>19</v>
-      </c>
       <c r="C82" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D82" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E82">
         <v>14.5</v>
@@ -4479,10 +4476,10 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="K82" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
@@ -4493,10 +4490,10 @@
         <v>14</v>
       </c>
       <c r="C83" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D83" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E83">
         <v>5.0000000000000001E-4</v>
@@ -4514,24 +4511,24 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>214</v>
+        <v>209</v>
       </c>
       <c r="K83" t="s">
-        <v>213</v>
+        <v>208</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
       <c r="B84" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
       <c r="C84" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D84" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E84">
         <v>0.05</v>
@@ -4549,24 +4546,24 @@
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
       <c r="K84" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B85" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
       <c r="C85" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D85" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E85">
         <v>5</v>
@@ -4584,24 +4581,24 @@
         <v>1</v>
       </c>
       <c r="J85" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="K85" t="s">
-        <v>189</v>
+        <v>184</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B86" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C86" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D86" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E86">
         <v>0</v>
@@ -4619,24 +4616,24 @@
         <v>1</v>
       </c>
       <c r="J86" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="K86" t="s">
-        <v>193</v>
+        <v>188</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B87" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="C87" t="s">
-        <v>205</v>
+        <v>200</v>
       </c>
       <c r="D87" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E87">
         <v>90</v>
@@ -4654,10 +4651,10 @@
         <v>1</v>
       </c>
       <c r="J87" t="s">
-        <v>198</v>
+        <v>193</v>
       </c>
       <c r="K87" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
1. Added ms_coverage_by_depth metrics (replaces mosdepth) 2. Adjusted resource allocation for 12 samples on m6i.32xlarge
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DB69382-78DE-4BFB-AE92-BF0EB76DF3C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EF54474-ED57-44DB-BBC6-FF599AEE2217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$86</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="241">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="245">
   <si>
     <t>nn_lower</t>
   </si>
@@ -759,6 +759,18 @@
   </si>
   <si>
     <t>Minimum IQR lower quartile for base quality at any position in reads (Phred score)</t>
+  </si>
+  <si>
+    <t>ms_coverage_at_depth_threshold</t>
+  </si>
+  <si>
+    <t>Percentage of genome with depth &gt; 40X</t>
+  </si>
+  <si>
+    <t>_coverage_by_depth.json</t>
+  </si>
+  <si>
+    <t>pct_coverage.40X</t>
   </si>
 </sst>
 </file>
@@ -1629,7 +1641,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K87"/>
+  <dimension ref="A1:K88"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" customWidth="1"/>
@@ -2711,10 +2723,10 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>133</v>
+        <v>241</v>
       </c>
       <c r="B32" t="s">
-        <v>92</v>
+        <v>242</v>
       </c>
       <c r="C32" t="s">
         <v>66</v>
@@ -2723,68 +2735,68 @@
         <v>31</v>
       </c>
       <c r="E32">
-        <v>125</v>
+        <v>21.75</v>
       </c>
       <c r="F32">
-        <v>175</v>
+        <v>29</v>
       </c>
       <c r="G32">
-        <v>140</v>
+        <v>26.1</v>
       </c>
       <c r="H32">
-        <v>160</v>
+        <v>29</v>
       </c>
       <c r="I32" t="b">
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>154</v>
+        <v>243</v>
       </c>
       <c r="K32" t="s">
-        <v>186</v>
+        <v>244</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>30</v>
+        <v>133</v>
       </c>
       <c r="B33" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C33" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="D33" t="s">
         <v>31</v>
       </c>
       <c r="E33">
-        <v>1.2999999999999999E-3</v>
+        <v>125</v>
       </c>
       <c r="F33">
-        <v>1.9E-3</v>
+        <v>175</v>
       </c>
       <c r="G33">
-        <v>1.4E-3</v>
+        <v>140</v>
       </c>
       <c r="H33">
-        <v>1.8E-3</v>
+        <v>160</v>
       </c>
       <c r="I33" t="b">
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>176</v>
+        <v>154</v>
       </c>
       <c r="K33" t="s">
-        <v>170</v>
+        <v>186</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="B34" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C34" t="s">
         <v>68</v>
@@ -2793,16 +2805,16 @@
         <v>31</v>
       </c>
       <c r="E34">
-        <v>4</v>
+        <v>1.2999999999999999E-3</v>
       </c>
       <c r="F34">
-        <v>10</v>
+        <v>1.9E-3</v>
       </c>
       <c r="G34">
-        <v>4.3</v>
+        <v>1.4E-3</v>
       </c>
       <c r="H34">
-        <v>8.5</v>
+        <v>1.8E-3</v>
       </c>
       <c r="I34" t="b">
         <v>1</v>
@@ -2811,15 +2823,15 @@
         <v>176</v>
       </c>
       <c r="K34" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B35" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C35" t="s">
         <v>68</v>
@@ -2828,16 +2840,16 @@
         <v>31</v>
       </c>
       <c r="E35">
-        <v>0.5</v>
+        <v>4</v>
       </c>
       <c r="F35">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G35">
-        <v>0.6</v>
+        <v>4.3</v>
       </c>
       <c r="H35">
-        <v>0.94</v>
+        <v>8.5</v>
       </c>
       <c r="I35" t="b">
         <v>1</v>
@@ -2846,15 +2858,15 @@
         <v>176</v>
       </c>
       <c r="K35" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B36" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C36" t="s">
         <v>68</v>
@@ -2863,16 +2875,16 @@
         <v>31</v>
       </c>
       <c r="E36">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="F36">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G36">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="H36">
-        <v>0</v>
+        <v>0.94</v>
       </c>
       <c r="I36" t="b">
         <v>1</v>
@@ -2881,15 +2893,15 @@
         <v>176</v>
       </c>
       <c r="K36" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B37" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C37" t="s">
         <v>68</v>
@@ -2898,16 +2910,16 @@
         <v>31</v>
       </c>
       <c r="E37">
-        <v>1.9</v>
+        <v>0</v>
       </c>
       <c r="F37">
-        <v>2.2000000000000002</v>
+        <v>0</v>
       </c>
       <c r="G37">
-        <v>2.0499999999999998</v>
+        <v>0</v>
       </c>
       <c r="H37">
-        <v>2.15</v>
+        <v>0</v>
       </c>
       <c r="I37" t="b">
         <v>1</v>
@@ -2916,15 +2928,15 @@
         <v>176</v>
       </c>
       <c r="K37" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B38" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C38" t="s">
         <v>68</v>
@@ -2933,16 +2945,16 @@
         <v>31</v>
       </c>
       <c r="E38">
-        <v>1.2</v>
+        <v>1.9</v>
       </c>
       <c r="F38">
-        <v>2.1</v>
+        <v>2.2000000000000002</v>
       </c>
       <c r="G38">
-        <v>1.3</v>
+        <v>2.0499999999999998</v>
       </c>
       <c r="H38">
-        <v>2</v>
+        <v>2.15</v>
       </c>
       <c r="I38" t="b">
         <v>1</v>
@@ -2951,97 +2963,97 @@
         <v>176</v>
       </c>
       <c r="K38" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>71</v>
+        <v>10</v>
       </c>
       <c r="B39" t="s">
-        <v>4</v>
+        <v>98</v>
       </c>
       <c r="C39" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D39" t="s">
         <v>31</v>
       </c>
       <c r="E39">
-        <v>70</v>
+        <v>1.2</v>
       </c>
       <c r="F39">
-        <v>90</v>
+        <v>2.1</v>
       </c>
       <c r="G39">
-        <v>70</v>
+        <v>1.3</v>
       </c>
       <c r="H39">
-        <v>80</v>
+        <v>2</v>
       </c>
       <c r="I39" t="b">
         <v>1</v>
       </c>
       <c r="J39" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="K39" t="s">
-        <v>190</v>
+        <v>174</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>25</v>
+        <v>71</v>
       </c>
       <c r="B40" t="s">
-        <v>47</v>
+        <v>4</v>
       </c>
       <c r="C40" t="s">
-        <v>58</v>
+        <v>69</v>
       </c>
       <c r="D40" t="s">
         <v>31</v>
       </c>
       <c r="E40">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F40">
-        <v>1000</v>
+        <v>90</v>
+      </c>
+      <c r="G40">
+        <v>70</v>
+      </c>
+      <c r="H40">
+        <v>80</v>
       </c>
       <c r="I40" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J40" t="s">
-        <v>70</v>
+        <v>189</v>
       </c>
       <c r="K40" t="s">
-        <v>70</v>
+        <v>190</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
       <c r="B41" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C41" t="s">
         <v>58</v>
       </c>
       <c r="D41" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E41">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F41">
-        <v>0.3</v>
-      </c>
-      <c r="G41">
-        <v>0</v>
-      </c>
-      <c r="H41">
-        <v>0.2</v>
+        <v>1000</v>
       </c>
       <c r="I41" t="b">
         <v>0</v>
@@ -3055,28 +3067,28 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="B42" t="s">
-        <v>197</v>
+        <v>48</v>
       </c>
       <c r="C42" t="s">
         <v>58</v>
       </c>
       <c r="D42" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E42">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F42">
-        <v>100</v>
+        <v>0.3</v>
       </c>
       <c r="G42">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H42">
-        <v>100</v>
+        <v>0.2</v>
       </c>
       <c r="I42" t="b">
         <v>0</v>
@@ -3090,10 +3102,10 @@
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="B43" t="s">
-        <v>50</v>
+        <v>197</v>
       </c>
       <c r="C43" t="s">
         <v>58</v>
@@ -3102,10 +3114,16 @@
         <v>31</v>
       </c>
       <c r="E43">
-        <v>4.3</v>
-      </c>
-      <c r="F43" t="s">
-        <v>5</v>
+        <v>80</v>
+      </c>
+      <c r="F43">
+        <v>100</v>
+      </c>
+      <c r="G43">
+        <v>95</v>
+      </c>
+      <c r="H43">
+        <v>100</v>
       </c>
       <c r="I43" t="b">
         <v>0</v>
@@ -3119,28 +3137,22 @@
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B44" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C44" t="s">
         <v>58</v>
       </c>
       <c r="D44" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E44">
-        <v>0</v>
-      </c>
-      <c r="F44">
-        <v>0.3</v>
-      </c>
-      <c r="G44">
-        <v>0</v>
-      </c>
-      <c r="H44">
-        <v>0.2</v>
+        <v>4.3</v>
+      </c>
+      <c r="F44" t="s">
+        <v>5</v>
       </c>
       <c r="I44" t="b">
         <v>0</v>
@@ -3154,28 +3166,28 @@
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>198</v>
+        <v>48</v>
       </c>
       <c r="C45" t="s">
         <v>58</v>
       </c>
       <c r="D45" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E45">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F45">
-        <v>100</v>
+        <v>0.3</v>
       </c>
       <c r="G45">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H45">
-        <v>100</v>
+        <v>0.2</v>
       </c>
       <c r="I45" t="b">
         <v>0</v>
@@ -3189,10 +3201,10 @@
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C46" t="s">
         <v>58</v>
@@ -3201,16 +3213,16 @@
         <v>31</v>
       </c>
       <c r="E46">
-        <v>1</v>
+        <v>80</v>
       </c>
       <c r="F46">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="G46">
-        <v>1</v>
+        <v>95</v>
       </c>
       <c r="H46">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I46" t="b">
         <v>0</v>
@@ -3224,10 +3236,10 @@
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>23</v>
+        <v>199</v>
       </c>
       <c r="C47" t="s">
         <v>58</v>
@@ -3236,16 +3248,16 @@
         <v>31</v>
       </c>
       <c r="E47">
-        <v>544</v>
+        <v>1</v>
       </c>
       <c r="F47">
-        <v>624</v>
+        <v>1</v>
       </c>
       <c r="G47">
-        <v>564</v>
+        <v>1</v>
       </c>
       <c r="H47">
-        <v>604</v>
+        <v>1</v>
       </c>
       <c r="I47" t="b">
         <v>0</v>
@@ -3259,10 +3271,10 @@
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B48" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C48" t="s">
         <v>58</v>
@@ -3271,16 +3283,16 @@
         <v>31</v>
       </c>
       <c r="E48">
-        <v>98</v>
+        <v>544</v>
       </c>
       <c r="F48">
-        <v>100</v>
+        <v>624</v>
       </c>
       <c r="G48">
-        <v>100</v>
+        <v>564</v>
       </c>
       <c r="H48">
-        <v>100</v>
+        <v>604</v>
       </c>
       <c r="I48" t="b">
         <v>0</v>
@@ -3294,45 +3306,45 @@
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
+        <v>27</v>
+      </c>
+      <c r="B49" t="s">
+        <v>24</v>
+      </c>
+      <c r="C49" t="s">
+        <v>58</v>
+      </c>
+      <c r="D49" t="s">
+        <v>31</v>
+      </c>
+      <c r="E49">
+        <v>98</v>
+      </c>
+      <c r="F49">
+        <v>100</v>
+      </c>
+      <c r="G49">
+        <v>100</v>
+      </c>
+      <c r="H49">
+        <v>100</v>
+      </c>
+      <c r="I49" t="b">
+        <v>0</v>
+      </c>
+      <c r="J49" t="s">
+        <v>70</v>
+      </c>
+      <c r="K49" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
         <v>103</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B50" t="s">
         <v>237</v>
-      </c>
-      <c r="C49" t="s">
-        <v>62</v>
-      </c>
-      <c r="D49" t="s">
-        <v>75</v>
-      </c>
-      <c r="E49">
-        <v>35</v>
-      </c>
-      <c r="F49">
-        <v>40</v>
-      </c>
-      <c r="G49">
-        <v>39</v>
-      </c>
-      <c r="H49">
-        <v>40</v>
-      </c>
-      <c r="I49" t="b">
-        <v>1</v>
-      </c>
-      <c r="J49" t="s">
-        <v>155</v>
-      </c>
-      <c r="K49" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>104</v>
-      </c>
-      <c r="B50" t="s">
-        <v>238</v>
       </c>
       <c r="C50" t="s">
         <v>62</v>
@@ -3356,18 +3368,18 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="K50" t="s">
         <v>161</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B51" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C51" t="s">
         <v>62</v>
@@ -3376,30 +3388,30 @@
         <v>75</v>
       </c>
       <c r="E51">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F51">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G51">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="H51">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="I51" t="b">
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K51" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B52" t="s">
         <v>236</v>
@@ -3426,7 +3438,7 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="K52" t="s">
         <v>163</v>
@@ -3434,10 +3446,10 @@
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="B53" t="s">
-        <v>101</v>
+        <v>236</v>
       </c>
       <c r="C53" t="s">
         <v>62</v>
@@ -3446,30 +3458,30 @@
         <v>75</v>
       </c>
       <c r="E53">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F53">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="G53">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="H53">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="I53" t="b">
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K53" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>111</v>
+        <v>102</v>
       </c>
       <c r="B54" t="s">
         <v>101</v>
@@ -3496,7 +3508,7 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="K54" t="s">
         <v>164</v>
@@ -3504,10 +3516,10 @@
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B55" t="s">
-        <v>122</v>
+        <v>101</v>
       </c>
       <c r="C55" t="s">
         <v>62</v>
@@ -3516,30 +3528,30 @@
         <v>75</v>
       </c>
       <c r="E55">
-        <v>2850</v>
-      </c>
-      <c r="F55" t="s">
-        <v>5</v>
+        <v>150</v>
+      </c>
+      <c r="F55">
+        <v>150</v>
       </c>
       <c r="G55">
-        <v>3000</v>
-      </c>
-      <c r="H55" t="s">
-        <v>5</v>
+        <v>150</v>
+      </c>
+      <c r="H55">
+        <v>150</v>
       </c>
       <c r="I55" t="b">
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="K55" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B56" t="s">
         <v>122</v>
@@ -3566,7 +3578,7 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="K56" t="s">
         <v>160</v>
@@ -3574,42 +3586,42 @@
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>211</v>
+        <v>113</v>
       </c>
       <c r="B57" t="s">
-        <v>240</v>
+        <v>122</v>
       </c>
       <c r="C57" t="s">
         <v>62</v>
       </c>
       <c r="D57" t="s">
-        <v>31</v>
+        <v>75</v>
       </c>
       <c r="E57">
-        <v>30</v>
-      </c>
-      <c r="F57">
-        <v>40</v>
+        <v>2850</v>
+      </c>
+      <c r="F57" t="s">
+        <v>5</v>
       </c>
       <c r="G57">
-        <v>35</v>
-      </c>
-      <c r="H57">
-        <v>40</v>
+        <v>3000</v>
+      </c>
+      <c r="H57" t="s">
+        <v>5</v>
       </c>
       <c r="I57" t="b">
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="K57" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B58" t="s">
         <v>240</v>
@@ -3636,7 +3648,7 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K58" t="s">
         <v>162</v>
@@ -3644,10 +3656,10 @@
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>114</v>
+        <v>212</v>
       </c>
       <c r="B59" t="s">
-        <v>124</v>
+        <v>240</v>
       </c>
       <c r="C59" t="s">
         <v>62</v>
@@ -3656,30 +3668,30 @@
         <v>31</v>
       </c>
       <c r="E59">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F59">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="G59">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H59">
-        <v>0.1</v>
+        <v>40</v>
       </c>
       <c r="I59" t="b">
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="K59" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B60" t="s">
         <v>124</v>
@@ -3706,7 +3718,7 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K60" t="s">
         <v>165</v>
@@ -3714,10 +3726,10 @@
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B61" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C61" t="s">
         <v>62</v>
@@ -3729,27 +3741,27 @@
         <v>0</v>
       </c>
       <c r="F61">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="G61">
         <v>0</v>
       </c>
       <c r="H61">
-        <v>20</v>
+        <v>0.1</v>
       </c>
       <c r="I61" t="b">
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="K61" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B62" t="s">
         <v>125</v>
@@ -3776,7 +3788,7 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K62" t="s">
         <v>166</v>
@@ -3784,10 +3796,10 @@
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B63" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C63" t="s">
         <v>62</v>
@@ -3799,27 +3811,27 @@
         <v>0</v>
       </c>
       <c r="F63">
+        <v>30</v>
+      </c>
+      <c r="G63">
+        <v>0</v>
+      </c>
+      <c r="H63">
         <v>20</v>
       </c>
-      <c r="G63">
-        <v>0</v>
-      </c>
-      <c r="H63">
-        <v>10</v>
-      </c>
       <c r="I63" t="b">
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="K63" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B64" t="s">
         <v>126</v>
@@ -3846,7 +3858,7 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K64" t="s">
         <v>167</v>
@@ -3854,10 +3866,10 @@
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B65" t="s">
-        <v>239</v>
+        <v>126</v>
       </c>
       <c r="C65" t="s">
         <v>62</v>
@@ -3869,27 +3881,27 @@
         <v>0</v>
       </c>
       <c r="F65">
+        <v>20</v>
+      </c>
+      <c r="G65">
+        <v>0</v>
+      </c>
+      <c r="H65">
         <v>10</v>
       </c>
-      <c r="G65">
-        <v>0</v>
-      </c>
-      <c r="H65">
-        <v>5</v>
-      </c>
       <c r="I65" t="b">
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="K65" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B66" t="s">
         <v>239</v>
@@ -3916,7 +3928,7 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="K66" t="s">
         <v>168</v>
@@ -3924,45 +3936,45 @@
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>72</v>
+        <v>121</v>
       </c>
       <c r="B67" t="s">
-        <v>224</v>
+        <v>239</v>
       </c>
       <c r="C67" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D67" t="s">
-        <v>75</v>
+        <v>31</v>
       </c>
       <c r="E67">
         <v>0</v>
       </c>
       <c r="F67">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G67">
         <v>0</v>
       </c>
       <c r="H67">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I67" t="b">
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>222</v>
+        <v>158</v>
       </c>
       <c r="K67" t="s">
-        <v>223</v>
+        <v>168</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>129</v>
+        <v>72</v>
       </c>
       <c r="B68" t="s">
-        <v>130</v>
+        <v>224</v>
       </c>
       <c r="C68" t="s">
         <v>64</v>
@@ -3974,13 +3986,13 @@
         <v>0</v>
       </c>
       <c r="F68">
-        <v>0.1</v>
+        <v>25</v>
       </c>
       <c r="G68">
         <v>0</v>
       </c>
       <c r="H68">
-        <v>0.05</v>
+        <v>10</v>
       </c>
       <c r="I68" t="b">
         <v>1</v>
@@ -3989,50 +4001,50 @@
         <v>222</v>
       </c>
       <c r="K68" t="s">
-        <v>177</v>
+        <v>223</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>201</v>
+        <v>129</v>
       </c>
       <c r="B69" t="s">
-        <v>202</v>
+        <v>130</v>
       </c>
       <c r="C69" t="s">
         <v>64</v>
       </c>
       <c r="D69" t="s">
-        <v>31</v>
+        <v>75</v>
       </c>
       <c r="E69">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F69">
-        <v>30</v>
+        <v>0.1</v>
       </c>
       <c r="G69">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H69">
-        <v>15</v>
+        <v>0.05</v>
       </c>
       <c r="I69" t="b">
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>210</v>
+        <v>222</v>
       </c>
       <c r="K69" t="s">
-        <v>225</v>
+        <v>177</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>228</v>
+        <v>201</v>
       </c>
       <c r="B70" t="s">
-        <v>215</v>
+        <v>202</v>
       </c>
       <c r="C70" t="s">
         <v>64</v>
@@ -4041,33 +4053,33 @@
         <v>31</v>
       </c>
       <c r="E70">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F70">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="G70">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H70">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="I70" t="b">
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>226</v>
+        <v>210</v>
       </c>
       <c r="K70" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>73</v>
+        <v>228</v>
       </c>
       <c r="B71" t="s">
-        <v>203</v>
+        <v>215</v>
       </c>
       <c r="C71" t="s">
         <v>64</v>
@@ -4076,33 +4088,33 @@
         <v>31</v>
       </c>
       <c r="E71">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F71">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="G71">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="H71">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="I71" t="b">
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>206</v>
+        <v>226</v>
       </c>
       <c r="K71" t="s">
-        <v>205</v>
+        <v>227</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B72" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C72" t="s">
         <v>64</v>
@@ -4111,13 +4123,13 @@
         <v>31</v>
       </c>
       <c r="E72">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="F72">
         <v>99</v>
       </c>
       <c r="G72">
-        <v>92.5</v>
+        <v>90</v>
       </c>
       <c r="H72">
         <v>99</v>
@@ -4126,7 +4138,7 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K72" t="s">
         <v>205</v>
@@ -4134,45 +4146,45 @@
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B73" t="s">
-        <v>90</v>
+        <v>204</v>
       </c>
       <c r="C73" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="D73" t="s">
         <v>31</v>
       </c>
       <c r="E73">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="F73">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G73">
-        <v>95</v>
+        <v>92.5</v>
       </c>
       <c r="H73">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I73" t="b">
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>146</v>
+        <v>207</v>
       </c>
       <c r="K73" t="s">
-        <v>185</v>
+        <v>205</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B74" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C74" t="s">
         <v>61</v>
@@ -4181,13 +4193,13 @@
         <v>31</v>
       </c>
       <c r="E74">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="F74">
         <v>100</v>
       </c>
       <c r="G74">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="H74">
         <v>100</v>
@@ -4199,15 +4211,15 @@
         <v>146</v>
       </c>
       <c r="K74" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B75" t="s">
-        <v>131</v>
+        <v>91</v>
       </c>
       <c r="C75" t="s">
         <v>61</v>
@@ -4216,68 +4228,68 @@
         <v>31</v>
       </c>
       <c r="E75">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="F75">
-        <v>175</v>
+        <v>100</v>
       </c>
       <c r="G75">
-        <v>140</v>
+        <v>75</v>
       </c>
       <c r="H75">
-        <v>160</v>
+        <v>100</v>
       </c>
       <c r="I75" t="b">
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="K75" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>143</v>
+        <v>78</v>
       </c>
       <c r="B76" t="s">
-        <v>218</v>
+        <v>131</v>
       </c>
       <c r="C76" t="s">
-        <v>67</v>
+        <v>61</v>
       </c>
       <c r="D76" t="s">
         <v>31</v>
       </c>
       <c r="E76">
-        <v>50</v>
+        <v>125</v>
       </c>
       <c r="F76">
-        <v>55</v>
+        <v>175</v>
       </c>
       <c r="G76">
-        <v>50</v>
+        <v>140</v>
       </c>
       <c r="H76">
-        <v>52.5</v>
+        <v>160</v>
       </c>
       <c r="I76" t="b">
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>178</v>
+        <v>147</v>
       </c>
       <c r="K76" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="B77" t="s">
-        <v>194</v>
+        <v>218</v>
       </c>
       <c r="C77" t="s">
         <v>67</v>
@@ -4286,33 +4298,33 @@
         <v>31</v>
       </c>
       <c r="E77">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="F77">
-        <v>100</v>
+        <v>55</v>
       </c>
       <c r="G77">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="H77">
-        <v>100</v>
+        <v>52.5</v>
       </c>
       <c r="I77" t="b">
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>192</v>
+        <v>178</v>
       </c>
       <c r="K77" t="s">
-        <v>191</v>
+        <v>179</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="B78" t="s">
-        <v>15</v>
+        <v>194</v>
       </c>
       <c r="C78" t="s">
         <v>67</v>
@@ -4321,13 +4333,13 @@
         <v>31</v>
       </c>
       <c r="E78">
-        <v>99</v>
+        <v>60</v>
       </c>
       <c r="F78">
         <v>100</v>
       </c>
       <c r="G78">
-        <v>99.5</v>
+        <v>90</v>
       </c>
       <c r="H78">
         <v>100</v>
@@ -4336,18 +4348,18 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>182</v>
+        <v>192</v>
       </c>
       <c r="K78" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="B79" t="s">
-        <v>136</v>
+        <v>15</v>
       </c>
       <c r="C79" t="s">
         <v>67</v>
@@ -4356,16 +4368,16 @@
         <v>31</v>
       </c>
       <c r="E79">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="F79">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="G79">
-        <v>0</v>
+        <v>99.5</v>
       </c>
       <c r="H79">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="I79" t="b">
         <v>1</v>
@@ -4374,15 +4386,15 @@
         <v>182</v>
       </c>
       <c r="K79" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="B80" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="C80" t="s">
         <v>67</v>
@@ -4391,33 +4403,33 @@
         <v>31</v>
       </c>
       <c r="E80">
-        <v>0.5</v>
-      </c>
-      <c r="F80" t="s">
+        <v>0</v>
+      </c>
+      <c r="F80">
+        <v>15</v>
+      </c>
+      <c r="G80">
+        <v>0</v>
+      </c>
+      <c r="H80">
         <v>5</v>
       </c>
-      <c r="G80">
-        <v>1</v>
-      </c>
-      <c r="H80" t="s">
-        <v>5</v>
-      </c>
       <c r="I80" t="b">
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>193</v>
+        <v>182</v>
       </c>
       <c r="K80" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>19</v>
+        <v>139</v>
       </c>
       <c r="B81" t="s">
-        <v>20</v>
+        <v>140</v>
       </c>
       <c r="C81" t="s">
         <v>67</v>
@@ -4426,33 +4438,33 @@
         <v>31</v>
       </c>
       <c r="E81">
-        <v>0</v>
-      </c>
-      <c r="F81">
-        <v>0</v>
+        <v>0.5</v>
+      </c>
+      <c r="F81" t="s">
+        <v>5</v>
       </c>
       <c r="G81">
-        <v>0</v>
-      </c>
-      <c r="H81">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H81" t="s">
+        <v>5</v>
       </c>
       <c r="I81" t="b">
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>148</v>
+        <v>193</v>
       </c>
       <c r="K81" t="s">
-        <v>169</v>
+        <v>183</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B82" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C82" t="s">
         <v>67</v>
@@ -4461,33 +4473,33 @@
         <v>31</v>
       </c>
       <c r="E82">
-        <v>14.5</v>
+        <v>0</v>
       </c>
       <c r="F82">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G82">
-        <v>26.1</v>
+        <v>0</v>
       </c>
       <c r="H82">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I82" t="b">
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>193</v>
+        <v>148</v>
       </c>
       <c r="K82" t="s">
-        <v>17</v>
+        <v>169</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B83" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C83" t="s">
         <v>67</v>
@@ -4496,68 +4508,68 @@
         <v>31</v>
       </c>
       <c r="E83">
-        <v>5.0000000000000001E-4</v>
+        <v>14.5</v>
       </c>
       <c r="F83">
-        <v>8.0000000000000004E-4</v>
+        <v>100</v>
       </c>
       <c r="G83">
-        <v>2.0000000000000001E-4</v>
+        <v>26.1</v>
       </c>
       <c r="H83">
-        <v>5.0000000000000001E-4</v>
+        <v>100</v>
       </c>
       <c r="I83" t="b">
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>209</v>
+        <v>193</v>
       </c>
       <c r="K83" t="s">
-        <v>208</v>
+        <v>17</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>229</v>
+        <v>13</v>
       </c>
       <c r="B84" t="s">
-        <v>230</v>
+        <v>14</v>
       </c>
       <c r="C84" t="s">
-        <v>200</v>
+        <v>67</v>
       </c>
       <c r="D84" t="s">
         <v>31</v>
       </c>
       <c r="E84">
-        <v>0.05</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="F84">
-        <v>0.08</v>
+        <v>8.0000000000000004E-4</v>
       </c>
       <c r="G84">
-        <v>0.02</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="H84">
-        <v>0.05</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="I84" t="b">
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>232</v>
+        <v>209</v>
       </c>
       <c r="K84" t="s">
-        <v>233</v>
+        <v>208</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>16</v>
+        <v>229</v>
       </c>
       <c r="B85" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="C85" t="s">
         <v>200</v>
@@ -4566,33 +4578,33 @@
         <v>31</v>
       </c>
       <c r="E85">
-        <v>5</v>
+        <v>0.05</v>
       </c>
       <c r="F85">
-        <v>100</v>
+        <v>0.08</v>
       </c>
       <c r="G85">
-        <v>20</v>
+        <v>0.02</v>
       </c>
       <c r="H85">
-        <v>100</v>
+        <v>0.05</v>
       </c>
       <c r="I85" t="b">
         <v>1</v>
       </c>
       <c r="J85" t="s">
-        <v>193</v>
+        <v>232</v>
       </c>
       <c r="K85" t="s">
-        <v>184</v>
+        <v>233</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="B86" t="s">
-        <v>21</v>
+        <v>231</v>
       </c>
       <c r="C86" t="s">
         <v>200</v>
@@ -4601,33 +4613,33 @@
         <v>31</v>
       </c>
       <c r="E86">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F86">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="G86">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H86">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="I86" t="b">
         <v>1</v>
       </c>
       <c r="J86" t="s">
-        <v>159</v>
+        <v>193</v>
       </c>
       <c r="K86" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>56</v>
+        <v>22</v>
       </c>
       <c r="B87" t="s">
-        <v>216</v>
+        <v>21</v>
       </c>
       <c r="C87" t="s">
         <v>200</v>
@@ -4636,29 +4648,64 @@
         <v>31</v>
       </c>
       <c r="E87">
+        <v>0</v>
+      </c>
+      <c r="F87">
+        <v>95</v>
+      </c>
+      <c r="G87">
+        <v>0</v>
+      </c>
+      <c r="H87">
+        <v>80</v>
+      </c>
+      <c r="I87" t="b">
+        <v>1</v>
+      </c>
+      <c r="J87" t="s">
+        <v>159</v>
+      </c>
+      <c r="K87" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>56</v>
+      </c>
+      <c r="B88" t="s">
+        <v>216</v>
+      </c>
+      <c r="C88" t="s">
+        <v>200</v>
+      </c>
+      <c r="D88" t="s">
+        <v>31</v>
+      </c>
+      <c r="E88">
         <v>90</v>
       </c>
-      <c r="F87">
+      <c r="F88">
         <v>100</v>
       </c>
-      <c r="G87">
+      <c r="G88">
         <v>95</v>
       </c>
-      <c r="H87">
+      <c r="H88">
         <v>100</v>
       </c>
-      <c r="I87" t="b">
-        <v>1</v>
-      </c>
-      <c r="J87" t="s">
+      <c r="I88" t="b">
+        <v>1</v>
+      </c>
+      <c r="J88" t="s">
         <v>193</v>
       </c>
-      <c r="K87" t="s">
+      <c r="K88" t="s">
         <v>56</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K85" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K86" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated component metrics for DNA yield variability
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EF54474-ED57-44DB-BBC6-FF599AEE2217}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8958431-9DC5-4FD8-889B-F9BA36EC42F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -155,9 +155,6 @@
     <t>Name</t>
   </si>
   <si>
-    <t>Variability in DNA extraction yield (normalised interquartile range). UL of 95% CI must meet target.</t>
-  </si>
-  <si>
     <t>ex_fragmented_DNA_size</t>
   </si>
   <si>
@@ -182,9 +179,6 @@
     <t>Quantity of DNA (ng) after enzymatic fragmentation</t>
   </si>
   <si>
-    <t>Variability in DNA quantity post fragmentation (normalised interquartile range). UL of 95% CI must meet target.</t>
-  </si>
-  <si>
     <t>ex_amplified_DNA_conc</t>
   </si>
   <si>
@@ -203,9 +197,6 @@
     <t>ms_ligated_DNA_yield_variability</t>
   </si>
   <si>
-    <t>Variability in DNA quantity post adaptor ligation (normalised interquartile range). UL of 95% CI must meet target.</t>
-  </si>
-  <si>
     <t>coverage_overlap_ex_ms</t>
   </si>
   <si>
@@ -771,6 +762,15 @@
   </si>
   <si>
     <t>pct_coverage.40X</t>
+  </si>
+  <si>
+    <t>Variability in DNA extraction yield (normalised interquartile range)</t>
+  </si>
+  <si>
+    <t>Variability in DNA quantity post fragmentation (normalised interquartile range)</t>
+  </si>
+  <si>
+    <t>Variability in DNA quantity post adaptor ligation (normalised interquartile range)</t>
   </si>
 </sst>
 </file>
@@ -1645,7 +1645,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" customWidth="1"/>
-    <col min="2" max="2" width="103.140625" customWidth="1"/>
+    <col min="2" max="2" width="123.140625" customWidth="1"/>
     <col min="3" max="4" width="35.28515625" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
@@ -1683,21 +1683,21 @@
         <v>37</v>
       </c>
       <c r="J1" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
       <c r="K1" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B2" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C2" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D2" t="s">
         <v>31</v>
@@ -1712,21 +1712,21 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K2" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B3" t="s">
-        <v>39</v>
+        <v>242</v>
       </c>
       <c r="C3" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D3" t="s">
         <v>32</v>
@@ -1747,21 +1747,21 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K3" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B4" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="D4" t="s">
         <v>31</v>
@@ -1782,21 +1782,21 @@
         <v>0</v>
       </c>
       <c r="J4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K4" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="B5" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C5" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D5" t="s">
         <v>31</v>
@@ -1811,21 +1811,21 @@
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K5" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>48</v>
+        <v>243</v>
       </c>
       <c r="C6" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D6" t="s">
         <v>32</v>
@@ -1846,21 +1846,21 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K6" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B7" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C7" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D7" t="s">
         <v>31</v>
@@ -1875,21 +1875,21 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K7" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>244</v>
       </c>
       <c r="C8" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D8" t="s">
         <v>32</v>
@@ -1910,10 +1910,10 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K8" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -1921,10 +1921,10 @@
         <v>28</v>
       </c>
       <c r="B9" t="s">
-        <v>79</v>
+        <v>76</v>
       </c>
       <c r="C9" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D9" t="s">
         <v>31</v>
@@ -1945,10 +1945,10 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K9" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -1956,10 +1956,10 @@
         <v>29</v>
       </c>
       <c r="B10" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="C10" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D10" t="s">
         <v>31</v>
@@ -1980,10 +1980,10 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K10" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -1991,10 +1991,10 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C11" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D11" t="s">
         <v>31</v>
@@ -2015,10 +2015,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="K11" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -2026,10 +2026,10 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C12" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D12" t="s">
         <v>31</v>
@@ -2050,21 +2050,21 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="K12" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="B13" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C13" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D13" t="s">
         <v>31</v>
@@ -2085,21 +2085,21 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="K13" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="B14" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C14" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D14" t="s">
         <v>31</v>
@@ -2120,21 +2120,21 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="K14" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B15" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C15" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D15" t="s">
         <v>31</v>
@@ -2155,21 +2155,21 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="K15" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B16" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C16" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D16" t="s">
         <v>31</v>
@@ -2190,21 +2190,21 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="K16" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B17" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C17" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D17" t="s">
         <v>31</v>
@@ -2225,21 +2225,21 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="K17" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B18" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C18" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D18" t="s">
         <v>31</v>
@@ -2260,21 +2260,21 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="K18" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B19" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="C19" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D19" t="s">
         <v>31</v>
@@ -2295,21 +2295,21 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K19" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B20" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="C20" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="D20" t="s">
         <v>31</v>
@@ -2330,21 +2330,21 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="K20" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B21" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C21" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D21" t="s">
         <v>31</v>
@@ -2365,21 +2365,21 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K21" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B22" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C22" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D22" t="s">
         <v>31</v>
@@ -2400,21 +2400,21 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="K22" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B23" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C23" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D23" t="s">
         <v>31</v>
@@ -2435,21 +2435,21 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K23" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B24" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C24" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D24" t="s">
         <v>31</v>
@@ -2470,21 +2470,21 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="K24" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B25" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C25" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D25" t="s">
         <v>31</v>
@@ -2505,21 +2505,21 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K25" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="B26" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C26" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D26" t="s">
         <v>31</v>
@@ -2540,21 +2540,21 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="K26" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="B27" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="C27" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D27" t="s">
         <v>31</v>
@@ -2575,21 +2575,21 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="K27" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B28" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="C28" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="D28" t="s">
         <v>31</v>
@@ -2610,21 +2610,21 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="K28" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B29" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="C29" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="D29" t="s">
         <v>31</v>
@@ -2645,21 +2645,21 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="B30" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="C30" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D30" t="s">
         <v>31</v>
@@ -2680,21 +2680,21 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="K30" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="B31" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
       <c r="C31" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D31" t="s">
         <v>31</v>
@@ -2715,21 +2715,21 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="K31" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="B32" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="C32" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D32" t="s">
         <v>31</v>
@@ -2750,21 +2750,21 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="K32" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="B33" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="C33" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="D33" t="s">
         <v>31</v>
@@ -2785,10 +2785,10 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="K33" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
@@ -2796,10 +2796,10 @@
         <v>30</v>
       </c>
       <c r="B34" t="s">
-        <v>93</v>
+        <v>90</v>
       </c>
       <c r="C34" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D34" t="s">
         <v>31</v>
@@ -2820,10 +2820,10 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="K34" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -2831,10 +2831,10 @@
         <v>6</v>
       </c>
       <c r="B35" t="s">
-        <v>94</v>
+        <v>91</v>
       </c>
       <c r="C35" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D35" t="s">
         <v>31</v>
@@ -2855,10 +2855,10 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="K35" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -2866,10 +2866,10 @@
         <v>7</v>
       </c>
       <c r="B36" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="C36" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D36" t="s">
         <v>31</v>
@@ -2890,10 +2890,10 @@
         <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="K36" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
@@ -2901,10 +2901,10 @@
         <v>8</v>
       </c>
       <c r="B37" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="C37" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D37" t="s">
         <v>31</v>
@@ -2925,10 +2925,10 @@
         <v>1</v>
       </c>
       <c r="J37" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="K37" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
@@ -2936,10 +2936,10 @@
         <v>9</v>
       </c>
       <c r="B38" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="C38" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D38" t="s">
         <v>31</v>
@@ -2960,10 +2960,10 @@
         <v>1</v>
       </c>
       <c r="J38" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="K38" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
@@ -2971,10 +2971,10 @@
         <v>10</v>
       </c>
       <c r="B39" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C39" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="D39" t="s">
         <v>31</v>
@@ -2995,21 +2995,21 @@
         <v>1</v>
       </c>
       <c r="J39" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="K39" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="B40" t="s">
         <v>4</v>
       </c>
       <c r="C40" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="D40" t="s">
         <v>31</v>
@@ -3030,10 +3030,10 @@
         <v>1</v>
       </c>
       <c r="J40" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="K40" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
@@ -3041,10 +3041,10 @@
         <v>25</v>
       </c>
       <c r="B41" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C41" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D41" t="s">
         <v>31</v>
@@ -3059,10 +3059,10 @@
         <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K41" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
@@ -3070,10 +3070,10 @@
         <v>33</v>
       </c>
       <c r="B42" t="s">
-        <v>48</v>
+        <v>243</v>
       </c>
       <c r="C42" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D42" t="s">
         <v>32</v>
@@ -3094,21 +3094,21 @@
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K42" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B43" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C43" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D43" t="s">
         <v>31</v>
@@ -3129,21 +3129,21 @@
         <v>0</v>
       </c>
       <c r="J43" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K43" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="B44" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C44" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D44" t="s">
         <v>31</v>
@@ -3158,21 +3158,21 @@
         <v>0</v>
       </c>
       <c r="J44" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K44" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>48</v>
+        <v>243</v>
       </c>
       <c r="C45" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D45" t="s">
         <v>32</v>
@@ -3181,33 +3181,33 @@
         <v>0</v>
       </c>
       <c r="F45">
+        <v>0.4</v>
+      </c>
+      <c r="G45">
+        <v>0</v>
+      </c>
+      <c r="H45">
         <v>0.3</v>
       </c>
-      <c r="G45">
-        <v>0</v>
-      </c>
-      <c r="H45">
-        <v>0.2</v>
-      </c>
       <c r="I45" t="b">
         <v>0</v>
       </c>
       <c r="J45" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K45" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B46" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C46" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D46" t="s">
         <v>31</v>
@@ -3228,21 +3228,21 @@
         <v>0</v>
       </c>
       <c r="J46" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K46" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B47" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C47" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D47" t="s">
         <v>31</v>
@@ -3263,10 +3263,10 @@
         <v>0</v>
       </c>
       <c r="J47" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K47" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
@@ -3277,7 +3277,7 @@
         <v>23</v>
       </c>
       <c r="C48" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D48" t="s">
         <v>31</v>
@@ -3298,10 +3298,10 @@
         <v>0</v>
       </c>
       <c r="J48" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K48" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
@@ -3312,7 +3312,7 @@
         <v>24</v>
       </c>
       <c r="C49" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="D49" t="s">
         <v>31</v>
@@ -3333,24 +3333,24 @@
         <v>0</v>
       </c>
       <c r="J49" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="K49" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B50" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="C50" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D50" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E50">
         <v>35</v>
@@ -3368,24 +3368,24 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K50" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="51" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B51" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="C51" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D51" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E51">
         <v>35</v>
@@ -3403,24 +3403,24 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="K51" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B52" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C52" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D52" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E52">
         <v>0</v>
@@ -3438,24 +3438,24 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K52" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B53" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="C53" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D53" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E53">
         <v>0</v>
@@ -3473,24 +3473,24 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="K53" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B54" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C54" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D54" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E54">
         <v>150</v>
@@ -3508,24 +3508,24 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K54" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="B55" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C55" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D55" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E55">
         <v>150</v>
@@ -3543,24 +3543,24 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="K55" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="B56" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C56" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D56" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E56">
         <v>2850</v>
@@ -3578,24 +3578,24 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="K56" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="B57" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="C57" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D57" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E57">
         <v>2850</v>
@@ -3613,21 +3613,21 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="K57" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="B58" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="C58" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D58" t="s">
         <v>31</v>
@@ -3648,21 +3648,21 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="K58" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B59" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="C59" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D59" t="s">
         <v>31</v>
@@ -3683,21 +3683,21 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="K59" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="B60" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C60" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D60" t="s">
         <v>31</v>
@@ -3718,21 +3718,21 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="K60" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="B61" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="C61" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D61" t="s">
         <v>31</v>
@@ -3753,21 +3753,21 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="K61" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="B62" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C62" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D62" t="s">
         <v>31</v>
@@ -3788,21 +3788,21 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="K62" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="B63" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C63" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D63" t="s">
         <v>31</v>
@@ -3823,21 +3823,21 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="K63" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="B64" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C64" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D64" t="s">
         <v>31</v>
@@ -3858,21 +3858,21 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="K64" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="B65" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="C65" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D65" t="s">
         <v>31</v>
@@ -3893,21 +3893,21 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="K65" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="B66" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="C66" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D66" t="s">
         <v>31</v>
@@ -3928,21 +3928,21 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="K66" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B67" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="C67" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="D67" t="s">
         <v>31</v>
@@ -3963,24 +3963,24 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="K67" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
+        <v>69</v>
+      </c>
+      <c r="B68" t="s">
+        <v>221</v>
+      </c>
+      <c r="C68" t="s">
+        <v>61</v>
+      </c>
+      <c r="D68" t="s">
         <v>72</v>
-      </c>
-      <c r="B68" t="s">
-        <v>224</v>
-      </c>
-      <c r="C68" t="s">
-        <v>64</v>
-      </c>
-      <c r="D68" t="s">
-        <v>75</v>
       </c>
       <c r="E68">
         <v>0</v>
@@ -3998,24 +3998,24 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="K68" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B69" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C69" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D69" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="E69">
         <v>0</v>
@@ -4033,21 +4033,21 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="K69" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B70" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="C70" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D70" t="s">
         <v>31</v>
@@ -4068,21 +4068,21 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="K70" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="B71" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C71" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D71" t="s">
         <v>31</v>
@@ -4103,21 +4103,21 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="K71" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B72" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C72" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D72" t="s">
         <v>31</v>
@@ -4138,21 +4138,21 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="K72" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B73" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="C73" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="D73" t="s">
         <v>31</v>
@@ -4173,21 +4173,21 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="K73" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="B74" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="C74" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D74" t="s">
         <v>31</v>
@@ -4208,21 +4208,21 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="K74" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="B75" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="C75" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D75" t="s">
         <v>31</v>
@@ -4243,21 +4243,21 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="K75" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="B76" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C76" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D76" t="s">
         <v>31</v>
@@ -4278,21 +4278,21 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="K76" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="B77" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C77" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D77" t="s">
         <v>31</v>
@@ -4313,21 +4313,21 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="K77" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B78" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C78" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D78" t="s">
         <v>31</v>
@@ -4348,21 +4348,21 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="K78" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B79" t="s">
         <v>15</v>
       </c>
       <c r="C79" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D79" t="s">
         <v>31</v>
@@ -4383,21 +4383,21 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="K79" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="B80" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C80" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D80" t="s">
         <v>31</v>
@@ -4418,21 +4418,21 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="K80" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="B81" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C81" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D81" t="s">
         <v>31</v>
@@ -4453,10 +4453,10 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="K81" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
@@ -4467,7 +4467,7 @@
         <v>20</v>
       </c>
       <c r="C82" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D82" t="s">
         <v>31</v>
@@ -4488,10 +4488,10 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="K82" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
@@ -4502,7 +4502,7 @@
         <v>18</v>
       </c>
       <c r="C83" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D83" t="s">
         <v>31</v>
@@ -4523,7 +4523,7 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="K83" t="s">
         <v>17</v>
@@ -4537,7 +4537,7 @@
         <v>14</v>
       </c>
       <c r="C84" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D84" t="s">
         <v>31</v>
@@ -4558,21 +4558,21 @@
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="K84" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B85" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="C85" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D85" t="s">
         <v>31</v>
@@ -4593,10 +4593,10 @@
         <v>1</v>
       </c>
       <c r="J85" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="K85" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
@@ -4604,10 +4604,10 @@
         <v>16</v>
       </c>
       <c r="B86" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="C86" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D86" t="s">
         <v>31</v>
@@ -4628,10 +4628,10 @@
         <v>1</v>
       </c>
       <c r="J86" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="K86" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.25">
@@ -4642,7 +4642,7 @@
         <v>21</v>
       </c>
       <c r="C87" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D87" t="s">
         <v>31</v>
@@ -4663,21 +4663,21 @@
         <v>1</v>
       </c>
       <c r="J87" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="K87" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B88" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C88" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D88" t="s">
         <v>31</v>
@@ -4698,10 +4698,10 @@
         <v>1</v>
       </c>
       <c r="J88" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="K88" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated targets for ms coverage at depth threshold and removed hardcoded depth value
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8958431-9DC5-4FD8-889B-F9BA36EC42F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68CB76BB-89F2-45F8-A6FD-640F5715532E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -755,15 +755,9 @@
     <t>ms_coverage_at_depth_threshold</t>
   </si>
   <si>
-    <t>Percentage of genome with depth &gt; 40X</t>
-  </si>
-  <si>
     <t>_coverage_by_depth.json</t>
   </si>
   <si>
-    <t>pct_coverage.40X</t>
-  </si>
-  <si>
     <t>Variability in DNA extraction yield (normalised interquartile range)</t>
   </si>
   <si>
@@ -771,6 +765,12 @@
   </si>
   <si>
     <t>Variability in DNA quantity post adaptor ligation (normalised interquartile range)</t>
+  </si>
+  <si>
+    <t>pct_coverage_min_depth</t>
+  </si>
+  <si>
+    <t>Percentage of genome with depth &gt;= minimum MS depth value defined in config</t>
   </si>
 </sst>
 </file>
@@ -1723,7 +1723,7 @@
         <v>41</v>
       </c>
       <c r="B3" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C3" t="s">
         <v>54</v>
@@ -1822,7 +1822,7 @@
         <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C6" t="s">
         <v>56</v>
@@ -1886,7 +1886,7 @@
         <v>52</v>
       </c>
       <c r="B8" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C8" t="s">
         <v>56</v>
@@ -2726,7 +2726,7 @@
         <v>238</v>
       </c>
       <c r="B32" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="C32" t="s">
         <v>63</v>
@@ -2738,22 +2738,22 @@
         <v>21.75</v>
       </c>
       <c r="F32">
-        <v>29</v>
+        <v>100</v>
       </c>
       <c r="G32">
         <v>26.1</v>
       </c>
       <c r="H32">
-        <v>29</v>
+        <v>100</v>
       </c>
       <c r="I32" t="b">
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="K32" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -3070,7 +3070,7 @@
         <v>33</v>
       </c>
       <c r="B42" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C42" t="s">
         <v>55</v>
@@ -3169,7 +3169,7 @@
         <v>43</v>
       </c>
       <c r="B45" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C45" t="s">
         <v>55</v>

</xml_diff>

<commit_message>
Fixed region definition in ms_candidate_germ_variants
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68CB76BB-89F2-45F8-A6FD-640F5715532E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20836419-948E-4ED5-A5A8-9DCD71467FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -2817,7 +2817,7 @@
         <v>1.8E-3</v>
       </c>
       <c r="I34" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J34" t="s">
         <v>173</v>
@@ -2852,7 +2852,7 @@
         <v>8.5</v>
       </c>
       <c r="I35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J35" t="s">
         <v>173</v>
@@ -2887,7 +2887,7 @@
         <v>0.94</v>
       </c>
       <c r="I36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J36" t="s">
         <v>173</v>
@@ -2922,7 +2922,7 @@
         <v>0</v>
       </c>
       <c r="I37" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J37" t="s">
         <v>173</v>
@@ -2957,7 +2957,7 @@
         <v>2.15</v>
       </c>
       <c r="I38" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J38" t="s">
         <v>173</v>
@@ -2992,7 +2992,7 @@
         <v>2</v>
       </c>
       <c r="I39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J39" t="s">
         <v>173</v>

</xml_diff>

<commit_message>
Updated component metric thresholds (ex_bases_trimmed, coverage_overlap_ex_ms)
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20836419-948E-4ED5-A5A8-9DCD71467FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AF8D20C-EECA-4786-B788-CEB994176079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="1200" yWindow="1210" windowWidth="18010" windowHeight="18910" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -1642,19 +1642,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
   <dimension ref="A1:K88"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="35.140625" customWidth="1"/>
-    <col min="2" max="2" width="123.140625" customWidth="1"/>
-    <col min="3" max="4" width="35.28515625" customWidth="1"/>
+    <col min="1" max="1" width="35.1796875" customWidth="1"/>
+    <col min="2" max="2" width="123.1796875" customWidth="1"/>
+    <col min="3" max="4" width="35.26953125" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" customWidth="1"/>
-    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="76.85546875" customWidth="1"/>
+    <col min="9" max="9" width="12.81640625" customWidth="1"/>
+    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="76.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>38</v>
       </c>
@@ -1689,7 +1689,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>40</v>
       </c>
@@ -1718,7 +1718,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>41</v>
       </c>
@@ -1753,7 +1753,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>42</v>
       </c>
@@ -1788,7 +1788,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>50</v>
       </c>
@@ -1817,7 +1817,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>49</v>
       </c>
@@ -1852,7 +1852,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>51</v>
       </c>
@@ -1881,7 +1881,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>52</v>
       </c>
@@ -1916,7 +1916,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>28</v>
       </c>
@@ -1951,7 +1951,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -1986,7 +1986,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -2021,7 +2021,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>12</v>
       </c>
@@ -2056,7 +2056,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>106</v>
       </c>
@@ -2091,7 +2091,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>107</v>
       </c>
@@ -2126,7 +2126,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>104</v>
       </c>
@@ -2161,7 +2161,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>105</v>
       </c>
@@ -2196,7 +2196,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -2231,7 +2231,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>97</v>
       </c>
@@ -2266,7 +2266,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>210</v>
       </c>
@@ -2301,7 +2301,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>211</v>
       </c>
@@ -2336,7 +2336,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>78</v>
       </c>
@@ -2371,7 +2371,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>79</v>
       </c>
@@ -2406,7 +2406,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>80</v>
       </c>
@@ -2441,7 +2441,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>81</v>
       </c>
@@ -2476,7 +2476,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>82</v>
       </c>
@@ -2511,7 +2511,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>83</v>
       </c>
@@ -2546,7 +2546,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>84</v>
       </c>
@@ -2581,7 +2581,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>85</v>
       </c>
@@ -2616,7 +2616,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>86</v>
       </c>
@@ -2651,7 +2651,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>132</v>
       </c>
@@ -2686,7 +2686,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>131</v>
       </c>
@@ -2721,7 +2721,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>238</v>
       </c>
@@ -2756,7 +2756,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>130</v>
       </c>
@@ -2791,7 +2791,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>30</v>
       </c>
@@ -2826,7 +2826,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>6</v>
       </c>
@@ -2861,7 +2861,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>7</v>
       </c>
@@ -2896,7 +2896,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>8</v>
       </c>
@@ -2931,7 +2931,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>9</v>
       </c>
@@ -2966,7 +2966,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>10</v>
       </c>
@@ -3001,7 +3001,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>68</v>
       </c>
@@ -3036,7 +3036,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>25</v>
       </c>
@@ -3065,7 +3065,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>33</v>
       </c>
@@ -3100,7 +3100,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>39</v>
       </c>
@@ -3135,7 +3135,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>47</v>
       </c>
@@ -3164,7 +3164,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>43</v>
       </c>
@@ -3199,7 +3199,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>44</v>
       </c>
@@ -3234,7 +3234,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>45</v>
       </c>
@@ -3269,7 +3269,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>26</v>
       </c>
@@ -3304,7 +3304,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>27</v>
       </c>
@@ -3339,7 +3339,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>100</v>
       </c>
@@ -3374,7 +3374,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="51" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>101</v>
       </c>
@@ -3409,7 +3409,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>102</v>
       </c>
@@ -3444,7 +3444,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>103</v>
       </c>
@@ -3479,7 +3479,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>99</v>
       </c>
@@ -3514,7 +3514,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>108</v>
       </c>
@@ -3549,7 +3549,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>109</v>
       </c>
@@ -3584,7 +3584,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>110</v>
       </c>
@@ -3619,7 +3619,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>208</v>
       </c>
@@ -3654,7 +3654,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>209</v>
       </c>
@@ -3689,7 +3689,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>111</v>
       </c>
@@ -3724,7 +3724,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>112</v>
       </c>
@@ -3759,7 +3759,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>113</v>
       </c>
@@ -3794,7 +3794,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>114</v>
       </c>
@@ -3829,7 +3829,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>115</v>
       </c>
@@ -3864,7 +3864,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>116</v>
       </c>
@@ -3899,7 +3899,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>117</v>
       </c>
@@ -3934,7 +3934,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>118</v>
       </c>
@@ -3969,7 +3969,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>69</v>
       </c>
@@ -4004,7 +4004,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>126</v>
       </c>
@@ -4039,7 +4039,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>198</v>
       </c>
@@ -4056,13 +4056,13 @@
         <v>1</v>
       </c>
       <c r="F70">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G70">
         <v>1</v>
       </c>
       <c r="H70">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="I70" t="b">
         <v>1</v>
@@ -4074,7 +4074,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>225</v>
       </c>
@@ -4109,7 +4109,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>70</v>
       </c>
@@ -4144,7 +4144,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>71</v>
       </c>
@@ -4179,7 +4179,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>74</v>
       </c>
@@ -4214,7 +4214,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>73</v>
       </c>
@@ -4249,7 +4249,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>75</v>
       </c>
@@ -4284,7 +4284,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>140</v>
       </c>
@@ -4319,7 +4319,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>129</v>
       </c>
@@ -4354,7 +4354,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>135</v>
       </c>
@@ -4389,7 +4389,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>134</v>
       </c>
@@ -4424,7 +4424,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>136</v>
       </c>
@@ -4459,7 +4459,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>19</v>
       </c>
@@ -4494,7 +4494,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>17</v>
       </c>
@@ -4529,7 +4529,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>13</v>
       </c>
@@ -4564,7 +4564,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A85" t="s">
         <v>226</v>
       </c>
@@ -4599,7 +4599,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A86" t="s">
         <v>16</v>
       </c>
@@ -4634,7 +4634,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A87" t="s">
         <v>22</v>
       </c>
@@ -4669,7 +4669,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A88" t="s">
         <v>53</v>
       </c>
@@ -4683,13 +4683,13 @@
         <v>31</v>
       </c>
       <c r="E88">
-        <v>90</v>
+        <v>33</v>
       </c>
       <c r="F88">
         <v>100</v>
       </c>
       <c r="G88">
-        <v>95</v>
+        <v>67</v>
       </c>
       <c r="H88">
         <v>100</v>

</xml_diff>

<commit_message>
Renamed germline calling to germline risk
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3AF8D20C-EECA-4786-B788-CEB994176079}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18343491-7A9E-47B5-9158-4801C1E4434A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1200" yWindow="1210" windowWidth="18010" windowHeight="18910" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$80</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="545" uniqueCount="245">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="225">
   <si>
     <t>nn_lower</t>
   </si>
@@ -56,21 +56,6 @@
     <t>Inf</t>
   </si>
   <si>
-    <t>ms_SNV_indel_ratio</t>
-  </si>
-  <si>
-    <t>ms_insertion_deletion_ratio</t>
-  </si>
-  <si>
-    <t>ms_MNP_other_variants</t>
-  </si>
-  <si>
-    <t>ms_transition_transversion_ratio</t>
-  </si>
-  <si>
-    <t>ms_het_hom_ratio</t>
-  </si>
-  <si>
     <t>ms_total_reads_r1</t>
   </si>
   <si>
@@ -128,9 +113,6 @@
     <t>ms_tape_station_area</t>
   </si>
   <si>
-    <t>ms_germline_variant_rate</t>
-  </si>
-  <si>
     <t>Sample</t>
   </si>
   <si>
@@ -233,9 +215,6 @@
     <t>EX create DSC</t>
   </si>
   <si>
-    <t>MS Call germline variants</t>
-  </si>
-  <si>
     <t>Mask regions</t>
   </si>
   <si>
@@ -308,24 +287,6 @@
     <t>Median insert size (start of R1 to end of R2) as determined during alignment (bp)</t>
   </si>
   <si>
-    <t>Percentage of genomic positions where germline variants have been called</t>
-  </si>
-  <si>
-    <t>Ratio of called SNVs to called INDELs</t>
-  </si>
-  <si>
-    <t>Ratio of called insertions to called deletions</t>
-  </si>
-  <si>
-    <t>Number of MNP or other variants after decomposition</t>
-  </si>
-  <si>
-    <t>Ratio of called transitions to called transversions</t>
-  </si>
-  <si>
-    <t>Ratio of called heterozygous variants to called homozygous variants</t>
-  </si>
-  <si>
     <t>ms_raw_read_length_r1</t>
   </si>
   <si>
@@ -537,27 +498,6 @@
   </si>
   <si>
     <t>softclip_bases_per_read_percentiles.90th_percentile</t>
-  </si>
-  <si>
-    <t>germline_variant_rate</t>
-  </si>
-  <si>
-    <t>insertion_deletion_ratio</t>
-  </si>
-  <si>
-    <t>MNP_other_variants</t>
-  </si>
-  <si>
-    <t>transition_transversion_ratio</t>
-  </si>
-  <si>
-    <t>het_hom_ratio</t>
-  </si>
-  <si>
-    <t>snv_indel_ratio</t>
-  </si>
-  <si>
-    <t>_candidate_variant_metrics_summary.json</t>
   </si>
   <si>
     <t>gini_coefficient</t>
@@ -1641,7 +1581,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K88"/>
+  <dimension ref="A1:K82"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.1796875" customWidth="1"/>
@@ -1656,16 +1596,16 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="B1" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -1680,27 +1620,27 @@
         <v>3</v>
       </c>
       <c r="I1" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="J1" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="K1" t="s">
-        <v>142</v>
+        <v>129</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>218</v>
+        <v>198</v>
       </c>
       <c r="C2" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E2">
         <v>2500</v>
@@ -1712,24 +1652,24 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="K2" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="C3" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="D3" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1747,24 +1687,24 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="K3" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="B4" t="s">
-        <v>193</v>
+        <v>173</v>
       </c>
       <c r="C4" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="D4" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E4">
         <v>90</v>
@@ -1782,24 +1722,24 @@
         <v>0</v>
       </c>
       <c r="J4" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="K4" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
+        <v>44</v>
+      </c>
+      <c r="B5" t="s">
+        <v>197</v>
+      </c>
+      <c r="C5" t="s">
         <v>50</v>
       </c>
-      <c r="B5" t="s">
-        <v>217</v>
-      </c>
-      <c r="C5" t="s">
-        <v>56</v>
-      </c>
       <c r="D5" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E5">
         <v>90</v>
@@ -1811,24 +1751,24 @@
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="K5" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>241</v>
+        <v>221</v>
       </c>
       <c r="C6" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D6" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1846,24 +1786,24 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="K6" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>216</v>
+        <v>196</v>
       </c>
       <c r="C7" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D7" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E7">
         <v>45</v>
@@ -1875,24 +1815,24 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="K7" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>242</v>
+        <v>222</v>
       </c>
       <c r="C8" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D8" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -1910,24 +1850,24 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="K8" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>76</v>
+        <v>69</v>
       </c>
       <c r="C9" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D9" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E9">
         <v>280</v>
@@ -1945,24 +1885,24 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="K9" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="C10" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D10" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E10">
         <v>95</v>
@@ -1980,24 +1920,24 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="K10" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
       <c r="C11" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="D11" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E11">
         <v>200</v>
@@ -2015,24 +1955,24 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
       <c r="K11" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>120</v>
+        <v>107</v>
       </c>
       <c r="C12" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="D12" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E12">
         <v>200</v>
@@ -2050,24 +1990,24 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="K12" t="s">
-        <v>157</v>
+        <v>144</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="B13" t="s">
-        <v>234</v>
+        <v>214</v>
       </c>
       <c r="C13" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D13" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E13">
         <v>35</v>
@@ -2085,24 +2025,24 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
       <c r="K13" t="s">
-        <v>158</v>
+        <v>145</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="B14" t="s">
-        <v>235</v>
+        <v>215</v>
       </c>
       <c r="C14" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D14" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E14">
         <v>35</v>
@@ -2120,24 +2060,24 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="K14" t="s">
-        <v>158</v>
+        <v>145</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="B15" t="s">
-        <v>233</v>
+        <v>213</v>
       </c>
       <c r="C15" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="D15" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -2155,24 +2095,24 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
       <c r="K15" t="s">
-        <v>160</v>
+        <v>147</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="B16" t="s">
-        <v>233</v>
+        <v>213</v>
       </c>
       <c r="C16" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="D16" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -2190,24 +2130,24 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
+        <v>134</v>
+      </c>
+      <c r="K16" t="s">
         <v>147</v>
-      </c>
-      <c r="K16" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="B17" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="C17" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D17" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E17">
         <v>150</v>
@@ -2225,24 +2165,24 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
       <c r="K17" t="s">
-        <v>161</v>
+        <v>148</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
-        <v>97</v>
+        <v>84</v>
       </c>
       <c r="B18" t="s">
-        <v>98</v>
+        <v>85</v>
       </c>
       <c r="C18" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D18" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E18">
         <v>150</v>
@@ -2260,24 +2200,24 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="K18" t="s">
-        <v>161</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>210</v>
+        <v>190</v>
       </c>
       <c r="B19" t="s">
-        <v>237</v>
+        <v>217</v>
       </c>
       <c r="C19" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="D19" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E19">
         <v>30</v>
@@ -2295,24 +2235,24 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="K19" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>211</v>
+        <v>191</v>
       </c>
       <c r="B20" t="s">
-        <v>237</v>
+        <v>217</v>
       </c>
       <c r="C20" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="D20" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E20">
         <v>30</v>
@@ -2330,24 +2270,24 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="K20" t="s">
-        <v>159</v>
+        <v>146</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
-        <v>78</v>
+        <v>71</v>
       </c>
       <c r="B21" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="C21" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D21" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -2365,24 +2305,24 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="K21" t="s">
-        <v>162</v>
+        <v>149</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="B22" t="s">
-        <v>124</v>
+        <v>111</v>
       </c>
       <c r="C22" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D22" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -2400,24 +2340,24 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
+        <v>136</v>
+      </c>
+      <c r="K22" t="s">
         <v>149</v>
-      </c>
-      <c r="K22" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
-        <v>80</v>
+        <v>73</v>
       </c>
       <c r="B23" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="C23" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D23" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -2435,24 +2375,24 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="K23" t="s">
-        <v>163</v>
+        <v>150</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
-        <v>81</v>
+        <v>74</v>
       </c>
       <c r="B24" t="s">
-        <v>122</v>
+        <v>109</v>
       </c>
       <c r="C24" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D24" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -2470,24 +2410,24 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="K24" t="s">
-        <v>163</v>
+        <v>150</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
-        <v>82</v>
+        <v>75</v>
       </c>
       <c r="B25" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="C25" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D25" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -2505,24 +2445,24 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="K25" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="B26" t="s">
-        <v>123</v>
+        <v>110</v>
       </c>
       <c r="C26" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D26" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E26">
         <v>0</v>
@@ -2540,24 +2480,24 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="K26" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="B27" t="s">
-        <v>236</v>
+        <v>216</v>
       </c>
       <c r="C27" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D27" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -2575,24 +2515,24 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="K27" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
-        <v>85</v>
+        <v>78</v>
       </c>
       <c r="B28" t="s">
-        <v>236</v>
+        <v>216</v>
       </c>
       <c r="C28" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D28" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -2610,24 +2550,24 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="K28" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>86</v>
+        <v>79</v>
       </c>
       <c r="B29" t="s">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="C29" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="D29" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -2645,24 +2585,24 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>192</v>
+        <v>172</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>214</v>
+        <v>194</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
-        <v>132</v>
+        <v>119</v>
       </c>
       <c r="B30" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="C30" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D30" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E30">
         <v>90</v>
@@ -2680,24 +2620,24 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
       <c r="K30" t="s">
-        <v>182</v>
+        <v>162</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
-        <v>131</v>
+        <v>118</v>
       </c>
       <c r="B31" t="s">
-        <v>139</v>
+        <v>126</v>
       </c>
       <c r="C31" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D31" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -2715,24 +2655,24 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>232</v>
+        <v>212</v>
       </c>
       <c r="K31" t="s">
-        <v>231</v>
+        <v>211</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>238</v>
+        <v>218</v>
       </c>
       <c r="B32" t="s">
-        <v>244</v>
+        <v>224</v>
       </c>
       <c r="C32" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D32" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E32">
         <v>21.75</v>
@@ -2750,24 +2690,24 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>239</v>
+        <v>219</v>
       </c>
       <c r="K32" t="s">
-        <v>243</v>
+        <v>223</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>130</v>
+        <v>117</v>
       </c>
       <c r="B33" t="s">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="C33" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D33" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E33">
         <v>125</v>
@@ -2785,42 +2725,42 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>151</v>
+        <v>138</v>
       </c>
       <c r="K33" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
-        <v>30</v>
+        <v>61</v>
       </c>
       <c r="B34" t="s">
+        <v>4</v>
+      </c>
+      <c r="C34" t="s">
+        <v>59</v>
+      </c>
+      <c r="D34" t="s">
+        <v>25</v>
+      </c>
+      <c r="E34">
+        <v>70</v>
+      </c>
+      <c r="F34">
         <v>90</v>
       </c>
-      <c r="C34" t="s">
-        <v>65</v>
-      </c>
-      <c r="D34" t="s">
-        <v>31</v>
-      </c>
-      <c r="E34">
-        <v>1.2999999999999999E-3</v>
-      </c>
-      <c r="F34">
-        <v>1.9E-3</v>
-      </c>
       <c r="G34">
-        <v>1.4E-3</v>
+        <v>70</v>
       </c>
       <c r="H34">
-        <v>1.8E-3</v>
+        <v>80</v>
       </c>
       <c r="I34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="K34" t="s">
         <v>167</v>
@@ -2828,299 +2768,293 @@
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="B35" t="s">
-        <v>91</v>
+        <v>40</v>
       </c>
       <c r="C35" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="D35" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E35">
-        <v>4</v>
+        <v>75</v>
       </c>
       <c r="F35">
-        <v>10</v>
-      </c>
-      <c r="G35">
-        <v>4.3</v>
-      </c>
-      <c r="H35">
-        <v>8.5</v>
+        <v>1000</v>
       </c>
       <c r="I35" t="b">
         <v>0</v>
       </c>
       <c r="J35" t="s">
-        <v>173</v>
+        <v>60</v>
       </c>
       <c r="K35" t="s">
-        <v>172</v>
+        <v>60</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="B36" t="s">
-        <v>92</v>
+        <v>221</v>
       </c>
       <c r="C36" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="D36" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E36">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="F36">
-        <v>1</v>
+        <v>0.3</v>
       </c>
       <c r="G36">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="H36">
-        <v>0.94</v>
+        <v>0.2</v>
       </c>
       <c r="I36" t="b">
         <v>0</v>
       </c>
       <c r="J36" t="s">
-        <v>173</v>
+        <v>60</v>
       </c>
       <c r="K36" t="s">
-        <v>168</v>
+        <v>60</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>8</v>
+        <v>33</v>
       </c>
       <c r="B37" t="s">
-        <v>93</v>
+        <v>174</v>
       </c>
       <c r="C37" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="D37" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E37">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F37">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G37">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="H37">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I37" t="b">
         <v>0</v>
       </c>
       <c r="J37" t="s">
-        <v>173</v>
+        <v>60</v>
       </c>
       <c r="K37" t="s">
-        <v>169</v>
+        <v>60</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="B38" t="s">
-        <v>94</v>
+        <v>42</v>
       </c>
       <c r="C38" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="D38" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E38">
-        <v>1.9</v>
-      </c>
-      <c r="F38">
-        <v>2.2000000000000002</v>
-      </c>
-      <c r="G38">
-        <v>2.0499999999999998</v>
-      </c>
-      <c r="H38">
-        <v>2.15</v>
+        <v>4.3</v>
+      </c>
+      <c r="F38" t="s">
+        <v>5</v>
       </c>
       <c r="I38" t="b">
         <v>0</v>
       </c>
       <c r="J38" t="s">
-        <v>173</v>
+        <v>60</v>
       </c>
       <c r="K38" t="s">
-        <v>170</v>
+        <v>60</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>10</v>
+        <v>37</v>
       </c>
       <c r="B39" t="s">
-        <v>95</v>
+        <v>221</v>
       </c>
       <c r="C39" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="D39" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="E39">
-        <v>1.2</v>
+        <v>0</v>
       </c>
       <c r="F39">
-        <v>2.1</v>
+        <v>0.4</v>
       </c>
       <c r="G39">
-        <v>1.3</v>
+        <v>0</v>
       </c>
       <c r="H39">
-        <v>2</v>
+        <v>0.3</v>
       </c>
       <c r="I39" t="b">
         <v>0</v>
       </c>
       <c r="J39" t="s">
-        <v>173</v>
+        <v>60</v>
       </c>
       <c r="K39" t="s">
-        <v>171</v>
+        <v>60</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>68</v>
+        <v>38</v>
       </c>
       <c r="B40" t="s">
-        <v>4</v>
+        <v>175</v>
       </c>
       <c r="C40" t="s">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="D40" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E40">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="F40">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G40">
-        <v>70</v>
+        <v>95</v>
       </c>
       <c r="H40">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="I40" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J40" t="s">
-        <v>186</v>
+        <v>60</v>
       </c>
       <c r="K40" t="s">
-        <v>187</v>
+        <v>60</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="B41" t="s">
-        <v>46</v>
+        <v>176</v>
       </c>
       <c r="C41" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D41" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E41">
-        <v>75</v>
+        <v>1</v>
       </c>
       <c r="F41">
-        <v>1000</v>
+        <v>1</v>
+      </c>
+      <c r="G41">
+        <v>1</v>
+      </c>
+      <c r="H41">
+        <v>1</v>
       </c>
       <c r="I41" t="b">
         <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="K41" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="B42" t="s">
-        <v>241</v>
+        <v>18</v>
       </c>
       <c r="C42" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D42" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
       <c r="E42">
-        <v>0</v>
+        <v>544</v>
       </c>
       <c r="F42">
-        <v>0.3</v>
+        <v>624</v>
       </c>
       <c r="G42">
-        <v>0</v>
+        <v>564</v>
       </c>
       <c r="H42">
-        <v>0.2</v>
+        <v>604</v>
       </c>
       <c r="I42" t="b">
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="K42" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="B43" t="s">
-        <v>194</v>
+        <v>19</v>
       </c>
       <c r="C43" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="D43" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E43">
-        <v>80</v>
+        <v>98</v>
       </c>
       <c r="F43">
         <v>100</v>
       </c>
       <c r="G43">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="H43">
         <v>100</v>
@@ -3129,753 +3063,759 @@
         <v>0</v>
       </c>
       <c r="J43" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="K43" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>47</v>
+        <v>87</v>
       </c>
       <c r="B44" t="s">
-        <v>48</v>
+        <v>214</v>
       </c>
       <c r="C44" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D44" t="s">
-        <v>31</v>
+        <v>65</v>
       </c>
       <c r="E44">
-        <v>4.3</v>
-      </c>
-      <c r="F44" t="s">
-        <v>5</v>
+        <v>35</v>
+      </c>
+      <c r="F44">
+        <v>40</v>
+      </c>
+      <c r="G44">
+        <v>39</v>
+      </c>
+      <c r="H44">
+        <v>40</v>
       </c>
       <c r="I44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J44" t="s">
-        <v>67</v>
+        <v>139</v>
       </c>
       <c r="K44" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
-        <v>43</v>
+        <v>88</v>
       </c>
       <c r="B45" t="s">
-        <v>241</v>
+        <v>215</v>
       </c>
       <c r="C45" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D45" t="s">
-        <v>32</v>
+        <v>65</v>
       </c>
       <c r="E45">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F45">
-        <v>0.4</v>
+        <v>40</v>
       </c>
       <c r="G45">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="H45">
-        <v>0.3</v>
+        <v>40</v>
       </c>
       <c r="I45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="K45" t="s">
-        <v>67</v>
+        <v>145</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>44</v>
+        <v>89</v>
       </c>
       <c r="B46" t="s">
-        <v>195</v>
+        <v>213</v>
       </c>
       <c r="C46" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D46" t="s">
-        <v>31</v>
+        <v>65</v>
       </c>
       <c r="E46">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F46">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G46">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H46">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="I46" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>67</v>
+        <v>139</v>
       </c>
       <c r="K46" t="s">
-        <v>67</v>
+        <v>147</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="B47" t="s">
-        <v>196</v>
+        <v>213</v>
       </c>
       <c r="C47" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D47" t="s">
-        <v>31</v>
+        <v>65</v>
       </c>
       <c r="E47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F47">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G47">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H47">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="I47" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="K47" t="s">
-        <v>67</v>
+        <v>147</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>26</v>
+        <v>86</v>
       </c>
       <c r="B48" t="s">
-        <v>23</v>
+        <v>85</v>
       </c>
       <c r="C48" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D48" t="s">
-        <v>31</v>
+        <v>65</v>
       </c>
       <c r="E48">
-        <v>544</v>
+        <v>150</v>
       </c>
       <c r="F48">
-        <v>624</v>
+        <v>150</v>
       </c>
       <c r="G48">
-        <v>564</v>
+        <v>150</v>
       </c>
       <c r="H48">
-        <v>604</v>
+        <v>150</v>
       </c>
       <c r="I48" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>67</v>
+        <v>139</v>
       </c>
       <c r="K48" t="s">
-        <v>67</v>
+        <v>148</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>27</v>
+        <v>95</v>
       </c>
       <c r="B49" t="s">
-        <v>24</v>
+        <v>85</v>
       </c>
       <c r="C49" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D49" t="s">
-        <v>31</v>
+        <v>65</v>
       </c>
       <c r="E49">
-        <v>98</v>
+        <v>150</v>
       </c>
       <c r="F49">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="G49">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="H49">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="I49" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>67</v>
+        <v>140</v>
       </c>
       <c r="K49" t="s">
-        <v>67</v>
+        <v>148</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="B50" t="s">
-        <v>234</v>
+        <v>106</v>
       </c>
       <c r="C50" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D50" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="E50">
-        <v>35</v>
-      </c>
-      <c r="F50">
-        <v>40</v>
+        <v>2850</v>
+      </c>
+      <c r="F50" t="s">
+        <v>5</v>
       </c>
       <c r="G50">
-        <v>39</v>
-      </c>
-      <c r="H50">
-        <v>40</v>
+        <v>3000</v>
+      </c>
+      <c r="H50" t="s">
+        <v>5</v>
       </c>
       <c r="I50" t="b">
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>152</v>
+        <v>139</v>
       </c>
       <c r="K50" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="B51" t="s">
-        <v>235</v>
+        <v>106</v>
       </c>
       <c r="C51" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D51" t="s">
-        <v>72</v>
+        <v>65</v>
       </c>
       <c r="E51">
-        <v>35</v>
-      </c>
-      <c r="F51">
-        <v>40</v>
+        <v>2850</v>
+      </c>
+      <c r="F51" t="s">
+        <v>5</v>
       </c>
       <c r="G51">
-        <v>39</v>
-      </c>
-      <c r="H51">
-        <v>40</v>
+        <v>3000</v>
+      </c>
+      <c r="H51" t="s">
+        <v>5</v>
       </c>
       <c r="I51" t="b">
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>153</v>
+        <v>140</v>
       </c>
       <c r="K51" t="s">
-        <v>158</v>
+        <v>144</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>102</v>
+        <v>188</v>
       </c>
       <c r="B52" t="s">
-        <v>233</v>
+        <v>217</v>
       </c>
       <c r="C52" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D52" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="E52">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F52">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G52">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H52">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="I52" t="b">
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="K52" t="s">
-        <v>160</v>
+        <v>146</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>103</v>
+        <v>189</v>
       </c>
       <c r="B53" t="s">
-        <v>233</v>
+        <v>217</v>
       </c>
       <c r="C53" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D53" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="E53">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F53">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G53">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H53">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="I53" t="b">
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="K53" t="s">
-        <v>160</v>
+        <v>146</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B54" t="s">
-        <v>98</v>
+        <v>108</v>
       </c>
       <c r="C54" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D54" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="E54">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F54">
-        <v>150</v>
+        <v>1</v>
       </c>
       <c r="G54">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="H54">
-        <v>150</v>
+        <v>0.1</v>
       </c>
       <c r="I54" t="b">
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="K54" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
+        <v>99</v>
+      </c>
+      <c r="B55" t="s">
         <v>108</v>
       </c>
-      <c r="B55" t="s">
-        <v>98</v>
-      </c>
       <c r="C55" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D55" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="E55">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F55">
-        <v>150</v>
+        <v>1</v>
       </c>
       <c r="G55">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="H55">
-        <v>150</v>
+        <v>0.1</v>
       </c>
       <c r="I55" t="b">
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="K55" t="s">
-        <v>161</v>
+        <v>149</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
+        <v>100</v>
+      </c>
+      <c r="B56" t="s">
         <v>109</v>
       </c>
-      <c r="B56" t="s">
-        <v>119</v>
-      </c>
       <c r="C56" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D56" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="E56">
-        <v>2850</v>
-      </c>
-      <c r="F56" t="s">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="F56">
+        <v>30</v>
       </c>
       <c r="G56">
-        <v>3000</v>
-      </c>
-      <c r="H56" t="s">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="H56">
+        <v>20</v>
       </c>
       <c r="I56" t="b">
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="K56" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="B57" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="C57" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D57" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="E57">
-        <v>2850</v>
-      </c>
-      <c r="F57" t="s">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="F57">
+        <v>30</v>
       </c>
       <c r="G57">
-        <v>3000</v>
-      </c>
-      <c r="H57" t="s">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="H57">
+        <v>20</v>
       </c>
       <c r="I57" t="b">
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>153</v>
+        <v>142</v>
       </c>
       <c r="K57" t="s">
-        <v>157</v>
+        <v>150</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>208</v>
+        <v>102</v>
       </c>
       <c r="B58" t="s">
-        <v>237</v>
+        <v>110</v>
       </c>
       <c r="C58" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D58" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E58">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F58">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="G58">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H58">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="I58" t="b">
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="K58" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>209</v>
+        <v>103</v>
       </c>
       <c r="B59" t="s">
-        <v>237</v>
+        <v>110</v>
       </c>
       <c r="C59" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D59" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E59">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F59">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="G59">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H59">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="I59" t="b">
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="K59" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>111</v>
+        <v>104</v>
       </c>
       <c r="B60" t="s">
-        <v>121</v>
+        <v>216</v>
       </c>
       <c r="C60" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D60" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E60">
         <v>0</v>
       </c>
       <c r="F60">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G60">
         <v>0</v>
       </c>
       <c r="H60">
-        <v>0.1</v>
+        <v>5</v>
       </c>
       <c r="I60" t="b">
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>154</v>
+        <v>141</v>
       </c>
       <c r="K60" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>112</v>
+        <v>105</v>
       </c>
       <c r="B61" t="s">
-        <v>121</v>
+        <v>216</v>
       </c>
       <c r="C61" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D61" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E61">
         <v>0</v>
       </c>
       <c r="F61">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="G61">
         <v>0</v>
       </c>
       <c r="H61">
-        <v>0.1</v>
+        <v>5</v>
       </c>
       <c r="I61" t="b">
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>155</v>
+        <v>142</v>
       </c>
       <c r="K61" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
-        <v>113</v>
+        <v>62</v>
       </c>
       <c r="B62" t="s">
-        <v>122</v>
+        <v>201</v>
       </c>
       <c r="C62" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D62" t="s">
-        <v>31</v>
+        <v>65</v>
       </c>
       <c r="E62">
         <v>0</v>
       </c>
       <c r="F62">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="G62">
         <v>0</v>
       </c>
       <c r="H62">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I62" t="b">
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>154</v>
+        <v>199</v>
       </c>
       <c r="K62" t="s">
-        <v>163</v>
+        <v>200</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
+        <v>113</v>
+      </c>
+      <c r="B63" t="s">
         <v>114</v>
       </c>
-      <c r="B63" t="s">
-        <v>122</v>
-      </c>
       <c r="C63" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D63" t="s">
-        <v>31</v>
+        <v>65</v>
       </c>
       <c r="E63">
         <v>0</v>
       </c>
       <c r="F63">
-        <v>30</v>
+        <v>0.1</v>
       </c>
       <c r="G63">
         <v>0</v>
       </c>
       <c r="H63">
-        <v>20</v>
+        <v>0.05</v>
       </c>
       <c r="I63" t="b">
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>155</v>
+        <v>199</v>
       </c>
       <c r="K63" t="s">
-        <v>163</v>
+        <v>154</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>115</v>
+        <v>178</v>
       </c>
       <c r="B64" t="s">
-        <v>123</v>
+        <v>179</v>
       </c>
       <c r="C64" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D64" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E64">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F64">
+        <v>40</v>
+      </c>
+      <c r="G64">
+        <v>1</v>
+      </c>
+      <c r="H64">
         <v>20</v>
       </c>
-      <c r="G64">
-        <v>0</v>
-      </c>
-      <c r="H64">
-        <v>10</v>
-      </c>
       <c r="I64" t="b">
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>154</v>
+        <v>187</v>
       </c>
       <c r="K64" t="s">
-        <v>164</v>
+        <v>202</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>116</v>
+        <v>205</v>
       </c>
       <c r="B65" t="s">
-        <v>123</v>
+        <v>192</v>
       </c>
       <c r="C65" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D65" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E65">
         <v>0</v>
@@ -3893,819 +3833,609 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>155</v>
+        <v>203</v>
       </c>
       <c r="K65" t="s">
-        <v>164</v>
+        <v>204</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>117</v>
+        <v>63</v>
       </c>
       <c r="B66" t="s">
-        <v>236</v>
+        <v>180</v>
       </c>
       <c r="C66" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D66" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E66">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F66">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="G66">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="H66">
-        <v>5</v>
+        <v>99</v>
       </c>
       <c r="I66" t="b">
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>154</v>
+        <v>183</v>
       </c>
       <c r="K66" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>118</v>
+        <v>64</v>
       </c>
       <c r="B67" t="s">
-        <v>236</v>
+        <v>181</v>
       </c>
       <c r="C67" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="D67" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E67">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="F67">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="G67">
-        <v>0</v>
+        <v>92.5</v>
       </c>
       <c r="H67">
-        <v>5</v>
+        <v>99</v>
       </c>
       <c r="I67" t="b">
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>155</v>
+        <v>184</v>
       </c>
       <c r="K67" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B68" t="s">
-        <v>221</v>
+        <v>80</v>
       </c>
       <c r="C68" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="D68" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="E68">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F68">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="G68">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="H68">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="I68" t="b">
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>219</v>
+        <v>130</v>
       </c>
       <c r="K68" t="s">
-        <v>220</v>
+        <v>162</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
-        <v>126</v>
+        <v>66</v>
       </c>
       <c r="B69" t="s">
-        <v>127</v>
+        <v>81</v>
       </c>
       <c r="C69" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="D69" t="s">
-        <v>72</v>
+        <v>25</v>
       </c>
       <c r="E69">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F69">
-        <v>0.1</v>
+        <v>100</v>
       </c>
       <c r="G69">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="H69">
-        <v>0.05</v>
+        <v>100</v>
       </c>
       <c r="I69" t="b">
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>219</v>
+        <v>130</v>
       </c>
       <c r="K69" t="s">
-        <v>174</v>
+        <v>164</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>198</v>
+        <v>68</v>
       </c>
       <c r="B70" t="s">
-        <v>199</v>
+        <v>115</v>
       </c>
       <c r="C70" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="D70" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E70">
-        <v>1</v>
+        <v>125</v>
       </c>
       <c r="F70">
-        <v>40</v>
+        <v>175</v>
       </c>
       <c r="G70">
-        <v>1</v>
+        <v>140</v>
       </c>
       <c r="H70">
-        <v>20</v>
+        <v>160</v>
       </c>
       <c r="I70" t="b">
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>207</v>
+        <v>131</v>
       </c>
       <c r="K70" t="s">
-        <v>222</v>
+        <v>163</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>225</v>
+        <v>127</v>
       </c>
       <c r="B71" t="s">
-        <v>212</v>
+        <v>195</v>
       </c>
       <c r="C71" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D71" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E71">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="F71">
-        <v>20</v>
+        <v>55</v>
       </c>
       <c r="G71">
-        <v>0</v>
+        <v>50</v>
       </c>
       <c r="H71">
-        <v>10</v>
+        <v>52.5</v>
       </c>
       <c r="I71" t="b">
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>223</v>
+        <v>155</v>
       </c>
       <c r="K71" t="s">
-        <v>224</v>
+        <v>156</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>70</v>
+        <v>116</v>
       </c>
       <c r="B72" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="C72" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D72" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E72">
-        <v>80</v>
+        <v>60</v>
       </c>
       <c r="F72">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G72">
         <v>90</v>
       </c>
       <c r="H72">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I72" t="b">
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>203</v>
+        <v>169</v>
       </c>
       <c r="K72" t="s">
-        <v>202</v>
+        <v>168</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>71</v>
+        <v>122</v>
       </c>
       <c r="B73" t="s">
-        <v>201</v>
+        <v>10</v>
       </c>
       <c r="C73" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="D73" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E73">
-        <v>85</v>
+        <v>99</v>
       </c>
       <c r="F73">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G73">
-        <v>92.5</v>
+        <v>99.5</v>
       </c>
       <c r="H73">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I73" t="b">
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>204</v>
+        <v>159</v>
       </c>
       <c r="K73" t="s">
-        <v>202</v>
+        <v>157</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>74</v>
+        <v>121</v>
       </c>
       <c r="B74" t="s">
-        <v>87</v>
+        <v>120</v>
       </c>
       <c r="C74" t="s">
         <v>58</v>
       </c>
       <c r="D74" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E74">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="F74">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="G74">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H74">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="I74" t="b">
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>143</v>
+        <v>159</v>
       </c>
       <c r="K74" t="s">
-        <v>182</v>
+        <v>158</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>73</v>
+        <v>123</v>
       </c>
       <c r="B75" t="s">
-        <v>88</v>
+        <v>124</v>
       </c>
       <c r="C75" t="s">
         <v>58</v>
       </c>
       <c r="D75" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E75">
-        <v>50</v>
-      </c>
-      <c r="F75">
-        <v>100</v>
+        <v>0.5</v>
+      </c>
+      <c r="F75" t="s">
+        <v>5</v>
       </c>
       <c r="G75">
-        <v>75</v>
-      </c>
-      <c r="H75">
-        <v>100</v>
+        <v>1</v>
+      </c>
+      <c r="H75" t="s">
+        <v>5</v>
       </c>
       <c r="I75" t="b">
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>143</v>
+        <v>170</v>
       </c>
       <c r="K75" t="s">
-        <v>184</v>
+        <v>160</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>75</v>
+        <v>14</v>
       </c>
       <c r="B76" t="s">
-        <v>128</v>
+        <v>15</v>
       </c>
       <c r="C76" t="s">
         <v>58</v>
       </c>
       <c r="D76" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E76">
-        <v>125</v>
+        <v>0</v>
       </c>
       <c r="F76">
-        <v>175</v>
+        <v>0</v>
       </c>
       <c r="G76">
-        <v>140</v>
+        <v>0</v>
       </c>
       <c r="H76">
-        <v>160</v>
+        <v>0</v>
       </c>
       <c r="I76" t="b">
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>144</v>
+        <v>132</v>
       </c>
       <c r="K76" t="s">
-        <v>183</v>
+        <v>153</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>140</v>
+        <v>12</v>
       </c>
       <c r="B77" t="s">
-        <v>215</v>
+        <v>13</v>
       </c>
       <c r="C77" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="D77" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E77">
-        <v>50</v>
+        <v>14.5</v>
       </c>
       <c r="F77">
-        <v>55</v>
+        <v>100</v>
       </c>
       <c r="G77">
-        <v>50</v>
+        <v>26.1</v>
       </c>
       <c r="H77">
-        <v>52.5</v>
+        <v>100</v>
       </c>
       <c r="I77" t="b">
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>175</v>
+        <v>170</v>
       </c>
       <c r="K77" t="s">
-        <v>176</v>
+        <v>12</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
-        <v>129</v>
+        <v>8</v>
       </c>
       <c r="B78" t="s">
-        <v>191</v>
+        <v>9</v>
       </c>
       <c r="C78" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="D78" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E78">
-        <v>60</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="F78">
-        <v>100</v>
+        <v>8.0000000000000004E-4</v>
       </c>
       <c r="G78">
-        <v>90</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="H78">
-        <v>100</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="I78" t="b">
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="K78" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>135</v>
+        <v>206</v>
       </c>
       <c r="B79" t="s">
-        <v>15</v>
+        <v>207</v>
       </c>
       <c r="C79" t="s">
-        <v>64</v>
+        <v>177</v>
       </c>
       <c r="D79" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E79">
-        <v>99</v>
+        <v>0.05</v>
       </c>
       <c r="F79">
-        <v>100</v>
+        <v>0.08</v>
       </c>
       <c r="G79">
-        <v>99.5</v>
+        <v>0.02</v>
       </c>
       <c r="H79">
-        <v>100</v>
+        <v>0.05</v>
       </c>
       <c r="I79" t="b">
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>179</v>
+        <v>209</v>
       </c>
       <c r="K79" t="s">
-        <v>177</v>
+        <v>210</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>134</v>
+        <v>11</v>
       </c>
       <c r="B80" t="s">
-        <v>133</v>
+        <v>208</v>
       </c>
       <c r="C80" t="s">
-        <v>64</v>
+        <v>177</v>
       </c>
       <c r="D80" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E80">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F80">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="G80">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H80">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="I80" t="b">
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>179</v>
+        <v>170</v>
       </c>
       <c r="K80" t="s">
-        <v>178</v>
+        <v>161</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
-        <v>136</v>
+        <v>17</v>
       </c>
       <c r="B81" t="s">
-        <v>137</v>
+        <v>16</v>
       </c>
       <c r="C81" t="s">
-        <v>64</v>
+        <v>177</v>
       </c>
       <c r="D81" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E81">
-        <v>0.5</v>
-      </c>
-      <c r="F81" t="s">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="F81">
+        <v>95</v>
       </c>
       <c r="G81">
-        <v>1</v>
-      </c>
-      <c r="H81" t="s">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="H81">
+        <v>80</v>
       </c>
       <c r="I81" t="b">
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>190</v>
+        <v>143</v>
       </c>
       <c r="K81" t="s">
-        <v>180</v>
+        <v>165</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>19</v>
+        <v>47</v>
       </c>
       <c r="B82" t="s">
-        <v>20</v>
+        <v>193</v>
       </c>
       <c r="C82" t="s">
-        <v>64</v>
+        <v>177</v>
       </c>
       <c r="D82" t="s">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="E82">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="F82">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G82">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="H82">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I82" t="b">
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>145</v>
+        <v>170</v>
       </c>
       <c r="K82" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A83" t="s">
-        <v>17</v>
-      </c>
-      <c r="B83" t="s">
-        <v>18</v>
-      </c>
-      <c r="C83" t="s">
-        <v>64</v>
-      </c>
-      <c r="D83" t="s">
-        <v>31</v>
-      </c>
-      <c r="E83">
-        <v>14.5</v>
-      </c>
-      <c r="F83">
-        <v>100</v>
-      </c>
-      <c r="G83">
-        <v>26.1</v>
-      </c>
-      <c r="H83">
-        <v>100</v>
-      </c>
-      <c r="I83" t="b">
-        <v>1</v>
-      </c>
-      <c r="J83" t="s">
-        <v>190</v>
-      </c>
-      <c r="K83" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A84" t="s">
-        <v>13</v>
-      </c>
-      <c r="B84" t="s">
-        <v>14</v>
-      </c>
-      <c r="C84" t="s">
-        <v>64</v>
-      </c>
-      <c r="D84" t="s">
-        <v>31</v>
-      </c>
-      <c r="E84">
-        <v>5.0000000000000001E-4</v>
-      </c>
-      <c r="F84">
-        <v>8.0000000000000004E-4</v>
-      </c>
-      <c r="G84">
-        <v>2.0000000000000001E-4</v>
-      </c>
-      <c r="H84">
-        <v>5.0000000000000001E-4</v>
-      </c>
-      <c r="I84" t="b">
-        <v>1</v>
-      </c>
-      <c r="J84" t="s">
-        <v>206</v>
-      </c>
-      <c r="K84" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A85" t="s">
-        <v>226</v>
-      </c>
-      <c r="B85" t="s">
-        <v>227</v>
-      </c>
-      <c r="C85" t="s">
-        <v>197</v>
-      </c>
-      <c r="D85" t="s">
-        <v>31</v>
-      </c>
-      <c r="E85">
-        <v>0.05</v>
-      </c>
-      <c r="F85">
-        <v>0.08</v>
-      </c>
-      <c r="G85">
-        <v>0.02</v>
-      </c>
-      <c r="H85">
-        <v>0.05</v>
-      </c>
-      <c r="I85" t="b">
-        <v>1</v>
-      </c>
-      <c r="J85" t="s">
-        <v>229</v>
-      </c>
-      <c r="K85" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A86" t="s">
-        <v>16</v>
-      </c>
-      <c r="B86" t="s">
-        <v>228</v>
-      </c>
-      <c r="C86" t="s">
-        <v>197</v>
-      </c>
-      <c r="D86" t="s">
-        <v>31</v>
-      </c>
-      <c r="E86">
-        <v>5</v>
-      </c>
-      <c r="F86">
-        <v>100</v>
-      </c>
-      <c r="G86">
-        <v>20</v>
-      </c>
-      <c r="H86">
-        <v>100</v>
-      </c>
-      <c r="I86" t="b">
-        <v>1</v>
-      </c>
-      <c r="J86" t="s">
-        <v>190</v>
-      </c>
-      <c r="K86" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A87" t="s">
-        <v>22</v>
-      </c>
-      <c r="B87" t="s">
-        <v>21</v>
-      </c>
-      <c r="C87" t="s">
-        <v>197</v>
-      </c>
-      <c r="D87" t="s">
-        <v>31</v>
-      </c>
-      <c r="E87">
-        <v>0</v>
-      </c>
-      <c r="F87">
-        <v>95</v>
-      </c>
-      <c r="G87">
-        <v>0</v>
-      </c>
-      <c r="H87">
-        <v>80</v>
-      </c>
-      <c r="I87" t="b">
-        <v>1</v>
-      </c>
-      <c r="J87" t="s">
-        <v>156</v>
-      </c>
-      <c r="K87" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A88" t="s">
-        <v>53</v>
-      </c>
-      <c r="B88" t="s">
-        <v>213</v>
-      </c>
-      <c r="C88" t="s">
-        <v>197</v>
-      </c>
-      <c r="D88" t="s">
-        <v>31</v>
-      </c>
-      <c r="E88">
-        <v>33</v>
-      </c>
-      <c r="F88">
-        <v>100</v>
-      </c>
-      <c r="G88">
-        <v>67</v>
-      </c>
-      <c r="H88">
-        <v>100</v>
-      </c>
-      <c r="I88" t="b">
-        <v>1</v>
-      </c>
-      <c r="J88" t="s">
-        <v>190</v>
-      </c>
-      <c r="K88" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K86" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K80" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Changed ideal and nn limits for ex_reads_lost_call_dsc
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\jamesphie\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18343491-7A9E-47B5-9158-4801C1E4434A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E12D9541-9562-4270-94EC-0E2B05146D8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -1582,19 +1582,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
   <dimension ref="A1:K82"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.1796875" customWidth="1"/>
-    <col min="2" max="2" width="123.1796875" customWidth="1"/>
-    <col min="3" max="4" width="35.26953125" customWidth="1"/>
+    <col min="1" max="1" width="35.140625" customWidth="1"/>
+    <col min="2" max="2" width="123.140625" customWidth="1"/>
+    <col min="3" max="4" width="35.28515625" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.81640625" customWidth="1"/>
-    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="76.81640625" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="76.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>32</v>
       </c>
@@ -1629,7 +1629,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -1658,7 +1658,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>35</v>
       </c>
@@ -1693,7 +1693,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -1728,7 +1728,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>44</v>
       </c>
@@ -1757,7 +1757,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -1792,7 +1792,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>45</v>
       </c>
@@ -1821,7 +1821,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>46</v>
       </c>
@@ -1856,7 +1856,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1891,7 +1891,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -1926,7 +1926,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -1961,7 +1961,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -1996,7 +1996,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>93</v>
       </c>
@@ -2031,7 +2031,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>94</v>
       </c>
@@ -2066,7 +2066,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>91</v>
       </c>
@@ -2101,7 +2101,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>92</v>
       </c>
@@ -2136,7 +2136,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>83</v>
       </c>
@@ -2171,7 +2171,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>84</v>
       </c>
@@ -2206,7 +2206,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>190</v>
       </c>
@@ -2241,7 +2241,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>191</v>
       </c>
@@ -2276,7 +2276,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>71</v>
       </c>
@@ -2311,7 +2311,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>72</v>
       </c>
@@ -2346,7 +2346,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>73</v>
       </c>
@@ -2381,7 +2381,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>74</v>
       </c>
@@ -2416,7 +2416,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>75</v>
       </c>
@@ -2451,7 +2451,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>76</v>
       </c>
@@ -2486,7 +2486,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>77</v>
       </c>
@@ -2521,7 +2521,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>78</v>
       </c>
@@ -2556,7 +2556,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>79</v>
       </c>
@@ -2591,7 +2591,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>119</v>
       </c>
@@ -2626,7 +2626,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>118</v>
       </c>
@@ -2661,7 +2661,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>218</v>
       </c>
@@ -2696,7 +2696,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>117</v>
       </c>
@@ -2731,7 +2731,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>61</v>
       </c>
@@ -2766,7 +2766,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>20</v>
       </c>
@@ -2795,7 +2795,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>27</v>
       </c>
@@ -2830,7 +2830,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>33</v>
       </c>
@@ -2865,7 +2865,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>41</v>
       </c>
@@ -2894,7 +2894,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>37</v>
       </c>
@@ -2929,7 +2929,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>38</v>
       </c>
@@ -2964,7 +2964,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>39</v>
       </c>
@@ -2999,7 +2999,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>21</v>
       </c>
@@ -3034,7 +3034,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>22</v>
       </c>
@@ -3069,7 +3069,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>87</v>
       </c>
@@ -3104,7 +3104,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>88</v>
       </c>
@@ -3139,7 +3139,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>89</v>
       </c>
@@ -3174,7 +3174,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>90</v>
       </c>
@@ -3209,7 +3209,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>86</v>
       </c>
@@ -3244,7 +3244,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>95</v>
       </c>
@@ -3279,7 +3279,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>96</v>
       </c>
@@ -3314,7 +3314,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>97</v>
       </c>
@@ -3349,7 +3349,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>188</v>
       </c>
@@ -3384,7 +3384,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>189</v>
       </c>
@@ -3419,7 +3419,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>98</v>
       </c>
@@ -3454,7 +3454,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>99</v>
       </c>
@@ -3489,7 +3489,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>100</v>
       </c>
@@ -3524,7 +3524,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>101</v>
       </c>
@@ -3559,7 +3559,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>102</v>
       </c>
@@ -3594,7 +3594,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>103</v>
       </c>
@@ -3629,7 +3629,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>104</v>
       </c>
@@ -3664,7 +3664,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>105</v>
       </c>
@@ -3699,7 +3699,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>62</v>
       </c>
@@ -3734,7 +3734,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>113</v>
       </c>
@@ -3769,7 +3769,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>178</v>
       </c>
@@ -3804,7 +3804,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>205</v>
       </c>
@@ -3839,7 +3839,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>63</v>
       </c>
@@ -3874,7 +3874,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>64</v>
       </c>
@@ -3909,7 +3909,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>67</v>
       </c>
@@ -3944,7 +3944,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>66</v>
       </c>
@@ -3979,7 +3979,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>68</v>
       </c>
@@ -4014,7 +4014,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>127</v>
       </c>
@@ -4031,13 +4031,13 @@
         <v>50</v>
       </c>
       <c r="F71">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="G71">
         <v>50</v>
       </c>
       <c r="H71">
-        <v>52.5</v>
+        <v>60</v>
       </c>
       <c r="I71" t="b">
         <v>1</v>
@@ -4049,7 +4049,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>116</v>
       </c>
@@ -4084,7 +4084,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>122</v>
       </c>
@@ -4119,7 +4119,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>121</v>
       </c>
@@ -4154,7 +4154,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>123</v>
       </c>
@@ -4189,7 +4189,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>14</v>
       </c>
@@ -4224,7 +4224,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>12</v>
       </c>
@@ -4259,7 +4259,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -4294,7 +4294,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>206</v>
       </c>
@@ -4329,7 +4329,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>11</v>
       </c>
@@ -4364,7 +4364,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>17</v>
       </c>
@@ -4399,7 +4399,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>47</v>
       </c>

</xml_diff>

<commit_message>
Added mean quality filter rule to ms_filter_fastq
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\jamesphie\codec-opensource\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E12D9541-9562-4270-94EC-0E2B05146D8E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8313D711-6932-4253-BE9A-CDEA1651B409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$81</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="225">
   <si>
     <t>nn_lower</t>
   </si>
@@ -413,9 +413,6 @@
     <t>Mean duplex depth of final DSC passed to variant calling</t>
   </si>
   <si>
-    <t>Percentage of raw reads filtered by length threshold</t>
-  </si>
-  <si>
     <t>Fraction of mapped reads that are marked as duplicates</t>
   </si>
   <si>
@@ -554,9 +551,6 @@
     <t>Percentage of reads that are unique following initial alignment</t>
   </si>
   <si>
-    <t>_filtered_fq_metrics.txt</t>
-  </si>
-  <si>
     <t>Percentage of fragments that fall within the expected size range on gel elextrophoresis (10,000-50,000 bp)</t>
   </si>
   <si>
@@ -620,9 +614,6 @@
     <t>Percentage of all sequenced bases with 1. MS depth &gt; half MS depth theshold and 2. EX duplex depth &gt; 0</t>
   </si>
   <si>
-    <t>^Pairs that were too short:\s+[\d,]+\s+\((?P&lt;percent&gt;[\d.]+)%\)\s*$</t>
-  </si>
-  <si>
     <t>Percentage of reads lost from creation of DSC</t>
   </si>
   <si>
@@ -711,6 +702,15 @@
   </si>
   <si>
     <t>Percentage of genome with depth &gt;= minimum MS depth value defined in config</t>
+  </si>
+  <si>
+    <t>ms_reads_filtered_quality</t>
+  </si>
+  <si>
+    <t>_length_filter_metrics.txt</t>
+  </si>
+  <si>
+    <t>_quality_filter_metrics.txt</t>
   </si>
 </sst>
 </file>
@@ -1194,9 +1194,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1581,20 +1580,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K82"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:K83"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="35.140625" customWidth="1"/>
-    <col min="2" max="2" width="123.140625" customWidth="1"/>
-    <col min="3" max="4" width="35.28515625" customWidth="1"/>
+    <col min="1" max="1" width="35.1796875" customWidth="1"/>
+    <col min="2" max="2" width="123.1796875" customWidth="1"/>
+    <col min="3" max="4" width="35.26953125" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" customWidth="1"/>
-    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="76.85546875" customWidth="1"/>
+    <col min="9" max="9" width="12.81640625" customWidth="1"/>
+    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="76.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>32</v>
       </c>
@@ -1623,18 +1622,18 @@
         <v>31</v>
       </c>
       <c r="J1" t="s">
+        <v>127</v>
+      </c>
+      <c r="K1" t="s">
         <v>128</v>
       </c>
-      <c r="K1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C2" t="s">
         <v>48</v>
@@ -1658,12 +1657,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C3" t="s">
         <v>48</v>
@@ -1693,12 +1692,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>36</v>
       </c>
       <c r="B4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C4" t="s">
         <v>48</v>
@@ -1728,12 +1727,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C5" t="s">
         <v>50</v>
@@ -1757,12 +1756,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C6" t="s">
         <v>50</v>
@@ -1792,12 +1791,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C7" t="s">
         <v>50</v>
@@ -1821,12 +1820,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="C8" t="s">
         <v>50</v>
@@ -1856,7 +1855,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1891,7 +1890,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -1926,7 +1925,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -1955,13 +1954,13 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K11" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -1990,18 +1989,18 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K12" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>93</v>
       </c>
       <c r="B13" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C13" t="s">
         <v>51</v>
@@ -2025,18 +2024,18 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K13" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>94</v>
       </c>
       <c r="B14" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C14" t="s">
         <v>51</v>
@@ -2060,18 +2059,18 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K14" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>91</v>
       </c>
       <c r="B15" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C15" t="s">
         <v>54</v>
@@ -2095,18 +2094,18 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K15" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>92</v>
       </c>
       <c r="B16" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C16" t="s">
         <v>54</v>
@@ -2130,13 +2129,13 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K16" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>83</v>
       </c>
@@ -2165,13 +2164,13 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K17" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>84</v>
       </c>
@@ -2200,18 +2199,18 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K18" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B19" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C19" t="s">
         <v>54</v>
@@ -2235,18 +2234,18 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K19" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B20" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C20" t="s">
         <v>54</v>
@@ -2270,13 +2269,13 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K20" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>71</v>
       </c>
@@ -2305,13 +2304,13 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K21" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>72</v>
       </c>
@@ -2340,13 +2339,13 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K22" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>73</v>
       </c>
@@ -2375,13 +2374,13 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K23" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>74</v>
       </c>
@@ -2410,13 +2409,13 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K24" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>75</v>
       </c>
@@ -2445,13 +2444,13 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K25" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>76</v>
       </c>
@@ -2480,18 +2479,18 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K26" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>77</v>
       </c>
       <c r="B27" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C27" t="s">
         <v>51</v>
@@ -2515,18 +2514,18 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K27" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>78</v>
       </c>
       <c r="B28" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C28" t="s">
         <v>51</v>
@@ -2550,18 +2549,18 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K28" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>79</v>
       </c>
       <c r="B29" t="s">
-        <v>125</v>
+        <v>178</v>
       </c>
       <c r="C29" t="s">
         <v>56</v>
@@ -2570,68 +2569,68 @@
         <v>25</v>
       </c>
       <c r="E29">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F29">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="G29">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="H29">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="I29" t="b">
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>172</v>
-      </c>
-      <c r="K29" s="1" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+        <v>223</v>
+      </c>
+      <c r="K29" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
+        <v>222</v>
+      </c>
+      <c r="B30" t="s">
+        <v>179</v>
+      </c>
+      <c r="C30" t="s">
+        <v>56</v>
+      </c>
+      <c r="D30" t="s">
+        <v>25</v>
+      </c>
+      <c r="E30">
+        <v>85</v>
+      </c>
+      <c r="F30">
+        <v>99</v>
+      </c>
+      <c r="G30">
+        <v>92.5</v>
+      </c>
+      <c r="H30">
+        <v>99</v>
+      </c>
+      <c r="I30" t="b">
+        <v>1</v>
+      </c>
+      <c r="J30" t="s">
+        <v>224</v>
+      </c>
+      <c r="K30" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
         <v>119</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B31" t="s">
         <v>112</v>
-      </c>
-      <c r="C30" t="s">
-        <v>57</v>
-      </c>
-      <c r="D30" t="s">
-        <v>25</v>
-      </c>
-      <c r="E30">
-        <v>90</v>
-      </c>
-      <c r="F30">
-        <v>100</v>
-      </c>
-      <c r="G30">
-        <v>95</v>
-      </c>
-      <c r="H30">
-        <v>100</v>
-      </c>
-      <c r="I30" t="b">
-        <v>1</v>
-      </c>
-      <c r="J30" t="s">
-        <v>137</v>
-      </c>
-      <c r="K30" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>118</v>
-      </c>
-      <c r="B31" t="s">
-        <v>126</v>
       </c>
       <c r="C31" t="s">
         <v>57</v>
@@ -2640,33 +2639,33 @@
         <v>25</v>
       </c>
       <c r="E31">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F31">
-        <v>0.1</v>
+        <v>100</v>
       </c>
       <c r="G31">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="H31">
-        <v>0.03</v>
+        <v>100</v>
       </c>
       <c r="I31" t="b">
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>212</v>
+        <v>136</v>
       </c>
       <c r="K31" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>218</v>
+        <v>118</v>
       </c>
       <c r="B32" t="s">
-        <v>224</v>
+        <v>125</v>
       </c>
       <c r="C32" t="s">
         <v>57</v>
@@ -2675,33 +2674,33 @@
         <v>25</v>
       </c>
       <c r="E32">
-        <v>21.75</v>
+        <v>0</v>
       </c>
       <c r="F32">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G32">
-        <v>26.1</v>
+        <v>0</v>
       </c>
       <c r="H32">
-        <v>100</v>
+        <v>0.03</v>
       </c>
       <c r="I32" t="b">
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>219</v>
+        <v>209</v>
       </c>
       <c r="K32" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
-        <v>117</v>
+        <v>215</v>
       </c>
       <c r="B33" t="s">
-        <v>82</v>
+        <v>221</v>
       </c>
       <c r="C33" t="s">
         <v>57</v>
@@ -2710,115 +2709,115 @@
         <v>25</v>
       </c>
       <c r="E33">
+        <v>21.75</v>
+      </c>
+      <c r="F33">
+        <v>100</v>
+      </c>
+      <c r="G33">
+        <v>26.1</v>
+      </c>
+      <c r="H33">
+        <v>100</v>
+      </c>
+      <c r="I33" t="b">
+        <v>1</v>
+      </c>
+      <c r="J33" t="s">
+        <v>216</v>
+      </c>
+      <c r="K33" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>117</v>
+      </c>
+      <c r="B34" t="s">
+        <v>82</v>
+      </c>
+      <c r="C34" t="s">
+        <v>57</v>
+      </c>
+      <c r="D34" t="s">
+        <v>25</v>
+      </c>
+      <c r="E34">
         <v>125</v>
       </c>
-      <c r="F33">
+      <c r="F34">
         <v>175</v>
       </c>
-      <c r="G33">
+      <c r="G34">
         <v>140</v>
       </c>
-      <c r="H33">
+      <c r="H34">
         <v>160</v>
       </c>
-      <c r="I33" t="b">
-        <v>1</v>
-      </c>
-      <c r="J33" t="s">
-        <v>138</v>
-      </c>
-      <c r="K33" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
+      <c r="I34" t="b">
+        <v>1</v>
+      </c>
+      <c r="J34" t="s">
+        <v>137</v>
+      </c>
+      <c r="K34" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
         <v>61</v>
       </c>
-      <c r="B34" t="s">
+      <c r="B35" t="s">
         <v>4</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C35" t="s">
         <v>59</v>
       </c>
-      <c r="D34" t="s">
-        <v>25</v>
-      </c>
-      <c r="E34">
+      <c r="D35" t="s">
+        <v>25</v>
+      </c>
+      <c r="E35">
         <v>70</v>
       </c>
-      <c r="F34">
+      <c r="F35">
         <v>90</v>
       </c>
-      <c r="G34">
+      <c r="G35">
         <v>70</v>
       </c>
-      <c r="H34">
+      <c r="H35">
         <v>80</v>
       </c>
-      <c r="I34" t="b">
-        <v>1</v>
-      </c>
-      <c r="J34" t="s">
+      <c r="I35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J35" t="s">
+        <v>165</v>
+      </c>
+      <c r="K35" t="s">
         <v>166</v>
       </c>
-      <c r="K34" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
         <v>20</v>
       </c>
-      <c r="B35" t="s">
+      <c r="B36" t="s">
         <v>40</v>
-      </c>
-      <c r="C35" t="s">
-        <v>49</v>
-      </c>
-      <c r="D35" t="s">
-        <v>25</v>
-      </c>
-      <c r="E35">
-        <v>75</v>
-      </c>
-      <c r="F35">
-        <v>1000</v>
-      </c>
-      <c r="I35" t="b">
-        <v>0</v>
-      </c>
-      <c r="J35" t="s">
-        <v>60</v>
-      </c>
-      <c r="K35" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>27</v>
-      </c>
-      <c r="B36" t="s">
-        <v>221</v>
       </c>
       <c r="C36" t="s">
         <v>49</v>
       </c>
       <c r="D36" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E36">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F36">
-        <v>0.3</v>
-      </c>
-      <c r="G36">
-        <v>0</v>
-      </c>
-      <c r="H36">
-        <v>0.2</v>
+        <v>1000</v>
       </c>
       <c r="I36" t="b">
         <v>0</v>
@@ -2830,30 +2829,30 @@
         <v>60</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B37" t="s">
-        <v>174</v>
+        <v>218</v>
       </c>
       <c r="C37" t="s">
         <v>49</v>
       </c>
       <c r="D37" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E37">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F37">
-        <v>100</v>
+        <v>0.3</v>
       </c>
       <c r="G37">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H37">
-        <v>100</v>
+        <v>0.2</v>
       </c>
       <c r="I37" t="b">
         <v>0</v>
@@ -2865,12 +2864,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="B38" t="s">
-        <v>42</v>
+        <v>172</v>
       </c>
       <c r="C38" t="s">
         <v>49</v>
@@ -2879,10 +2878,16 @@
         <v>25</v>
       </c>
       <c r="E38">
-        <v>4.3</v>
-      </c>
-      <c r="F38" t="s">
-        <v>5</v>
+        <v>80</v>
+      </c>
+      <c r="F38">
+        <v>100</v>
+      </c>
+      <c r="G38">
+        <v>95</v>
+      </c>
+      <c r="H38">
+        <v>100</v>
       </c>
       <c r="I38" t="b">
         <v>0</v>
@@ -2894,30 +2899,24 @@
         <v>60</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B39" t="s">
-        <v>221</v>
+        <v>42</v>
       </c>
       <c r="C39" t="s">
         <v>49</v>
       </c>
       <c r="D39" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E39">
-        <v>0</v>
-      </c>
-      <c r="F39">
-        <v>0.4</v>
-      </c>
-      <c r="G39">
-        <v>0</v>
-      </c>
-      <c r="H39">
-        <v>0.3</v>
+        <v>4.3</v>
+      </c>
+      <c r="F39" t="s">
+        <v>5</v>
       </c>
       <c r="I39" t="b">
         <v>0</v>
@@ -2929,30 +2928,30 @@
         <v>60</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B40" t="s">
-        <v>175</v>
+        <v>218</v>
       </c>
       <c r="C40" t="s">
         <v>49</v>
       </c>
       <c r="D40" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E40">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F40">
-        <v>100</v>
+        <v>0.4</v>
       </c>
       <c r="G40">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H40">
-        <v>100</v>
+        <v>0.3</v>
       </c>
       <c r="I40" t="b">
         <v>0</v>
@@ -2964,12 +2963,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B41" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="C41" t="s">
         <v>49</v>
@@ -2978,16 +2977,16 @@
         <v>25</v>
       </c>
       <c r="E41">
-        <v>1</v>
+        <v>80</v>
       </c>
       <c r="F41">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="G41">
-        <v>1</v>
+        <v>95</v>
       </c>
       <c r="H41">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I41" t="b">
         <v>0</v>
@@ -2999,12 +2998,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="B42" t="s">
-        <v>18</v>
+        <v>174</v>
       </c>
       <c r="C42" t="s">
         <v>49</v>
@@ -3013,16 +3012,16 @@
         <v>25</v>
       </c>
       <c r="E42">
-        <v>544</v>
+        <v>1</v>
       </c>
       <c r="F42">
-        <v>624</v>
+        <v>1</v>
       </c>
       <c r="G42">
-        <v>564</v>
+        <v>1</v>
       </c>
       <c r="H42">
-        <v>604</v>
+        <v>1</v>
       </c>
       <c r="I42" t="b">
         <v>0</v>
@@ -3034,12 +3033,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B43" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C43" t="s">
         <v>49</v>
@@ -3048,16 +3047,16 @@
         <v>25</v>
       </c>
       <c r="E43">
-        <v>98</v>
+        <v>544</v>
       </c>
       <c r="F43">
-        <v>100</v>
+        <v>624</v>
       </c>
       <c r="G43">
-        <v>100</v>
+        <v>564</v>
       </c>
       <c r="H43">
-        <v>100</v>
+        <v>604</v>
       </c>
       <c r="I43" t="b">
         <v>0</v>
@@ -3069,47 +3068,47 @@
         <v>60</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
+        <v>22</v>
+      </c>
+      <c r="B44" t="s">
+        <v>19</v>
+      </c>
+      <c r="C44" t="s">
+        <v>49</v>
+      </c>
+      <c r="D44" t="s">
+        <v>25</v>
+      </c>
+      <c r="E44">
+        <v>98</v>
+      </c>
+      <c r="F44">
+        <v>100</v>
+      </c>
+      <c r="G44">
+        <v>100</v>
+      </c>
+      <c r="H44">
+        <v>100</v>
+      </c>
+      <c r="I44" t="b">
+        <v>0</v>
+      </c>
+      <c r="J44" t="s">
+        <v>60</v>
+      </c>
+      <c r="K44" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
         <v>87</v>
       </c>
-      <c r="B44" t="s">
-        <v>214</v>
-      </c>
-      <c r="C44" t="s">
-        <v>53</v>
-      </c>
-      <c r="D44" t="s">
-        <v>65</v>
-      </c>
-      <c r="E44">
-        <v>35</v>
-      </c>
-      <c r="F44">
-        <v>40</v>
-      </c>
-      <c r="G44">
-        <v>39</v>
-      </c>
-      <c r="H44">
-        <v>40</v>
-      </c>
-      <c r="I44" t="b">
-        <v>1</v>
-      </c>
-      <c r="J44" t="s">
-        <v>139</v>
-      </c>
-      <c r="K44" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>88</v>
-      </c>
       <c r="B45" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="C45" t="s">
         <v>53</v>
@@ -3133,18 +3132,18 @@
         <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="K45" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B46" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C46" t="s">
         <v>53</v>
@@ -3153,16 +3152,16 @@
         <v>65</v>
       </c>
       <c r="E46">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F46">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G46">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="H46">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="I46" t="b">
         <v>1</v>
@@ -3171,15 +3170,15 @@
         <v>139</v>
       </c>
       <c r="K46" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B47" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C47" t="s">
         <v>53</v>
@@ -3203,18 +3202,18 @@
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="K47" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B48" t="s">
-        <v>85</v>
+        <v>210</v>
       </c>
       <c r="C48" t="s">
         <v>53</v>
@@ -3223,16 +3222,16 @@
         <v>65</v>
       </c>
       <c r="E48">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F48">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="G48">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="H48">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="I48" t="b">
         <v>1</v>
@@ -3241,12 +3240,12 @@
         <v>139</v>
       </c>
       <c r="K48" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="B49" t="s">
         <v>85</v>
@@ -3273,18 +3272,18 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="K49" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B50" t="s">
-        <v>106</v>
+        <v>85</v>
       </c>
       <c r="C50" t="s">
         <v>53</v>
@@ -3293,16 +3292,16 @@
         <v>65</v>
       </c>
       <c r="E50">
-        <v>2850</v>
-      </c>
-      <c r="F50" t="s">
-        <v>5</v>
+        <v>150</v>
+      </c>
+      <c r="F50">
+        <v>150</v>
       </c>
       <c r="G50">
-        <v>3000</v>
-      </c>
-      <c r="H50" t="s">
-        <v>5</v>
+        <v>150</v>
+      </c>
+      <c r="H50">
+        <v>150</v>
       </c>
       <c r="I50" t="b">
         <v>1</v>
@@ -3311,12 +3310,12 @@
         <v>139</v>
       </c>
       <c r="K50" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B51" t="s">
         <v>106</v>
@@ -3343,53 +3342,53 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="K51" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
-        <v>188</v>
+        <v>97</v>
       </c>
       <c r="B52" t="s">
-        <v>217</v>
+        <v>106</v>
       </c>
       <c r="C52" t="s">
         <v>53</v>
       </c>
       <c r="D52" t="s">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="E52">
-        <v>30</v>
-      </c>
-      <c r="F52">
-        <v>40</v>
+        <v>2850</v>
+      </c>
+      <c r="F52" t="s">
+        <v>5</v>
       </c>
       <c r="G52">
-        <v>35</v>
-      </c>
-      <c r="H52">
-        <v>40</v>
+        <v>3000</v>
+      </c>
+      <c r="H52" t="s">
+        <v>5</v>
       </c>
       <c r="I52" t="b">
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="K52" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="B53" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="C53" t="s">
         <v>53</v>
@@ -3413,18 +3412,18 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="K53" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>98</v>
+        <v>187</v>
       </c>
       <c r="B54" t="s">
-        <v>108</v>
+        <v>214</v>
       </c>
       <c r="C54" t="s">
         <v>53</v>
@@ -3433,16 +3432,16 @@
         <v>25</v>
       </c>
       <c r="E54">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F54">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="G54">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H54">
-        <v>0.1</v>
+        <v>40</v>
       </c>
       <c r="I54" t="b">
         <v>1</v>
@@ -3451,12 +3450,12 @@
         <v>141</v>
       </c>
       <c r="K54" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B55" t="s">
         <v>108</v>
@@ -3483,18 +3482,18 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="K55" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B56" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C56" t="s">
         <v>53</v>
@@ -3506,13 +3505,13 @@
         <v>0</v>
       </c>
       <c r="F56">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="G56">
         <v>0</v>
       </c>
       <c r="H56">
-        <v>20</v>
+        <v>0.1</v>
       </c>
       <c r="I56" t="b">
         <v>1</v>
@@ -3521,12 +3520,12 @@
         <v>141</v>
       </c>
       <c r="K56" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="B57" t="s">
         <v>109</v>
@@ -3553,18 +3552,18 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="K57" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="B58" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C58" t="s">
         <v>53</v>
@@ -3576,13 +3575,13 @@
         <v>0</v>
       </c>
       <c r="F58">
+        <v>30</v>
+      </c>
+      <c r="G58">
+        <v>0</v>
+      </c>
+      <c r="H58">
         <v>20</v>
-      </c>
-      <c r="G58">
-        <v>0</v>
-      </c>
-      <c r="H58">
-        <v>10</v>
       </c>
       <c r="I58" t="b">
         <v>1</v>
@@ -3591,12 +3590,12 @@
         <v>141</v>
       </c>
       <c r="K58" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B59" t="s">
         <v>110</v>
@@ -3623,18 +3622,18 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="K59" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B60" t="s">
-        <v>216</v>
+        <v>110</v>
       </c>
       <c r="C60" t="s">
         <v>53</v>
@@ -3646,13 +3645,13 @@
         <v>0</v>
       </c>
       <c r="F60">
+        <v>20</v>
+      </c>
+      <c r="G60">
+        <v>0</v>
+      </c>
+      <c r="H60">
         <v>10</v>
-      </c>
-      <c r="G60">
-        <v>0</v>
-      </c>
-      <c r="H60">
-        <v>5</v>
       </c>
       <c r="I60" t="b">
         <v>1</v>
@@ -3661,15 +3660,15 @@
         <v>141</v>
       </c>
       <c r="K60" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B61" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C61" t="s">
         <v>53</v>
@@ -3693,53 +3692,53 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="K61" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
+        <v>105</v>
+      </c>
+      <c r="B62" t="s">
+        <v>213</v>
+      </c>
+      <c r="C62" t="s">
+        <v>53</v>
+      </c>
+      <c r="D62" t="s">
+        <v>25</v>
+      </c>
+      <c r="E62">
+        <v>0</v>
+      </c>
+      <c r="F62">
+        <v>10</v>
+      </c>
+      <c r="G62">
+        <v>0</v>
+      </c>
+      <c r="H62">
+        <v>5</v>
+      </c>
+      <c r="I62" t="b">
+        <v>1</v>
+      </c>
+      <c r="J62" t="s">
+        <v>141</v>
+      </c>
+      <c r="K62" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A63" t="s">
         <v>62</v>
       </c>
-      <c r="B62" t="s">
-        <v>201</v>
-      </c>
-      <c r="C62" t="s">
-        <v>55</v>
-      </c>
-      <c r="D62" t="s">
-        <v>65</v>
-      </c>
-      <c r="E62">
-        <v>0</v>
-      </c>
-      <c r="F62">
-        <v>25</v>
-      </c>
-      <c r="G62">
-        <v>0</v>
-      </c>
-      <c r="H62">
-        <v>10</v>
-      </c>
-      <c r="I62" t="b">
-        <v>1</v>
-      </c>
-      <c r="J62" t="s">
-        <v>199</v>
-      </c>
-      <c r="K62" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>113</v>
-      </c>
       <c r="B63" t="s">
-        <v>114</v>
+        <v>198</v>
       </c>
       <c r="C63" t="s">
         <v>55</v>
@@ -3751,65 +3750,65 @@
         <v>0</v>
       </c>
       <c r="F63">
-        <v>0.1</v>
+        <v>25</v>
       </c>
       <c r="G63">
         <v>0</v>
       </c>
       <c r="H63">
-        <v>0.05</v>
+        <v>10</v>
       </c>
       <c r="I63" t="b">
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="K63" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
-        <v>178</v>
+        <v>113</v>
       </c>
       <c r="B64" t="s">
-        <v>179</v>
+        <v>114</v>
       </c>
       <c r="C64" t="s">
         <v>55</v>
       </c>
       <c r="D64" t="s">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="E64">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F64">
-        <v>40</v>
+        <v>0.1</v>
       </c>
       <c r="G64">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H64">
-        <v>20</v>
+        <v>0.05</v>
       </c>
       <c r="I64" t="b">
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>187</v>
+        <v>196</v>
       </c>
       <c r="K64" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>205</v>
+        <v>176</v>
       </c>
       <c r="B65" t="s">
-        <v>192</v>
+        <v>177</v>
       </c>
       <c r="C65" t="s">
         <v>55</v>
@@ -3818,33 +3817,33 @@
         <v>25</v>
       </c>
       <c r="E65">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F65">
+        <v>40</v>
+      </c>
+      <c r="G65">
+        <v>1</v>
+      </c>
+      <c r="H65">
         <v>20</v>
       </c>
-      <c r="G65">
-        <v>0</v>
-      </c>
-      <c r="H65">
-        <v>10</v>
-      </c>
       <c r="I65" t="b">
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>203</v>
+        <v>185</v>
       </c>
       <c r="K65" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>63</v>
+        <v>202</v>
       </c>
       <c r="B66" t="s">
-        <v>180</v>
+        <v>190</v>
       </c>
       <c r="C66" t="s">
         <v>55</v>
@@ -3853,33 +3852,33 @@
         <v>25</v>
       </c>
       <c r="E66">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F66">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="G66">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="H66">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="I66" t="b">
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>183</v>
+        <v>200</v>
       </c>
       <c r="K66" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B67" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C67" t="s">
         <v>55</v>
@@ -3888,13 +3887,13 @@
         <v>25</v>
       </c>
       <c r="E67">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="F67">
         <v>99</v>
       </c>
       <c r="G67">
-        <v>92.5</v>
+        <v>90</v>
       </c>
       <c r="H67">
         <v>99</v>
@@ -3903,53 +3902,53 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="K67" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A68" t="s">
+        <v>64</v>
+      </c>
+      <c r="B68" t="s">
+        <v>179</v>
+      </c>
+      <c r="C68" t="s">
+        <v>55</v>
+      </c>
+      <c r="D68" t="s">
+        <v>25</v>
+      </c>
+      <c r="E68">
+        <v>85</v>
+      </c>
+      <c r="F68">
+        <v>99</v>
+      </c>
+      <c r="G68">
+        <v>92.5</v>
+      </c>
+      <c r="H68">
+        <v>99</v>
+      </c>
+      <c r="I68" t="b">
+        <v>1</v>
+      </c>
+      <c r="J68" t="s">
         <v>182</v>
       </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
+      <c r="K68" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A69" t="s">
         <v>67</v>
       </c>
-      <c r="B68" t="s">
+      <c r="B69" t="s">
         <v>80</v>
-      </c>
-      <c r="C68" t="s">
-        <v>52</v>
-      </c>
-      <c r="D68" t="s">
-        <v>25</v>
-      </c>
-      <c r="E68">
-        <v>90</v>
-      </c>
-      <c r="F68">
-        <v>100</v>
-      </c>
-      <c r="G68">
-        <v>95</v>
-      </c>
-      <c r="H68">
-        <v>100</v>
-      </c>
-      <c r="I68" t="b">
-        <v>1</v>
-      </c>
-      <c r="J68" t="s">
-        <v>130</v>
-      </c>
-      <c r="K68" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>66</v>
-      </c>
-      <c r="B69" t="s">
-        <v>81</v>
       </c>
       <c r="C69" t="s">
         <v>52</v>
@@ -3958,13 +3957,13 @@
         <v>25</v>
       </c>
       <c r="E69">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="F69">
         <v>100</v>
       </c>
       <c r="G69">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="H69">
         <v>100</v>
@@ -3973,18 +3972,18 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K69" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B70" t="s">
-        <v>115</v>
+        <v>81</v>
       </c>
       <c r="C70" t="s">
         <v>52</v>
@@ -3993,68 +3992,68 @@
         <v>25</v>
       </c>
       <c r="E70">
-        <v>125</v>
+        <v>50</v>
       </c>
       <c r="F70">
-        <v>175</v>
+        <v>100</v>
       </c>
       <c r="G70">
-        <v>140</v>
+        <v>75</v>
       </c>
       <c r="H70">
-        <v>160</v>
+        <v>100</v>
       </c>
       <c r="I70" t="b">
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K70" t="s">
         <v>163</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
-        <v>127</v>
+        <v>68</v>
       </c>
       <c r="B71" t="s">
-        <v>195</v>
+        <v>115</v>
       </c>
       <c r="C71" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D71" t="s">
         <v>25</v>
       </c>
       <c r="E71">
-        <v>50</v>
+        <v>125</v>
       </c>
       <c r="F71">
-        <v>70</v>
+        <v>175</v>
       </c>
       <c r="G71">
-        <v>50</v>
+        <v>140</v>
       </c>
       <c r="H71">
-        <v>60</v>
+        <v>160</v>
       </c>
       <c r="I71" t="b">
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>155</v>
+        <v>130</v>
       </c>
       <c r="K71" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>116</v>
+        <v>126</v>
       </c>
       <c r="B72" t="s">
-        <v>171</v>
+        <v>192</v>
       </c>
       <c r="C72" t="s">
         <v>58</v>
@@ -4063,33 +4062,33 @@
         <v>25</v>
       </c>
       <c r="E72">
+        <v>50</v>
+      </c>
+      <c r="F72">
+        <v>70</v>
+      </c>
+      <c r="G72">
+        <v>50</v>
+      </c>
+      <c r="H72">
         <v>60</v>
       </c>
-      <c r="F72">
-        <v>100</v>
-      </c>
-      <c r="G72">
-        <v>90</v>
-      </c>
-      <c r="H72">
-        <v>100</v>
-      </c>
       <c r="I72" t="b">
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>169</v>
+        <v>154</v>
       </c>
       <c r="K72" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="B73" t="s">
-        <v>10</v>
+        <v>170</v>
       </c>
       <c r="C73" t="s">
         <v>58</v>
@@ -4098,13 +4097,13 @@
         <v>25</v>
       </c>
       <c r="E73">
-        <v>99</v>
+        <v>60</v>
       </c>
       <c r="F73">
         <v>100</v>
       </c>
       <c r="G73">
-        <v>99.5</v>
+        <v>90</v>
       </c>
       <c r="H73">
         <v>100</v>
@@ -4113,18 +4112,18 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="K73" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B74" t="s">
-        <v>120</v>
+        <v>10</v>
       </c>
       <c r="C74" t="s">
         <v>58</v>
@@ -4133,33 +4132,33 @@
         <v>25</v>
       </c>
       <c r="E74">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="F74">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="G74">
-        <v>0</v>
+        <v>99.5</v>
       </c>
       <c r="H74">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="I74" t="b">
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="K74" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="B75" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="C75" t="s">
         <v>58</v>
@@ -4168,33 +4167,33 @@
         <v>25</v>
       </c>
       <c r="E75">
-        <v>0.5</v>
-      </c>
-      <c r="F75" t="s">
+        <v>0</v>
+      </c>
+      <c r="F75">
+        <v>15</v>
+      </c>
+      <c r="G75">
+        <v>0</v>
+      </c>
+      <c r="H75">
         <v>5</v>
       </c>
-      <c r="G75">
-        <v>1</v>
-      </c>
-      <c r="H75" t="s">
-        <v>5</v>
-      </c>
       <c r="I75" t="b">
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>170</v>
+        <v>158</v>
       </c>
       <c r="K75" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
-        <v>14</v>
+        <v>123</v>
       </c>
       <c r="B76" t="s">
-        <v>15</v>
+        <v>124</v>
       </c>
       <c r="C76" t="s">
         <v>58</v>
@@ -4203,33 +4202,33 @@
         <v>25</v>
       </c>
       <c r="E76">
-        <v>0</v>
-      </c>
-      <c r="F76">
-        <v>0</v>
+        <v>0.5</v>
+      </c>
+      <c r="F76" t="s">
+        <v>5</v>
       </c>
       <c r="G76">
-        <v>0</v>
-      </c>
-      <c r="H76">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H76" t="s">
+        <v>5</v>
       </c>
       <c r="I76" t="b">
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>132</v>
+        <v>169</v>
       </c>
       <c r="K76" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B77" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C77" t="s">
         <v>58</v>
@@ -4238,33 +4237,33 @@
         <v>25</v>
       </c>
       <c r="E77">
-        <v>14.5</v>
+        <v>0</v>
       </c>
       <c r="F77">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G77">
-        <v>26.1</v>
+        <v>0</v>
       </c>
       <c r="H77">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I77" t="b">
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>170</v>
+        <v>131</v>
       </c>
       <c r="K77" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A78" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A78" t="s">
-        <v>8</v>
-      </c>
       <c r="B78" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C78" t="s">
         <v>58</v>
@@ -4273,169 +4272,204 @@
         <v>25</v>
       </c>
       <c r="E78">
+        <v>14.5</v>
+      </c>
+      <c r="F78">
+        <v>100</v>
+      </c>
+      <c r="G78">
+        <v>26.1</v>
+      </c>
+      <c r="H78">
+        <v>100</v>
+      </c>
+      <c r="I78" t="b">
+        <v>1</v>
+      </c>
+      <c r="J78" t="s">
+        <v>169</v>
+      </c>
+      <c r="K78" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A79" t="s">
+        <v>8</v>
+      </c>
+      <c r="B79" t="s">
+        <v>9</v>
+      </c>
+      <c r="C79" t="s">
+        <v>58</v>
+      </c>
+      <c r="D79" t="s">
+        <v>25</v>
+      </c>
+      <c r="E79">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="F78">
+      <c r="F79">
         <v>8.0000000000000004E-4</v>
       </c>
-      <c r="G78">
+      <c r="G79">
         <v>2.0000000000000001E-4</v>
       </c>
-      <c r="H78">
+      <c r="H79">
         <v>5.0000000000000001E-4</v>
       </c>
-      <c r="I78" t="b">
-        <v>1</v>
-      </c>
-      <c r="J78" t="s">
-        <v>186</v>
-      </c>
-      <c r="K78" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A79" t="s">
+      <c r="I79" t="b">
+        <v>1</v>
+      </c>
+      <c r="J79" t="s">
+        <v>184</v>
+      </c>
+      <c r="K79" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A80" t="s">
+        <v>203</v>
+      </c>
+      <c r="B80" t="s">
+        <v>204</v>
+      </c>
+      <c r="C80" t="s">
+        <v>175</v>
+      </c>
+      <c r="D80" t="s">
+        <v>25</v>
+      </c>
+      <c r="E80">
+        <v>0.05</v>
+      </c>
+      <c r="F80">
+        <v>0.08</v>
+      </c>
+      <c r="G80">
+        <v>0.02</v>
+      </c>
+      <c r="H80">
+        <v>0.05</v>
+      </c>
+      <c r="I80" t="b">
+        <v>1</v>
+      </c>
+      <c r="J80" t="s">
         <v>206</v>
       </c>
-      <c r="B79" t="s">
+      <c r="K80" t="s">
         <v>207</v>
       </c>
-      <c r="C79" t="s">
-        <v>177</v>
-      </c>
-      <c r="D79" t="s">
-        <v>25</v>
-      </c>
-      <c r="E79">
-        <v>0.05</v>
-      </c>
-      <c r="F79">
-        <v>0.08</v>
-      </c>
-      <c r="G79">
-        <v>0.02</v>
-      </c>
-      <c r="H79">
-        <v>0.05</v>
-      </c>
-      <c r="I79" t="b">
-        <v>1</v>
-      </c>
-      <c r="J79" t="s">
-        <v>209</v>
-      </c>
-      <c r="K79" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A80" t="s">
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A81" t="s">
         <v>11</v>
       </c>
-      <c r="B80" t="s">
-        <v>208</v>
-      </c>
-      <c r="C80" t="s">
-        <v>177</v>
-      </c>
-      <c r="D80" t="s">
-        <v>25</v>
-      </c>
-      <c r="E80">
+      <c r="B81" t="s">
+        <v>205</v>
+      </c>
+      <c r="C81" t="s">
+        <v>175</v>
+      </c>
+      <c r="D81" t="s">
+        <v>25</v>
+      </c>
+      <c r="E81">
         <v>5</v>
       </c>
-      <c r="F80">
+      <c r="F81">
         <v>100</v>
       </c>
-      <c r="G80">
+      <c r="G81">
         <v>20</v>
       </c>
-      <c r="H80">
+      <c r="H81">
         <v>100</v>
       </c>
-      <c r="I80" t="b">
-        <v>1</v>
-      </c>
-      <c r="J80" t="s">
-        <v>170</v>
-      </c>
-      <c r="K80" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A81" t="s">
+      <c r="I81" t="b">
+        <v>1</v>
+      </c>
+      <c r="J81" t="s">
+        <v>169</v>
+      </c>
+      <c r="K81" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A82" t="s">
         <v>17</v>
       </c>
-      <c r="B81" t="s">
+      <c r="B82" t="s">
         <v>16</v>
       </c>
-      <c r="C81" t="s">
-        <v>177</v>
-      </c>
-      <c r="D81" t="s">
-        <v>25</v>
-      </c>
-      <c r="E81">
-        <v>0</v>
-      </c>
-      <c r="F81">
+      <c r="C82" t="s">
+        <v>175</v>
+      </c>
+      <c r="D82" t="s">
+        <v>25</v>
+      </c>
+      <c r="E82">
+        <v>0</v>
+      </c>
+      <c r="F82">
         <v>95</v>
       </c>
-      <c r="G81">
-        <v>0</v>
-      </c>
-      <c r="H81">
+      <c r="G82">
+        <v>0</v>
+      </c>
+      <c r="H82">
         <v>80</v>
       </c>
-      <c r="I81" t="b">
-        <v>1</v>
-      </c>
-      <c r="J81" t="s">
-        <v>143</v>
-      </c>
-      <c r="K81" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A82" t="s">
+      <c r="I82" t="b">
+        <v>1</v>
+      </c>
+      <c r="J82" t="s">
+        <v>142</v>
+      </c>
+      <c r="K82" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A83" t="s">
         <v>47</v>
       </c>
-      <c r="B82" t="s">
-        <v>193</v>
-      </c>
-      <c r="C82" t="s">
-        <v>177</v>
-      </c>
-      <c r="D82" t="s">
-        <v>25</v>
-      </c>
-      <c r="E82">
+      <c r="B83" t="s">
+        <v>191</v>
+      </c>
+      <c r="C83" t="s">
+        <v>175</v>
+      </c>
+      <c r="D83" t="s">
+        <v>25</v>
+      </c>
+      <c r="E83">
         <v>33</v>
       </c>
-      <c r="F82">
+      <c r="F83">
         <v>100</v>
       </c>
-      <c r="G82">
+      <c r="G83">
         <v>67</v>
       </c>
-      <c r="H82">
+      <c r="H83">
         <v>100</v>
       </c>
-      <c r="I82" t="b">
-        <v>1</v>
-      </c>
-      <c r="J82" t="s">
-        <v>170</v>
-      </c>
-      <c r="K82" t="s">
+      <c r="I83" t="b">
+        <v>1</v>
+      </c>
+      <c r="J83" t="s">
+        <v>169</v>
+      </c>
+      <c r="K83" t="s">
         <v>47</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K80" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K81" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
1. Updated low depth mask to use effective depth after accounting for low base quality 2. Added germline risk masking rate component metric 3. Updated resource allocation
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -5,18 +5,18 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8313D711-6932-4253-BE9A-CDEA1651B409}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD19655F-4079-4AEF-9964-53AB0454C2E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$82</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="228">
   <si>
     <t>nn_lower</t>
   </si>
@@ -191,9 +191,6 @@
     <t>MS library preparation</t>
   </si>
   <si>
-    <t>MS Sequencing</t>
-  </si>
-  <si>
     <t>EX alignment</t>
   </si>
   <si>
@@ -215,9 +212,6 @@
     <t>EX create DSC</t>
   </si>
   <si>
-    <t>Mask regions</t>
-  </si>
-  <si>
     <t>NA</t>
   </si>
   <si>
@@ -711,6 +705,21 @@
   </si>
   <si>
     <t>_quality_filter_metrics.txt</t>
+  </si>
+  <si>
+    <t>MS mask regions</t>
+  </si>
+  <si>
+    <t>germline_variant_rate</t>
+  </si>
+  <si>
+    <t>_germ_risk_variant_metrics_summary.json</t>
+  </si>
+  <si>
+    <t>ms_germline_risk_masking_rate</t>
+  </si>
+  <si>
+    <t>Proportion of genomic positions masked due to risk of being a germline variant</t>
   </si>
 </sst>
 </file>
@@ -1580,20 +1589,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K83"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K84"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.1796875" customWidth="1"/>
-    <col min="2" max="2" width="123.1796875" customWidth="1"/>
-    <col min="3" max="4" width="35.26953125" customWidth="1"/>
+    <col min="1" max="1" width="35.140625" customWidth="1"/>
+    <col min="2" max="2" width="123.140625" customWidth="1"/>
+    <col min="3" max="4" width="35.28515625" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.81640625" customWidth="1"/>
-    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="76.81640625" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="76.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>32</v>
       </c>
@@ -1622,18 +1631,18 @@
         <v>31</v>
       </c>
       <c r="J1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="K1" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C2" t="s">
         <v>48</v>
@@ -1651,18 +1660,18 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C3" t="s">
         <v>48</v>
@@ -1686,18 +1695,18 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K3" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>36</v>
       </c>
       <c r="B4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C4" t="s">
         <v>48</v>
@@ -1721,18 +1730,18 @@
         <v>0</v>
       </c>
       <c r="J4" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K4" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C5" t="s">
         <v>50</v>
@@ -1750,18 +1759,18 @@
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K5" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C6" t="s">
         <v>50</v>
@@ -1785,18 +1794,18 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K6" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C7" t="s">
         <v>50</v>
@@ -1814,18 +1823,18 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K7" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="C8" t="s">
         <v>50</v>
@@ -1849,18 +1858,18 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K8" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C9" t="s">
         <v>50</v>
@@ -1884,18 +1893,18 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K9" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="C10" t="s">
         <v>50</v>
@@ -1919,21 +1928,21 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K10" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D11" t="s">
         <v>25</v>
@@ -1954,21 +1963,21 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K11" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D12" t="s">
         <v>25</v>
@@ -1989,21 +1998,21 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K12" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B13" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C13" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D13" t="s">
         <v>25</v>
@@ -2024,21 +2033,21 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K13" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B14" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C14" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D14" t="s">
         <v>25</v>
@@ -2059,21 +2068,21 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K14" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B15" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D15" t="s">
         <v>25</v>
@@ -2094,21 +2103,21 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K15" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B16" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C16" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D16" t="s">
         <v>25</v>
@@ -2129,21 +2138,21 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K16" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>81</v>
+      </c>
+      <c r="B17" t="s">
         <v>83</v>
       </c>
-      <c r="B17" t="s">
-        <v>85</v>
-      </c>
       <c r="C17" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D17" t="s">
         <v>25</v>
@@ -2164,21 +2173,21 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K17" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B18" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C18" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D18" t="s">
         <v>25</v>
@@ -2199,21 +2208,21 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K18" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B19" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C19" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D19" t="s">
         <v>25</v>
@@ -2234,21 +2243,21 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K19" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B20" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C20" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D20" t="s">
         <v>25</v>
@@ -2269,21 +2278,21 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K20" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B21" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C21" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D21" t="s">
         <v>25</v>
@@ -2304,21 +2313,21 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K21" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B22" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C22" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D22" t="s">
         <v>25</v>
@@ -2339,21 +2348,21 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K22" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B23" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C23" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D23" t="s">
         <v>25</v>
@@ -2374,21 +2383,21 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K23" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B24" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C24" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D24" t="s">
         <v>25</v>
@@ -2409,21 +2418,21 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K24" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B25" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C25" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D25" t="s">
         <v>25</v>
@@ -2444,21 +2453,21 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K25" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B26" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C26" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D26" t="s">
         <v>25</v>
@@ -2479,21 +2488,21 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K26" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B27" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C27" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D27" t="s">
         <v>25</v>
@@ -2514,21 +2523,21 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K27" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B28" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C28" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D28" t="s">
         <v>25</v>
@@ -2549,21 +2558,21 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K28" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="B29" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C29" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D29" t="s">
         <v>25</v>
@@ -2584,21 +2593,21 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="K29" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B30" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C30" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D30" t="s">
         <v>25</v>
@@ -2619,21 +2628,21 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="K30" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B31" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C31" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D31" t="s">
         <v>25</v>
@@ -2654,21 +2663,21 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="K31" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B32" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C32" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D32" t="s">
         <v>25</v>
@@ -2689,21 +2698,21 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="K32" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B33" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C33" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D33" t="s">
         <v>25</v>
@@ -2724,21 +2733,21 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="K33" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B34" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C34" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D34" t="s">
         <v>25</v>
@@ -2759,152 +2768,152 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="K34" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>61</v>
+        <v>226</v>
       </c>
       <c r="B35" t="s">
+        <v>227</v>
+      </c>
+      <c r="C35" t="s">
+        <v>223</v>
+      </c>
+      <c r="D35" t="s">
+        <v>25</v>
+      </c>
+      <c r="E35">
+        <v>1.5E-3</v>
+      </c>
+      <c r="F35">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="G35">
+        <v>1.5E-3</v>
+      </c>
+      <c r="H35">
+        <v>3.0000000000000001E-3</v>
+      </c>
+      <c r="I35" t="b">
+        <v>1</v>
+      </c>
+      <c r="J35" t="s">
+        <v>225</v>
+      </c>
+      <c r="K35" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>59</v>
+      </c>
+      <c r="B36" t="s">
         <v>4</v>
       </c>
-      <c r="C35" t="s">
-        <v>59</v>
-      </c>
-      <c r="D35" t="s">
-        <v>25</v>
-      </c>
-      <c r="E35">
+      <c r="C36" t="s">
+        <v>223</v>
+      </c>
+      <c r="D36" t="s">
+        <v>25</v>
+      </c>
+      <c r="E36">
         <v>70</v>
       </c>
-      <c r="F35">
+      <c r="F36">
         <v>90</v>
       </c>
-      <c r="G35">
+      <c r="G36">
         <v>70</v>
       </c>
-      <c r="H35">
+      <c r="H36">
         <v>80</v>
       </c>
-      <c r="I35" t="b">
-        <v>1</v>
-      </c>
-      <c r="J35" t="s">
-        <v>165</v>
-      </c>
-      <c r="K35" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A36" t="s">
+      <c r="I36" t="b">
+        <v>1</v>
+      </c>
+      <c r="J36" t="s">
+        <v>163</v>
+      </c>
+      <c r="K36" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
         <v>20</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B37" t="s">
         <v>40</v>
-      </c>
-      <c r="C36" t="s">
-        <v>49</v>
-      </c>
-      <c r="D36" t="s">
-        <v>25</v>
-      </c>
-      <c r="E36">
-        <v>75</v>
-      </c>
-      <c r="F36">
-        <v>1000</v>
-      </c>
-      <c r="I36" t="b">
-        <v>0</v>
-      </c>
-      <c r="J36" t="s">
-        <v>60</v>
-      </c>
-      <c r="K36" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A37" t="s">
-        <v>27</v>
-      </c>
-      <c r="B37" t="s">
-        <v>218</v>
       </c>
       <c r="C37" t="s">
         <v>49</v>
       </c>
       <c r="D37" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E37">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F37">
-        <v>0.3</v>
-      </c>
-      <c r="G37">
-        <v>0</v>
-      </c>
-      <c r="H37">
-        <v>0.2</v>
+        <v>1000</v>
       </c>
       <c r="I37" t="b">
         <v>0</v>
       </c>
       <c r="J37" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K37" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B38" t="s">
-        <v>172</v>
+        <v>216</v>
       </c>
       <c r="C38" t="s">
         <v>49</v>
       </c>
       <c r="D38" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E38">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F38">
-        <v>100</v>
+        <v>0.3</v>
       </c>
       <c r="G38">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H38">
-        <v>100</v>
+        <v>0.2</v>
       </c>
       <c r="I38" t="b">
         <v>0</v>
       </c>
       <c r="J38" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K38" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>41</v>
+        <v>33</v>
       </c>
       <c r="B39" t="s">
-        <v>42</v>
+        <v>170</v>
       </c>
       <c r="C39" t="s">
         <v>49</v>
@@ -2913,97 +2922,97 @@
         <v>25</v>
       </c>
       <c r="E39">
-        <v>4.3</v>
-      </c>
-      <c r="F39" t="s">
-        <v>5</v>
+        <v>80</v>
+      </c>
+      <c r="F39">
+        <v>100</v>
+      </c>
+      <c r="G39">
+        <v>95</v>
+      </c>
+      <c r="H39">
+        <v>100</v>
       </c>
       <c r="I39" t="b">
         <v>0</v>
       </c>
       <c r="J39" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K39" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B40" t="s">
-        <v>218</v>
+        <v>42</v>
       </c>
       <c r="C40" t="s">
         <v>49</v>
       </c>
       <c r="D40" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E40">
-        <v>0</v>
-      </c>
-      <c r="F40">
-        <v>0.4</v>
-      </c>
-      <c r="G40">
-        <v>0</v>
-      </c>
-      <c r="H40">
-        <v>0.3</v>
+        <v>4.3</v>
+      </c>
+      <c r="F40" t="s">
+        <v>5</v>
       </c>
       <c r="I40" t="b">
         <v>0</v>
       </c>
       <c r="J40" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K40" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B41" t="s">
-        <v>173</v>
+        <v>216</v>
       </c>
       <c r="C41" t="s">
         <v>49</v>
       </c>
       <c r="D41" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E41">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="F41">
-        <v>100</v>
+        <v>0.4</v>
       </c>
       <c r="G41">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H41">
-        <v>100</v>
+        <v>0.3</v>
       </c>
       <c r="I41" t="b">
         <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K41" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B42" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="C42" t="s">
         <v>49</v>
@@ -3012,33 +3021,33 @@
         <v>25</v>
       </c>
       <c r="E42">
-        <v>1</v>
+        <v>80</v>
       </c>
       <c r="F42">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="G42">
-        <v>1</v>
+        <v>95</v>
       </c>
       <c r="H42">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I42" t="b">
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K42" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>21</v>
+        <v>39</v>
       </c>
       <c r="B43" t="s">
-        <v>18</v>
+        <v>172</v>
       </c>
       <c r="C43" t="s">
         <v>49</v>
@@ -3047,33 +3056,33 @@
         <v>25</v>
       </c>
       <c r="E43">
-        <v>544</v>
+        <v>1</v>
       </c>
       <c r="F43">
-        <v>624</v>
+        <v>1</v>
       </c>
       <c r="G43">
-        <v>564</v>
+        <v>1</v>
       </c>
       <c r="H43">
-        <v>604</v>
+        <v>1</v>
       </c>
       <c r="I43" t="b">
         <v>0</v>
       </c>
       <c r="J43" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="K43" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B44" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C44" t="s">
         <v>49</v>
@@ -3082,74 +3091,74 @@
         <v>25</v>
       </c>
       <c r="E44">
+        <v>544</v>
+      </c>
+      <c r="F44">
+        <v>624</v>
+      </c>
+      <c r="G44">
+        <v>564</v>
+      </c>
+      <c r="H44">
+        <v>604</v>
+      </c>
+      <c r="I44" t="b">
+        <v>0</v>
+      </c>
+      <c r="J44" t="s">
+        <v>58</v>
+      </c>
+      <c r="K44" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>22</v>
+      </c>
+      <c r="B45" t="s">
+        <v>19</v>
+      </c>
+      <c r="C45" t="s">
+        <v>49</v>
+      </c>
+      <c r="D45" t="s">
+        <v>25</v>
+      </c>
+      <c r="E45">
         <v>98</v>
       </c>
-      <c r="F44">
+      <c r="F45">
         <v>100</v>
       </c>
-      <c r="G44">
+      <c r="G45">
         <v>100</v>
       </c>
-      <c r="H44">
+      <c r="H45">
         <v>100</v>
       </c>
-      <c r="I44" t="b">
-        <v>0</v>
-      </c>
-      <c r="J44" t="s">
-        <v>60</v>
-      </c>
-      <c r="K44" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A45" t="s">
-        <v>87</v>
-      </c>
-      <c r="B45" t="s">
-        <v>211</v>
-      </c>
-      <c r="C45" t="s">
-        <v>53</v>
-      </c>
-      <c r="D45" t="s">
-        <v>65</v>
-      </c>
-      <c r="E45">
-        <v>35</v>
-      </c>
-      <c r="F45">
-        <v>40</v>
-      </c>
-      <c r="G45">
-        <v>39</v>
-      </c>
-      <c r="H45">
-        <v>40</v>
-      </c>
       <c r="I45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J45" t="s">
-        <v>138</v>
+        <v>58</v>
       </c>
       <c r="K45" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="B46" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="C46" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D46" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E46">
         <v>35</v>
@@ -3167,59 +3176,59 @@
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="K46" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B47" t="s">
         <v>210</v>
       </c>
       <c r="C47" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D47" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E47">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F47">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G47">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="H47">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="I47" t="b">
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K47" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B48" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C48" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D48" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E48">
         <v>0</v>
@@ -3237,59 +3246,59 @@
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="K48" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B49" t="s">
-        <v>85</v>
+        <v>208</v>
       </c>
       <c r="C49" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D49" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E49">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F49">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="G49">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="H49">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="I49" t="b">
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K49" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="B50" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C50" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D50" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E50">
         <v>150</v>
@@ -3307,59 +3316,59 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="K50" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="B51" t="s">
-        <v>106</v>
+        <v>83</v>
       </c>
       <c r="C51" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D51" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E51">
-        <v>2850</v>
-      </c>
-      <c r="F51" t="s">
-        <v>5</v>
+        <v>150</v>
+      </c>
+      <c r="F51">
+        <v>150</v>
       </c>
       <c r="G51">
-        <v>3000</v>
-      </c>
-      <c r="H51" t="s">
-        <v>5</v>
+        <v>150</v>
+      </c>
+      <c r="H51">
+        <v>150</v>
       </c>
       <c r="I51" t="b">
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K51" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="B52" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C52" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D52" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E52">
         <v>2850</v>
@@ -3377,56 +3386,56 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="K52" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>186</v>
+        <v>95</v>
       </c>
       <c r="B53" t="s">
-        <v>214</v>
+        <v>104</v>
       </c>
       <c r="C53" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D53" t="s">
-        <v>25</v>
+        <v>63</v>
       </c>
       <c r="E53">
-        <v>30</v>
-      </c>
-      <c r="F53">
-        <v>40</v>
+        <v>2850</v>
+      </c>
+      <c r="F53" t="s">
+        <v>5</v>
       </c>
       <c r="G53">
-        <v>35</v>
-      </c>
-      <c r="H53">
-        <v>40</v>
+        <v>3000</v>
+      </c>
+      <c r="H53" t="s">
+        <v>5</v>
       </c>
       <c r="I53" t="b">
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="K53" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="B54" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="C54" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D54" t="s">
         <v>25</v>
@@ -3447,56 +3456,56 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="K54" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>98</v>
+        <v>185</v>
       </c>
       <c r="B55" t="s">
-        <v>108</v>
+        <v>212</v>
       </c>
       <c r="C55" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D55" t="s">
         <v>25</v>
       </c>
       <c r="E55">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F55">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="G55">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H55">
-        <v>0.1</v>
+        <v>40</v>
       </c>
       <c r="I55" t="b">
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K55" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="B56" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C56" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D56" t="s">
         <v>25</v>
@@ -3517,21 +3526,21 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="K56" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="B57" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C57" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D57" t="s">
         <v>25</v>
@@ -3540,33 +3549,33 @@
         <v>0</v>
       </c>
       <c r="F57">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="G57">
         <v>0</v>
       </c>
       <c r="H57">
-        <v>20</v>
+        <v>0.1</v>
       </c>
       <c r="I57" t="b">
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K57" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="B58" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C58" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D58" t="s">
         <v>25</v>
@@ -3587,21 +3596,21 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="K58" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="B59" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C59" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D59" t="s">
         <v>25</v>
@@ -3610,33 +3619,33 @@
         <v>0</v>
       </c>
       <c r="F59">
+        <v>30</v>
+      </c>
+      <c r="G59">
+        <v>0</v>
+      </c>
+      <c r="H59">
         <v>20</v>
       </c>
-      <c r="G59">
-        <v>0</v>
-      </c>
-      <c r="H59">
-        <v>10</v>
-      </c>
       <c r="I59" t="b">
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K59" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="B60" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C60" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D60" t="s">
         <v>25</v>
@@ -3657,21 +3666,21 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="K60" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="B61" t="s">
-        <v>213</v>
+        <v>108</v>
       </c>
       <c r="C61" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D61" t="s">
         <v>25</v>
@@ -3680,33 +3689,33 @@
         <v>0</v>
       </c>
       <c r="F61">
+        <v>20</v>
+      </c>
+      <c r="G61">
+        <v>0</v>
+      </c>
+      <c r="H61">
         <v>10</v>
       </c>
-      <c r="G61">
-        <v>0</v>
-      </c>
-      <c r="H61">
-        <v>5</v>
-      </c>
       <c r="I61" t="b">
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K61" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="B62" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C62" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D62" t="s">
         <v>25</v>
@@ -3727,208 +3736,208 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="K62" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>103</v>
+      </c>
+      <c r="B63" t="s">
+        <v>211</v>
+      </c>
+      <c r="C63" t="s">
+        <v>52</v>
+      </c>
+      <c r="D63" t="s">
+        <v>25</v>
+      </c>
+      <c r="E63">
+        <v>0</v>
+      </c>
+      <c r="F63">
+        <v>10</v>
+      </c>
+      <c r="G63">
+        <v>0</v>
+      </c>
+      <c r="H63">
+        <v>5</v>
+      </c>
+      <c r="I63" t="b">
+        <v>1</v>
+      </c>
+      <c r="J63" t="s">
+        <v>139</v>
+      </c>
+      <c r="K63" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>60</v>
+      </c>
+      <c r="B64" t="s">
+        <v>196</v>
+      </c>
+      <c r="C64" t="s">
+        <v>54</v>
+      </c>
+      <c r="D64" t="s">
+        <v>63</v>
+      </c>
+      <c r="E64">
+        <v>0</v>
+      </c>
+      <c r="F64">
+        <v>25</v>
+      </c>
+      <c r="G64">
+        <v>0</v>
+      </c>
+      <c r="H64">
+        <v>10</v>
+      </c>
+      <c r="I64" t="b">
+        <v>1</v>
+      </c>
+      <c r="J64" t="s">
+        <v>194</v>
+      </c>
+      <c r="K64" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>111</v>
+      </c>
+      <c r="B65" t="s">
+        <v>112</v>
+      </c>
+      <c r="C65" t="s">
+        <v>54</v>
+      </c>
+      <c r="D65" t="s">
+        <v>63</v>
+      </c>
+      <c r="E65">
+        <v>0</v>
+      </c>
+      <c r="F65">
+        <v>0.1</v>
+      </c>
+      <c r="G65">
+        <v>0</v>
+      </c>
+      <c r="H65">
+        <v>0.05</v>
+      </c>
+      <c r="I65" t="b">
+        <v>1</v>
+      </c>
+      <c r="J65" t="s">
+        <v>194</v>
+      </c>
+      <c r="K65" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A63" t="s">
-        <v>62</v>
-      </c>
-      <c r="B63" t="s">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>174</v>
+      </c>
+      <c r="B66" t="s">
+        <v>175</v>
+      </c>
+      <c r="C66" t="s">
+        <v>54</v>
+      </c>
+      <c r="D66" t="s">
+        <v>25</v>
+      </c>
+      <c r="E66">
+        <v>1</v>
+      </c>
+      <c r="F66">
+        <v>40</v>
+      </c>
+      <c r="G66">
+        <v>1</v>
+      </c>
+      <c r="H66">
+        <v>20</v>
+      </c>
+      <c r="I66" t="b">
+        <v>1</v>
+      </c>
+      <c r="J66" t="s">
+        <v>183</v>
+      </c>
+      <c r="K66" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>200</v>
+      </c>
+      <c r="B67" t="s">
+        <v>188</v>
+      </c>
+      <c r="C67" t="s">
+        <v>54</v>
+      </c>
+      <c r="D67" t="s">
+        <v>25</v>
+      </c>
+      <c r="E67">
+        <v>0</v>
+      </c>
+      <c r="F67">
+        <v>20</v>
+      </c>
+      <c r="G67">
+        <v>0</v>
+      </c>
+      <c r="H67">
+        <v>10</v>
+      </c>
+      <c r="I67" t="b">
+        <v>1</v>
+      </c>
+      <c r="J67" t="s">
         <v>198</v>
       </c>
-      <c r="C63" t="s">
-        <v>55</v>
-      </c>
-      <c r="D63" t="s">
-        <v>65</v>
-      </c>
-      <c r="E63">
-        <v>0</v>
-      </c>
-      <c r="F63">
-        <v>25</v>
-      </c>
-      <c r="G63">
-        <v>0</v>
-      </c>
-      <c r="H63">
-        <v>10</v>
-      </c>
-      <c r="I63" t="b">
-        <v>1</v>
-      </c>
-      <c r="J63" t="s">
-        <v>196</v>
-      </c>
-      <c r="K63" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A64" t="s">
-        <v>113</v>
-      </c>
-      <c r="B64" t="s">
-        <v>114</v>
-      </c>
-      <c r="C64" t="s">
-        <v>55</v>
-      </c>
-      <c r="D64" t="s">
-        <v>65</v>
-      </c>
-      <c r="E64">
-        <v>0</v>
-      </c>
-      <c r="F64">
-        <v>0.1</v>
-      </c>
-      <c r="G64">
-        <v>0</v>
-      </c>
-      <c r="H64">
-        <v>0.05</v>
-      </c>
-      <c r="I64" t="b">
-        <v>1</v>
-      </c>
-      <c r="J64" t="s">
-        <v>196</v>
-      </c>
-      <c r="K64" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A65" t="s">
+      <c r="K67" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>61</v>
+      </c>
+      <c r="B68" t="s">
         <v>176</v>
       </c>
-      <c r="B65" t="s">
-        <v>177</v>
-      </c>
-      <c r="C65" t="s">
-        <v>55</v>
-      </c>
-      <c r="D65" t="s">
-        <v>25</v>
-      </c>
-      <c r="E65">
-        <v>1</v>
-      </c>
-      <c r="F65">
-        <v>40</v>
-      </c>
-      <c r="G65">
-        <v>1</v>
-      </c>
-      <c r="H65">
-        <v>20</v>
-      </c>
-      <c r="I65" t="b">
-        <v>1</v>
-      </c>
-      <c r="J65" t="s">
-        <v>185</v>
-      </c>
-      <c r="K65" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
-        <v>202</v>
-      </c>
-      <c r="B66" t="s">
-        <v>190</v>
-      </c>
-      <c r="C66" t="s">
-        <v>55</v>
-      </c>
-      <c r="D66" t="s">
-        <v>25</v>
-      </c>
-      <c r="E66">
-        <v>0</v>
-      </c>
-      <c r="F66">
-        <v>20</v>
-      </c>
-      <c r="G66">
-        <v>0</v>
-      </c>
-      <c r="H66">
-        <v>10</v>
-      </c>
-      <c r="I66" t="b">
-        <v>1</v>
-      </c>
-      <c r="J66" t="s">
-        <v>200</v>
-      </c>
-      <c r="K66" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A67" t="s">
-        <v>63</v>
-      </c>
-      <c r="B67" t="s">
-        <v>178</v>
-      </c>
-      <c r="C67" t="s">
-        <v>55</v>
-      </c>
-      <c r="D67" t="s">
-        <v>25</v>
-      </c>
-      <c r="E67">
+      <c r="C68" t="s">
+        <v>54</v>
+      </c>
+      <c r="D68" t="s">
+        <v>25</v>
+      </c>
+      <c r="E68">
         <v>80</v>
-      </c>
-      <c r="F67">
-        <v>99</v>
-      </c>
-      <c r="G67">
-        <v>90</v>
-      </c>
-      <c r="H67">
-        <v>99</v>
-      </c>
-      <c r="I67" t="b">
-        <v>1</v>
-      </c>
-      <c r="J67" t="s">
-        <v>181</v>
-      </c>
-      <c r="K67" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A68" t="s">
-        <v>64</v>
-      </c>
-      <c r="B68" t="s">
-        <v>179</v>
-      </c>
-      <c r="C68" t="s">
-        <v>55</v>
-      </c>
-      <c r="D68" t="s">
-        <v>25</v>
-      </c>
-      <c r="E68">
-        <v>85</v>
       </c>
       <c r="F68">
         <v>99</v>
       </c>
       <c r="G68">
-        <v>92.5</v>
+        <v>90</v>
       </c>
       <c r="H68">
         <v>99</v>
@@ -3937,68 +3946,68 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="K68" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>62</v>
+      </c>
+      <c r="B69" t="s">
+        <v>177</v>
+      </c>
+      <c r="C69" t="s">
+        <v>54</v>
+      </c>
+      <c r="D69" t="s">
+        <v>25</v>
+      </c>
+      <c r="E69">
+        <v>85</v>
+      </c>
+      <c r="F69">
+        <v>99</v>
+      </c>
+      <c r="G69">
+        <v>92.5</v>
+      </c>
+      <c r="H69">
+        <v>99</v>
+      </c>
+      <c r="I69" t="b">
+        <v>1</v>
+      </c>
+      <c r="J69" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A69" t="s">
-        <v>67</v>
-      </c>
-      <c r="B69" t="s">
-        <v>80</v>
-      </c>
-      <c r="C69" t="s">
-        <v>52</v>
-      </c>
-      <c r="D69" t="s">
-        <v>25</v>
-      </c>
-      <c r="E69">
+      <c r="K69" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>65</v>
+      </c>
+      <c r="B70" t="s">
+        <v>78</v>
+      </c>
+      <c r="C70" t="s">
+        <v>51</v>
+      </c>
+      <c r="D70" t="s">
+        <v>25</v>
+      </c>
+      <c r="E70">
         <v>90</v>
-      </c>
-      <c r="F69">
-        <v>100</v>
-      </c>
-      <c r="G69">
-        <v>95</v>
-      </c>
-      <c r="H69">
-        <v>100</v>
-      </c>
-      <c r="I69" t="b">
-        <v>1</v>
-      </c>
-      <c r="J69" t="s">
-        <v>129</v>
-      </c>
-      <c r="K69" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A70" t="s">
-        <v>66</v>
-      </c>
-      <c r="B70" t="s">
-        <v>81</v>
-      </c>
-      <c r="C70" t="s">
-        <v>52</v>
-      </c>
-      <c r="D70" t="s">
-        <v>25</v>
-      </c>
-      <c r="E70">
-        <v>50</v>
       </c>
       <c r="F70">
         <v>100</v>
       </c>
       <c r="G70">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="H70">
         <v>100</v>
@@ -4007,138 +4016,138 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K70" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="B71" t="s">
-        <v>115</v>
+        <v>79</v>
       </c>
       <c r="C71" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D71" t="s">
         <v>25</v>
       </c>
       <c r="E71">
+        <v>50</v>
+      </c>
+      <c r="F71">
+        <v>100</v>
+      </c>
+      <c r="G71">
+        <v>75</v>
+      </c>
+      <c r="H71">
+        <v>100</v>
+      </c>
+      <c r="I71" t="b">
+        <v>1</v>
+      </c>
+      <c r="J71" t="s">
+        <v>127</v>
+      </c>
+      <c r="K71" t="s">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>66</v>
+      </c>
+      <c r="B72" t="s">
+        <v>113</v>
+      </c>
+      <c r="C72" t="s">
+        <v>51</v>
+      </c>
+      <c r="D72" t="s">
+        <v>25</v>
+      </c>
+      <c r="E72">
         <v>125</v>
       </c>
-      <c r="F71">
+      <c r="F72">
         <v>175</v>
       </c>
-      <c r="G71">
+      <c r="G72">
         <v>140</v>
       </c>
-      <c r="H71">
+      <c r="H72">
         <v>160</v>
       </c>
-      <c r="I71" t="b">
-        <v>1</v>
-      </c>
-      <c r="J71" t="s">
-        <v>130</v>
-      </c>
-      <c r="K71" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A72" t="s">
-        <v>126</v>
-      </c>
-      <c r="B72" t="s">
-        <v>192</v>
-      </c>
-      <c r="C72" t="s">
-        <v>58</v>
-      </c>
-      <c r="D72" t="s">
-        <v>25</v>
-      </c>
-      <c r="E72">
+      <c r="I72" t="b">
+        <v>1</v>
+      </c>
+      <c r="J72" t="s">
+        <v>128</v>
+      </c>
+      <c r="K72" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>124</v>
+      </c>
+      <c r="B73" t="s">
+        <v>190</v>
+      </c>
+      <c r="C73" t="s">
+        <v>57</v>
+      </c>
+      <c r="D73" t="s">
+        <v>25</v>
+      </c>
+      <c r="E73">
         <v>50</v>
       </c>
-      <c r="F72">
+      <c r="F73">
         <v>70</v>
       </c>
-      <c r="G72">
+      <c r="G73">
         <v>50</v>
       </c>
-      <c r="H72">
+      <c r="H73">
         <v>60</v>
       </c>
-      <c r="I72" t="b">
-        <v>1</v>
-      </c>
-      <c r="J72" t="s">
-        <v>154</v>
-      </c>
-      <c r="K72" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A73" t="s">
-        <v>116</v>
-      </c>
-      <c r="B73" t="s">
-        <v>170</v>
-      </c>
-      <c r="C73" t="s">
-        <v>58</v>
-      </c>
-      <c r="D73" t="s">
-        <v>25</v>
-      </c>
-      <c r="E73">
+      <c r="I73" t="b">
+        <v>1</v>
+      </c>
+      <c r="J73" t="s">
+        <v>152</v>
+      </c>
+      <c r="K73" t="s">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>114</v>
+      </c>
+      <c r="B74" t="s">
+        <v>168</v>
+      </c>
+      <c r="C74" t="s">
+        <v>57</v>
+      </c>
+      <c r="D74" t="s">
+        <v>25</v>
+      </c>
+      <c r="E74">
         <v>60</v>
-      </c>
-      <c r="F73">
-        <v>100</v>
-      </c>
-      <c r="G73">
-        <v>90</v>
-      </c>
-      <c r="H73">
-        <v>100</v>
-      </c>
-      <c r="I73" t="b">
-        <v>1</v>
-      </c>
-      <c r="J73" t="s">
-        <v>168</v>
-      </c>
-      <c r="K73" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A74" t="s">
-        <v>122</v>
-      </c>
-      <c r="B74" t="s">
-        <v>10</v>
-      </c>
-      <c r="C74" t="s">
-        <v>58</v>
-      </c>
-      <c r="D74" t="s">
-        <v>25</v>
-      </c>
-      <c r="E74">
-        <v>99</v>
       </c>
       <c r="F74">
         <v>100</v>
       </c>
       <c r="G74">
-        <v>99.5</v>
+        <v>90</v>
       </c>
       <c r="H74">
         <v>100</v>
@@ -4147,329 +4156,364 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
+        <v>166</v>
+      </c>
+      <c r="K74" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>120</v>
+      </c>
+      <c r="B75" t="s">
+        <v>10</v>
+      </c>
+      <c r="C75" t="s">
+        <v>57</v>
+      </c>
+      <c r="D75" t="s">
+        <v>25</v>
+      </c>
+      <c r="E75">
+        <v>99</v>
+      </c>
+      <c r="F75">
+        <v>100</v>
+      </c>
+      <c r="G75">
+        <v>99.5</v>
+      </c>
+      <c r="H75">
+        <v>100</v>
+      </c>
+      <c r="I75" t="b">
+        <v>1</v>
+      </c>
+      <c r="J75" t="s">
+        <v>156</v>
+      </c>
+      <c r="K75" t="s">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>119</v>
+      </c>
+      <c r="B76" t="s">
+        <v>118</v>
+      </c>
+      <c r="C76" t="s">
+        <v>57</v>
+      </c>
+      <c r="D76" t="s">
+        <v>25</v>
+      </c>
+      <c r="E76">
+        <v>0</v>
+      </c>
+      <c r="F76">
+        <v>15</v>
+      </c>
+      <c r="G76">
+        <v>0</v>
+      </c>
+      <c r="H76">
+        <v>5</v>
+      </c>
+      <c r="I76" t="b">
+        <v>1</v>
+      </c>
+      <c r="J76" t="s">
+        <v>156</v>
+      </c>
+      <c r="K76" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>121</v>
+      </c>
+      <c r="B77" t="s">
+        <v>122</v>
+      </c>
+      <c r="C77" t="s">
+        <v>57</v>
+      </c>
+      <c r="D77" t="s">
+        <v>25</v>
+      </c>
+      <c r="E77">
+        <v>0.5</v>
+      </c>
+      <c r="F77" t="s">
+        <v>5</v>
+      </c>
+      <c r="G77">
+        <v>1</v>
+      </c>
+      <c r="H77" t="s">
+        <v>5</v>
+      </c>
+      <c r="I77" t="b">
+        <v>1</v>
+      </c>
+      <c r="J77" t="s">
+        <v>167</v>
+      </c>
+      <c r="K77" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>14</v>
+      </c>
+      <c r="B78" t="s">
+        <v>15</v>
+      </c>
+      <c r="C78" t="s">
+        <v>57</v>
+      </c>
+      <c r="D78" t="s">
+        <v>25</v>
+      </c>
+      <c r="E78">
+        <v>0</v>
+      </c>
+      <c r="F78">
+        <v>0</v>
+      </c>
+      <c r="G78">
+        <v>0</v>
+      </c>
+      <c r="H78">
+        <v>0</v>
+      </c>
+      <c r="I78" t="b">
+        <v>1</v>
+      </c>
+      <c r="J78" t="s">
+        <v>129</v>
+      </c>
+      <c r="K78" t="s">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>12</v>
+      </c>
+      <c r="B79" t="s">
+        <v>13</v>
+      </c>
+      <c r="C79" t="s">
+        <v>57</v>
+      </c>
+      <c r="D79" t="s">
+        <v>25</v>
+      </c>
+      <c r="E79">
+        <v>14.5</v>
+      </c>
+      <c r="F79">
+        <v>100</v>
+      </c>
+      <c r="G79">
+        <v>26.1</v>
+      </c>
+      <c r="H79">
+        <v>100</v>
+      </c>
+      <c r="I79" t="b">
+        <v>1</v>
+      </c>
+      <c r="J79" t="s">
+        <v>167</v>
+      </c>
+      <c r="K79" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>8</v>
+      </c>
+      <c r="B80" t="s">
+        <v>9</v>
+      </c>
+      <c r="C80" t="s">
+        <v>57</v>
+      </c>
+      <c r="D80" t="s">
+        <v>25</v>
+      </c>
+      <c r="E80">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="F80">
+        <v>8.0000000000000004E-4</v>
+      </c>
+      <c r="G80">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="H80">
+        <v>5.0000000000000001E-4</v>
+      </c>
+      <c r="I80" t="b">
+        <v>1</v>
+      </c>
+      <c r="J80" t="s">
+        <v>182</v>
+      </c>
+      <c r="K80" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>201</v>
+      </c>
+      <c r="B81" t="s">
+        <v>202</v>
+      </c>
+      <c r="C81" t="s">
+        <v>173</v>
+      </c>
+      <c r="D81" t="s">
+        <v>25</v>
+      </c>
+      <c r="E81">
+        <v>0.05</v>
+      </c>
+      <c r="F81">
+        <v>0.08</v>
+      </c>
+      <c r="G81">
+        <v>0.02</v>
+      </c>
+      <c r="H81">
+        <v>0.05</v>
+      </c>
+      <c r="I81" t="b">
+        <v>1</v>
+      </c>
+      <c r="J81" t="s">
+        <v>204</v>
+      </c>
+      <c r="K81" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>11</v>
+      </c>
+      <c r="B82" t="s">
+        <v>203</v>
+      </c>
+      <c r="C82" t="s">
+        <v>173</v>
+      </c>
+      <c r="D82" t="s">
+        <v>25</v>
+      </c>
+      <c r="E82">
+        <v>5</v>
+      </c>
+      <c r="F82">
+        <v>100</v>
+      </c>
+      <c r="G82">
+        <v>20</v>
+      </c>
+      <c r="H82">
+        <v>100</v>
+      </c>
+      <c r="I82" t="b">
+        <v>1</v>
+      </c>
+      <c r="J82" t="s">
+        <v>167</v>
+      </c>
+      <c r="K82" t="s">
         <v>158</v>
       </c>
-      <c r="K74" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A75" t="s">
-        <v>121</v>
-      </c>
-      <c r="B75" t="s">
-        <v>120</v>
-      </c>
-      <c r="C75" t="s">
-        <v>58</v>
-      </c>
-      <c r="D75" t="s">
-        <v>25</v>
-      </c>
-      <c r="E75">
-        <v>0</v>
-      </c>
-      <c r="F75">
-        <v>15</v>
-      </c>
-      <c r="G75">
-        <v>0</v>
-      </c>
-      <c r="H75">
-        <v>5</v>
-      </c>
-      <c r="I75" t="b">
-        <v>1</v>
-      </c>
-      <c r="J75" t="s">
-        <v>158</v>
-      </c>
-      <c r="K75" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A76" t="s">
-        <v>123</v>
-      </c>
-      <c r="B76" t="s">
-        <v>124</v>
-      </c>
-      <c r="C76" t="s">
-        <v>58</v>
-      </c>
-      <c r="D76" t="s">
-        <v>25</v>
-      </c>
-      <c r="E76">
-        <v>0.5</v>
-      </c>
-      <c r="F76" t="s">
-        <v>5</v>
-      </c>
-      <c r="G76">
-        <v>1</v>
-      </c>
-      <c r="H76" t="s">
-        <v>5</v>
-      </c>
-      <c r="I76" t="b">
-        <v>1</v>
-      </c>
-      <c r="J76" t="s">
-        <v>169</v>
-      </c>
-      <c r="K76" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A77" t="s">
-        <v>14</v>
-      </c>
-      <c r="B77" t="s">
-        <v>15</v>
-      </c>
-      <c r="C77" t="s">
-        <v>58</v>
-      </c>
-      <c r="D77" t="s">
-        <v>25</v>
-      </c>
-      <c r="E77">
-        <v>0</v>
-      </c>
-      <c r="F77">
-        <v>0</v>
-      </c>
-      <c r="G77">
-        <v>0</v>
-      </c>
-      <c r="H77">
-        <v>0</v>
-      </c>
-      <c r="I77" t="b">
-        <v>1</v>
-      </c>
-      <c r="J77" t="s">
-        <v>131</v>
-      </c>
-      <c r="K77" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A78" t="s">
-        <v>12</v>
-      </c>
-      <c r="B78" t="s">
-        <v>13</v>
-      </c>
-      <c r="C78" t="s">
-        <v>58</v>
-      </c>
-      <c r="D78" t="s">
-        <v>25</v>
-      </c>
-      <c r="E78">
-        <v>14.5</v>
-      </c>
-      <c r="F78">
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>17</v>
+      </c>
+      <c r="B83" t="s">
+        <v>16</v>
+      </c>
+      <c r="C83" t="s">
+        <v>173</v>
+      </c>
+      <c r="D83" t="s">
+        <v>25</v>
+      </c>
+      <c r="E83">
+        <v>0</v>
+      </c>
+      <c r="F83">
+        <v>95</v>
+      </c>
+      <c r="G83">
+        <v>0</v>
+      </c>
+      <c r="H83">
+        <v>80</v>
+      </c>
+      <c r="I83" t="b">
+        <v>1</v>
+      </c>
+      <c r="J83" t="s">
+        <v>140</v>
+      </c>
+      <c r="K83" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>47</v>
+      </c>
+      <c r="B84" t="s">
+        <v>189</v>
+      </c>
+      <c r="C84" t="s">
+        <v>173</v>
+      </c>
+      <c r="D84" t="s">
+        <v>25</v>
+      </c>
+      <c r="E84">
+        <v>33</v>
+      </c>
+      <c r="F84">
         <v>100</v>
       </c>
-      <c r="G78">
-        <v>26.1</v>
-      </c>
-      <c r="H78">
+      <c r="G84">
+        <v>67</v>
+      </c>
+      <c r="H84">
         <v>100</v>
       </c>
-      <c r="I78" t="b">
-        <v>1</v>
-      </c>
-      <c r="J78" t="s">
-        <v>169</v>
-      </c>
-      <c r="K78" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A79" t="s">
-        <v>8</v>
-      </c>
-      <c r="B79" t="s">
-        <v>9</v>
-      </c>
-      <c r="C79" t="s">
-        <v>58</v>
-      </c>
-      <c r="D79" t="s">
-        <v>25</v>
-      </c>
-      <c r="E79">
-        <v>5.0000000000000001E-4</v>
-      </c>
-      <c r="F79">
-        <v>8.0000000000000004E-4</v>
-      </c>
-      <c r="G79">
-        <v>2.0000000000000001E-4</v>
-      </c>
-      <c r="H79">
-        <v>5.0000000000000001E-4</v>
-      </c>
-      <c r="I79" t="b">
-        <v>1</v>
-      </c>
-      <c r="J79" t="s">
-        <v>184</v>
-      </c>
-      <c r="K79" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A80" t="s">
-        <v>203</v>
-      </c>
-      <c r="B80" t="s">
-        <v>204</v>
-      </c>
-      <c r="C80" t="s">
-        <v>175</v>
-      </c>
-      <c r="D80" t="s">
-        <v>25</v>
-      </c>
-      <c r="E80">
-        <v>0.05</v>
-      </c>
-      <c r="F80">
-        <v>0.08</v>
-      </c>
-      <c r="G80">
-        <v>0.02</v>
-      </c>
-      <c r="H80">
-        <v>0.05</v>
-      </c>
-      <c r="I80" t="b">
-        <v>1</v>
-      </c>
-      <c r="J80" t="s">
-        <v>206</v>
-      </c>
-      <c r="K80" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A81" t="s">
-        <v>11</v>
-      </c>
-      <c r="B81" t="s">
-        <v>205</v>
-      </c>
-      <c r="C81" t="s">
-        <v>175</v>
-      </c>
-      <c r="D81" t="s">
-        <v>25</v>
-      </c>
-      <c r="E81">
-        <v>5</v>
-      </c>
-      <c r="F81">
-        <v>100</v>
-      </c>
-      <c r="G81">
-        <v>20</v>
-      </c>
-      <c r="H81">
-        <v>100</v>
-      </c>
-      <c r="I81" t="b">
-        <v>1</v>
-      </c>
-      <c r="J81" t="s">
-        <v>169</v>
-      </c>
-      <c r="K81" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A82" t="s">
-        <v>17</v>
-      </c>
-      <c r="B82" t="s">
-        <v>16</v>
-      </c>
-      <c r="C82" t="s">
-        <v>175</v>
-      </c>
-      <c r="D82" t="s">
-        <v>25</v>
-      </c>
-      <c r="E82">
-        <v>0</v>
-      </c>
-      <c r="F82">
-        <v>95</v>
-      </c>
-      <c r="G82">
-        <v>0</v>
-      </c>
-      <c r="H82">
-        <v>80</v>
-      </c>
-      <c r="I82" t="b">
-        <v>1</v>
-      </c>
-      <c r="J82" t="s">
-        <v>142</v>
-      </c>
-      <c r="K82" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A83" t="s">
+      <c r="I84" t="b">
+        <v>1</v>
+      </c>
+      <c r="J84" t="s">
+        <v>167</v>
+      </c>
+      <c r="K84" t="s">
         <v>47</v>
       </c>
-      <c r="B83" t="s">
-        <v>191</v>
-      </c>
-      <c r="C83" t="s">
-        <v>175</v>
-      </c>
-      <c r="D83" t="s">
-        <v>25</v>
-      </c>
-      <c r="E83">
-        <v>33</v>
-      </c>
-      <c r="F83">
-        <v>100</v>
-      </c>
-      <c r="G83">
-        <v>67</v>
-      </c>
-      <c r="H83">
-        <v>100</v>
-      </c>
-      <c r="I83" t="b">
-        <v>1</v>
-      </c>
-      <c r="J83" t="s">
-        <v>169</v>
-      </c>
-      <c r="K83" t="s">
-        <v>47</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K81" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K82" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Added metadata spreadsheet for technical controls (e.g. NTCs)
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD19655F-4079-4AEF-9964-53AB0454C2E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96E506E6-AA54-4ED1-8D96-2C936D9B1D6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -1590,19 +1590,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
   <dimension ref="A1:K84"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="35.140625" customWidth="1"/>
-    <col min="2" max="2" width="123.140625" customWidth="1"/>
-    <col min="3" max="4" width="35.28515625" customWidth="1"/>
+    <col min="1" max="1" width="35.1796875" customWidth="1"/>
+    <col min="2" max="2" width="123.1796875" customWidth="1"/>
+    <col min="3" max="4" width="35.26953125" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" customWidth="1"/>
-    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="76.85546875" customWidth="1"/>
+    <col min="9" max="9" width="12.81640625" customWidth="1"/>
+    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="76.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>32</v>
       </c>
@@ -1637,7 +1637,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>35</v>
       </c>
@@ -1701,7 +1701,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -1736,7 +1736,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>44</v>
       </c>
@@ -1765,7 +1765,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>45</v>
       </c>
@@ -1829,7 +1829,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>46</v>
       </c>
@@ -1864,7 +1864,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1899,7 +1899,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -1934,7 +1934,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -1969,7 +1969,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -2004,7 +2004,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>91</v>
       </c>
@@ -2039,7 +2039,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>92</v>
       </c>
@@ -2074,7 +2074,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>89</v>
       </c>
@@ -2109,7 +2109,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>90</v>
       </c>
@@ -2144,7 +2144,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>81</v>
       </c>
@@ -2179,7 +2179,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>82</v>
       </c>
@@ -2214,7 +2214,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>186</v>
       </c>
@@ -2249,7 +2249,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>187</v>
       </c>
@@ -2284,7 +2284,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>69</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>70</v>
       </c>
@@ -2354,7 +2354,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>71</v>
       </c>
@@ -2389,7 +2389,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>72</v>
       </c>
@@ -2424,7 +2424,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>73</v>
       </c>
@@ -2459,7 +2459,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>74</v>
       </c>
@@ -2494,7 +2494,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>75</v>
       </c>
@@ -2529,7 +2529,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>76</v>
       </c>
@@ -2564,7 +2564,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>77</v>
       </c>
@@ -2599,7 +2599,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>220</v>
       </c>
@@ -2634,7 +2634,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>117</v>
       </c>
@@ -2669,7 +2669,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>116</v>
       </c>
@@ -2704,7 +2704,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>213</v>
       </c>
@@ -2739,7 +2739,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>115</v>
       </c>
@@ -2774,7 +2774,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>226</v>
       </c>
@@ -2809,7 +2809,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>59</v>
       </c>
@@ -2844,7 +2844,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>20</v>
       </c>
@@ -2873,7 +2873,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>27</v>
       </c>
@@ -2908,7 +2908,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>33</v>
       </c>
@@ -2943,7 +2943,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>41</v>
       </c>
@@ -2972,7 +2972,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>37</v>
       </c>
@@ -3007,7 +3007,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>38</v>
       </c>
@@ -3042,7 +3042,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>39</v>
       </c>
@@ -3077,7 +3077,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>21</v>
       </c>
@@ -3112,7 +3112,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>22</v>
       </c>
@@ -3147,7 +3147,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>85</v>
       </c>
@@ -3182,7 +3182,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>86</v>
       </c>
@@ -3217,7 +3217,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>87</v>
       </c>
@@ -3252,7 +3252,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>88</v>
       </c>
@@ -3287,7 +3287,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>84</v>
       </c>
@@ -3322,7 +3322,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>93</v>
       </c>
@@ -3357,7 +3357,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>94</v>
       </c>
@@ -3392,7 +3392,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>95</v>
       </c>
@@ -3427,7 +3427,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>184</v>
       </c>
@@ -3462,7 +3462,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>185</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>96</v>
       </c>
@@ -3532,7 +3532,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>97</v>
       </c>
@@ -3567,7 +3567,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>98</v>
       </c>
@@ -3602,7 +3602,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>99</v>
       </c>
@@ -3637,7 +3637,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>100</v>
       </c>
@@ -3672,7 +3672,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>101</v>
       </c>
@@ -3707,7 +3707,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>102</v>
       </c>
@@ -3742,7 +3742,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>103</v>
       </c>
@@ -3777,7 +3777,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>60</v>
       </c>
@@ -3803,7 +3803,7 @@
         <v>10</v>
       </c>
       <c r="I64" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J64" t="s">
         <v>194</v>
@@ -3812,7 +3812,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>111</v>
       </c>
@@ -3838,7 +3838,7 @@
         <v>0.05</v>
       </c>
       <c r="I65" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J65" t="s">
         <v>194</v>
@@ -3847,7 +3847,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>174</v>
       </c>
@@ -3882,7 +3882,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>200</v>
       </c>
@@ -3917,7 +3917,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>61</v>
       </c>
@@ -3952,7 +3952,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>62</v>
       </c>
@@ -3987,7 +3987,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>65</v>
       </c>
@@ -4022,7 +4022,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>64</v>
       </c>
@@ -4057,7 +4057,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>66</v>
       </c>
@@ -4092,7 +4092,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>124</v>
       </c>
@@ -4127,7 +4127,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>114</v>
       </c>
@@ -4162,7 +4162,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>120</v>
       </c>
@@ -4197,7 +4197,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>119</v>
       </c>
@@ -4232,7 +4232,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>121</v>
       </c>
@@ -4267,7 +4267,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>14</v>
       </c>
@@ -4302,7 +4302,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>12</v>
       </c>
@@ -4337,7 +4337,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>8</v>
       </c>
@@ -4372,7 +4372,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>201</v>
       </c>
@@ -4407,7 +4407,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>11</v>
       </c>
@@ -4442,7 +4442,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>17</v>
       </c>
@@ -4477,7 +4477,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A84" t="s">
         <v>47</v>
       </c>

</xml_diff>

<commit_message>
Fixed regex in ex_demux_counts_and_gini script
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96E506E6-AA54-4ED1-8D96-2C936D9B1D6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCB1DA4E-F356-4F76-84A7-C3306573E291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -1590,19 +1590,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
   <dimension ref="A1:K84"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.1796875" customWidth="1"/>
-    <col min="2" max="2" width="123.1796875" customWidth="1"/>
-    <col min="3" max="4" width="35.26953125" customWidth="1"/>
+    <col min="1" max="1" width="35.140625" customWidth="1"/>
+    <col min="2" max="2" width="123.140625" customWidth="1"/>
+    <col min="3" max="4" width="35.28515625" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.81640625" customWidth="1"/>
-    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="76.81640625" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="76.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>32</v>
       </c>
@@ -1637,7 +1637,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -1666,7 +1666,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>35</v>
       </c>
@@ -1701,7 +1701,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -1736,7 +1736,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>44</v>
       </c>
@@ -1765,7 +1765,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -1800,7 +1800,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>45</v>
       </c>
@@ -1829,7 +1829,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>46</v>
       </c>
@@ -1864,7 +1864,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1899,7 +1899,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -1934,7 +1934,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -1969,7 +1969,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -2004,7 +2004,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>91</v>
       </c>
@@ -2039,7 +2039,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>92</v>
       </c>
@@ -2074,7 +2074,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>89</v>
       </c>
@@ -2109,7 +2109,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>90</v>
       </c>
@@ -2144,7 +2144,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>81</v>
       </c>
@@ -2179,7 +2179,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>82</v>
       </c>
@@ -2214,7 +2214,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>186</v>
       </c>
@@ -2249,7 +2249,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>187</v>
       </c>
@@ -2284,7 +2284,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>69</v>
       </c>
@@ -2319,7 +2319,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>70</v>
       </c>
@@ -2354,7 +2354,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>71</v>
       </c>
@@ -2389,7 +2389,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>72</v>
       </c>
@@ -2424,7 +2424,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>73</v>
       </c>
@@ -2459,7 +2459,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>74</v>
       </c>
@@ -2494,7 +2494,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>75</v>
       </c>
@@ -2529,7 +2529,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>76</v>
       </c>
@@ -2564,7 +2564,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>77</v>
       </c>
@@ -2599,7 +2599,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>220</v>
       </c>
@@ -2634,7 +2634,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>117</v>
       </c>
@@ -2669,7 +2669,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>116</v>
       </c>
@@ -2704,7 +2704,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>213</v>
       </c>
@@ -2739,7 +2739,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>115</v>
       </c>
@@ -2774,7 +2774,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>226</v>
       </c>
@@ -2809,7 +2809,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>59</v>
       </c>
@@ -2844,7 +2844,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>20</v>
       </c>
@@ -2873,7 +2873,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>27</v>
       </c>
@@ -2908,7 +2908,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>33</v>
       </c>
@@ -2943,7 +2943,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>41</v>
       </c>
@@ -2972,7 +2972,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>37</v>
       </c>
@@ -3007,7 +3007,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>38</v>
       </c>
@@ -3042,7 +3042,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>39</v>
       </c>
@@ -3077,7 +3077,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>21</v>
       </c>
@@ -3112,7 +3112,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>22</v>
       </c>
@@ -3147,7 +3147,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>85</v>
       </c>
@@ -3182,7 +3182,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>86</v>
       </c>
@@ -3217,7 +3217,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>87</v>
       </c>
@@ -3252,7 +3252,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>88</v>
       </c>
@@ -3287,7 +3287,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>84</v>
       </c>
@@ -3322,7 +3322,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>93</v>
       </c>
@@ -3357,7 +3357,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>94</v>
       </c>
@@ -3392,7 +3392,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>95</v>
       </c>
@@ -3427,7 +3427,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>184</v>
       </c>
@@ -3462,7 +3462,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>185</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>96</v>
       </c>
@@ -3532,7 +3532,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>97</v>
       </c>
@@ -3567,7 +3567,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>98</v>
       </c>
@@ -3602,7 +3602,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>99</v>
       </c>
@@ -3637,7 +3637,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>100</v>
       </c>
@@ -3672,7 +3672,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>101</v>
       </c>
@@ -3707,7 +3707,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>102</v>
       </c>
@@ -3742,7 +3742,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>103</v>
       </c>
@@ -3777,7 +3777,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>60</v>
       </c>
@@ -3803,7 +3803,7 @@
         <v>10</v>
       </c>
       <c r="I64" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J64" t="s">
         <v>194</v>
@@ -3812,7 +3812,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>111</v>
       </c>
@@ -3838,7 +3838,7 @@
         <v>0.05</v>
       </c>
       <c r="I65" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J65" t="s">
         <v>194</v>
@@ -3847,7 +3847,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>174</v>
       </c>
@@ -3882,7 +3882,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>200</v>
       </c>
@@ -3917,7 +3917,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>61</v>
       </c>
@@ -3952,7 +3952,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>62</v>
       </c>
@@ -3987,7 +3987,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>65</v>
       </c>
@@ -4022,7 +4022,7 @@
         <v>159</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>64</v>
       </c>
@@ -4057,7 +4057,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>66</v>
       </c>
@@ -4092,7 +4092,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>124</v>
       </c>
@@ -4127,7 +4127,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>114</v>
       </c>
@@ -4162,7 +4162,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>120</v>
       </c>
@@ -4197,7 +4197,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>119</v>
       </c>
@@ -4232,7 +4232,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>121</v>
       </c>
@@ -4267,7 +4267,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>14</v>
       </c>
@@ -4302,7 +4302,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>12</v>
       </c>
@@ -4337,7 +4337,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>8</v>
       </c>
@@ -4372,7 +4372,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>201</v>
       </c>
@@ -4407,7 +4407,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>11</v>
       </c>
@@ -4442,7 +4442,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>17</v>
       </c>
@@ -4477,7 +4477,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>47</v>
       </c>

</xml_diff>

<commit_message>
Added reads for test technical controls to test lane fastqs
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCB1DA4E-F356-4F76-84A7-C3306573E291}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE159B88-AA7C-42AB-8D7C-31F0BFE08D8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="960" yWindow="4830" windowWidth="17280" windowHeight="10005" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -374,9 +374,6 @@
     <t>ex_lane_demux_read_gini</t>
   </si>
   <si>
-    <t>Gini coefficient of demultiplexed sample read count</t>
-  </si>
-  <si>
     <t>Median insert size (start of R1 to end of R2) as determined by initial alignment (bp)</t>
   </si>
   <si>
@@ -720,6 +717,9 @@
   </si>
   <si>
     <t>Proportion of genomic positions masked due to risk of being a germline variant</t>
+  </si>
+  <si>
+    <t>Gini coefficient for inequality between ex_samples</t>
   </si>
 </sst>
 </file>
@@ -1631,10 +1631,10 @@
         <v>31</v>
       </c>
       <c r="J1" t="s">
+        <v>124</v>
+      </c>
+      <c r="K1" t="s">
         <v>125</v>
-      </c>
-      <c r="K1" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -1642,7 +1642,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C2" t="s">
         <v>48</v>
@@ -1671,7 +1671,7 @@
         <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C3" t="s">
         <v>48</v>
@@ -1706,7 +1706,7 @@
         <v>36</v>
       </c>
       <c r="B4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C4" t="s">
         <v>48</v>
@@ -1741,7 +1741,7 @@
         <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C5" t="s">
         <v>50</v>
@@ -1770,7 +1770,7 @@
         <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C6" t="s">
         <v>50</v>
@@ -1805,7 +1805,7 @@
         <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="C7" t="s">
         <v>50</v>
@@ -1834,7 +1834,7 @@
         <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C8" t="s">
         <v>50</v>
@@ -1963,10 +1963,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K11" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1998,10 +1998,10 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="K12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -2009,7 +2009,7 @@
         <v>91</v>
       </c>
       <c r="B13" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C13" t="s">
         <v>53</v>
@@ -2033,10 +2033,10 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K13" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -2044,7 +2044,7 @@
         <v>92</v>
       </c>
       <c r="B14" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C14" t="s">
         <v>53</v>
@@ -2068,10 +2068,10 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="K14" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -2079,7 +2079,7 @@
         <v>89</v>
       </c>
       <c r="B15" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C15" t="s">
         <v>53</v>
@@ -2103,10 +2103,10 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K15" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
@@ -2114,7 +2114,7 @@
         <v>90</v>
       </c>
       <c r="B16" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C16" t="s">
         <v>53</v>
@@ -2138,10 +2138,10 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="K16" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -2173,10 +2173,10 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -2208,18 +2208,18 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="K18" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B19" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C19" t="s">
         <v>53</v>
@@ -2243,18 +2243,18 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K19" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B20" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C20" t="s">
         <v>53</v>
@@ -2278,10 +2278,10 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K20" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
@@ -2313,10 +2313,10 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K21" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
@@ -2348,10 +2348,10 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K22" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
@@ -2383,10 +2383,10 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K23" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
@@ -2418,10 +2418,10 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K24" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
@@ -2453,10 +2453,10 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K25" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
@@ -2488,10 +2488,10 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K26" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
@@ -2499,7 +2499,7 @@
         <v>75</v>
       </c>
       <c r="B27" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C27" t="s">
         <v>53</v>
@@ -2523,10 +2523,10 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K27" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
@@ -2534,7 +2534,7 @@
         <v>76</v>
       </c>
       <c r="B28" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C28" t="s">
         <v>53</v>
@@ -2558,10 +2558,10 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="K28" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
@@ -2569,7 +2569,7 @@
         <v>77</v>
       </c>
       <c r="B29" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C29" t="s">
         <v>55</v>
@@ -2593,18 +2593,18 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="K29" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B30" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C30" t="s">
         <v>55</v>
@@ -2628,15 +2628,15 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="K30" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B31" t="s">
         <v>110</v>
@@ -2663,18 +2663,18 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="K31" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B32" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C32" t="s">
         <v>56</v>
@@ -2698,18 +2698,18 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K32" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B33" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C33" t="s">
         <v>56</v>
@@ -2733,15 +2733,15 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="K33" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B34" t="s">
         <v>80</v>
@@ -2768,21 +2768,21 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="K34" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
+        <v>225</v>
+      </c>
+      <c r="B35" t="s">
         <v>226</v>
       </c>
-      <c r="B35" t="s">
-        <v>227</v>
-      </c>
       <c r="C35" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D35" t="s">
         <v>25</v>
@@ -2803,10 +2803,10 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="K35" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -2817,7 +2817,7 @@
         <v>4</v>
       </c>
       <c r="C36" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D36" t="s">
         <v>25</v>
@@ -2838,10 +2838,10 @@
         <v>1</v>
       </c>
       <c r="J36" t="s">
+        <v>162</v>
+      </c>
+      <c r="K36" t="s">
         <v>163</v>
-      </c>
-      <c r="K36" t="s">
-        <v>164</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
@@ -2878,7 +2878,7 @@
         <v>27</v>
       </c>
       <c r="B38" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C38" t="s">
         <v>49</v>
@@ -2913,7 +2913,7 @@
         <v>33</v>
       </c>
       <c r="B39" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C39" t="s">
         <v>49</v>
@@ -2977,7 +2977,7 @@
         <v>37</v>
       </c>
       <c r="B41" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C41" t="s">
         <v>49</v>
@@ -3012,7 +3012,7 @@
         <v>38</v>
       </c>
       <c r="B42" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="C42" t="s">
         <v>49</v>
@@ -3047,7 +3047,7 @@
         <v>39</v>
       </c>
       <c r="B43" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C43" t="s">
         <v>49</v>
@@ -3152,7 +3152,7 @@
         <v>85</v>
       </c>
       <c r="B46" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C46" t="s">
         <v>52</v>
@@ -3176,10 +3176,10 @@
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K46" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3187,7 +3187,7 @@
         <v>86</v>
       </c>
       <c r="B47" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C47" t="s">
         <v>52</v>
@@ -3211,10 +3211,10 @@
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="K47" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
@@ -3222,7 +3222,7 @@
         <v>87</v>
       </c>
       <c r="B48" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C48" t="s">
         <v>52</v>
@@ -3246,10 +3246,10 @@
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K48" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
@@ -3257,7 +3257,7 @@
         <v>88</v>
       </c>
       <c r="B49" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C49" t="s">
         <v>52</v>
@@ -3281,10 +3281,10 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="K49" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
@@ -3316,10 +3316,10 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K50" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
@@ -3351,10 +3351,10 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="K51" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
@@ -3386,10 +3386,10 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="K52" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
@@ -3421,18 +3421,18 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="K53" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B54" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C54" t="s">
         <v>52</v>
@@ -3456,18 +3456,18 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K54" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B55" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C55" t="s">
         <v>52</v>
@@ -3491,10 +3491,10 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K55" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
@@ -3526,10 +3526,10 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K56" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
@@ -3561,10 +3561,10 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K57" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
@@ -3596,10 +3596,10 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K58" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
@@ -3631,10 +3631,10 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K59" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
@@ -3666,10 +3666,10 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K60" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
@@ -3701,10 +3701,10 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K61" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
@@ -3712,7 +3712,7 @@
         <v>102</v>
       </c>
       <c r="B62" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C62" t="s">
         <v>52</v>
@@ -3736,10 +3736,10 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="K62" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
@@ -3747,7 +3747,7 @@
         <v>103</v>
       </c>
       <c r="B63" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C63" t="s">
         <v>52</v>
@@ -3771,10 +3771,10 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="K63" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
@@ -3782,7 +3782,7 @@
         <v>60</v>
       </c>
       <c r="B64" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C64" t="s">
         <v>54</v>
@@ -3806,10 +3806,10 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
+        <v>193</v>
+      </c>
+      <c r="K64" t="s">
         <v>194</v>
-      </c>
-      <c r="K64" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
@@ -3817,7 +3817,7 @@
         <v>111</v>
       </c>
       <c r="B65" t="s">
-        <v>112</v>
+        <v>227</v>
       </c>
       <c r="C65" t="s">
         <v>54</v>
@@ -3841,18 +3841,18 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="K65" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
+        <v>173</v>
+      </c>
+      <c r="B66" t="s">
         <v>174</v>
-      </c>
-      <c r="B66" t="s">
-        <v>175</v>
       </c>
       <c r="C66" t="s">
         <v>54</v>
@@ -3876,18 +3876,18 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="K66" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B67" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C67" t="s">
         <v>54</v>
@@ -3911,10 +3911,10 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
+        <v>197</v>
+      </c>
+      <c r="K67" t="s">
         <v>198</v>
-      </c>
-      <c r="K67" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
@@ -3922,7 +3922,7 @@
         <v>61</v>
       </c>
       <c r="B68" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C68" t="s">
         <v>54</v>
@@ -3946,10 +3946,10 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="K68" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
@@ -3957,7 +3957,7 @@
         <v>62</v>
       </c>
       <c r="B69" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C69" t="s">
         <v>54</v>
@@ -3981,10 +3981,10 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="K69" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
@@ -4016,10 +4016,10 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="K70" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
@@ -4051,10 +4051,10 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="K71" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
@@ -4062,7 +4062,7 @@
         <v>66</v>
       </c>
       <c r="B72" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C72" t="s">
         <v>51</v>
@@ -4086,18 +4086,18 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K72" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B73" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C73" t="s">
         <v>57</v>
@@ -4121,18 +4121,18 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
+        <v>151</v>
+      </c>
+      <c r="K73" t="s">
         <v>152</v>
-      </c>
-      <c r="K73" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B74" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C74" t="s">
         <v>57</v>
@@ -4156,15 +4156,15 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="K74" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B75" t="s">
         <v>10</v>
@@ -4191,18 +4191,18 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="K75" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B76" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C76" t="s">
         <v>57</v>
@@ -4226,18 +4226,18 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="K76" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
+        <v>120</v>
+      </c>
+      <c r="B77" t="s">
         <v>121</v>
-      </c>
-      <c r="B77" t="s">
-        <v>122</v>
       </c>
       <c r="C77" t="s">
         <v>57</v>
@@ -4261,10 +4261,10 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K77" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
@@ -4296,10 +4296,10 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K78" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
@@ -4331,7 +4331,7 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K79" t="s">
         <v>12</v>
@@ -4366,21 +4366,21 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="K80" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
+        <v>200</v>
+      </c>
+      <c r="B81" t="s">
         <v>201</v>
       </c>
-      <c r="B81" t="s">
-        <v>202</v>
-      </c>
       <c r="C81" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D81" t="s">
         <v>25</v>
@@ -4401,10 +4401,10 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
+        <v>203</v>
+      </c>
+      <c r="K81" t="s">
         <v>204</v>
-      </c>
-      <c r="K81" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
@@ -4412,10 +4412,10 @@
         <v>11</v>
       </c>
       <c r="B82" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C82" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D82" t="s">
         <v>25</v>
@@ -4436,10 +4436,10 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K82" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
@@ -4450,7 +4450,7 @@
         <v>16</v>
       </c>
       <c r="C83" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D83" t="s">
         <v>25</v>
@@ -4471,10 +4471,10 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="K83" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
@@ -4482,10 +4482,10 @@
         <v>47</v>
       </c>
       <c r="B84" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C84" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D84" t="s">
         <v>25</v>
@@ -4506,7 +4506,7 @@
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K84" t="s">
         <v>47</v>

</xml_diff>

<commit_message>
Merged two filter commands into one for ex_ and ms_filter_fastq
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE159B88-AA7C-42AB-8D7C-31F0BFE08D8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B817D27-CB3B-425F-A31E-032B2525744E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="960" yWindow="4830" windowWidth="17280" windowHeight="10005" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$80</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="223">
   <si>
     <t>nn_lower</t>
   </si>
@@ -221,12 +221,6 @@
     <t>ex_reads_lost_demux</t>
   </si>
   <si>
-    <t>ex_reads_filtered_length</t>
-  </si>
-  <si>
-    <t>ex_reads_filtered_quality</t>
-  </si>
-  <si>
     <t>Lane</t>
   </si>
   <si>
@@ -269,9 +263,6 @@
     <t>ms_filtered_per_base_N_content_r2</t>
   </si>
   <si>
-    <t>ms_reads_filtered_length</t>
-  </si>
-  <si>
     <t>Percentage of reads successfully mapped to reference genome, post initial alignment</t>
   </si>
   <si>
@@ -563,21 +554,9 @@
     <t>Percentage of bases lost during trimming</t>
   </si>
   <si>
-    <t>Percentage of reads that retained after length filtering</t>
-  </si>
-  <si>
-    <t>Percentage of reads that are retained after mean quality filtering</t>
-  </si>
-  <si>
     <t>(?m)^\s*Both Surviving Read Percent:\s*(?P&lt;value&gt;100(?:\.0+)?|(?:\d{1,2})(?:\.\d+)?)\s*$</t>
   </si>
   <si>
-    <t>_filter_length.txt</t>
-  </si>
-  <si>
-    <t>_filter_quality.txt</t>
-  </si>
-  <si>
     <t>^duplex_disagreement_rate\s+([0-9]*\.?[0-9]+)</t>
   </si>
   <si>
@@ -695,15 +674,6 @@
     <t>Percentage of genome with depth &gt;= minimum MS depth value defined in config</t>
   </si>
   <si>
-    <t>ms_reads_filtered_quality</t>
-  </si>
-  <si>
-    <t>_length_filter_metrics.txt</t>
-  </si>
-  <si>
-    <t>_quality_filter_metrics.txt</t>
-  </si>
-  <si>
     <t>MS mask regions</t>
   </si>
   <si>
@@ -720,6 +690,21 @@
   </si>
   <si>
     <t>Gini coefficient for inequality between ex_samples</t>
+  </si>
+  <si>
+    <t>ex_reads_filtered_length_quality</t>
+  </si>
+  <si>
+    <t>Percentage of reads that retained after length and quality filtering</t>
+  </si>
+  <si>
+    <t>_filter_metrics_ex.txt</t>
+  </si>
+  <si>
+    <t>ms_reads_filtered_length_quality</t>
+  </si>
+  <si>
+    <t>_filter_metrics_ms.txt</t>
   </si>
 </sst>
 </file>
@@ -1589,7 +1574,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K84"/>
+  <dimension ref="A1:K82"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" customWidth="1"/>
@@ -1631,10 +1616,10 @@
         <v>31</v>
       </c>
       <c r="J1" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="K1" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -1642,7 +1627,7 @@
         <v>34</v>
       </c>
       <c r="B2" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="C2" t="s">
         <v>48</v>
@@ -1671,7 +1656,7 @@
         <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>214</v>
+        <v>207</v>
       </c>
       <c r="C3" t="s">
         <v>48</v>
@@ -1706,7 +1691,7 @@
         <v>36</v>
       </c>
       <c r="B4" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="C4" t="s">
         <v>48</v>
@@ -1741,7 +1726,7 @@
         <v>44</v>
       </c>
       <c r="B5" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="C5" t="s">
         <v>50</v>
@@ -1770,7 +1755,7 @@
         <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="C6" t="s">
         <v>50</v>
@@ -1805,7 +1790,7 @@
         <v>45</v>
       </c>
       <c r="B7" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="C7" t="s">
         <v>50</v>
@@ -1834,7 +1819,7 @@
         <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="C8" t="s">
         <v>50</v>
@@ -1869,7 +1854,7 @@
         <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C9" t="s">
         <v>50</v>
@@ -1904,7 +1889,7 @@
         <v>24</v>
       </c>
       <c r="B10" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="C10" t="s">
         <v>50</v>
@@ -1939,7 +1924,7 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C11" t="s">
         <v>53</v>
@@ -1963,10 +1948,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="K11" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1974,7 +1959,7 @@
         <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>105</v>
+        <v>102</v>
       </c>
       <c r="C12" t="s">
         <v>53</v>
@@ -1998,18 +1983,18 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="K12" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>91</v>
+        <v>88</v>
       </c>
       <c r="B13" t="s">
-        <v>208</v>
+        <v>201</v>
       </c>
       <c r="C13" t="s">
         <v>53</v>
@@ -2033,18 +2018,18 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="K13" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="B14" t="s">
-        <v>209</v>
+        <v>202</v>
       </c>
       <c r="C14" t="s">
         <v>53</v>
@@ -2068,18 +2053,18 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="K14" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>89</v>
+        <v>86</v>
       </c>
       <c r="B15" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="C15" t="s">
         <v>53</v>
@@ -2103,18 +2088,18 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="K15" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>90</v>
+        <v>87</v>
       </c>
       <c r="B16" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="C16" t="s">
         <v>53</v>
@@ -2138,18 +2123,18 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="K16" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B17" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C17" t="s">
         <v>53</v>
@@ -2173,18 +2158,18 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="K17" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B18" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C18" t="s">
         <v>53</v>
@@ -2208,18 +2193,18 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="K18" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="B19" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="C19" t="s">
         <v>53</v>
@@ -2243,18 +2228,18 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="K19" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="B20" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="C20" t="s">
         <v>53</v>
@@ -2278,18 +2263,18 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="K20" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B21" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C21" t="s">
         <v>53</v>
@@ -2313,18 +2298,18 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="K21" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B22" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="C22" t="s">
         <v>53</v>
@@ -2348,18 +2333,18 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="K22" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B23" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C23" t="s">
         <v>53</v>
@@ -2383,18 +2368,18 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="K23" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B24" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C24" t="s">
         <v>53</v>
@@ -2418,18 +2403,18 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="K24" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B25" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C25" t="s">
         <v>53</v>
@@ -2453,18 +2438,18 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="K25" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B26" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C26" t="s">
         <v>53</v>
@@ -2488,18 +2473,18 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="K26" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B27" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="C27" t="s">
         <v>53</v>
@@ -2523,18 +2508,18 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="K27" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B28" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="C28" t="s">
         <v>53</v>
@@ -2558,18 +2543,18 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="K28" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>77</v>
+        <v>221</v>
       </c>
       <c r="B29" t="s">
-        <v>175</v>
+        <v>219</v>
       </c>
       <c r="C29" t="s">
         <v>55</v>
@@ -2593,53 +2578,53 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="K29" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>219</v>
+        <v>113</v>
       </c>
       <c r="B30" t="s">
-        <v>176</v>
+        <v>107</v>
       </c>
       <c r="C30" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="D30" t="s">
         <v>25</v>
       </c>
       <c r="E30">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="F30">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G30">
-        <v>92.5</v>
+        <v>95</v>
       </c>
       <c r="H30">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I30" t="b">
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>221</v>
+        <v>130</v>
       </c>
       <c r="K30" t="s">
-        <v>177</v>
+        <v>155</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="B31" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="C31" t="s">
         <v>56</v>
@@ -2648,33 +2633,33 @@
         <v>25</v>
       </c>
       <c r="E31">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="F31">
-        <v>100</v>
+        <v>0.1</v>
       </c>
       <c r="G31">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H31">
-        <v>100</v>
+        <v>0.03</v>
       </c>
       <c r="I31" t="b">
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>133</v>
+        <v>199</v>
       </c>
       <c r="K31" t="s">
-        <v>158</v>
+        <v>198</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>115</v>
+        <v>205</v>
       </c>
       <c r="B32" t="s">
-        <v>122</v>
+        <v>211</v>
       </c>
       <c r="C32" t="s">
         <v>56</v>
@@ -2683,16 +2668,16 @@
         <v>25</v>
       </c>
       <c r="E32">
-        <v>0</v>
+        <v>21.75</v>
       </c>
       <c r="F32">
-        <v>0.1</v>
+        <v>100</v>
       </c>
       <c r="G32">
-        <v>0</v>
+        <v>26.1</v>
       </c>
       <c r="H32">
-        <v>0.03</v>
+        <v>100</v>
       </c>
       <c r="I32" t="b">
         <v>1</v>
@@ -2701,15 +2686,15 @@
         <v>206</v>
       </c>
       <c r="K32" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>212</v>
+        <v>111</v>
       </c>
       <c r="B33" t="s">
-        <v>218</v>
+        <v>77</v>
       </c>
       <c r="C33" t="s">
         <v>56</v>
@@ -2718,150 +2703,150 @@
         <v>25</v>
       </c>
       <c r="E33">
-        <v>21.75</v>
+        <v>125</v>
       </c>
       <c r="F33">
-        <v>100</v>
+        <v>175</v>
       </c>
       <c r="G33">
-        <v>26.1</v>
+        <v>140</v>
       </c>
       <c r="H33">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="I33" t="b">
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>213</v>
+        <v>131</v>
       </c>
       <c r="K33" t="s">
-        <v>217</v>
+        <v>156</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>114</v>
+        <v>215</v>
       </c>
       <c r="B34" t="s">
-        <v>80</v>
+        <v>216</v>
       </c>
       <c r="C34" t="s">
-        <v>56</v>
+        <v>212</v>
       </c>
       <c r="D34" t="s">
         <v>25</v>
       </c>
       <c r="E34">
-        <v>125</v>
+        <v>1.5E-3</v>
       </c>
       <c r="F34">
-        <v>175</v>
+        <v>1.4999999999999999E-2</v>
       </c>
       <c r="G34">
-        <v>140</v>
+        <v>1.5E-3</v>
       </c>
       <c r="H34">
-        <v>160</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="I34" t="b">
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>134</v>
+        <v>214</v>
       </c>
       <c r="K34" t="s">
-        <v>159</v>
+        <v>213</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>225</v>
+        <v>59</v>
       </c>
       <c r="B35" t="s">
-        <v>226</v>
+        <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="D35" t="s">
         <v>25</v>
       </c>
       <c r="E35">
-        <v>1.5E-3</v>
+        <v>70</v>
       </c>
       <c r="F35">
-        <v>1.4999999999999999E-2</v>
+        <v>90</v>
       </c>
       <c r="G35">
-        <v>1.5E-3</v>
+        <v>70</v>
       </c>
       <c r="H35">
-        <v>3.0000000000000001E-3</v>
+        <v>80</v>
       </c>
       <c r="I35" t="b">
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>224</v>
+        <v>159</v>
       </c>
       <c r="K35" t="s">
-        <v>223</v>
+        <v>160</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>59</v>
+        <v>20</v>
       </c>
       <c r="B36" t="s">
-        <v>4</v>
+        <v>40</v>
       </c>
       <c r="C36" t="s">
-        <v>222</v>
+        <v>49</v>
       </c>
       <c r="D36" t="s">
         <v>25</v>
       </c>
       <c r="E36">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="F36">
-        <v>90</v>
-      </c>
-      <c r="G36">
-        <v>70</v>
-      </c>
-      <c r="H36">
-        <v>80</v>
+        <v>1000</v>
       </c>
       <c r="I36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J36" t="s">
-        <v>162</v>
+        <v>58</v>
       </c>
       <c r="K36" t="s">
-        <v>163</v>
+        <v>58</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="B37" t="s">
-        <v>40</v>
+        <v>208</v>
       </c>
       <c r="C37" t="s">
         <v>49</v>
       </c>
       <c r="D37" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E37">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="F37">
-        <v>1000</v>
+        <v>0.3</v>
+      </c>
+      <c r="G37">
+        <v>0</v>
+      </c>
+      <c r="H37">
+        <v>0.2</v>
       </c>
       <c r="I37" t="b">
         <v>0</v>
@@ -2875,28 +2860,28 @@
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B38" t="s">
-        <v>215</v>
+        <v>166</v>
       </c>
       <c r="C38" t="s">
         <v>49</v>
       </c>
       <c r="D38" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E38">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F38">
-        <v>0.3</v>
+        <v>100</v>
       </c>
       <c r="G38">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="H38">
-        <v>0.2</v>
+        <v>100</v>
       </c>
       <c r="I38" t="b">
         <v>0</v>
@@ -2910,10 +2895,10 @@
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="B39" t="s">
-        <v>169</v>
+        <v>42</v>
       </c>
       <c r="C39" t="s">
         <v>49</v>
@@ -2922,16 +2907,10 @@
         <v>25</v>
       </c>
       <c r="E39">
-        <v>80</v>
-      </c>
-      <c r="F39">
-        <v>100</v>
-      </c>
-      <c r="G39">
-        <v>95</v>
-      </c>
-      <c r="H39">
-        <v>100</v>
+        <v>4.3</v>
+      </c>
+      <c r="F39" t="s">
+        <v>5</v>
       </c>
       <c r="I39" t="b">
         <v>0</v>
@@ -2945,22 +2924,28 @@
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>41</v>
+        <v>37</v>
       </c>
       <c r="B40" t="s">
-        <v>42</v>
+        <v>208</v>
       </c>
       <c r="C40" t="s">
         <v>49</v>
       </c>
       <c r="D40" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E40">
-        <v>4.3</v>
-      </c>
-      <c r="F40" t="s">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="F40">
+        <v>0.4</v>
+      </c>
+      <c r="G40">
+        <v>0</v>
+      </c>
+      <c r="H40">
+        <v>0.3</v>
       </c>
       <c r="I40" t="b">
         <v>0</v>
@@ -2974,28 +2959,28 @@
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B41" t="s">
-        <v>215</v>
+        <v>167</v>
       </c>
       <c r="C41" t="s">
         <v>49</v>
       </c>
       <c r="D41" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E41">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F41">
-        <v>0.4</v>
+        <v>100</v>
       </c>
       <c r="G41">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="H41">
-        <v>0.3</v>
+        <v>100</v>
       </c>
       <c r="I41" t="b">
         <v>0</v>
@@ -3009,10 +2994,10 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B42" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C42" t="s">
         <v>49</v>
@@ -3021,16 +3006,16 @@
         <v>25</v>
       </c>
       <c r="E42">
-        <v>80</v>
+        <v>1</v>
       </c>
       <c r="F42">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G42">
-        <v>95</v>
+        <v>1</v>
       </c>
       <c r="H42">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="I42" t="b">
         <v>0</v>
@@ -3044,10 +3029,10 @@
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>39</v>
+        <v>21</v>
       </c>
       <c r="B43" t="s">
-        <v>171</v>
+        <v>18</v>
       </c>
       <c r="C43" t="s">
         <v>49</v>
@@ -3056,16 +3041,16 @@
         <v>25</v>
       </c>
       <c r="E43">
-        <v>1</v>
+        <v>544</v>
       </c>
       <c r="F43">
-        <v>1</v>
+        <v>624</v>
       </c>
       <c r="G43">
-        <v>1</v>
+        <v>564</v>
       </c>
       <c r="H43">
-        <v>1</v>
+        <v>604</v>
       </c>
       <c r="I43" t="b">
         <v>0</v>
@@ -3079,10 +3064,10 @@
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B44" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C44" t="s">
         <v>49</v>
@@ -3091,16 +3076,16 @@
         <v>25</v>
       </c>
       <c r="E44">
-        <v>544</v>
+        <v>98</v>
       </c>
       <c r="F44">
-        <v>624</v>
+        <v>100</v>
       </c>
       <c r="G44">
-        <v>564</v>
+        <v>100</v>
       </c>
       <c r="H44">
-        <v>604</v>
+        <v>100</v>
       </c>
       <c r="I44" t="b">
         <v>0</v>
@@ -3114,51 +3099,51 @@
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>22</v>
+        <v>82</v>
       </c>
       <c r="B45" t="s">
-        <v>19</v>
+        <v>201</v>
       </c>
       <c r="C45" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D45" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="E45">
-        <v>98</v>
+        <v>35</v>
       </c>
       <c r="F45">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="G45">
-        <v>100</v>
+        <v>39</v>
       </c>
       <c r="H45">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="I45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>58</v>
+        <v>132</v>
       </c>
       <c r="K45" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B46" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
       <c r="C46" t="s">
         <v>52</v>
       </c>
       <c r="D46" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E46">
         <v>35</v>
@@ -3176,59 +3161,59 @@
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K46" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B47" t="s">
-        <v>209</v>
+        <v>200</v>
       </c>
       <c r="C47" t="s">
         <v>52</v>
       </c>
       <c r="D47" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E47">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="F47">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="G47">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="H47">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="I47" t="b">
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="K47" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B48" t="s">
-        <v>207</v>
+        <v>200</v>
       </c>
       <c r="C48" t="s">
         <v>52</v>
       </c>
       <c r="D48" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E48">
         <v>0</v>
@@ -3246,59 +3231,59 @@
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K48" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>88</v>
+        <v>81</v>
       </c>
       <c r="B49" t="s">
-        <v>207</v>
+        <v>80</v>
       </c>
       <c r="C49" t="s">
         <v>52</v>
       </c>
       <c r="D49" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E49">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="F49">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="G49">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="H49">
-        <v>5</v>
+        <v>150</v>
       </c>
       <c r="I49" t="b">
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="K49" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
       <c r="B50" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="C50" t="s">
         <v>52</v>
       </c>
       <c r="D50" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E50">
         <v>150</v>
@@ -3316,59 +3301,59 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K50" t="s">
-        <v>144</v>
+        <v>141</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B51" t="s">
-        <v>83</v>
+        <v>101</v>
       </c>
       <c r="C51" t="s">
         <v>52</v>
       </c>
       <c r="D51" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E51">
-        <v>150</v>
-      </c>
-      <c r="F51">
-        <v>150</v>
+        <v>2850</v>
+      </c>
+      <c r="F51" t="s">
+        <v>5</v>
       </c>
       <c r="G51">
-        <v>150</v>
-      </c>
-      <c r="H51">
-        <v>150</v>
+        <v>3000</v>
+      </c>
+      <c r="H51" t="s">
+        <v>5</v>
       </c>
       <c r="I51" t="b">
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
       <c r="K51" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B52" t="s">
-        <v>104</v>
+        <v>101</v>
       </c>
       <c r="C52" t="s">
         <v>52</v>
       </c>
       <c r="D52" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E52">
         <v>2850</v>
@@ -3386,53 +3371,53 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K52" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>95</v>
+        <v>176</v>
       </c>
       <c r="B53" t="s">
-        <v>104</v>
+        <v>204</v>
       </c>
       <c r="C53" t="s">
         <v>52</v>
       </c>
       <c r="D53" t="s">
-        <v>63</v>
+        <v>25</v>
       </c>
       <c r="E53">
-        <v>2850</v>
-      </c>
-      <c r="F53" t="s">
-        <v>5</v>
+        <v>30</v>
+      </c>
+      <c r="F53">
+        <v>40</v>
       </c>
       <c r="G53">
-        <v>3000</v>
-      </c>
-      <c r="H53" t="s">
-        <v>5</v>
+        <v>35</v>
+      </c>
+      <c r="H53">
+        <v>40</v>
       </c>
       <c r="I53" t="b">
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="K53" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="B54" t="s">
-        <v>211</v>
+        <v>204</v>
       </c>
       <c r="C54" t="s">
         <v>52</v>
@@ -3456,18 +3441,18 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="K54" t="s">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>184</v>
+        <v>93</v>
       </c>
       <c r="B55" t="s">
-        <v>211</v>
+        <v>103</v>
       </c>
       <c r="C55" t="s">
         <v>52</v>
@@ -3476,22 +3461,22 @@
         <v>25</v>
       </c>
       <c r="E55">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F55">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="G55">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H55">
-        <v>40</v>
+        <v>0.1</v>
       </c>
       <c r="I55" t="b">
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="K55" t="s">
         <v>142</v>
@@ -3499,10 +3484,10 @@
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B56" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C56" t="s">
         <v>52</v>
@@ -3526,18 +3511,18 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="K56" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B57" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C57" t="s">
         <v>52</v>
@@ -3549,30 +3534,30 @@
         <v>0</v>
       </c>
       <c r="F57">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="G57">
         <v>0</v>
       </c>
       <c r="H57">
-        <v>0.1</v>
+        <v>20</v>
       </c>
       <c r="I57" t="b">
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="K57" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B58" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="C58" t="s">
         <v>52</v>
@@ -3596,18 +3581,18 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="K58" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B59" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C59" t="s">
         <v>52</v>
@@ -3619,30 +3604,30 @@
         <v>0</v>
       </c>
       <c r="F59">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G59">
         <v>0</v>
       </c>
       <c r="H59">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I59" t="b">
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="K59" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="B60" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C60" t="s">
         <v>52</v>
@@ -3666,18 +3651,18 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="K60" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="B61" t="s">
-        <v>108</v>
+        <v>203</v>
       </c>
       <c r="C61" t="s">
         <v>52</v>
@@ -3689,30 +3674,30 @@
         <v>0</v>
       </c>
       <c r="F61">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G61">
         <v>0</v>
       </c>
       <c r="H61">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I61" t="b">
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="K61" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="B62" t="s">
-        <v>210</v>
+        <v>203</v>
       </c>
       <c r="C62" t="s">
         <v>52</v>
@@ -3736,123 +3721,123 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="K62" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>103</v>
+        <v>60</v>
       </c>
       <c r="B63" t="s">
-        <v>210</v>
+        <v>188</v>
       </c>
       <c r="C63" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D63" t="s">
-        <v>25</v>
+        <v>61</v>
       </c>
       <c r="E63">
         <v>0</v>
       </c>
       <c r="F63">
+        <v>25</v>
+      </c>
+      <c r="G63">
+        <v>0</v>
+      </c>
+      <c r="H63">
         <v>10</v>
       </c>
-      <c r="G63">
-        <v>0</v>
-      </c>
-      <c r="H63">
-        <v>5</v>
-      </c>
       <c r="I63" t="b">
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>138</v>
+        <v>186</v>
       </c>
       <c r="K63" t="s">
-        <v>148</v>
+        <v>187</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>60</v>
+        <v>108</v>
       </c>
       <c r="B64" t="s">
-        <v>195</v>
+        <v>217</v>
       </c>
       <c r="C64" t="s">
         <v>54</v>
       </c>
       <c r="D64" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E64">
         <v>0</v>
       </c>
       <c r="F64">
-        <v>25</v>
+        <v>0.1</v>
       </c>
       <c r="G64">
         <v>0</v>
       </c>
       <c r="H64">
-        <v>10</v>
+        <v>0.05</v>
       </c>
       <c r="I64" t="b">
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="K64" t="s">
-        <v>194</v>
+        <v>147</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>111</v>
+        <v>170</v>
       </c>
       <c r="B65" t="s">
-        <v>227</v>
+        <v>171</v>
       </c>
       <c r="C65" t="s">
         <v>54</v>
       </c>
       <c r="D65" t="s">
-        <v>63</v>
+        <v>25</v>
       </c>
       <c r="E65">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F65">
-        <v>0.1</v>
+        <v>40</v>
       </c>
       <c r="G65">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H65">
-        <v>0.05</v>
+        <v>20</v>
       </c>
       <c r="I65" t="b">
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>193</v>
+        <v>175</v>
       </c>
       <c r="K65" t="s">
-        <v>150</v>
+        <v>189</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>173</v>
+        <v>192</v>
       </c>
       <c r="B66" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="C66" t="s">
         <v>54</v>
@@ -3861,33 +3846,33 @@
         <v>25</v>
       </c>
       <c r="E66">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F66">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="G66">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H66">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I66" t="b">
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="K66" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="B67" t="s">
-        <v>187</v>
+        <v>219</v>
       </c>
       <c r="C67" t="s">
         <v>54</v>
@@ -3896,60 +3881,60 @@
         <v>25</v>
       </c>
       <c r="E67">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="F67">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="G67">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="H67">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="I67" t="b">
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>197</v>
+        <v>220</v>
       </c>
       <c r="K67" t="s">
-        <v>198</v>
+        <v>172</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B68" t="s">
-        <v>175</v>
+        <v>75</v>
       </c>
       <c r="C68" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D68" t="s">
         <v>25</v>
       </c>
       <c r="E68">
-        <v>80</v>
+        <v>90</v>
       </c>
       <c r="F68">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G68">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="H68">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I68" t="b">
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>178</v>
+        <v>123</v>
       </c>
       <c r="K68" t="s">
-        <v>177</v>
+        <v>155</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
@@ -3957,42 +3942,42 @@
         <v>62</v>
       </c>
       <c r="B69" t="s">
-        <v>176</v>
+        <v>76</v>
       </c>
       <c r="C69" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="D69" t="s">
         <v>25</v>
       </c>
       <c r="E69">
-        <v>85</v>
+        <v>50</v>
       </c>
       <c r="F69">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G69">
-        <v>92.5</v>
+        <v>75</v>
       </c>
       <c r="H69">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I69" t="b">
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>179</v>
+        <v>123</v>
       </c>
       <c r="K69" t="s">
-        <v>177</v>
+        <v>157</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B70" t="s">
-        <v>78</v>
+        <v>109</v>
       </c>
       <c r="C70" t="s">
         <v>51</v>
@@ -4001,36 +3986,36 @@
         <v>25</v>
       </c>
       <c r="E70">
-        <v>90</v>
+        <v>125</v>
       </c>
       <c r="F70">
-        <v>100</v>
+        <v>175</v>
       </c>
       <c r="G70">
-        <v>95</v>
+        <v>140</v>
       </c>
       <c r="H70">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="I70" t="b">
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K70" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>64</v>
+        <v>120</v>
       </c>
       <c r="B71" t="s">
-        <v>79</v>
+        <v>182</v>
       </c>
       <c r="C71" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D71" t="s">
         <v>25</v>
@@ -4039,65 +4024,65 @@
         <v>50</v>
       </c>
       <c r="F71">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="G71">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="H71">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="I71" t="b">
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>126</v>
+        <v>148</v>
       </c>
       <c r="K71" t="s">
-        <v>160</v>
+        <v>149</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>66</v>
+        <v>110</v>
       </c>
       <c r="B72" t="s">
-        <v>112</v>
+        <v>164</v>
       </c>
       <c r="C72" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="D72" t="s">
         <v>25</v>
       </c>
       <c r="E72">
-        <v>125</v>
+        <v>60</v>
       </c>
       <c r="F72">
-        <v>175</v>
+        <v>100</v>
       </c>
       <c r="G72">
-        <v>140</v>
+        <v>90</v>
       </c>
       <c r="H72">
-        <v>160</v>
+        <v>100</v>
       </c>
       <c r="I72" t="b">
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>127</v>
+        <v>162</v>
       </c>
       <c r="K72" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="B73" t="s">
-        <v>189</v>
+        <v>10</v>
       </c>
       <c r="C73" t="s">
         <v>57</v>
@@ -4106,33 +4091,33 @@
         <v>25</v>
       </c>
       <c r="E73">
-        <v>50</v>
+        <v>99</v>
       </c>
       <c r="F73">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="G73">
-        <v>50</v>
+        <v>99.5</v>
       </c>
       <c r="H73">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="I73" t="b">
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K73" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B74" t="s">
-        <v>167</v>
+        <v>114</v>
       </c>
       <c r="C74" t="s">
         <v>57</v>
@@ -4141,33 +4126,33 @@
         <v>25</v>
       </c>
       <c r="E74">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="F74">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="G74">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="H74">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="I74" t="b">
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>165</v>
+        <v>152</v>
       </c>
       <c r="K74" t="s">
-        <v>164</v>
+        <v>151</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="B75" t="s">
-        <v>10</v>
+        <v>118</v>
       </c>
       <c r="C75" t="s">
         <v>57</v>
@@ -4176,22 +4161,22 @@
         <v>25</v>
       </c>
       <c r="E75">
-        <v>99</v>
-      </c>
-      <c r="F75">
-        <v>100</v>
+        <v>0.5</v>
+      </c>
+      <c r="F75" t="s">
+        <v>5</v>
       </c>
       <c r="G75">
-        <v>99.5</v>
-      </c>
-      <c r="H75">
-        <v>100</v>
+        <v>1</v>
+      </c>
+      <c r="H75" t="s">
+        <v>5</v>
       </c>
       <c r="I75" t="b">
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="K75" t="s">
         <v>153</v>
@@ -4199,10 +4184,10 @@
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>118</v>
+        <v>14</v>
       </c>
       <c r="B76" t="s">
-        <v>117</v>
+        <v>15</v>
       </c>
       <c r="C76" t="s">
         <v>57</v>
@@ -4214,30 +4199,30 @@
         <v>0</v>
       </c>
       <c r="F76">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="G76">
         <v>0</v>
       </c>
       <c r="H76">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I76" t="b">
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>155</v>
+        <v>125</v>
       </c>
       <c r="K76" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>120</v>
+        <v>12</v>
       </c>
       <c r="B77" t="s">
-        <v>121</v>
+        <v>13</v>
       </c>
       <c r="C77" t="s">
         <v>57</v>
@@ -4246,33 +4231,33 @@
         <v>25</v>
       </c>
       <c r="E77">
-        <v>0.5</v>
-      </c>
-      <c r="F77" t="s">
-        <v>5</v>
+        <v>14.5</v>
+      </c>
+      <c r="F77">
+        <v>100</v>
       </c>
       <c r="G77">
-        <v>1</v>
-      </c>
-      <c r="H77" t="s">
-        <v>5</v>
+        <v>26.1</v>
+      </c>
+      <c r="H77">
+        <v>100</v>
       </c>
       <c r="I77" t="b">
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="K77" t="s">
-        <v>156</v>
+        <v>12</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="B78" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="C78" t="s">
         <v>57</v>
@@ -4281,153 +4266,153 @@
         <v>25</v>
       </c>
       <c r="E78">
-        <v>0</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="F78">
-        <v>0</v>
+        <v>8.0000000000000004E-4</v>
       </c>
       <c r="G78">
-        <v>0</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="H78">
-        <v>0</v>
+        <v>5.0000000000000001E-4</v>
       </c>
       <c r="I78" t="b">
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>128</v>
+        <v>174</v>
       </c>
       <c r="K78" t="s">
-        <v>149</v>
+        <v>173</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>12</v>
+        <v>193</v>
       </c>
       <c r="B79" t="s">
-        <v>13</v>
+        <v>194</v>
       </c>
       <c r="C79" t="s">
-        <v>57</v>
+        <v>169</v>
       </c>
       <c r="D79" t="s">
         <v>25</v>
       </c>
       <c r="E79">
-        <v>14.5</v>
+        <v>0.05</v>
       </c>
       <c r="F79">
-        <v>100</v>
+        <v>0.08</v>
       </c>
       <c r="G79">
-        <v>26.1</v>
+        <v>0.02</v>
       </c>
       <c r="H79">
-        <v>100</v>
+        <v>0.05</v>
       </c>
       <c r="I79" t="b">
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>166</v>
+        <v>196</v>
       </c>
       <c r="K79" t="s">
-        <v>12</v>
+        <v>197</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="B80" t="s">
-        <v>9</v>
+        <v>195</v>
       </c>
       <c r="C80" t="s">
-        <v>57</v>
+        <v>169</v>
       </c>
       <c r="D80" t="s">
         <v>25</v>
       </c>
       <c r="E80">
-        <v>5.0000000000000001E-4</v>
+        <v>5</v>
       </c>
       <c r="F80">
-        <v>8.0000000000000004E-4</v>
+        <v>100</v>
       </c>
       <c r="G80">
-        <v>2.0000000000000001E-4</v>
+        <v>20</v>
       </c>
       <c r="H80">
-        <v>5.0000000000000001E-4</v>
+        <v>100</v>
       </c>
       <c r="I80" t="b">
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>181</v>
+        <v>163</v>
       </c>
       <c r="K80" t="s">
-        <v>180</v>
+        <v>154</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>200</v>
+        <v>17</v>
       </c>
       <c r="B81" t="s">
-        <v>201</v>
+        <v>16</v>
       </c>
       <c r="C81" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="D81" t="s">
         <v>25</v>
       </c>
       <c r="E81">
-        <v>0.05</v>
+        <v>0</v>
       </c>
       <c r="F81">
-        <v>0.08</v>
+        <v>95</v>
       </c>
       <c r="G81">
-        <v>0.02</v>
+        <v>0</v>
       </c>
       <c r="H81">
-        <v>0.05</v>
+        <v>80</v>
       </c>
       <c r="I81" t="b">
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>203</v>
+        <v>136</v>
       </c>
       <c r="K81" t="s">
-        <v>204</v>
+        <v>158</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>11</v>
+        <v>47</v>
       </c>
       <c r="B82" t="s">
-        <v>202</v>
+        <v>181</v>
       </c>
       <c r="C82" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="D82" t="s">
         <v>25</v>
       </c>
       <c r="E82">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="F82">
         <v>100</v>
       </c>
       <c r="G82">
-        <v>20</v>
+        <v>67</v>
       </c>
       <c r="H82">
         <v>100</v>
@@ -4436,84 +4421,14 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="K82" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>17</v>
-      </c>
-      <c r="B83" t="s">
-        <v>16</v>
-      </c>
-      <c r="C83" t="s">
-        <v>172</v>
-      </c>
-      <c r="D83" t="s">
-        <v>25</v>
-      </c>
-      <c r="E83">
-        <v>0</v>
-      </c>
-      <c r="F83">
-        <v>95</v>
-      </c>
-      <c r="G83">
-        <v>0</v>
-      </c>
-      <c r="H83">
-        <v>80</v>
-      </c>
-      <c r="I83" t="b">
-        <v>1</v>
-      </c>
-      <c r="J83" t="s">
-        <v>139</v>
-      </c>
-      <c r="K83" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
         <v>47</v>
       </c>
-      <c r="B84" t="s">
-        <v>188</v>
-      </c>
-      <c r="C84" t="s">
-        <v>172</v>
-      </c>
-      <c r="D84" t="s">
-        <v>25</v>
-      </c>
-      <c r="E84">
-        <v>33</v>
-      </c>
-      <c r="F84">
-        <v>100</v>
-      </c>
-      <c r="G84">
-        <v>67</v>
-      </c>
-      <c r="H84">
-        <v>100</v>
-      </c>
-      <c r="I84" t="b">
-        <v>1</v>
-      </c>
-      <c r="J84" t="s">
-        <v>166</v>
-      </c>
-      <c r="K84" t="s">
-        <v>47</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K82" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K80" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated thresholds for filter component metrics
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B817D27-CB3B-425F-A31E-032B2525744E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC205ECD-0A80-4056-9EC3-6742DF84C0FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -2563,13 +2563,13 @@
         <v>25</v>
       </c>
       <c r="E29">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="F29">
         <v>99</v>
       </c>
       <c r="G29">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="H29">
         <v>99</v>
@@ -3881,13 +3881,13 @@
         <v>25</v>
       </c>
       <c r="E67">
-        <v>80</v>
+        <v>70</v>
       </c>
       <c r="F67">
         <v>99</v>
       </c>
       <c r="G67">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="H67">
         <v>99</v>

</xml_diff>

<commit_message>
Rebased component_level_metrics changes for variant call eligible disagree rate
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\codec-opensource\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\jamesphie\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC205ECD-0A80-4056-9EC3-6742DF84C0FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7813D0D-797C-4744-BF26-FF11480F7186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -617,21 +617,9 @@
     <t>ex_zero_length_reads</t>
   </si>
   <si>
-    <t>ex_N_bases_variant_call_eligible</t>
-  </si>
-  <si>
-    <t>Percentage of N bases in bases eligible for variant calling (duplex depth &gt; 0, unmasked, QUAL &gt; min_base_quality)</t>
-  </si>
-  <si>
     <t>Percentage of genome eligible for variant calling (duplex depth &gt; 0, unmasked, QUAL &gt; min_base_quality)</t>
   </si>
   <si>
-    <t>_percent_eligible_N_bases.json</t>
-  </si>
-  <si>
-    <t>post_consensus_percent_N</t>
-  </si>
-  <si>
     <t>duplication_rate</t>
   </si>
   <si>
@@ -705,6 +693,18 @@
   </si>
   <si>
     <t>_filter_metrics_ms.txt</t>
+  </si>
+  <si>
+    <t>ex_variant_call_eligible_disagree_rate</t>
+  </si>
+  <si>
+    <t>Watson and Crick disagreement rate among bases eligible for somatic variant calling</t>
+  </si>
+  <si>
+    <t>_variant_call_disagree_metrics.json</t>
+  </si>
+  <si>
+    <t>observed_disagreement_rate</t>
   </si>
 </sst>
 </file>
@@ -1656,7 +1656,7 @@
         <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="C3" t="s">
         <v>48</v>
@@ -1755,7 +1755,7 @@
         <v>43</v>
       </c>
       <c r="B6" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="C6" t="s">
         <v>50</v>
@@ -1819,7 +1819,7 @@
         <v>46</v>
       </c>
       <c r="B8" t="s">
-        <v>209</v>
+        <v>205</v>
       </c>
       <c r="C8" t="s">
         <v>50</v>
@@ -1994,7 +1994,7 @@
         <v>88</v>
       </c>
       <c r="B13" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C13" t="s">
         <v>53</v>
@@ -2029,7 +2029,7 @@
         <v>89</v>
       </c>
       <c r="B14" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C14" t="s">
         <v>53</v>
@@ -2064,7 +2064,7 @@
         <v>86</v>
       </c>
       <c r="B15" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C15" t="s">
         <v>53</v>
@@ -2099,7 +2099,7 @@
         <v>87</v>
       </c>
       <c r="B16" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C16" t="s">
         <v>53</v>
@@ -2204,7 +2204,7 @@
         <v>178</v>
       </c>
       <c r="B19" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C19" t="s">
         <v>53</v>
@@ -2239,7 +2239,7 @@
         <v>179</v>
       </c>
       <c r="B20" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C20" t="s">
         <v>53</v>
@@ -2484,7 +2484,7 @@
         <v>73</v>
       </c>
       <c r="B27" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C27" t="s">
         <v>53</v>
@@ -2519,7 +2519,7 @@
         <v>74</v>
       </c>
       <c r="B28" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C28" t="s">
         <v>53</v>
@@ -2551,10 +2551,10 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="B29" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="C29" t="s">
         <v>55</v>
@@ -2578,7 +2578,7 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="K29" t="s">
         <v>172</v>
@@ -2648,18 +2648,18 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>199</v>
+        <v>195</v>
       </c>
       <c r="K31" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="B32" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="C32" t="s">
         <v>56</v>
@@ -2683,10 +2683,10 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
+        <v>202</v>
+      </c>
+      <c r="K32" t="s">
         <v>206</v>
-      </c>
-      <c r="K32" t="s">
-        <v>210</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -2726,13 +2726,13 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="B34" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="C34" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="D34" t="s">
         <v>25</v>
@@ -2753,10 +2753,10 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="K34" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -2767,7 +2767,7 @@
         <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="D35" t="s">
         <v>25</v>
@@ -2828,7 +2828,7 @@
         <v>27</v>
       </c>
       <c r="B37" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="C37" t="s">
         <v>49</v>
@@ -2927,7 +2927,7 @@
         <v>37</v>
       </c>
       <c r="B40" t="s">
-        <v>208</v>
+        <v>204</v>
       </c>
       <c r="C40" t="s">
         <v>49</v>
@@ -3102,7 +3102,7 @@
         <v>82</v>
       </c>
       <c r="B45" t="s">
-        <v>201</v>
+        <v>197</v>
       </c>
       <c r="C45" t="s">
         <v>52</v>
@@ -3137,7 +3137,7 @@
         <v>83</v>
       </c>
       <c r="B46" t="s">
-        <v>202</v>
+        <v>198</v>
       </c>
       <c r="C46" t="s">
         <v>52</v>
@@ -3172,7 +3172,7 @@
         <v>84</v>
       </c>
       <c r="B47" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C47" t="s">
         <v>52</v>
@@ -3207,7 +3207,7 @@
         <v>85</v>
       </c>
       <c r="B48" t="s">
-        <v>200</v>
+        <v>196</v>
       </c>
       <c r="C48" t="s">
         <v>52</v>
@@ -3382,7 +3382,7 @@
         <v>176</v>
       </c>
       <c r="B53" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C53" t="s">
         <v>52</v>
@@ -3417,7 +3417,7 @@
         <v>177</v>
       </c>
       <c r="B54" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C54" t="s">
         <v>52</v>
@@ -3662,7 +3662,7 @@
         <v>99</v>
       </c>
       <c r="B61" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C61" t="s">
         <v>52</v>
@@ -3697,7 +3697,7 @@
         <v>100</v>
       </c>
       <c r="B62" t="s">
-        <v>203</v>
+        <v>199</v>
       </c>
       <c r="C62" t="s">
         <v>52</v>
@@ -3767,7 +3767,7 @@
         <v>108</v>
       </c>
       <c r="B64" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="C64" t="s">
         <v>54</v>
@@ -3869,10 +3869,10 @@
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="B67" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="C67" t="s">
         <v>54</v>
@@ -3896,7 +3896,7 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="K67" t="s">
         <v>172</v>
@@ -4266,16 +4266,16 @@
         <v>25</v>
       </c>
       <c r="E78">
-        <v>5.0000000000000001E-4</v>
+        <v>1.2E-2</v>
       </c>
       <c r="F78">
-        <v>8.0000000000000004E-4</v>
+        <v>7.0000000000000001E-3</v>
       </c>
       <c r="G78">
-        <v>2.0000000000000001E-4</v>
+        <v>3.0000000000000001E-3</v>
       </c>
       <c r="H78">
-        <v>5.0000000000000001E-4</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="I78" t="b">
         <v>1</v>
@@ -4289,10 +4289,10 @@
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>193</v>
+        <v>219</v>
       </c>
       <c r="B79" t="s">
-        <v>194</v>
+        <v>220</v>
       </c>
       <c r="C79" t="s">
         <v>169</v>
@@ -4301,25 +4301,25 @@
         <v>25</v>
       </c>
       <c r="E79">
-        <v>0.05</v>
+        <v>1.1999999999999999E-3</v>
       </c>
       <c r="F79">
-        <v>0.08</v>
+        <v>6.9999999999999999E-4</v>
       </c>
       <c r="G79">
-        <v>0.02</v>
+        <v>2.9999999999999997E-4</v>
       </c>
       <c r="H79">
-        <v>0.05</v>
+        <v>5.9999999999999995E-4</v>
       </c>
       <c r="I79" t="b">
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>196</v>
+        <v>221</v>
       </c>
       <c r="K79" t="s">
-        <v>197</v>
+        <v>222</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
@@ -4327,7 +4327,7 @@
         <v>11</v>
       </c>
       <c r="B80" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C80" t="s">
         <v>169</v>

</xml_diff>

<commit_message>
Updated targets for ex_variant_call_eligible_disagree_rate, based on 20251002 Required strand disagreement rates analysis
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-24.04\home\jamesphie\codec-opensource\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7813D0D-797C-4744-BF26-FF11480F7186}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C400125-7A80-43BB-A6A2-41EC36C36557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -1575,19 +1575,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
   <dimension ref="A1:K82"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="35.140625" customWidth="1"/>
-    <col min="2" max="2" width="123.140625" customWidth="1"/>
-    <col min="3" max="4" width="35.28515625" customWidth="1"/>
+    <col min="1" max="1" width="35.1796875" customWidth="1"/>
+    <col min="2" max="2" width="123.1796875" customWidth="1"/>
+    <col min="3" max="4" width="35.26953125" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" customWidth="1"/>
-    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="76.85546875" customWidth="1"/>
+    <col min="9" max="9" width="12.81640625" customWidth="1"/>
+    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="76.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>32</v>
       </c>
@@ -1622,7 +1622,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>34</v>
       </c>
@@ -1651,7 +1651,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>35</v>
       </c>
@@ -1686,7 +1686,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>36</v>
       </c>
@@ -1721,7 +1721,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>44</v>
       </c>
@@ -1750,7 +1750,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -1785,7 +1785,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>45</v>
       </c>
@@ -1814,7 +1814,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>46</v>
       </c>
@@ -1849,7 +1849,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1884,7 +1884,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>24</v>
       </c>
@@ -1919,7 +1919,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -1954,7 +1954,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -1989,7 +1989,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>88</v>
       </c>
@@ -2024,7 +2024,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>89</v>
       </c>
@@ -2059,7 +2059,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>86</v>
       </c>
@@ -2094,7 +2094,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>87</v>
       </c>
@@ -2129,7 +2129,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>78</v>
       </c>
@@ -2164,7 +2164,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>79</v>
       </c>
@@ -2199,7 +2199,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>178</v>
       </c>
@@ -2234,7 +2234,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>179</v>
       </c>
@@ -2269,7 +2269,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>67</v>
       </c>
@@ -2304,7 +2304,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>68</v>
       </c>
@@ -2339,7 +2339,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>69</v>
       </c>
@@ -2374,7 +2374,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>70</v>
       </c>
@@ -2409,7 +2409,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>71</v>
       </c>
@@ -2444,7 +2444,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>72</v>
       </c>
@@ -2479,7 +2479,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>73</v>
       </c>
@@ -2514,7 +2514,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>74</v>
       </c>
@@ -2549,7 +2549,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>217</v>
       </c>
@@ -2584,7 +2584,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>113</v>
       </c>
@@ -2619,7 +2619,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>112</v>
       </c>
@@ -2654,7 +2654,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>201</v>
       </c>
@@ -2689,7 +2689,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>111</v>
       </c>
@@ -2724,7 +2724,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>211</v>
       </c>
@@ -2759,7 +2759,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>59</v>
       </c>
@@ -2794,7 +2794,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>20</v>
       </c>
@@ -2823,7 +2823,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>27</v>
       </c>
@@ -2858,7 +2858,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>33</v>
       </c>
@@ -2893,7 +2893,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>41</v>
       </c>
@@ -2922,7 +2922,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>37</v>
       </c>
@@ -2957,7 +2957,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>38</v>
       </c>
@@ -2992,7 +2992,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>39</v>
       </c>
@@ -3027,7 +3027,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>21</v>
       </c>
@@ -3062,7 +3062,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>22</v>
       </c>
@@ -3097,7 +3097,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>82</v>
       </c>
@@ -3132,7 +3132,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>83</v>
       </c>
@@ -3167,7 +3167,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>84</v>
       </c>
@@ -3202,7 +3202,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>85</v>
       </c>
@@ -3237,7 +3237,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>81</v>
       </c>
@@ -3272,7 +3272,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>90</v>
       </c>
@@ -3307,7 +3307,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>91</v>
       </c>
@@ -3342,7 +3342,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>92</v>
       </c>
@@ -3377,7 +3377,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
         <v>176</v>
       </c>
@@ -3412,7 +3412,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
         <v>177</v>
       </c>
@@ -3447,7 +3447,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>93</v>
       </c>
@@ -3482,7 +3482,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>94</v>
       </c>
@@ -3517,7 +3517,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>95</v>
       </c>
@@ -3552,7 +3552,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>96</v>
       </c>
@@ -3587,7 +3587,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>97</v>
       </c>
@@ -3622,7 +3622,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>98</v>
       </c>
@@ -3657,7 +3657,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>99</v>
       </c>
@@ -3692,7 +3692,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>100</v>
       </c>
@@ -3727,7 +3727,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>60</v>
       </c>
@@ -3762,7 +3762,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>108</v>
       </c>
@@ -3797,7 +3797,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
         <v>170</v>
       </c>
@@ -3832,7 +3832,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
         <v>192</v>
       </c>
@@ -3867,7 +3867,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
         <v>214</v>
       </c>
@@ -3902,7 +3902,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>63</v>
       </c>
@@ -3937,7 +3937,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>62</v>
       </c>
@@ -3972,7 +3972,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>64</v>
       </c>
@@ -4007,7 +4007,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>120</v>
       </c>
@@ -4042,7 +4042,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
         <v>110</v>
       </c>
@@ -4077,7 +4077,7 @@
         <v>161</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>116</v>
       </c>
@@ -4112,7 +4112,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>115</v>
       </c>
@@ -4147,7 +4147,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
         <v>117</v>
       </c>
@@ -4182,7 +4182,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>14</v>
       </c>
@@ -4217,7 +4217,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
         <v>12</v>
       </c>
@@ -4252,7 +4252,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -4287,7 +4287,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
         <v>219</v>
       </c>
@@ -4301,16 +4301,16 @@
         <v>25</v>
       </c>
       <c r="E79">
-        <v>1.1999999999999999E-3</v>
+        <v>3.2679999999999997E-4</v>
       </c>
       <c r="F79">
-        <v>6.9999999999999999E-4</v>
+        <v>5.6599999999999999E-4</v>
       </c>
       <c r="G79">
-        <v>2.9999999999999997E-4</v>
+        <v>2.5179999999999999E-4</v>
       </c>
       <c r="H79">
-        <v>5.9999999999999995E-4</v>
+        <v>3.2679999999999997E-4</v>
       </c>
       <c r="I79" t="b">
         <v>1</v>
@@ -4322,7 +4322,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
         <v>11</v>
       </c>
@@ -4357,7 +4357,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>17</v>
       </c>
@@ -4392,7 +4392,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
         <v>47</v>
       </c>

</xml_diff>

<commit_message>
Updated thresholds for ex_variant_call_eligible_disagree_rate
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C400125-7A80-43BB-A6A2-41EC36C36557}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F5BC0F0-2AC2-43FB-B6AE-C263CDA9EECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -1188,8 +1188,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -4287,38 +4288,38 @@
         <v>173</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A79" t="s">
+    <row r="79" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.35">
+      <c r="A79" s="1" t="s">
         <v>219</v>
       </c>
-      <c r="B79" t="s">
+      <c r="B79" s="1" t="s">
         <v>220</v>
       </c>
-      <c r="C79" t="s">
+      <c r="C79" s="1" t="s">
         <v>169</v>
       </c>
-      <c r="D79" t="s">
-        <v>25</v>
-      </c>
-      <c r="E79">
+      <c r="D79" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E79" s="1">
+        <v>0</v>
+      </c>
+      <c r="F79" s="1">
+        <v>5.6599999999999999E-4</v>
+      </c>
+      <c r="G79" s="1">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="H79" s="1">
         <v>3.2679999999999997E-4</v>
       </c>
-      <c r="F79">
-        <v>5.6599999999999999E-4</v>
-      </c>
-      <c r="G79">
-        <v>2.5179999999999999E-4</v>
-      </c>
-      <c r="H79">
-        <v>3.2679999999999997E-4</v>
-      </c>
-      <c r="I79" t="b">
-        <v>1</v>
-      </c>
-      <c r="J79" t="s">
+      <c r="I79" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="J79" s="1" t="s">
         <v>221</v>
       </c>
-      <c r="K79" t="s">
+      <c r="K79" s="1" t="s">
         <v>222</v>
       </c>
     </row>

</xml_diff>

<commit_message>
1. Updated external concordance definition and targets 2. Updated inaccurate component metric names
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\codec-opensource\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F5BC0F0-2AC2-43FB-B6AE-C263CDA9EECD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4CC4416-11BA-4B9C-93DC-8683A5386089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -89,9 +89,6 @@
     <t>Percentage of reads lost between start and end of ex pipeline</t>
   </si>
   <si>
-    <t>ex_lane_total_read_loss</t>
-  </si>
-  <si>
     <t>Mean length of the largest peak</t>
   </si>
   <si>
@@ -368,9 +365,6 @@
     <t>Median insert size (start of R1 to end of R2) as determined by initial alignment (bp)</t>
   </si>
   <si>
-    <t>ex_duplication_rate_initial_alignment</t>
-  </si>
-  <si>
     <t>ms_insert_size_alignment</t>
   </si>
   <si>
@@ -705,6 +699,12 @@
   </si>
   <si>
     <t>observed_disagreement_rate</t>
+  </si>
+  <si>
+    <t>ex_unique_reads_initial_alignment</t>
+  </si>
+  <si>
+    <t>ex_total_read_loss</t>
   </si>
 </sst>
 </file>
@@ -1188,9 +1188,8 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1576,30 +1575,30 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
   <dimension ref="A1:K82"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.1796875" customWidth="1"/>
-    <col min="2" max="2" width="123.1796875" customWidth="1"/>
-    <col min="3" max="4" width="35.26953125" customWidth="1"/>
+    <col min="1" max="1" width="35.140625" customWidth="1"/>
+    <col min="2" max="2" width="123.140625" customWidth="1"/>
+    <col min="3" max="4" width="35.28515625" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.81640625" customWidth="1"/>
-    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="76.81640625" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="76.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C1" t="s">
         <v>28</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>29</v>
-      </c>
-      <c r="D1" t="s">
-        <v>30</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -1614,27 +1613,27 @@
         <v>3</v>
       </c>
       <c r="I1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="J1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="K1" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E2">
         <v>2500</v>
@@ -1646,24 +1645,24 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C3" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1681,24 +1680,24 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E4">
         <v>90</v>
@@ -1716,24 +1715,24 @@
         <v>0</v>
       </c>
       <c r="J4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K4" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E5">
         <v>90</v>
@@ -1745,24 +1744,24 @@
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K5" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1780,24 +1779,24 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K6" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E7">
         <v>45</v>
@@ -1809,24 +1808,24 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K7" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -1844,24 +1843,24 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K8" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C9" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D9" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E9">
         <v>280</v>
@@ -1879,24 +1878,24 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K9" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D10" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E10">
         <v>95</v>
@@ -1914,24 +1913,24 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K10" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C11" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E11">
         <v>200</v>
@@ -1949,24 +1948,24 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K11" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C12" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D12" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E12">
         <v>200</v>
@@ -1984,24 +1983,24 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="K12" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B13" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C13" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D13" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E13">
         <v>35</v>
@@ -2019,24 +2018,24 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K13" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B14" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C14" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E14">
         <v>35</v>
@@ -2054,24 +2053,24 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="K14" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B15" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C15" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -2089,24 +2088,24 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K15" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B16" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D16" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -2124,24 +2123,24 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="K16" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B17" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C17" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D17" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E17">
         <v>150</v>
@@ -2159,24 +2158,24 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K17" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>78</v>
+      </c>
+      <c r="B18" t="s">
         <v>79</v>
       </c>
-      <c r="B18" t="s">
-        <v>80</v>
-      </c>
       <c r="C18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E18">
         <v>150</v>
@@ -2194,24 +2193,24 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="K18" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B19" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D19" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E19">
         <v>30</v>
@@ -2229,24 +2228,24 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K19" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B20" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C20" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D20" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E20">
         <v>30</v>
@@ -2264,24 +2263,24 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K20" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B21" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D21" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -2299,24 +2298,24 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K21" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B22" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C22" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D22" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -2334,24 +2333,24 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K22" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B23" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C23" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D23" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -2369,24 +2368,24 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K23" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B24" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C24" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D24" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -2404,24 +2403,24 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K24" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B25" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C25" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D25" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -2439,24 +2438,24 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K25" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B26" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C26" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D26" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E26">
         <v>0</v>
@@ -2474,24 +2473,24 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K26" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B27" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C27" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D27" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -2509,24 +2508,24 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K27" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B28" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C28" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D28" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -2544,24 +2543,24 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K28" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B29" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C29" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D29" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E29">
         <v>70</v>
@@ -2579,24 +2578,24 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="K29" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B30" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C30" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D30" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E30">
         <v>90</v>
@@ -2614,24 +2613,24 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K30" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="B31" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C31" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D31" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -2649,24 +2648,24 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="K31" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B32" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="C32" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D32" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E32">
         <v>21.75</v>
@@ -2684,24 +2683,24 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="K32" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B33" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C33" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D33" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E33">
         <v>125</v>
@@ -2719,24 +2718,24 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K33" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B34" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="C34" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D34" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E34">
         <v>1.5E-3</v>
@@ -2754,24 +2753,24 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="K34" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B35" t="s">
         <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D35" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E35">
         <v>70</v>
@@ -2789,24 +2788,24 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="K35" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B36" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C36" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D36" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E36">
         <v>75</v>
@@ -2818,24 +2817,24 @@
         <v>0</v>
       </c>
       <c r="J36" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K36" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B37" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C37" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D37" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E37">
         <v>0</v>
@@ -2853,24 +2852,24 @@
         <v>0</v>
       </c>
       <c r="J37" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K37" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B38" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C38" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D38" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E38">
         <v>80</v>
@@ -2888,24 +2887,24 @@
         <v>0</v>
       </c>
       <c r="J38" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K38" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>40</v>
+      </c>
+      <c r="B39" t="s">
         <v>41</v>
       </c>
-      <c r="B39" t="s">
-        <v>42</v>
-      </c>
       <c r="C39" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D39" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E39">
         <v>4.3</v>
@@ -2917,24 +2916,24 @@
         <v>0</v>
       </c>
       <c r="J39" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K39" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B40" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C40" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D40" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E40">
         <v>0</v>
@@ -2952,24 +2951,24 @@
         <v>0</v>
       </c>
       <c r="J40" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K40" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B41" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C41" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D41" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E41">
         <v>80</v>
@@ -2987,24 +2986,24 @@
         <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K41" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B42" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C42" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D42" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -3022,24 +3021,24 @@
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K42" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B43" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C43" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D43" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E43">
         <v>544</v>
@@ -3057,24 +3056,24 @@
         <v>0</v>
       </c>
       <c r="J43" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K43" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B44" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C44" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D44" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E44">
         <v>98</v>
@@ -3092,24 +3091,24 @@
         <v>0</v>
       </c>
       <c r="J44" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K44" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B45" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C45" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D45" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E45">
         <v>35</v>
@@ -3127,24 +3126,24 @@
         <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K45" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B46" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C46" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D46" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E46">
         <v>35</v>
@@ -3162,24 +3161,24 @@
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K46" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B47" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C47" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D47" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E47">
         <v>0</v>
@@ -3197,24 +3196,24 @@
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K47" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B48" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C48" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D48" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E48">
         <v>0</v>
@@ -3232,24 +3231,24 @@
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K48" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B49" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C49" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D49" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E49">
         <v>150</v>
@@ -3267,24 +3266,24 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K49" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B50" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C50" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D50" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E50">
         <v>150</v>
@@ -3302,24 +3301,24 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K50" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B51" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C51" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D51" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E51">
         <v>2850</v>
@@ -3337,24 +3336,24 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K51" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B52" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C52" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D52" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E52">
         <v>2850</v>
@@ -3372,24 +3371,24 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K52" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B53" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C53" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D53" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E53">
         <v>30</v>
@@ -3407,24 +3406,24 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K53" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B54" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C54" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D54" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E54">
         <v>30</v>
@@ -3442,24 +3441,24 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K54" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B55" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C55" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D55" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E55">
         <v>0</v>
@@ -3477,24 +3476,24 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K55" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B56" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C56" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D56" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E56">
         <v>0</v>
@@ -3512,24 +3511,24 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K56" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B57" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C57" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D57" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E57">
         <v>0</v>
@@ -3547,24 +3546,24 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K57" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B58" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C58" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D58" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E58">
         <v>0</v>
@@ -3582,24 +3581,24 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K58" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B59" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C59" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D59" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E59">
         <v>0</v>
@@ -3617,24 +3616,24 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K59" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="B60" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C60" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D60" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E60">
         <v>0</v>
@@ -3652,24 +3651,24 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K60" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="B61" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C61" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D61" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E61">
         <v>0</v>
@@ -3687,24 +3686,24 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K61" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B62" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="C62" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D62" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E62">
         <v>0</v>
@@ -3722,24 +3721,24 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="K62" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>59</v>
+      </c>
+      <c r="B63" t="s">
+        <v>186</v>
+      </c>
+      <c r="C63" t="s">
+        <v>53</v>
+      </c>
+      <c r="D63" t="s">
         <v>60</v>
-      </c>
-      <c r="B63" t="s">
-        <v>188</v>
-      </c>
-      <c r="C63" t="s">
-        <v>54</v>
-      </c>
-      <c r="D63" t="s">
-        <v>61</v>
       </c>
       <c r="E63">
         <v>0</v>
@@ -3757,24 +3756,24 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="K63" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B64" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C64" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D64" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E64">
         <v>0</v>
@@ -3792,24 +3791,24 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="K64" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B65" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C65" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D65" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E65">
         <v>1</v>
@@ -3827,24 +3826,24 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="K65" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B66" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C66" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D66" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E66">
         <v>0</v>
@@ -3862,24 +3861,24 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="K66" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B67" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="C67" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D67" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E67">
         <v>70</v>
@@ -3897,24 +3896,24 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="K67" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B68" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C68" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D68" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E68">
         <v>90</v>
@@ -3932,24 +3931,24 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="K68" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B69" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C69" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D69" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E69">
         <v>50</v>
@@ -3967,24 +3966,24 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="K69" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B70" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C70" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D70" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E70">
         <v>125</v>
@@ -4002,24 +4001,24 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="K70" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="B71" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C71" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D71" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E71">
         <v>50</v>
@@ -4037,24 +4036,24 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="K71" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>110</v>
+        <v>221</v>
       </c>
       <c r="B72" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C72" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D72" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E72">
         <v>60</v>
@@ -4072,24 +4071,24 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="K72" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B73" t="s">
         <v>10</v>
       </c>
       <c r="C73" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D73" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E73">
         <v>99</v>
@@ -4107,24 +4106,24 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="K73" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="B74" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C74" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D74" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E74">
         <v>0</v>
@@ -4142,24 +4141,24 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="K74" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="B75" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C75" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D75" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E75">
         <v>0.5</v>
@@ -4177,13 +4176,13 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="K75" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>14</v>
       </c>
@@ -4191,10 +4190,10 @@
         <v>15</v>
       </c>
       <c r="C76" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D76" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E76">
         <v>0</v>
@@ -4212,13 +4211,13 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K76" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>12</v>
       </c>
@@ -4226,10 +4225,10 @@
         <v>13</v>
       </c>
       <c r="C77" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D77" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E77">
         <v>14.5</v>
@@ -4247,13 +4246,13 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="K77" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -4261,10 +4260,10 @@
         <v>9</v>
       </c>
       <c r="C78" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D78" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E78">
         <v>1.2E-2</v>
@@ -4282,59 +4281,59 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="K78" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" s="1" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="A79" s="1" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>217</v>
+      </c>
+      <c r="B79" t="s">
+        <v>218</v>
+      </c>
+      <c r="C79" t="s">
+        <v>167</v>
+      </c>
+      <c r="D79" t="s">
+        <v>24</v>
+      </c>
+      <c r="E79">
+        <v>0</v>
+      </c>
+      <c r="F79">
+        <v>5.6599999999999999E-4</v>
+      </c>
+      <c r="G79">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="H79">
+        <v>3.2679999999999997E-4</v>
+      </c>
+      <c r="I79" t="b">
+        <v>1</v>
+      </c>
+      <c r="J79" t="s">
         <v>219</v>
       </c>
-      <c r="B79" s="1" t="s">
+      <c r="K79" t="s">
         <v>220</v>
       </c>
-      <c r="C79" s="1" t="s">
-        <v>169</v>
-      </c>
-      <c r="D79" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="E79" s="1">
-        <v>0</v>
-      </c>
-      <c r="F79" s="1">
-        <v>5.6599999999999999E-4</v>
-      </c>
-      <c r="G79" s="1">
-        <v>2.0000000000000001E-4</v>
-      </c>
-      <c r="H79" s="1">
-        <v>3.2679999999999997E-4</v>
-      </c>
-      <c r="I79" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="J79" s="1" t="s">
-        <v>221</v>
-      </c>
-      <c r="K79" s="1" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>11</v>
       </c>
       <c r="B80" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C80" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D80" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E80">
         <v>5</v>
@@ -4352,24 +4351,24 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="K80" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>17</v>
+        <v>222</v>
       </c>
       <c r="B81" t="s">
         <v>16</v>
       </c>
       <c r="C81" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D81" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E81">
         <v>0</v>
@@ -4387,24 +4386,24 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="K81" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B82" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C82" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="D82" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E82">
         <v>33</v>
@@ -4422,10 +4421,10 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="K82" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated thresholds for ex_duplex_base_disagreement
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4CC4416-11BA-4B9C-93DC-8683A5386089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55EF1CB1-8E1E-4507-94F9-0622EDD3DF79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -4266,13 +4266,13 @@
         <v>24</v>
       </c>
       <c r="E78">
+        <v>0</v>
+      </c>
+      <c r="F78">
         <v>1.2E-2</v>
       </c>
-      <c r="F78">
-        <v>7.0000000000000001E-3</v>
-      </c>
       <c r="G78">
-        <v>3.0000000000000001E-3</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="H78">
         <v>6.0000000000000001E-3</v>

</xml_diff>

<commit_message>
1. Modified thresholds for ex_insert_size metric 2. Changed ex_uniformity_snv_position metric from mean to 80th percentile, modified thresholds 3. Removed uniformity_chromosomal_SNV_rate metric 4. Removed inter_batch_precision metric
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55EF1CB1-8E1E-4507-94F9-0622EDD3DF79}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{674ED3A6-B0A3-4BEF-B989-095BB37EFB69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -3986,10 +3986,10 @@
         <v>24</v>
       </c>
       <c r="E70">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="F70">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="G70">
         <v>140</v>

</xml_diff>

<commit_message>
Added component metric for ex_duplex_overlap
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{674ED3A6-B0A3-4BEF-B989-095BB37EFB69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6653BEC-37C3-4C5F-93DB-5B158C64AFEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$80</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$81</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="227">
   <si>
     <t>nn_lower</t>
   </si>
@@ -705,6 +705,18 @@
   </si>
   <si>
     <t>ex_total_read_loss</t>
+  </si>
+  <si>
+    <t>ex_duplex_overlap</t>
+  </si>
+  <si>
+    <t>_duplex_overlap_metrics.json</t>
+  </si>
+  <si>
+    <t>50th percentile for length of overlap between R1 and R2 in each duplex sequence</t>
+  </si>
+  <si>
+    <t>overlap_percentiles.value.50</t>
   </si>
 </sst>
 </file>
@@ -1574,7 +1586,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K82"/>
+  <dimension ref="A1:K83"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" customWidth="1"/>
@@ -4289,45 +4301,45 @@
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="B79" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="C79" t="s">
-        <v>167</v>
+        <v>56</v>
       </c>
       <c r="D79" t="s">
         <v>24</v>
       </c>
       <c r="E79">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="F79">
-        <v>5.6599999999999999E-4</v>
+        <v>120</v>
       </c>
       <c r="G79">
-        <v>2.0000000000000001E-4</v>
+        <v>82.8</v>
       </c>
       <c r="H79">
-        <v>3.2679999999999997E-4</v>
+        <v>120</v>
       </c>
       <c r="I79" t="b">
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="K79" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>11</v>
+        <v>217</v>
       </c>
       <c r="B80" t="s">
-        <v>191</v>
+        <v>218</v>
       </c>
       <c r="C80" t="s">
         <v>167</v>
@@ -4336,33 +4348,33 @@
         <v>24</v>
       </c>
       <c r="E80">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F80">
-        <v>100</v>
+        <v>5.6599999999999999E-4</v>
       </c>
       <c r="G80">
-        <v>20</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="H80">
-        <v>100</v>
+        <v>3.2679999999999997E-4</v>
       </c>
       <c r="I80" t="b">
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>161</v>
+        <v>219</v>
       </c>
       <c r="K80" t="s">
-        <v>152</v>
+        <v>220</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>222</v>
+        <v>11</v>
       </c>
       <c r="B81" t="s">
-        <v>16</v>
+        <v>191</v>
       </c>
       <c r="C81" t="s">
         <v>167</v>
@@ -4371,33 +4383,33 @@
         <v>24</v>
       </c>
       <c r="E81">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F81">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="G81">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H81">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="I81" t="b">
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>134</v>
+        <v>161</v>
       </c>
       <c r="K81" t="s">
-        <v>156</v>
+        <v>152</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>46</v>
+        <v>222</v>
       </c>
       <c r="B82" t="s">
-        <v>179</v>
+        <v>16</v>
       </c>
       <c r="C82" t="s">
         <v>167</v>
@@ -4406,29 +4418,64 @@
         <v>24</v>
       </c>
       <c r="E82">
+        <v>0</v>
+      </c>
+      <c r="F82">
+        <v>95</v>
+      </c>
+      <c r="G82">
+        <v>0</v>
+      </c>
+      <c r="H82">
+        <v>80</v>
+      </c>
+      <c r="I82" t="b">
+        <v>1</v>
+      </c>
+      <c r="J82" t="s">
+        <v>134</v>
+      </c>
+      <c r="K82" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>46</v>
+      </c>
+      <c r="B83" t="s">
+        <v>179</v>
+      </c>
+      <c r="C83" t="s">
+        <v>167</v>
+      </c>
+      <c r="D83" t="s">
+        <v>24</v>
+      </c>
+      <c r="E83">
         <v>33</v>
       </c>
-      <c r="F82">
+      <c r="F83">
         <v>100</v>
       </c>
-      <c r="G82">
+      <c r="G83">
         <v>67</v>
       </c>
-      <c r="H82">
+      <c r="H83">
         <v>100</v>
       </c>
-      <c r="I82" t="b">
-        <v>1</v>
-      </c>
-      <c r="J82" t="s">
+      <c r="I83" t="b">
+        <v>1</v>
+      </c>
+      <c r="J83" t="s">
         <v>161</v>
       </c>
-      <c r="K82" t="s">
+      <c r="K83" t="s">
         <v>46</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K80" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K81" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
ex_dsc_coverage_metrics.py now calculates the percentage of bases with EX but not MS depth and vice versa
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6653BEC-37C3-4C5F-93DB-5B158C64AFEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84F5B1BE-59A3-453B-B544-AEC962AE2166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metrics!$A$1:$K$83</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="229">
   <si>
     <t>nn_lower</t>
   </si>
@@ -491,12 +491,6 @@
     <t>_dsc_remap_metrics.json</t>
   </si>
   <si>
-    <t>ex_mean_analyzable_duplex_depth</t>
-  </si>
-  <si>
-    <t>ex_dsc_coverage_wholegenome</t>
-  </si>
-  <si>
     <t>^\d+ \+ 0 mapped \((?P&lt;percent&gt;[\d.]+)% : N/A\)$</t>
   </si>
   <si>
@@ -717,6 +711,18 @@
   </si>
   <si>
     <t>overlap_percentiles.value.50</t>
+  </si>
+  <si>
+    <t>ex_mean_analyzable_duplex_depth.value</t>
+  </si>
+  <si>
+    <t>ex_duplex_coverage.value</t>
+  </si>
+  <si>
+    <t>ex_dsc_coverage_wholegenome.value</t>
+  </si>
+  <si>
+    <t>coverage_overlap_ex_ms.value</t>
   </si>
 </sst>
 </file>
@@ -1586,6 +1592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:K83"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1634,12 +1641,12 @@
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C2" t="s">
         <v>47</v>
@@ -1663,12 +1670,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C3" t="s">
         <v>47</v>
@@ -1698,12 +1705,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C4" t="s">
         <v>47</v>
@@ -1733,12 +1740,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>43</v>
       </c>
       <c r="B5" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C5" t="s">
         <v>49</v>
@@ -1762,12 +1769,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C6" t="s">
         <v>49</v>
@@ -1797,12 +1804,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C7" t="s">
         <v>49</v>
@@ -1826,12 +1833,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C8" t="s">
         <v>49</v>
@@ -1861,7 +1868,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1896,7 +1903,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -1931,7 +1938,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -1966,7 +1973,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -2001,12 +2008,12 @@
         <v>135</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>87</v>
       </c>
       <c r="B13" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C13" t="s">
         <v>52</v>
@@ -2036,12 +2043,12 @@
         <v>136</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>88</v>
       </c>
       <c r="B14" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C14" t="s">
         <v>52</v>
@@ -2071,12 +2078,12 @@
         <v>136</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>85</v>
       </c>
       <c r="B15" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C15" t="s">
         <v>52</v>
@@ -2106,12 +2113,12 @@
         <v>138</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>86</v>
       </c>
       <c r="B16" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C16" t="s">
         <v>52</v>
@@ -2141,7 +2148,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>77</v>
       </c>
@@ -2176,7 +2183,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>78</v>
       </c>
@@ -2211,12 +2218,12 @@
         <v>139</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B19" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C19" t="s">
         <v>52</v>
@@ -2246,12 +2253,12 @@
         <v>137</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B20" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C20" t="s">
         <v>52</v>
@@ -2281,7 +2288,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>66</v>
       </c>
@@ -2316,7 +2323,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>67</v>
       </c>
@@ -2351,7 +2358,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>68</v>
       </c>
@@ -2386,7 +2393,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>69</v>
       </c>
@@ -2421,7 +2428,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>70</v>
       </c>
@@ -2456,7 +2463,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>71</v>
       </c>
@@ -2491,12 +2498,12 @@
         <v>142</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>72</v>
       </c>
       <c r="B27" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C27" t="s">
         <v>52</v>
@@ -2526,12 +2533,12 @@
         <v>143</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>73</v>
       </c>
       <c r="B28" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C28" t="s">
         <v>52</v>
@@ -2561,12 +2568,12 @@
         <v>143</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B29" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C29" t="s">
         <v>54</v>
@@ -2590,13 +2597,13 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="K29" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>111</v>
       </c>
@@ -2628,10 +2635,10 @@
         <v>128</v>
       </c>
       <c r="K30" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>110</v>
       </c>
@@ -2660,18 +2667,18 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="K31" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B32" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C32" t="s">
         <v>55</v>
@@ -2695,13 +2702,13 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="K32" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>109</v>
       </c>
@@ -2733,18 +2740,18 @@
         <v>129</v>
       </c>
       <c r="K33" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B34" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C34" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="D34" t="s">
         <v>24</v>
@@ -2765,13 +2772,13 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="K34" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>58</v>
       </c>
@@ -2779,7 +2786,7 @@
         <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="D35" t="s">
         <v>24</v>
@@ -2800,13 +2807,13 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="K35" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>19</v>
       </c>
@@ -2835,12 +2842,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>26</v>
       </c>
       <c r="B37" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C37" t="s">
         <v>48</v>
@@ -2870,12 +2877,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>32</v>
       </c>
       <c r="B38" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C38" t="s">
         <v>48</v>
@@ -2905,7 +2912,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>40</v>
       </c>
@@ -2934,12 +2941,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>36</v>
       </c>
       <c r="B40" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C40" t="s">
         <v>48</v>
@@ -2969,12 +2976,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>37</v>
       </c>
       <c r="B41" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C41" t="s">
         <v>48</v>
@@ -3004,12 +3011,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>38</v>
       </c>
       <c r="B42" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C42" t="s">
         <v>48</v>
@@ -3039,7 +3046,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>20</v>
       </c>
@@ -3074,7 +3081,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>21</v>
       </c>
@@ -3109,12 +3116,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>81</v>
       </c>
       <c r="B45" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C45" t="s">
         <v>51</v>
@@ -3144,12 +3151,12 @@
         <v>136</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>82</v>
       </c>
       <c r="B46" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C46" t="s">
         <v>51</v>
@@ -3179,12 +3186,12 @@
         <v>136</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>83</v>
       </c>
       <c r="B47" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C47" t="s">
         <v>51</v>
@@ -3214,12 +3221,12 @@
         <v>138</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>84</v>
       </c>
       <c r="B48" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C48" t="s">
         <v>51</v>
@@ -3249,7 +3256,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>80</v>
       </c>
@@ -3284,7 +3291,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>89</v>
       </c>
@@ -3319,7 +3326,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>90</v>
       </c>
@@ -3354,7 +3361,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>91</v>
       </c>
@@ -3389,12 +3396,12 @@
         <v>135</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B53" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C53" t="s">
         <v>51</v>
@@ -3424,12 +3431,12 @@
         <v>137</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B54" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C54" t="s">
         <v>51</v>
@@ -3459,7 +3466,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>92</v>
       </c>
@@ -3494,7 +3501,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>93</v>
       </c>
@@ -3529,7 +3536,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>94</v>
       </c>
@@ -3564,7 +3571,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>95</v>
       </c>
@@ -3599,7 +3606,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>96</v>
       </c>
@@ -3634,7 +3641,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>97</v>
       </c>
@@ -3669,12 +3676,12 @@
         <v>142</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>98</v>
       </c>
       <c r="B61" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C61" t="s">
         <v>51</v>
@@ -3704,12 +3711,12 @@
         <v>143</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>99</v>
       </c>
       <c r="B62" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C62" t="s">
         <v>51</v>
@@ -3739,12 +3746,12 @@
         <v>143</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>59</v>
       </c>
       <c r="B63" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C63" t="s">
         <v>53</v>
@@ -3768,18 +3775,18 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="K63" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>107</v>
       </c>
       <c r="B64" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C64" t="s">
         <v>53</v>
@@ -3803,18 +3810,18 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="K64" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B65" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C65" t="s">
         <v>53</v>
@@ -3838,18 +3845,18 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="K65" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B66" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C66" t="s">
         <v>53</v>
@@ -3873,18 +3880,18 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="K66" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B67" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C67" t="s">
         <v>53</v>
@@ -3908,13 +3915,13 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="K67" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>62</v>
       </c>
@@ -3946,10 +3953,10 @@
         <v>121</v>
       </c>
       <c r="K68" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>61</v>
       </c>
@@ -3981,10 +3988,10 @@
         <v>121</v>
       </c>
       <c r="K69" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>63</v>
       </c>
@@ -4016,15 +4023,15 @@
         <v>122</v>
       </c>
       <c r="K70" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>118</v>
       </c>
       <c r="B71" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C71" t="s">
         <v>56</v>
@@ -4054,12 +4061,12 @@
         <v>147</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B72" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C72" t="s">
         <v>56</v>
@@ -4083,13 +4090,13 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="K72" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>114</v>
       </c>
@@ -4124,7 +4131,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>113</v>
       </c>
@@ -4188,13 +4195,13 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K75" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>14</v>
       </c>
@@ -4258,13 +4265,13 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K77" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -4293,18 +4300,18 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="K78" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
+        <v>221</v>
+      </c>
+      <c r="B79" t="s">
         <v>223</v>
-      </c>
-      <c r="B79" t="s">
-        <v>225</v>
       </c>
       <c r="C79" t="s">
         <v>56</v>
@@ -4328,21 +4335,21 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
+        <v>222</v>
+      </c>
+      <c r="K79" t="s">
         <v>224</v>
       </c>
-      <c r="K79" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="80" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B80" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C80" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D80" t="s">
         <v>24</v>
@@ -4363,10 +4370,10 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="K80" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
@@ -4374,10 +4381,10 @@
         <v>11</v>
       </c>
       <c r="B81" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C81" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D81" t="s">
         <v>24</v>
@@ -4398,21 +4405,21 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K81" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B82" t="s">
         <v>16</v>
       </c>
       <c r="C82" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D82" t="s">
         <v>24</v>
@@ -4436,7 +4443,7 @@
         <v>134</v>
       </c>
       <c r="K82" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
@@ -4444,10 +4451,10 @@
         <v>46</v>
       </c>
       <c r="B83" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C83" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="D83" t="s">
         <v>24</v>
@@ -4468,14 +4475,20 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="K83" t="s">
-        <v>46</v>
+        <v>228</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K81" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K83" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
+    <filterColumn colId="9">
+      <filters>
+        <filter val="_dsc_coverage_metrics.json"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Revert "ex_dsc_coverage_metrics.py now calculates the percentage of bases with EX but not MS depth and vice versa"
This reverts commit f845c52a09f24254e9d34bec07eecdf9c30a4ace.
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84F5B1BE-59A3-453B-B544-AEC962AE2166}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6653BEC-37C3-4C5F-93DB-5B158C64AFEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metrics!$A$1:$K$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$81</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="227">
   <si>
     <t>nn_lower</t>
   </si>
@@ -491,6 +491,12 @@
     <t>_dsc_remap_metrics.json</t>
   </si>
   <si>
+    <t>ex_mean_analyzable_duplex_depth</t>
+  </si>
+  <si>
+    <t>ex_dsc_coverage_wholegenome</t>
+  </si>
+  <si>
     <t>^\d+ \+ 0 mapped \((?P&lt;percent&gt;[\d.]+)% : N/A\)$</t>
   </si>
   <si>
@@ -711,18 +717,6 @@
   </si>
   <si>
     <t>overlap_percentiles.value.50</t>
-  </si>
-  <si>
-    <t>ex_mean_analyzable_duplex_depth.value</t>
-  </si>
-  <si>
-    <t>ex_duplex_coverage.value</t>
-  </si>
-  <si>
-    <t>ex_dsc_coverage_wholegenome.value</t>
-  </si>
-  <si>
-    <t>coverage_overlap_ex_ms.value</t>
   </si>
 </sst>
 </file>
@@ -1592,7 +1586,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:K83"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1641,12 +1634,12 @@
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C2" t="s">
         <v>47</v>
@@ -1670,12 +1663,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C3" t="s">
         <v>47</v>
@@ -1705,12 +1698,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="C4" t="s">
         <v>47</v>
@@ -1740,12 +1733,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>43</v>
       </c>
       <c r="B5" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="C5" t="s">
         <v>49</v>
@@ -1769,12 +1762,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C6" t="s">
         <v>49</v>
@@ -1804,12 +1797,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C7" t="s">
         <v>49</v>
@@ -1833,12 +1826,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="C8" t="s">
         <v>49</v>
@@ -1868,7 +1861,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1903,7 +1896,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -1938,7 +1931,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -1973,7 +1966,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -2008,12 +2001,12 @@
         <v>135</v>
       </c>
     </row>
-    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>87</v>
       </c>
       <c r="B13" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C13" t="s">
         <v>52</v>
@@ -2043,12 +2036,12 @@
         <v>136</v>
       </c>
     </row>
-    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>88</v>
       </c>
       <c r="B14" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C14" t="s">
         <v>52</v>
@@ -2078,12 +2071,12 @@
         <v>136</v>
       </c>
     </row>
-    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>85</v>
       </c>
       <c r="B15" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C15" t="s">
         <v>52</v>
@@ -2113,12 +2106,12 @@
         <v>138</v>
       </c>
     </row>
-    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>86</v>
       </c>
       <c r="B16" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C16" t="s">
         <v>52</v>
@@ -2148,7 +2141,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>77</v>
       </c>
@@ -2183,7 +2176,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>78</v>
       </c>
@@ -2218,12 +2211,12 @@
         <v>139</v>
       </c>
     </row>
-    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="B19" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C19" t="s">
         <v>52</v>
@@ -2253,12 +2246,12 @@
         <v>137</v>
       </c>
     </row>
-    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="B20" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C20" t="s">
         <v>52</v>
@@ -2288,7 +2281,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>66</v>
       </c>
@@ -2323,7 +2316,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>67</v>
       </c>
@@ -2358,7 +2351,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>68</v>
       </c>
@@ -2393,7 +2386,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>69</v>
       </c>
@@ -2428,7 +2421,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="25" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>70</v>
       </c>
@@ -2463,7 +2456,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>71</v>
       </c>
@@ -2498,12 +2491,12 @@
         <v>142</v>
       </c>
     </row>
-    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>72</v>
       </c>
       <c r="B27" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C27" t="s">
         <v>52</v>
@@ -2533,12 +2526,12 @@
         <v>143</v>
       </c>
     </row>
-    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>73</v>
       </c>
       <c r="B28" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C28" t="s">
         <v>52</v>
@@ -2568,12 +2561,12 @@
         <v>143</v>
       </c>
     </row>
-    <row r="29" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
+        <v>215</v>
+      </c>
+      <c r="B29" t="s">
         <v>213</v>
-      </c>
-      <c r="B29" t="s">
-        <v>211</v>
       </c>
       <c r="C29" t="s">
         <v>54</v>
@@ -2597,13 +2590,13 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="K29" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>111</v>
       </c>
@@ -2635,10 +2628,10 @@
         <v>128</v>
       </c>
       <c r="K30" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>110</v>
       </c>
@@ -2667,18 +2660,18 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="K31" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B32" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="C32" t="s">
         <v>55</v>
@@ -2702,13 +2695,13 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="K32" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>109</v>
       </c>
@@ -2740,18 +2733,18 @@
         <v>129</v>
       </c>
       <c r="K33" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="B34" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="C34" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D34" t="s">
         <v>24</v>
@@ -2772,13 +2765,13 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="K34" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>58</v>
       </c>
@@ -2786,7 +2779,7 @@
         <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="D35" t="s">
         <v>24</v>
@@ -2807,13 +2800,13 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="K35" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>19</v>
       </c>
@@ -2842,12 +2835,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>26</v>
       </c>
       <c r="B37" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C37" t="s">
         <v>48</v>
@@ -2877,12 +2870,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>32</v>
       </c>
       <c r="B38" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="C38" t="s">
         <v>48</v>
@@ -2912,7 +2905,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>40</v>
       </c>
@@ -2941,12 +2934,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>36</v>
       </c>
       <c r="B40" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="C40" t="s">
         <v>48</v>
@@ -2976,12 +2969,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="41" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>37</v>
       </c>
       <c r="B41" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C41" t="s">
         <v>48</v>
@@ -3011,12 +3004,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="42" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>38</v>
       </c>
       <c r="B42" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="C42" t="s">
         <v>48</v>
@@ -3046,7 +3039,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="43" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>20</v>
       </c>
@@ -3081,7 +3074,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>21</v>
       </c>
@@ -3116,12 +3109,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>81</v>
       </c>
       <c r="B45" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="C45" t="s">
         <v>51</v>
@@ -3151,12 +3144,12 @@
         <v>136</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>82</v>
       </c>
       <c r="B46" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="C46" t="s">
         <v>51</v>
@@ -3186,12 +3179,12 @@
         <v>136</v>
       </c>
     </row>
-    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>83</v>
       </c>
       <c r="B47" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C47" t="s">
         <v>51</v>
@@ -3221,12 +3214,12 @@
         <v>138</v>
       </c>
     </row>
-    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>84</v>
       </c>
       <c r="B48" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C48" t="s">
         <v>51</v>
@@ -3256,7 +3249,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="49" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>80</v>
       </c>
@@ -3291,7 +3284,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="50" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>89</v>
       </c>
@@ -3326,7 +3319,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="51" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>90</v>
       </c>
@@ -3361,7 +3354,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="52" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>91</v>
       </c>
@@ -3396,12 +3389,12 @@
         <v>135</v>
       </c>
     </row>
-    <row r="53" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="B53" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C53" t="s">
         <v>51</v>
@@ -3431,12 +3424,12 @@
         <v>137</v>
       </c>
     </row>
-    <row r="54" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B54" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="C54" t="s">
         <v>51</v>
@@ -3466,7 +3459,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="55" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>92</v>
       </c>
@@ -3501,7 +3494,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="56" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>93</v>
       </c>
@@ -3536,7 +3529,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="57" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>94</v>
       </c>
@@ -3571,7 +3564,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>95</v>
       </c>
@@ -3606,7 +3599,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="59" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>96</v>
       </c>
@@ -3641,7 +3634,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="60" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>97</v>
       </c>
@@ -3676,12 +3669,12 @@
         <v>142</v>
       </c>
     </row>
-    <row r="61" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>98</v>
       </c>
       <c r="B61" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C61" t="s">
         <v>51</v>
@@ -3711,12 +3704,12 @@
         <v>143</v>
       </c>
     </row>
-    <row r="62" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>99</v>
       </c>
       <c r="B62" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C62" t="s">
         <v>51</v>
@@ -3746,12 +3739,12 @@
         <v>143</v>
       </c>
     </row>
-    <row r="63" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>59</v>
       </c>
       <c r="B63" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C63" t="s">
         <v>53</v>
@@ -3775,18 +3768,18 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="K63" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>107</v>
       </c>
       <c r="B64" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="C64" t="s">
         <v>53</v>
@@ -3810,18 +3803,18 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="K64" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="65" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B65" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C65" t="s">
         <v>53</v>
@@ -3845,18 +3838,18 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="K65" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B66" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="C66" t="s">
         <v>53</v>
@@ -3880,18 +3873,18 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="K66" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B67" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C67" t="s">
         <v>53</v>
@@ -3915,13 +3908,13 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="K67" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>62</v>
       </c>
@@ -3953,10 +3946,10 @@
         <v>121</v>
       </c>
       <c r="K68" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>61</v>
       </c>
@@ -3988,10 +3981,10 @@
         <v>121</v>
       </c>
       <c r="K69" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>63</v>
       </c>
@@ -4023,15 +4016,15 @@
         <v>122</v>
       </c>
       <c r="K70" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>118</v>
       </c>
       <c r="B71" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C71" t="s">
         <v>56</v>
@@ -4061,12 +4054,12 @@
         <v>147</v>
       </c>
     </row>
-    <row r="72" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B72" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="C72" t="s">
         <v>56</v>
@@ -4090,13 +4083,13 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="K72" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>159</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>114</v>
       </c>
@@ -4131,7 +4124,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="74" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>113</v>
       </c>
@@ -4195,13 +4188,13 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="K75" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>14</v>
       </c>
@@ -4265,13 +4258,13 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="K77" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -4300,18 +4293,18 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="K78" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B79" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="C79" t="s">
         <v>56</v>
@@ -4335,21 +4328,21 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="K79" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="B80" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="C80" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D80" t="s">
         <v>24</v>
@@ -4370,10 +4363,10 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="K80" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
@@ -4381,10 +4374,10 @@
         <v>11</v>
       </c>
       <c r="B81" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="C81" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D81" t="s">
         <v>24</v>
@@ -4405,21 +4398,21 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="K81" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="B82" t="s">
         <v>16</v>
       </c>
       <c r="C82" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D82" t="s">
         <v>24</v>
@@ -4443,7 +4436,7 @@
         <v>134</v>
       </c>
       <c r="K82" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
@@ -4451,10 +4444,10 @@
         <v>46</v>
       </c>
       <c r="B83" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C83" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D83" t="s">
         <v>24</v>
@@ -4475,20 +4468,14 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="K83" t="s">
-        <v>228</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K83" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-    <filterColumn colId="9">
-      <filters>
-        <filter val="_dsc_coverage_metrics.json"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:K81" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated various component metric thresholds based on current data percentiles
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B6653BEC-37C3-4C5F-93DB-5B158C64AFEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB1CC405-31AF-461C-8316-854EB9AEC12B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -1680,7 +1680,7 @@
         <v>0</v>
       </c>
       <c r="F3">
-        <v>0.3</v>
+        <v>0.52</v>
       </c>
       <c r="G3">
         <v>0</v>
@@ -1712,7 +1712,7 @@
         <v>24</v>
       </c>
       <c r="E4">
-        <v>90</v>
+        <v>77.2</v>
       </c>
       <c r="F4">
         <v>100</v>
@@ -1747,7 +1747,7 @@
         <v>24</v>
       </c>
       <c r="E5">
-        <v>90</v>
+        <v>86.2</v>
       </c>
       <c r="F5">
         <v>1000</v>
@@ -1878,7 +1878,7 @@
         <v>280</v>
       </c>
       <c r="F9">
-        <v>320</v>
+        <v>375.5</v>
       </c>
       <c r="G9">
         <v>290</v>
@@ -1910,7 +1910,7 @@
         <v>24</v>
       </c>
       <c r="E10">
-        <v>95</v>
+        <v>87.9</v>
       </c>
       <c r="F10">
         <v>100</v>
@@ -2648,7 +2648,7 @@
         <v>0</v>
       </c>
       <c r="F31">
-        <v>0.1</v>
+        <v>0.17</v>
       </c>
       <c r="G31">
         <v>0</v>
@@ -2884,7 +2884,7 @@
         <v>24</v>
       </c>
       <c r="E38">
-        <v>80</v>
+        <v>71.3</v>
       </c>
       <c r="F38">
         <v>100</v>
@@ -2983,7 +2983,7 @@
         <v>24</v>
       </c>
       <c r="E41">
-        <v>80</v>
+        <v>35</v>
       </c>
       <c r="F41">
         <v>100</v>
@@ -3088,7 +3088,7 @@
         <v>24</v>
       </c>
       <c r="E44">
-        <v>98</v>
+        <v>94.9</v>
       </c>
       <c r="F44">
         <v>100</v>
@@ -4068,7 +4068,7 @@
         <v>24</v>
       </c>
       <c r="E72">
-        <v>60</v>
+        <v>58.3</v>
       </c>
       <c r="F72">
         <v>100</v>
@@ -4383,7 +4383,7 @@
         <v>24</v>
       </c>
       <c r="E81">
-        <v>5</v>
+        <v>4.9000000000000004</v>
       </c>
       <c r="F81">
         <v>100</v>

</xml_diff>

<commit_message>
Added ex_coverage_overlap_metrics and test, update d component metrics keys
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB1CC405-31AF-461C-8316-854EB9AEC12B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA43862C-1057-4FE8-A487-37F7D19A0AE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">Metrics!$A$1:$K$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metrics!$A$1:$K$83</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="230">
   <si>
     <t>nn_lower</t>
   </si>
@@ -494,9 +494,6 @@
     <t>ex_mean_analyzable_duplex_depth</t>
   </si>
   <si>
-    <t>ex_dsc_coverage_wholegenome</t>
-  </si>
-  <si>
     <t>^\d+ \+ 0 mapped \((?P&lt;percent&gt;[\d.]+)% : N/A\)$</t>
   </si>
   <si>
@@ -575,9 +572,6 @@
     <t>Reads with a length of zero after trimming (e.g. blank ligation)</t>
   </si>
   <si>
-    <t>Percentage of all sequenced bases with 1. MS depth &gt; half MS depth theshold and 2. EX duplex depth &gt; 0</t>
-  </si>
-  <si>
     <t>Percentage of reads lost from creation of DSC</t>
   </si>
   <si>
@@ -717,6 +711,21 @@
   </si>
   <si>
     <t>overlap_percentiles.value.50</t>
+  </si>
+  <si>
+    <t>ex_dsc_coverage_pct.value</t>
+  </si>
+  <si>
+    <t>ex_dsc_high_qual_unmasked_pct.value</t>
+  </si>
+  <si>
+    <t>_coverage_overlap_metrics.json</t>
+  </si>
+  <si>
+    <t>Percentage of all sequenced bases with 1. MS depth &gt; MS depth theshold and 2. EX duplex depth &gt; 0</t>
+  </si>
+  <si>
+    <t>ms_depth_vs_ex_depth.pct_overlap</t>
   </si>
 </sst>
 </file>
@@ -1586,6 +1595,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:K83"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1634,12 +1644,12 @@
         <v>120</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C2" t="s">
         <v>47</v>
@@ -1663,12 +1673,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="C3" t="s">
         <v>47</v>
@@ -1698,12 +1708,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C4" t="s">
         <v>47</v>
@@ -1733,12 +1743,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>43</v>
       </c>
       <c r="B5" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C5" t="s">
         <v>49</v>
@@ -1762,12 +1772,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C6" t="s">
         <v>49</v>
@@ -1797,12 +1807,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C7" t="s">
         <v>49</v>
@@ -1826,12 +1836,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="C8" t="s">
         <v>49</v>
@@ -1861,7 +1871,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1896,7 +1906,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -1931,7 +1941,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -1966,7 +1976,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -2001,12 +2011,12 @@
         <v>135</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>87</v>
       </c>
       <c r="B13" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C13" t="s">
         <v>52</v>
@@ -2036,12 +2046,12 @@
         <v>136</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>88</v>
       </c>
       <c r="B14" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C14" t="s">
         <v>52</v>
@@ -2071,12 +2081,12 @@
         <v>136</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>85</v>
       </c>
       <c r="B15" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C15" t="s">
         <v>52</v>
@@ -2106,12 +2116,12 @@
         <v>138</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>86</v>
       </c>
       <c r="B16" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C16" t="s">
         <v>52</v>
@@ -2141,7 +2151,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>77</v>
       </c>
@@ -2176,7 +2186,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>78</v>
       </c>
@@ -2211,12 +2221,12 @@
         <v>139</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B19" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C19" t="s">
         <v>52</v>
@@ -2246,12 +2256,12 @@
         <v>137</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B20" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C20" t="s">
         <v>52</v>
@@ -2281,7 +2291,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>66</v>
       </c>
@@ -2316,7 +2326,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>67</v>
       </c>
@@ -2351,7 +2361,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>68</v>
       </c>
@@ -2386,7 +2396,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>69</v>
       </c>
@@ -2421,7 +2431,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>70</v>
       </c>
@@ -2456,7 +2466,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>71</v>
       </c>
@@ -2491,12 +2501,12 @@
         <v>142</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>72</v>
       </c>
       <c r="B27" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C27" t="s">
         <v>52</v>
@@ -2526,12 +2536,12 @@
         <v>143</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>73</v>
       </c>
       <c r="B28" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C28" t="s">
         <v>52</v>
@@ -2561,12 +2571,12 @@
         <v>143</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B29" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C29" t="s">
         <v>54</v>
@@ -2590,13 +2600,13 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="K29" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>111</v>
       </c>
@@ -2628,10 +2638,10 @@
         <v>128</v>
       </c>
       <c r="K30" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>110</v>
       </c>
@@ -2660,18 +2670,18 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="K31" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B32" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C32" t="s">
         <v>55</v>
@@ -2695,13 +2705,13 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="K32" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>109</v>
       </c>
@@ -2733,18 +2743,18 @@
         <v>129</v>
       </c>
       <c r="K33" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B34" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="C34" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="D34" t="s">
         <v>24</v>
@@ -2765,13 +2775,13 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="K34" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>58</v>
       </c>
@@ -2779,7 +2789,7 @@
         <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="D35" t="s">
         <v>24</v>
@@ -2800,13 +2810,13 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
+        <v>156</v>
+      </c>
+      <c r="K35" t="s">
         <v>157</v>
       </c>
-      <c r="K35" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>19</v>
       </c>
@@ -2835,12 +2845,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>26</v>
       </c>
       <c r="B37" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C37" t="s">
         <v>48</v>
@@ -2870,12 +2880,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>32</v>
       </c>
       <c r="B38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C38" t="s">
         <v>48</v>
@@ -2905,7 +2915,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>40</v>
       </c>
@@ -2934,12 +2944,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>36</v>
       </c>
       <c r="B40" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C40" t="s">
         <v>48</v>
@@ -2969,12 +2979,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>37</v>
       </c>
       <c r="B41" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C41" t="s">
         <v>48</v>
@@ -3004,12 +3014,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>38</v>
       </c>
       <c r="B42" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C42" t="s">
         <v>48</v>
@@ -3039,7 +3049,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>20</v>
       </c>
@@ -3074,7 +3084,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>21</v>
       </c>
@@ -3109,12 +3119,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>81</v>
       </c>
       <c r="B45" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C45" t="s">
         <v>51</v>
@@ -3144,12 +3154,12 @@
         <v>136</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>82</v>
       </c>
       <c r="B46" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C46" t="s">
         <v>51</v>
@@ -3179,12 +3189,12 @@
         <v>136</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>83</v>
       </c>
       <c r="B47" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C47" t="s">
         <v>51</v>
@@ -3214,12 +3224,12 @@
         <v>138</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>84</v>
       </c>
       <c r="B48" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C48" t="s">
         <v>51</v>
@@ -3249,7 +3259,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>80</v>
       </c>
@@ -3284,7 +3294,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>89</v>
       </c>
@@ -3319,7 +3329,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>90</v>
       </c>
@@ -3354,7 +3364,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>91</v>
       </c>
@@ -3389,12 +3399,12 @@
         <v>135</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B53" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C53" t="s">
         <v>51</v>
@@ -3424,12 +3434,12 @@
         <v>137</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B54" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C54" t="s">
         <v>51</v>
@@ -3459,7 +3469,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>92</v>
       </c>
@@ -3494,7 +3504,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>93</v>
       </c>
@@ -3529,7 +3539,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>94</v>
       </c>
@@ -3564,7 +3574,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>95</v>
       </c>
@@ -3599,7 +3609,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>96</v>
       </c>
@@ -3634,7 +3644,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>97</v>
       </c>
@@ -3669,12 +3679,12 @@
         <v>142</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>98</v>
       </c>
       <c r="B61" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C61" t="s">
         <v>51</v>
@@ -3704,12 +3714,12 @@
         <v>143</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>99</v>
       </c>
       <c r="B62" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="C62" t="s">
         <v>51</v>
@@ -3739,12 +3749,12 @@
         <v>143</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>59</v>
       </c>
       <c r="B63" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C63" t="s">
         <v>53</v>
@@ -3768,18 +3778,18 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="K63" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>107</v>
       </c>
       <c r="B64" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="C64" t="s">
         <v>53</v>
@@ -3803,18 +3813,18 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="K64" t="s">
         <v>145</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>167</v>
+      </c>
+      <c r="B65" t="s">
         <v>168</v>
-      </c>
-      <c r="B65" t="s">
-        <v>169</v>
       </c>
       <c r="C65" t="s">
         <v>53</v>
@@ -3838,18 +3848,18 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="K65" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B66" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C66" t="s">
         <v>53</v>
@@ -3873,18 +3883,18 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="K66" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B67" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C67" t="s">
         <v>53</v>
@@ -3908,13 +3918,13 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="K67" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>62</v>
       </c>
@@ -3946,10 +3956,10 @@
         <v>121</v>
       </c>
       <c r="K68" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>61</v>
       </c>
@@ -3981,10 +3991,10 @@
         <v>121</v>
       </c>
       <c r="K69" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>63</v>
       </c>
@@ -4016,15 +4026,15 @@
         <v>122</v>
       </c>
       <c r="K70" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>118</v>
       </c>
       <c r="B71" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C71" t="s">
         <v>56</v>
@@ -4054,12 +4064,12 @@
         <v>147</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B72" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C72" t="s">
         <v>56</v>
@@ -4083,13 +4093,13 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="K72" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>114</v>
       </c>
@@ -4124,7 +4134,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>113</v>
       </c>
@@ -4188,13 +4198,13 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K75" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>14</v>
       </c>
@@ -4258,13 +4268,13 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K77" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -4293,18 +4303,18 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="K78" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
+        <v>221</v>
+      </c>
+      <c r="B79" t="s">
         <v>223</v>
-      </c>
-      <c r="B79" t="s">
-        <v>225</v>
       </c>
       <c r="C79" t="s">
         <v>56</v>
@@ -4328,21 +4338,21 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
+        <v>222</v>
+      </c>
+      <c r="K79" t="s">
         <v>224</v>
       </c>
-      <c r="K79" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="80" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B80" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="C80" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D80" t="s">
         <v>24</v>
@@ -4363,10 +4373,10 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="K80" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
@@ -4374,10 +4384,10 @@
         <v>11</v>
       </c>
       <c r="B81" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C81" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D81" t="s">
         <v>24</v>
@@ -4398,21 +4408,21 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K81" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B82" t="s">
         <v>16</v>
       </c>
       <c r="C82" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D82" t="s">
         <v>24</v>
@@ -4436,7 +4446,7 @@
         <v>134</v>
       </c>
       <c r="K82" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
@@ -4444,10 +4454,10 @@
         <v>46</v>
       </c>
       <c r="B83" t="s">
-        <v>179</v>
+        <v>228</v>
       </c>
       <c r="C83" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D83" t="s">
         <v>24</v>
@@ -4468,14 +4478,20 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>161</v>
+        <v>227</v>
       </c>
       <c r="K83" t="s">
-        <v>46</v>
+        <v>229</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K81" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K83" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
+    <filterColumn colId="9">
+      <filters>
+        <filter val="_dsc_coverage_metrics.json"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated median_duplex_depth component metric name and keys
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA43862C-1057-4FE8-A487-37F7D19A0AE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{120E98BF-950C-446B-A3ED-277E9C51D153}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="231">
   <si>
     <t>nn_lower</t>
   </si>
@@ -383,12 +383,6 @@
     <t>ex_mapped_dsc_realignment</t>
   </si>
   <si>
-    <t>ex_mean_duplex_depth</t>
-  </si>
-  <si>
-    <t>Mean duplex depth of final DSC passed to variant calling</t>
-  </si>
-  <si>
     <t>Fraction of mapped reads that are marked as duplicates</t>
   </si>
   <si>
@@ -491,9 +485,6 @@
     <t>_dsc_remap_metrics.json</t>
   </si>
   <si>
-    <t>ex_mean_analyzable_duplex_depth</t>
-  </si>
-  <si>
     <t>^\d+ \+ 0 mapped \((?P&lt;percent&gt;[\d.]+)% : N/A\)$</t>
   </si>
   <si>
@@ -726,6 +717,18 @@
   </si>
   <si>
     <t>ms_depth_vs_ex_depth.pct_overlap</t>
+  </si>
+  <si>
+    <t>Median duplex depth of positions eligible for variant calling</t>
+  </si>
+  <si>
+    <t>_depth_metrics.json</t>
+  </si>
+  <si>
+    <t>depth_percentiles.values.50th</t>
+  </si>
+  <si>
+    <t>ex_median_duplex_depth</t>
   </si>
 </sst>
 </file>
@@ -1595,21 +1598,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:K83"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="35.140625" customWidth="1"/>
-    <col min="2" max="2" width="123.140625" customWidth="1"/>
-    <col min="3" max="4" width="35.28515625" customWidth="1"/>
+    <col min="1" max="1" width="35.109375" customWidth="1"/>
+    <col min="2" max="2" width="123.109375" customWidth="1"/>
+    <col min="3" max="4" width="35.33203125" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" customWidth="1"/>
-    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="76.85546875" customWidth="1"/>
+    <col min="9" max="9" width="12.88671875" customWidth="1"/>
+    <col min="10" max="10" width="61.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="76.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>31</v>
       </c>
@@ -1638,18 +1640,18 @@
         <v>30</v>
       </c>
       <c r="J1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="K1" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="C2" t="s">
         <v>47</v>
@@ -1673,12 +1675,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="3" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="C3" t="s">
         <v>47</v>
@@ -1708,12 +1710,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="4" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="C4" t="s">
         <v>47</v>
@@ -1743,12 +1745,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="5" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>43</v>
       </c>
       <c r="B5" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="C5" t="s">
         <v>49</v>
@@ -1772,12 +1774,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="6" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>42</v>
       </c>
       <c r="B6" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C6" t="s">
         <v>49</v>
@@ -1807,12 +1809,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="C7" t="s">
         <v>49</v>
@@ -1836,12 +1838,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="8" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>45</v>
       </c>
       <c r="B8" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="C8" t="s">
         <v>49</v>
@@ -1871,7 +1873,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>22</v>
       </c>
@@ -1906,7 +1908,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="10" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>23</v>
       </c>
@@ -1941,7 +1943,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="11" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -1970,13 +1972,13 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="K11" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -2005,18 +2007,18 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K12" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>87</v>
       </c>
       <c r="B13" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C13" t="s">
         <v>52</v>
@@ -2040,18 +2042,18 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="K13" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>88</v>
       </c>
       <c r="B14" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C14" t="s">
         <v>52</v>
@@ -2075,18 +2077,18 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K14" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>85</v>
       </c>
       <c r="B15" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C15" t="s">
         <v>52</v>
@@ -2110,18 +2112,18 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="K15" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>86</v>
       </c>
       <c r="B16" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C16" t="s">
         <v>52</v>
@@ -2145,13 +2147,13 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K16" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>77</v>
       </c>
@@ -2180,13 +2182,13 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="K17" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>78</v>
       </c>
@@ -2215,18 +2217,18 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K18" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B19" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C19" t="s">
         <v>52</v>
@@ -2250,18 +2252,18 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K19" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="B20" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C20" t="s">
         <v>52</v>
@@ -2285,13 +2287,13 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="K20" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>66</v>
       </c>
@@ -2320,13 +2322,13 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K21" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>67</v>
       </c>
@@ -2355,13 +2357,13 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="K22" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>68</v>
       </c>
@@ -2390,13 +2392,13 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K23" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>69</v>
       </c>
@@ -2425,13 +2427,13 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="K24" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>70</v>
       </c>
@@ -2460,13 +2462,13 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K25" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>71</v>
       </c>
@@ -2495,18 +2497,18 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="K26" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>72</v>
       </c>
       <c r="B27" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C27" t="s">
         <v>52</v>
@@ -2530,18 +2532,18 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K27" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>73</v>
       </c>
       <c r="B28" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C28" t="s">
         <v>52</v>
@@ -2565,18 +2567,18 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="K28" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B29" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C29" t="s">
         <v>54</v>
@@ -2600,13 +2602,13 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="K29" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>111</v>
       </c>
@@ -2635,18 +2637,18 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K30" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>110</v>
       </c>
       <c r="B31" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C31" t="s">
         <v>55</v>
@@ -2670,18 +2672,18 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="K31" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="B32" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="C32" t="s">
         <v>55</v>
@@ -2705,13 +2707,13 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="K32" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>109</v>
       </c>
@@ -2740,21 +2742,21 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K33" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B34" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C34" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D34" t="s">
         <v>24</v>
@@ -2775,13 +2777,13 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="K34" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>58</v>
       </c>
@@ -2789,7 +2791,7 @@
         <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="D35" t="s">
         <v>24</v>
@@ -2810,13 +2812,13 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="K35" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="36" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>19</v>
       </c>
@@ -2845,12 +2847,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="37" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>26</v>
       </c>
       <c r="B37" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C37" t="s">
         <v>48</v>
@@ -2880,12 +2882,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="38" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>32</v>
       </c>
       <c r="B38" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="C38" t="s">
         <v>48</v>
@@ -2915,7 +2917,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="39" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>40</v>
       </c>
@@ -2944,12 +2946,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="40" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>36</v>
       </c>
       <c r="B40" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C40" t="s">
         <v>48</v>
@@ -2979,12 +2981,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="41" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>37</v>
       </c>
       <c r="B41" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="C41" t="s">
         <v>48</v>
@@ -3014,12 +3016,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="42" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>38</v>
       </c>
       <c r="B42" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="C42" t="s">
         <v>48</v>
@@ -3049,7 +3051,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="43" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>20</v>
       </c>
@@ -3084,7 +3086,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="44" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>21</v>
       </c>
@@ -3119,12 +3121,12 @@
         <v>57</v>
       </c>
     </row>
-    <row r="45" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>81</v>
       </c>
       <c r="B45" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C45" t="s">
         <v>51</v>
@@ -3148,18 +3150,18 @@
         <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K45" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>82</v>
       </c>
       <c r="B46" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C46" t="s">
         <v>51</v>
@@ -3183,18 +3185,18 @@
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K46" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>83</v>
       </c>
       <c r="B47" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C47" t="s">
         <v>51</v>
@@ -3218,18 +3220,18 @@
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K47" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>84</v>
       </c>
       <c r="B48" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C48" t="s">
         <v>51</v>
@@ -3253,13 +3255,13 @@
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K48" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>80</v>
       </c>
@@ -3288,13 +3290,13 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K49" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>89</v>
       </c>
@@ -3323,13 +3325,13 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K50" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>90</v>
       </c>
@@ -3358,13 +3360,13 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K51" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>91</v>
       </c>
@@ -3393,18 +3395,18 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K52" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="B53" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C53" t="s">
         <v>51</v>
@@ -3428,18 +3430,18 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K53" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="B54" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C54" t="s">
         <v>51</v>
@@ -3463,13 +3465,13 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K54" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>92</v>
       </c>
@@ -3498,13 +3500,13 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K55" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>93</v>
       </c>
@@ -3533,13 +3535,13 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K56" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>94</v>
       </c>
@@ -3568,13 +3570,13 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K57" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>95</v>
       </c>
@@ -3603,13 +3605,13 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K58" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>96</v>
       </c>
@@ -3638,13 +3640,13 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K59" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>97</v>
       </c>
@@ -3673,18 +3675,18 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K60" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>98</v>
       </c>
       <c r="B61" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C61" t="s">
         <v>51</v>
@@ -3708,18 +3710,18 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K61" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>99</v>
       </c>
       <c r="B62" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="C62" t="s">
         <v>51</v>
@@ -3743,18 +3745,18 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K62" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>59</v>
       </c>
       <c r="B63" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C63" t="s">
         <v>53</v>
@@ -3778,18 +3780,18 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="K63" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>107</v>
       </c>
       <c r="B64" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="C64" t="s">
         <v>53</v>
@@ -3813,18 +3815,18 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="K64" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B65" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="C65" t="s">
         <v>53</v>
@@ -3848,18 +3850,18 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="K65" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
         <v>185</v>
       </c>
-    </row>
-    <row r="66" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>188</v>
-      </c>
       <c r="B66" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C66" t="s">
         <v>53</v>
@@ -3883,18 +3885,18 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="K66" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B67" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C67" t="s">
         <v>53</v>
@@ -3918,13 +3920,13 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="K67" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>62</v>
       </c>
@@ -3953,13 +3955,13 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="K68" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>61</v>
       </c>
@@ -3988,13 +3990,13 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="K69" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>63</v>
       </c>
@@ -4023,18 +4025,18 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="K70" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="B71" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C71" t="s">
         <v>56</v>
@@ -4058,18 +4060,18 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="K71" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="B72" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C72" t="s">
         <v>56</v>
@@ -4093,13 +4095,13 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="K72" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>114</v>
       </c>
@@ -4128,13 +4130,13 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="K73" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>113</v>
       </c>
@@ -4163,18 +4165,18 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="K74" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
-        <v>115</v>
+        <v>230</v>
       </c>
       <c r="B75" t="s">
-        <v>116</v>
+        <v>227</v>
       </c>
       <c r="C75" t="s">
         <v>56</v>
@@ -4198,13 +4200,13 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>160</v>
+        <v>228</v>
       </c>
       <c r="K75" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>14</v>
       </c>
@@ -4233,13 +4235,13 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="K76" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>12</v>
       </c>
@@ -4268,13 +4270,13 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="K77" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -4303,18 +4305,18 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="K78" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="B79" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="C79" t="s">
         <v>56</v>
@@ -4338,21 +4340,21 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="K79" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="B80" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C80" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D80" t="s">
         <v>24</v>
@@ -4373,21 +4375,21 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="K80" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>11</v>
       </c>
       <c r="B81" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C81" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D81" t="s">
         <v>24</v>
@@ -4408,21 +4410,21 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="K81" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" hidden="1" x14ac:dyDescent="0.25">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B82" t="s">
         <v>16</v>
       </c>
       <c r="C82" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D82" t="s">
         <v>24</v>
@@ -4443,21 +4445,21 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="K82" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>46</v>
       </c>
       <c r="B83" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="C83" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D83" t="s">
         <v>24</v>
@@ -4478,20 +4480,14 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="K83" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K83" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-    <filterColumn colId="9">
-      <filters>
-        <filter val="_dsc_coverage_metrics.json"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:K83" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated component metrics for coverage and depth metrics
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB08DDD0-5FFC-4CCA-9FD0-BE21EBF640EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{238E799F-FE5D-4F56-9B20-18B946B31021}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="231">
   <si>
     <t>nn_lower</t>
   </si>
@@ -74,12 +74,6 @@
     <t>ex_variant_call_eligible</t>
   </si>
   <si>
-    <t>ex_duplex_coverage</t>
-  </si>
-  <si>
-    <t>Percentage of genome with duplex depth &gt; 0</t>
-  </si>
-  <si>
     <t>ex_dsc_softclipping</t>
   </si>
   <si>
@@ -596,9 +590,6 @@
     <t>ex_zero_length_reads</t>
   </si>
   <si>
-    <t>Percentage of genome eligible for variant calling (duplex depth &gt; 0, unmasked, QUAL &gt; min_base_quality)</t>
-  </si>
-  <si>
     <t>duplication_rate</t>
   </si>
   <si>
@@ -704,9 +695,6 @@
     <t>overlap_percentiles.value.50</t>
   </si>
   <si>
-    <t>ex_dsc_coverage_pct.value</t>
-  </si>
-  <si>
     <t>ex_dsc_high_qual_unmasked_pct.value</t>
   </si>
   <si>
@@ -728,7 +716,19 @@
     <t>ex_median_duplex_depth</t>
   </si>
   <si>
-    <t>Median duplex depth of covered positions that are eligible for variant calling</t>
+    <t>Percentage of genome with duplex depth &gt; 0 and QUAL &gt; min_base_quality</t>
+  </si>
+  <si>
+    <t>Percentage of genome eligible for variant calling (duplex depth &gt; 0, QUAL &gt; min_base_quality, unmasked)</t>
+  </si>
+  <si>
+    <t>ex_dsc_high_qual_pct.value</t>
+  </si>
+  <si>
+    <t>Median duplex depth for positions that are eligible for variant calling</t>
+  </si>
+  <si>
+    <t>ex_high_qual_coverage</t>
   </si>
 </sst>
 </file>
@@ -1613,16 +1613,16 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="B1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s">
         <v>27</v>
-      </c>
-      <c r="C1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D1" t="s">
-        <v>29</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -1637,27 +1637,27 @@
         <v>3</v>
       </c>
       <c r="I1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="J1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="K1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="B2" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E2">
         <v>2500</v>
@@ -1669,24 +1669,24 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K2" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="C3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D3" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1704,24 +1704,24 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K3" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="B4" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C4" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="D4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E4">
         <v>77.2</v>
@@ -1739,24 +1739,24 @@
         <v>0</v>
       </c>
       <c r="J4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K4" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="B5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E5">
         <v>86.2</v>
@@ -1768,24 +1768,24 @@
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K5" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="B6" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C6" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1803,24 +1803,24 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K6" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B7" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D7" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E7">
         <v>45</v>
@@ -1832,24 +1832,24 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="B8" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C8" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -1867,24 +1867,24 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K8" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B9" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C9" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E9">
         <v>280</v>
@@ -1902,24 +1902,24 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B10" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E10">
         <v>87.9</v>
@@ -1937,10 +1937,10 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K10" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -1948,13 +1948,13 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C11" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E11">
         <v>200</v>
@@ -1972,10 +1972,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="K11" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1983,13 +1983,13 @@
         <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C12" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D12" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E12">
         <v>200</v>
@@ -2007,24 +2007,24 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="K12" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="B13" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C13" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D13" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E13">
         <v>35</v>
@@ -2042,24 +2042,24 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="K13" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="B14" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C14" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D14" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E14">
         <v>35</v>
@@ -2077,24 +2077,24 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="K14" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B15" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C15" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D15" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -2112,24 +2112,24 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="K15" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="B16" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D16" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -2147,24 +2147,24 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="K16" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>75</v>
+      </c>
+      <c r="B17" t="s">
         <v>77</v>
       </c>
-      <c r="B17" t="s">
-        <v>79</v>
-      </c>
       <c r="C17" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D17" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E17">
         <v>150</v>
@@ -2182,24 +2182,24 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="K17" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B18" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C18" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D18" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E18">
         <v>150</v>
@@ -2217,24 +2217,24 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="K18" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B19" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C19" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D19" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E19">
         <v>30</v>
@@ -2252,24 +2252,24 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="K19" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B20" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C20" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D20" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E20">
         <v>30</v>
@@ -2287,24 +2287,24 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K20" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B21" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C21" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D21" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -2322,24 +2322,24 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="K21" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B22" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C22" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D22" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -2357,24 +2357,24 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K22" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B23" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C23" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D23" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -2392,24 +2392,24 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="K23" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B24" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C24" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D24" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -2427,24 +2427,24 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K24" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B25" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C25" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D25" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -2462,24 +2462,24 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="K25" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B26" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C26" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D26" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E26">
         <v>0</v>
@@ -2497,24 +2497,24 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K26" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B27" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C27" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D27" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -2532,24 +2532,24 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="K27" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B28" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C28" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D28" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -2567,24 +2567,24 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K28" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="B29" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C29" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D29" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E29">
         <v>70</v>
@@ -2602,24 +2602,24 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="K29" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="B30" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C30" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D30" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E30">
         <v>90</v>
@@ -2637,24 +2637,24 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="K30" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B31" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C31" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D31" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -2672,24 +2672,24 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="K31" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="B32" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="C32" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D32" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E32">
         <v>21.75</v>
@@ -2707,24 +2707,24 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="K32" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="B33" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="C33" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D33" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E33">
         <v>125</v>
@@ -2742,24 +2742,24 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="K33" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="B34" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="C34" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D34" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E34">
         <v>1.5E-3</v>
@@ -2777,24 +2777,24 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="K34" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B35" t="s">
         <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="D35" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E35">
         <v>70</v>
@@ -2812,24 +2812,24 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="K35" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B36" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C36" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D36" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E36">
         <v>75</v>
@@ -2841,24 +2841,24 @@
         <v>0</v>
       </c>
       <c r="J36" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K36" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B37" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C37" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D37" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E37">
         <v>0</v>
@@ -2876,24 +2876,24 @@
         <v>0</v>
       </c>
       <c r="J37" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K37" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="B38" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C38" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D38" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E38">
         <v>71.3</v>
@@ -2911,24 +2911,24 @@
         <v>0</v>
       </c>
       <c r="J38" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K38" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C39" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D39" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E39">
         <v>4.3</v>
@@ -2940,24 +2940,24 @@
         <v>0</v>
       </c>
       <c r="J39" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K39" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="B40" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="C40" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D40" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E40">
         <v>0</v>
@@ -2975,24 +2975,24 @@
         <v>0</v>
       </c>
       <c r="J40" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K40" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="B41" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C41" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D41" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E41">
         <v>35</v>
@@ -3010,24 +3010,24 @@
         <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K41" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B42" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C42" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D42" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -3045,24 +3045,24 @@
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K42" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B43" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C43" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D43" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E43">
         <v>544</v>
@@ -3080,24 +3080,24 @@
         <v>0</v>
       </c>
       <c r="J43" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K43" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B44" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C44" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D44" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E44">
         <v>94.9</v>
@@ -3115,24 +3115,24 @@
         <v>0</v>
       </c>
       <c r="J44" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="K44" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B45" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C45" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D45" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E45">
         <v>35</v>
@@ -3150,24 +3150,24 @@
         <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K45" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="B46" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C46" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D46" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E46">
         <v>35</v>
@@ -3185,24 +3185,24 @@
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K46" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B47" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C47" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D47" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E47">
         <v>0</v>
@@ -3220,24 +3220,24 @@
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K47" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B48" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="C48" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D48" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E48">
         <v>0</v>
@@ -3255,24 +3255,24 @@
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K48" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="B49" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C49" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D49" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E49">
         <v>150</v>
@@ -3290,24 +3290,24 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K49" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="B50" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C50" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D50" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E50">
         <v>150</v>
@@ -3325,24 +3325,24 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K50" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="B51" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C51" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D51" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E51">
         <v>2850</v>
@@ -3360,24 +3360,24 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="K51" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="B52" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C52" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D52" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E52">
         <v>2850</v>
@@ -3395,24 +3395,24 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="K52" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B53" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C53" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D53" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E53">
         <v>30</v>
@@ -3430,24 +3430,24 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K53" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B54" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="C54" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D54" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E54">
         <v>30</v>
@@ -3465,24 +3465,24 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K54" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="B55" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C55" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D55" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E55">
         <v>0</v>
@@ -3500,24 +3500,24 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K55" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="B56" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C56" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D56" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E56">
         <v>0</v>
@@ -3535,24 +3535,24 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K56" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="B57" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C57" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D57" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E57">
         <v>0</v>
@@ -3570,24 +3570,24 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K57" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="B58" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C58" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D58" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E58">
         <v>0</v>
@@ -3605,24 +3605,24 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K58" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="B59" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C59" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D59" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E59">
         <v>0</v>
@@ -3640,24 +3640,24 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K59" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="B60" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C60" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D60" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E60">
         <v>0</v>
@@ -3675,24 +3675,24 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K60" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="B61" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C61" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D61" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E61">
         <v>0</v>
@@ -3710,24 +3710,24 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="K61" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="B62" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C62" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D62" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E62">
         <v>0</v>
@@ -3745,24 +3745,24 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K62" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="B63" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C63" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D63" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E63">
         <v>0</v>
@@ -3780,24 +3780,24 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="K63" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B64" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="C64" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D64" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E64">
         <v>0</v>
@@ -3815,24 +3815,24 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="K64" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B65" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C65" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D65" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E65">
         <v>1</v>
@@ -3850,24 +3850,24 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="K65" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B66" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C66" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D66" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E66">
         <v>0</v>
@@ -3885,24 +3885,24 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="K66" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B67" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="C67" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D67" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E67">
         <v>70</v>
@@ -3920,24 +3920,24 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="K67" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B68" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="C68" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D68" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E68">
         <v>90</v>
@@ -3955,24 +3955,24 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="K68" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B69" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="C69" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D69" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E69">
         <v>50</v>
@@ -3990,24 +3990,24 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="K69" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B70" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C70" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D70" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E70">
         <v>120</v>
@@ -4025,24 +4025,24 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="K70" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="B71" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C71" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D71" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E71">
         <v>50</v>
@@ -4060,24 +4060,24 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="K71" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="B72" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C72" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D72" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E72">
         <v>58.3</v>
@@ -4095,24 +4095,24 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="K72" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="B73" t="s">
         <v>10</v>
       </c>
       <c r="C73" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D73" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E73">
         <v>99</v>
@@ -4130,24 +4130,24 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="K73" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="B74" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C74" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D74" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E74">
         <v>0</v>
@@ -4165,59 +4165,53 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="K74" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
+        <v>225</v>
+      </c>
+      <c r="B75" t="s">
         <v>229</v>
       </c>
-      <c r="B75" t="s">
-        <v>230</v>
-      </c>
       <c r="C75" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D75" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E75">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F75" t="s">
         <v>5</v>
       </c>
-      <c r="G75">
-        <v>1</v>
-      </c>
-      <c r="H75" t="s">
-        <v>5</v>
-      </c>
       <c r="I75" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="K75" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B76" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C76" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D76" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E76">
         <v>0</v>
@@ -4235,24 +4229,24 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="K76" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>12</v>
+        <v>230</v>
       </c>
       <c r="B77" t="s">
-        <v>13</v>
+        <v>226</v>
       </c>
       <c r="C77" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D77" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E77">
         <v>14.5</v>
@@ -4270,10 +4264,10 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="K77" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
@@ -4284,10 +4278,10 @@
         <v>9</v>
       </c>
       <c r="C78" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D78" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E78">
         <v>0</v>
@@ -4305,24 +4299,24 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="K78" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B79" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="C79" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D79" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E79">
         <v>69</v>
@@ -4340,24 +4334,24 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="K79" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="B80" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C80" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D80" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E80">
         <v>0</v>
@@ -4375,10 +4369,10 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="K80" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
@@ -4386,13 +4380,13 @@
         <v>11</v>
       </c>
       <c r="B81" t="s">
-        <v>186</v>
+        <v>227</v>
       </c>
       <c r="C81" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D81" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E81">
         <v>4.9000000000000004</v>
@@ -4410,24 +4404,24 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="K81" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="B82" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C82" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D82" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E82">
         <v>0</v>
@@ -4445,24 +4439,24 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="K82" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="B83" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="C83" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="D83" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="E83">
         <v>33</v>
@@ -4477,13 +4471,13 @@
         <v>100</v>
       </c>
       <c r="I83" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="K83" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated component metric thresholds for EX depth and coverage metrics
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{238E799F-FE5D-4F56-9B20-18B946B31021}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26A74E71-5FFE-43A3-90F2-A80DF6D71EA0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -80,9 +80,6 @@
     <t>Number of soft clipped bases for 90th percentile most softclipped reads</t>
   </si>
   <si>
-    <t>Percentage of reads lost between start and end of ex pipeline</t>
-  </si>
-  <si>
     <t>Mean length of the largest peak</t>
   </si>
   <si>
@@ -729,6 +726,9 @@
   </si>
   <si>
     <t>ex_high_qual_coverage</t>
+  </si>
+  <si>
+    <t>Percentage of reads lost between start and end of EX pipeline</t>
   </si>
 </sst>
 </file>
@@ -1613,16 +1613,16 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C1" t="s">
         <v>25</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>26</v>
-      </c>
-      <c r="D1" t="s">
-        <v>27</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -1637,27 +1637,27 @@
         <v>3</v>
       </c>
       <c r="I1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J1" t="s">
+        <v>114</v>
+      </c>
+      <c r="K1" t="s">
         <v>115</v>
-      </c>
-      <c r="K1" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E2">
         <v>2500</v>
@@ -1669,24 +1669,24 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K2" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B3" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="C3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1704,24 +1704,24 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K3" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E4">
         <v>77.2</v>
@@ -1739,24 +1739,24 @@
         <v>0</v>
       </c>
       <c r="J4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K4" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="C5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E5">
         <v>86.2</v>
@@ -1768,24 +1768,24 @@
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C6" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D6" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1803,24 +1803,24 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="C7" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D7" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E7">
         <v>45</v>
@@ -1832,24 +1832,24 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K7" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B8" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="C8" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D8" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -1867,24 +1867,24 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K8" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D9" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E9">
         <v>280</v>
@@ -1902,24 +1902,24 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E10">
         <v>87.9</v>
@@ -1937,10 +1937,10 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -1948,13 +1948,13 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C11" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E11">
         <v>200</v>
@@ -1972,10 +1972,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="K11" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1983,13 +1983,13 @@
         <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C12" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D12" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E12">
         <v>200</v>
@@ -2007,24 +2007,24 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="K12" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D13" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E13">
         <v>35</v>
@@ -2042,24 +2042,24 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="K13" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B14" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C14" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E14">
         <v>35</v>
@@ -2077,24 +2077,24 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="K14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B15" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -2112,24 +2112,24 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="K15" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B16" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C16" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -2147,24 +2147,24 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="K16" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B17" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C17" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D17" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E17">
         <v>150</v>
@@ -2182,24 +2182,24 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="K17" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>75</v>
+      </c>
+      <c r="B18" t="s">
         <v>76</v>
       </c>
-      <c r="B18" t="s">
-        <v>77</v>
-      </c>
       <c r="C18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E18">
         <v>150</v>
@@ -2217,24 +2217,24 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="K18" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B19" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C19" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E19">
         <v>30</v>
@@ -2252,24 +2252,24 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K19" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B20" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C20" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E20">
         <v>30</v>
@@ -2287,24 +2287,24 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K20" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B21" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C21" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D21" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -2322,24 +2322,24 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K21" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B22" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C22" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -2357,24 +2357,24 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K22" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B23" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C23" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -2392,24 +2392,24 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K23" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B24" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C24" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -2427,24 +2427,24 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K24" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B25" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C25" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D25" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -2462,24 +2462,24 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K25" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B26" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C26" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D26" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E26">
         <v>0</v>
@@ -2497,24 +2497,24 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K26" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B27" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C27" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D27" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -2532,24 +2532,24 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="K27" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B28" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C28" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D28" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -2567,24 +2567,24 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K28" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B29" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="C29" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D29" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E29">
         <v>70</v>
@@ -2602,24 +2602,24 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="K29" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B30" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C30" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D30" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E30">
         <v>90</v>
@@ -2637,24 +2637,24 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="K30" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="B31" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C31" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D31" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -2672,24 +2672,24 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K31" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B32" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C32" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D32" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E32">
         <v>21.75</v>
@@ -2707,24 +2707,24 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="K32" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B33" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C33" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D33" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E33">
         <v>125</v>
@@ -2742,24 +2742,24 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="K33" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
+        <v>200</v>
+      </c>
+      <c r="B34" t="s">
         <v>201</v>
       </c>
-      <c r="B34" t="s">
-        <v>202</v>
-      </c>
       <c r="C34" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D34" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E34">
         <v>1.5E-3</v>
@@ -2777,24 +2777,24 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="K34" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B35" t="s">
         <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D35" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E35">
         <v>70</v>
@@ -2812,24 +2812,24 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
+        <v>150</v>
+      </c>
+      <c r="K35" t="s">
         <v>151</v>
-      </c>
-      <c r="K35" t="s">
-        <v>152</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B36" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C36" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D36" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E36">
         <v>75</v>
@@ -2841,24 +2841,24 @@
         <v>0</v>
       </c>
       <c r="J36" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K36" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B37" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C37" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D37" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E37">
         <v>0</v>
@@ -2876,24 +2876,24 @@
         <v>0</v>
       </c>
       <c r="J37" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K37" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B38" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C38" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D38" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E38">
         <v>71.3</v>
@@ -2911,24 +2911,24 @@
         <v>0</v>
       </c>
       <c r="J38" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K38" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>37</v>
+      </c>
+      <c r="B39" t="s">
         <v>38</v>
       </c>
-      <c r="B39" t="s">
-        <v>39</v>
-      </c>
       <c r="C39" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D39" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E39">
         <v>4.3</v>
@@ -2940,24 +2940,24 @@
         <v>0</v>
       </c>
       <c r="J39" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K39" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B40" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="C40" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D40" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E40">
         <v>0</v>
@@ -2975,24 +2975,24 @@
         <v>0</v>
       </c>
       <c r="J40" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K40" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B41" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C41" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D41" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E41">
         <v>35</v>
@@ -3010,24 +3010,24 @@
         <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K41" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B42" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C42" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D42" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E42">
         <v>1</v>
@@ -3045,24 +3045,24 @@
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K42" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B43" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C43" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D43" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E43">
         <v>544</v>
@@ -3080,24 +3080,24 @@
         <v>0</v>
       </c>
       <c r="J43" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K43" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B44" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C44" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D44" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E44">
         <v>94.9</v>
@@ -3115,24 +3115,24 @@
         <v>0</v>
       </c>
       <c r="J44" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="K44" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B45" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C45" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D45" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E45">
         <v>35</v>
@@ -3150,24 +3150,24 @@
         <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K45" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B46" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C46" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D46" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E46">
         <v>35</v>
@@ -3185,24 +3185,24 @@
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="K46" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B47" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C47" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D47" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E47">
         <v>0</v>
@@ -3220,24 +3220,24 @@
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K47" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B48" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="C48" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D48" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E48">
         <v>0</v>
@@ -3255,24 +3255,24 @@
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="K48" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B49" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C49" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D49" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E49">
         <v>150</v>
@@ -3290,24 +3290,24 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K49" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B50" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C50" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D50" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E50">
         <v>150</v>
@@ -3325,24 +3325,24 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="K50" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B51" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C51" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D51" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E51">
         <v>2850</v>
@@ -3360,24 +3360,24 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K51" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B52" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C52" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D52" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E52">
         <v>2850</v>
@@ -3395,24 +3395,24 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="K52" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B53" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C53" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D53" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E53">
         <v>30</v>
@@ -3430,24 +3430,24 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K53" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B54" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C54" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D54" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E54">
         <v>30</v>
@@ -3465,24 +3465,24 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K54" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B55" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C55" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D55" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E55">
         <v>0</v>
@@ -3500,24 +3500,24 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K55" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B56" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C56" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D56" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E56">
         <v>0</v>
@@ -3535,24 +3535,24 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K56" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B57" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C57" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D57" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E57">
         <v>0</v>
@@ -3570,24 +3570,24 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K57" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B58" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C58" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D58" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E58">
         <v>0</v>
@@ -3605,24 +3605,24 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K58" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B59" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C59" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D59" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E59">
         <v>0</v>
@@ -3640,24 +3640,24 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K59" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B60" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C60" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D60" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E60">
         <v>0</v>
@@ -3675,24 +3675,24 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K60" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B61" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C61" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D61" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E61">
         <v>0</v>
@@ -3710,24 +3710,24 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K61" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B62" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C62" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D62" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E62">
         <v>0</v>
@@ -3745,24 +3745,24 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="K62" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
+        <v>56</v>
+      </c>
+      <c r="B63" t="s">
+        <v>178</v>
+      </c>
+      <c r="C63" t="s">
+        <v>50</v>
+      </c>
+      <c r="D63" t="s">
         <v>57</v>
-      </c>
-      <c r="B63" t="s">
-        <v>179</v>
-      </c>
-      <c r="C63" t="s">
-        <v>51</v>
-      </c>
-      <c r="D63" t="s">
-        <v>58</v>
       </c>
       <c r="E63">
         <v>0</v>
@@ -3780,24 +3780,24 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
+        <v>176</v>
+      </c>
+      <c r="K63" t="s">
         <v>177</v>
-      </c>
-      <c r="K63" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B64" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C64" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D64" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E64">
         <v>0</v>
@@ -3815,24 +3815,24 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="K64" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
+        <v>161</v>
+      </c>
+      <c r="B65" t="s">
         <v>162</v>
       </c>
-      <c r="B65" t="s">
-        <v>163</v>
-      </c>
       <c r="C65" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D65" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E65">
         <v>1</v>
@@ -3850,24 +3850,24 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="K65" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B66" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="C66" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D66" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E66">
         <v>0</v>
@@ -3885,24 +3885,24 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
+        <v>180</v>
+      </c>
+      <c r="K66" t="s">
         <v>181</v>
-      </c>
-      <c r="K66" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
+        <v>203</v>
+      </c>
+      <c r="B67" t="s">
         <v>204</v>
       </c>
-      <c r="B67" t="s">
-        <v>205</v>
-      </c>
       <c r="C67" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D67" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E67">
         <v>70</v>
@@ -3920,24 +3920,24 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="K67" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B68" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C68" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D68" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E68">
         <v>90</v>
@@ -3955,24 +3955,24 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K68" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B69" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C69" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D69" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E69">
         <v>50</v>
@@ -3990,24 +3990,24 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K69" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B70" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C70" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D70" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E70">
         <v>120</v>
@@ -4025,24 +4025,24 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K70" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B71" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C71" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D71" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E71">
         <v>50</v>
@@ -4060,24 +4060,24 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
+        <v>141</v>
+      </c>
+      <c r="K71" t="s">
         <v>142</v>
-      </c>
-      <c r="K71" t="s">
-        <v>143</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B72" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C72" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D72" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E72">
         <v>58.3</v>
@@ -4095,24 +4095,24 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K72" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B73" t="s">
         <v>10</v>
       </c>
       <c r="C73" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D73" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E73">
         <v>99</v>
@@ -4130,24 +4130,24 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K73" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B74" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C74" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D74" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E74">
         <v>0</v>
@@ -4165,24 +4165,24 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="K74" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B75" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="C75" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D75" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E75">
         <v>1</v>
@@ -4194,10 +4194,10 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
+        <v>222</v>
+      </c>
+      <c r="K75" t="s">
         <v>223</v>
-      </c>
-      <c r="K75" t="s">
-        <v>224</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
@@ -4208,10 +4208,10 @@
         <v>13</v>
       </c>
       <c r="C76" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D76" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E76">
         <v>0</v>
@@ -4229,24 +4229,24 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K76" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B77" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="C77" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D77" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E77">
         <v>14.5</v>
@@ -4264,10 +4264,10 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K77" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
@@ -4278,10 +4278,10 @@
         <v>9</v>
       </c>
       <c r="C78" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D78" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E78">
         <v>0</v>
@@ -4299,24 +4299,24 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="K78" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B79" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C79" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D79" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E79">
         <v>69</v>
@@ -4334,24 +4334,24 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="K79" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>208</v>
+      </c>
+      <c r="B80" t="s">
         <v>209</v>
       </c>
-      <c r="B80" t="s">
-        <v>210</v>
-      </c>
       <c r="C80" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D80" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E80">
         <v>0</v>
@@ -4369,10 +4369,10 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
+        <v>210</v>
+      </c>
+      <c r="K80" t="s">
         <v>211</v>
-      </c>
-      <c r="K80" t="s">
-        <v>212</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
@@ -4380,16 +4380,16 @@
         <v>11</v>
       </c>
       <c r="B81" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C81" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D81" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E81">
-        <v>4.9000000000000004</v>
+        <v>4</v>
       </c>
       <c r="F81">
         <v>100</v>
@@ -4404,24 +4404,24 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="K81" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B82" t="s">
-        <v>14</v>
+        <v>230</v>
       </c>
       <c r="C82" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D82" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E82">
         <v>0</v>
@@ -4439,24 +4439,24 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="K82" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B83" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C83" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D83" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E83">
         <v>33</v>
@@ -4474,10 +4474,10 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="K83" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Removed deprecated ms_germ_risk_variant_metrics and ms_germ_risk_variant_metrics_summary
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C943E337-5200-4374-A9B9-25D5F0965982}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE95B345-A8C2-48D5-BC56-1CAEF140A09A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metrics!$A$1:$K$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metrics!$A$1:$K$82</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="515" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="227">
   <si>
     <t>nn_lower</t>
   </si>
@@ -630,18 +630,6 @@
   </si>
   <si>
     <t>MS mask regions</t>
-  </si>
-  <si>
-    <t>germline_variant_rate</t>
-  </si>
-  <si>
-    <t>_germ_risk_variant_metrics_summary.json</t>
-  </si>
-  <si>
-    <t>ms_germline_risk_masking_rate</t>
-  </si>
-  <si>
-    <t>Proportion of genomic positions masked due to risk of being a germline variant</t>
   </si>
   <si>
     <t>Gini coefficient for inequality between ex_samples</t>
@@ -1598,7 +1586,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K83"/>
+  <dimension ref="A1:K82"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" customWidth="1"/>
@@ -2575,10 +2563,10 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="B29" t="s">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="C29" t="s">
         <v>51</v>
@@ -2602,7 +2590,7 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="K29" t="s">
         <v>163</v>
@@ -2750,10 +2738,10 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>200</v>
+        <v>55</v>
       </c>
       <c r="B34" t="s">
-        <v>201</v>
+        <v>4</v>
       </c>
       <c r="C34" t="s">
         <v>197</v>
@@ -2762,80 +2750,80 @@
         <v>21</v>
       </c>
       <c r="E34">
-        <v>1.5E-3</v>
+        <v>70</v>
       </c>
       <c r="F34">
-        <v>1.4999999999999999E-2</v>
+        <v>90</v>
       </c>
       <c r="G34">
-        <v>1.5E-3</v>
+        <v>70</v>
       </c>
       <c r="H34">
-        <v>3.0000000000000001E-3</v>
+        <v>80</v>
       </c>
       <c r="I34" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>199</v>
+        <v>150</v>
       </c>
       <c r="K34" t="s">
-        <v>198</v>
+        <v>151</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>55</v>
+        <v>16</v>
       </c>
       <c r="B35" t="s">
-        <v>4</v>
+        <v>36</v>
       </c>
       <c r="C35" t="s">
-        <v>197</v>
+        <v>45</v>
       </c>
       <c r="D35" t="s">
         <v>21</v>
       </c>
       <c r="E35">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="F35">
-        <v>90</v>
-      </c>
-      <c r="G35">
-        <v>70</v>
-      </c>
-      <c r="H35">
-        <v>80</v>
+        <v>1000</v>
       </c>
       <c r="I35" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J35" t="s">
-        <v>150</v>
+        <v>54</v>
       </c>
       <c r="K35" t="s">
-        <v>151</v>
+        <v>54</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="B36" t="s">
-        <v>36</v>
+        <v>193</v>
       </c>
       <c r="C36" t="s">
         <v>45</v>
       </c>
       <c r="D36" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E36">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="F36">
-        <v>1000</v>
+        <v>0.3</v>
+      </c>
+      <c r="G36">
+        <v>0</v>
+      </c>
+      <c r="H36">
+        <v>0.2</v>
       </c>
       <c r="I36" t="b">
         <v>0</v>
@@ -2849,28 +2837,28 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B37" t="s">
-        <v>193</v>
+        <v>157</v>
       </c>
       <c r="C37" t="s">
         <v>45</v>
       </c>
       <c r="D37" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E37">
-        <v>0</v>
+        <v>71.3</v>
       </c>
       <c r="F37">
-        <v>0.3</v>
+        <v>100</v>
       </c>
       <c r="G37">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="H37">
-        <v>0.2</v>
+        <v>100</v>
       </c>
       <c r="I37" t="b">
         <v>0</v>
@@ -2884,10 +2872,10 @@
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>157</v>
+        <v>38</v>
       </c>
       <c r="C38" t="s">
         <v>45</v>
@@ -2896,16 +2884,10 @@
         <v>21</v>
       </c>
       <c r="E38">
-        <v>71.3</v>
-      </c>
-      <c r="F38">
-        <v>100</v>
-      </c>
-      <c r="G38">
-        <v>95</v>
-      </c>
-      <c r="H38">
-        <v>100</v>
+        <v>4.3</v>
+      </c>
+      <c r="F38" t="s">
+        <v>5</v>
       </c>
       <c r="I38" t="b">
         <v>0</v>
@@ -2919,22 +2901,28 @@
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="B39" t="s">
-        <v>38</v>
+        <v>193</v>
       </c>
       <c r="C39" t="s">
         <v>45</v>
       </c>
       <c r="D39" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E39">
-        <v>4.3</v>
-      </c>
-      <c r="F39" t="s">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="F39">
+        <v>0.4</v>
+      </c>
+      <c r="G39">
+        <v>0</v>
+      </c>
+      <c r="H39">
+        <v>0.3</v>
       </c>
       <c r="I39" t="b">
         <v>0</v>
@@ -2948,28 +2936,28 @@
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B40" t="s">
-        <v>193</v>
+        <v>158</v>
       </c>
       <c r="C40" t="s">
         <v>45</v>
       </c>
       <c r="D40" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E40">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F40">
-        <v>0.4</v>
+        <v>100</v>
       </c>
       <c r="G40">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="H40">
-        <v>0.3</v>
+        <v>100</v>
       </c>
       <c r="I40" t="b">
         <v>0</v>
@@ -2983,10 +2971,10 @@
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B41" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C41" t="s">
         <v>45</v>
@@ -2995,16 +2983,16 @@
         <v>21</v>
       </c>
       <c r="E41">
-        <v>35</v>
+        <v>1</v>
       </c>
       <c r="F41">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G41">
-        <v>95</v>
+        <v>1</v>
       </c>
       <c r="H41">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="I41" t="b">
         <v>0</v>
@@ -3018,10 +3006,10 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>35</v>
+        <v>17</v>
       </c>
       <c r="B42" t="s">
-        <v>159</v>
+        <v>14</v>
       </c>
       <c r="C42" t="s">
         <v>45</v>
@@ -3030,16 +3018,16 @@
         <v>21</v>
       </c>
       <c r="E42">
-        <v>1</v>
+        <v>544</v>
       </c>
       <c r="F42">
-        <v>1</v>
+        <v>624</v>
       </c>
       <c r="G42">
-        <v>1</v>
+        <v>564</v>
       </c>
       <c r="H42">
-        <v>1</v>
+        <v>604</v>
       </c>
       <c r="I42" t="b">
         <v>0</v>
@@ -3053,10 +3041,10 @@
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B43" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C43" t="s">
         <v>45</v>
@@ -3065,16 +3053,16 @@
         <v>21</v>
       </c>
       <c r="E43">
-        <v>544</v>
+        <v>94.9</v>
       </c>
       <c r="F43">
-        <v>624</v>
+        <v>100</v>
       </c>
       <c r="G43">
-        <v>564</v>
+        <v>100</v>
       </c>
       <c r="H43">
-        <v>604</v>
+        <v>100</v>
       </c>
       <c r="I43" t="b">
         <v>0</v>
@@ -3088,45 +3076,45 @@
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>18</v>
+        <v>78</v>
       </c>
       <c r="B44" t="s">
-        <v>15</v>
+        <v>186</v>
       </c>
       <c r="C44" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="D44" t="s">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="E44">
-        <v>94.9</v>
+        <v>35</v>
       </c>
       <c r="F44">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="G44">
-        <v>100</v>
+        <v>39</v>
       </c>
       <c r="H44">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="I44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J44" t="s">
-        <v>54</v>
+        <v>125</v>
       </c>
       <c r="K44" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B45" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C45" t="s">
         <v>48</v>
@@ -3150,18 +3138,18 @@
         <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K45" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B46" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C46" t="s">
         <v>48</v>
@@ -3170,30 +3158,30 @@
         <v>57</v>
       </c>
       <c r="E46">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="F46">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="G46">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="H46">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="I46" t="b">
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K46" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B47" t="s">
         <v>185</v>
@@ -3220,7 +3208,7 @@
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K47" t="s">
         <v>133</v>
@@ -3228,10 +3216,10 @@
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B48" t="s">
-        <v>185</v>
+        <v>76</v>
       </c>
       <c r="C48" t="s">
         <v>48</v>
@@ -3240,30 +3228,30 @@
         <v>57</v>
       </c>
       <c r="E48">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="F48">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="G48">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="H48">
-        <v>5</v>
+        <v>150</v>
       </c>
       <c r="I48" t="b">
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K48" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="B49" t="s">
         <v>76</v>
@@ -3290,7 +3278,7 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K49" t="s">
         <v>134</v>
@@ -3298,10 +3286,10 @@
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="B50" t="s">
-        <v>76</v>
+        <v>97</v>
       </c>
       <c r="C50" t="s">
         <v>48</v>
@@ -3310,30 +3298,30 @@
         <v>57</v>
       </c>
       <c r="E50">
-        <v>150</v>
-      </c>
-      <c r="F50">
-        <v>150</v>
+        <v>2850</v>
+      </c>
+      <c r="F50" t="s">
+        <v>5</v>
       </c>
       <c r="G50">
-        <v>150</v>
-      </c>
-      <c r="H50">
-        <v>150</v>
+        <v>3000</v>
+      </c>
+      <c r="H50" t="s">
+        <v>5</v>
       </c>
       <c r="I50" t="b">
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="K50" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B51" t="s">
         <v>97</v>
@@ -3360,7 +3348,7 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="K51" t="s">
         <v>130</v>
@@ -3368,42 +3356,42 @@
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>88</v>
+        <v>167</v>
       </c>
       <c r="B52" t="s">
-        <v>97</v>
+        <v>189</v>
       </c>
       <c r="C52" t="s">
         <v>48</v>
       </c>
       <c r="D52" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="E52">
-        <v>2850</v>
-      </c>
-      <c r="F52" t="s">
-        <v>5</v>
+        <v>30</v>
+      </c>
+      <c r="F52">
+        <v>40</v>
       </c>
       <c r="G52">
-        <v>3000</v>
-      </c>
-      <c r="H52" t="s">
-        <v>5</v>
+        <v>35</v>
+      </c>
+      <c r="H52">
+        <v>40</v>
       </c>
       <c r="I52" t="b">
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="K52" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B53" t="s">
         <v>189</v>
@@ -3430,7 +3418,7 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K53" t="s">
         <v>132</v>
@@ -3438,10 +3426,10 @@
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>168</v>
+        <v>89</v>
       </c>
       <c r="B54" t="s">
-        <v>189</v>
+        <v>99</v>
       </c>
       <c r="C54" t="s">
         <v>48</v>
@@ -3450,30 +3438,30 @@
         <v>21</v>
       </c>
       <c r="E54">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F54">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="G54">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H54">
-        <v>40</v>
+        <v>0.1</v>
       </c>
       <c r="I54" t="b">
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K54" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B55" t="s">
         <v>99</v>
@@ -3500,7 +3488,7 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K55" t="s">
         <v>135</v>
@@ -3508,10 +3496,10 @@
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B56" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C56" t="s">
         <v>48</v>
@@ -3523,27 +3511,27 @@
         <v>0</v>
       </c>
       <c r="F56">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="G56">
         <v>0</v>
       </c>
       <c r="H56">
-        <v>0.1</v>
+        <v>20</v>
       </c>
       <c r="I56" t="b">
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K56" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B57" t="s">
         <v>100</v>
@@ -3570,7 +3558,7 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K57" t="s">
         <v>136</v>
@@ -3578,10 +3566,10 @@
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B58" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C58" t="s">
         <v>48</v>
@@ -3593,27 +3581,27 @@
         <v>0</v>
       </c>
       <c r="F58">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G58">
         <v>0</v>
       </c>
       <c r="H58">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I58" t="b">
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K58" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B59" t="s">
         <v>101</v>
@@ -3640,7 +3628,7 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K59" t="s">
         <v>137</v>
@@ -3648,10 +3636,10 @@
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B60" t="s">
-        <v>101</v>
+        <v>188</v>
       </c>
       <c r="C60" t="s">
         <v>48</v>
@@ -3663,27 +3651,27 @@
         <v>0</v>
       </c>
       <c r="F60">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G60">
         <v>0</v>
       </c>
       <c r="H60">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I60" t="b">
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="K60" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B61" t="s">
         <v>188</v>
@@ -3710,7 +3698,7 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="K61" t="s">
         <v>138</v>
@@ -3718,45 +3706,45 @@
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>96</v>
+        <v>56</v>
       </c>
       <c r="B62" t="s">
-        <v>188</v>
+        <v>178</v>
       </c>
       <c r="C62" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="D62" t="s">
-        <v>21</v>
+        <v>57</v>
       </c>
       <c r="E62">
         <v>0</v>
       </c>
       <c r="F62">
+        <v>25</v>
+      </c>
+      <c r="G62">
+        <v>0</v>
+      </c>
+      <c r="H62">
         <v>10</v>
       </c>
-      <c r="G62">
-        <v>0</v>
-      </c>
-      <c r="H62">
-        <v>5</v>
-      </c>
       <c r="I62" t="b">
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>128</v>
+        <v>176</v>
       </c>
       <c r="K62" t="s">
-        <v>138</v>
+        <v>177</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>56</v>
+        <v>104</v>
       </c>
       <c r="B63" t="s">
-        <v>178</v>
+        <v>198</v>
       </c>
       <c r="C63" t="s">
         <v>50</v>
@@ -3768,13 +3756,13 @@
         <v>0</v>
       </c>
       <c r="F63">
-        <v>25</v>
+        <v>0.1</v>
       </c>
       <c r="G63">
         <v>0</v>
       </c>
       <c r="H63">
-        <v>10</v>
+        <v>0.05</v>
       </c>
       <c r="I63" t="b">
         <v>1</v>
@@ -3783,50 +3771,50 @@
         <v>176</v>
       </c>
       <c r="K63" t="s">
-        <v>177</v>
+        <v>140</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>104</v>
+        <v>161</v>
       </c>
       <c r="B64" t="s">
-        <v>202</v>
+        <v>162</v>
       </c>
       <c r="C64" t="s">
         <v>50</v>
       </c>
       <c r="D64" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="E64">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F64">
-        <v>0.1</v>
+        <v>40</v>
       </c>
       <c r="G64">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H64">
-        <v>0.05</v>
+        <v>20</v>
       </c>
       <c r="I64" t="b">
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>176</v>
+        <v>166</v>
       </c>
       <c r="K64" t="s">
-        <v>140</v>
+        <v>179</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>161</v>
+        <v>182</v>
       </c>
       <c r="B65" t="s">
-        <v>162</v>
+        <v>171</v>
       </c>
       <c r="C65" t="s">
         <v>50</v>
@@ -3835,33 +3823,33 @@
         <v>21</v>
       </c>
       <c r="E65">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F65">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="G65">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H65">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I65" t="b">
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>166</v>
+        <v>180</v>
       </c>
       <c r="K65" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>182</v>
+        <v>199</v>
       </c>
       <c r="B66" t="s">
-        <v>171</v>
+        <v>200</v>
       </c>
       <c r="C66" t="s">
         <v>50</v>
@@ -3870,68 +3858,68 @@
         <v>21</v>
       </c>
       <c r="E66">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F66">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="G66">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="H66">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="I66" t="b">
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>180</v>
+        <v>201</v>
       </c>
       <c r="K66" t="s">
-        <v>181</v>
+        <v>163</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>203</v>
+        <v>59</v>
       </c>
       <c r="B67" t="s">
-        <v>204</v>
+        <v>71</v>
       </c>
       <c r="C67" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D67" t="s">
         <v>21</v>
       </c>
       <c r="E67">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="F67">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G67">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="H67">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I67" t="b">
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>205</v>
+        <v>116</v>
       </c>
       <c r="K67" t="s">
-        <v>163</v>
+        <v>146</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B68" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C68" t="s">
         <v>47</v>
@@ -3940,13 +3928,13 @@
         <v>21</v>
       </c>
       <c r="E68">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="F68">
         <v>100</v>
       </c>
       <c r="G68">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="H68">
         <v>100</v>
@@ -3958,15 +3946,15 @@
         <v>116</v>
       </c>
       <c r="K68" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B69" t="s">
-        <v>72</v>
+        <v>105</v>
       </c>
       <c r="C69" t="s">
         <v>47</v>
@@ -3975,68 +3963,68 @@
         <v>21</v>
       </c>
       <c r="E69">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="F69">
-        <v>100</v>
+        <v>180</v>
       </c>
       <c r="G69">
-        <v>75</v>
+        <v>140</v>
       </c>
       <c r="H69">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="I69" t="b">
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="K69" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
+        <v>113</v>
+      </c>
+      <c r="B70" t="s">
+        <v>172</v>
+      </c>
+      <c r="C70" t="s">
+        <v>53</v>
+      </c>
+      <c r="D70" t="s">
+        <v>21</v>
+      </c>
+      <c r="E70">
+        <v>50</v>
+      </c>
+      <c r="F70">
+        <v>70</v>
+      </c>
+      <c r="G70">
+        <v>50</v>
+      </c>
+      <c r="H70">
         <v>60</v>
       </c>
-      <c r="B70" t="s">
-        <v>105</v>
-      </c>
-      <c r="C70" t="s">
-        <v>47</v>
-      </c>
-      <c r="D70" t="s">
-        <v>21</v>
-      </c>
-      <c r="E70">
-        <v>120</v>
-      </c>
-      <c r="F70">
-        <v>180</v>
-      </c>
-      <c r="G70">
-        <v>140</v>
-      </c>
-      <c r="H70">
-        <v>160</v>
-      </c>
       <c r="I70" t="b">
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>117</v>
+        <v>141</v>
       </c>
       <c r="K70" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>113</v>
+        <v>208</v>
       </c>
       <c r="B71" t="s">
-        <v>172</v>
+        <v>155</v>
       </c>
       <c r="C71" t="s">
         <v>53</v>
@@ -4045,33 +4033,33 @@
         <v>21</v>
       </c>
       <c r="E71">
-        <v>50</v>
+        <v>58.3</v>
       </c>
       <c r="F71">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="G71">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="H71">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="I71" t="b">
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>141</v>
+        <v>153</v>
       </c>
       <c r="K71" t="s">
-        <v>142</v>
+        <v>152</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>212</v>
+        <v>111</v>
       </c>
       <c r="B72" t="s">
-        <v>155</v>
+        <v>10</v>
       </c>
       <c r="C72" t="s">
         <v>53</v>
@@ -4080,13 +4068,13 @@
         <v>21</v>
       </c>
       <c r="E72">
-        <v>58.3</v>
+        <v>99</v>
       </c>
       <c r="F72">
         <v>100</v>
       </c>
       <c r="G72">
-        <v>90</v>
+        <v>99.5</v>
       </c>
       <c r="H72">
         <v>100</v>
@@ -4095,18 +4083,18 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="K72" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B73" t="s">
-        <v>10</v>
+        <v>109</v>
       </c>
       <c r="C73" t="s">
         <v>53</v>
@@ -4115,16 +4103,16 @@
         <v>21</v>
       </c>
       <c r="E73">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="F73">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="G73">
-        <v>99.5</v>
+        <v>0</v>
       </c>
       <c r="H73">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="I73" t="b">
         <v>1</v>
@@ -4133,15 +4121,15 @@
         <v>145</v>
       </c>
       <c r="K73" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>110</v>
+        <v>220</v>
       </c>
       <c r="B74" t="s">
-        <v>109</v>
+        <v>224</v>
       </c>
       <c r="C74" t="s">
         <v>53</v>
@@ -4150,33 +4138,33 @@
         <v>21</v>
       </c>
       <c r="E74">
-        <v>0</v>
-      </c>
-      <c r="F74">
-        <v>15</v>
+        <v>1</v>
+      </c>
+      <c r="F74" t="s">
+        <v>5</v>
       </c>
       <c r="G74">
-        <v>0</v>
-      </c>
-      <c r="H74">
+        <v>1</v>
+      </c>
+      <c r="H74" t="s">
         <v>5</v>
       </c>
       <c r="I74" t="b">
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>145</v>
+        <v>218</v>
       </c>
       <c r="K74" t="s">
-        <v>144</v>
+        <v>219</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>224</v>
+        <v>12</v>
       </c>
       <c r="B75" t="s">
-        <v>228</v>
+        <v>13</v>
       </c>
       <c r="C75" t="s">
         <v>53</v>
@@ -4185,33 +4173,33 @@
         <v>21</v>
       </c>
       <c r="E75">
-        <v>1</v>
-      </c>
-      <c r="F75" t="s">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="F75">
+        <v>0</v>
       </c>
       <c r="G75">
-        <v>1</v>
-      </c>
-      <c r="H75" t="s">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="H75">
+        <v>0</v>
       </c>
       <c r="I75" t="b">
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>222</v>
+        <v>118</v>
       </c>
       <c r="K75" t="s">
-        <v>223</v>
+        <v>139</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>12</v>
+        <v>225</v>
       </c>
       <c r="B76" t="s">
-        <v>13</v>
+        <v>221</v>
       </c>
       <c r="C76" t="s">
         <v>53</v>
@@ -4220,33 +4208,33 @@
         <v>21</v>
       </c>
       <c r="E76">
-        <v>0</v>
+        <v>14.5</v>
       </c>
       <c r="F76">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G76">
-        <v>0</v>
+        <v>26.1</v>
       </c>
       <c r="H76">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I76" t="b">
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>118</v>
+        <v>154</v>
       </c>
       <c r="K76" t="s">
-        <v>139</v>
+        <v>223</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>229</v>
+        <v>8</v>
       </c>
       <c r="B77" t="s">
-        <v>225</v>
+        <v>9</v>
       </c>
       <c r="C77" t="s">
         <v>53</v>
@@ -4255,33 +4243,33 @@
         <v>21</v>
       </c>
       <c r="E77">
-        <v>14.5</v>
+        <v>0</v>
       </c>
       <c r="F77">
-        <v>100</v>
+        <v>1.2E-2</v>
       </c>
       <c r="G77">
-        <v>26.1</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="H77">
-        <v>100</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="I77" t="b">
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="K77" t="s">
-        <v>227</v>
+        <v>164</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>8</v>
+        <v>210</v>
       </c>
       <c r="B78" t="s">
-        <v>9</v>
+        <v>212</v>
       </c>
       <c r="C78" t="s">
         <v>53</v>
@@ -4290,68 +4278,68 @@
         <v>21</v>
       </c>
       <c r="E78">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="F78">
-        <v>1.2E-2</v>
+        <v>120</v>
       </c>
       <c r="G78">
-        <v>2.0000000000000001E-4</v>
+        <v>82.8</v>
       </c>
       <c r="H78">
-        <v>6.0000000000000001E-3</v>
+        <v>120</v>
       </c>
       <c r="I78" t="b">
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>165</v>
+        <v>211</v>
       </c>
       <c r="K78" t="s">
-        <v>164</v>
+        <v>213</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>214</v>
+        <v>204</v>
       </c>
       <c r="B79" t="s">
-        <v>216</v>
+        <v>205</v>
       </c>
       <c r="C79" t="s">
-        <v>53</v>
+        <v>160</v>
       </c>
       <c r="D79" t="s">
         <v>21</v>
       </c>
       <c r="E79">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="F79">
-        <v>120</v>
+        <v>5.6599999999999999E-4</v>
       </c>
       <c r="G79">
-        <v>82.8</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="H79">
-        <v>120</v>
+        <v>3.2679999999999997E-4</v>
       </c>
       <c r="I79" t="b">
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="K79" t="s">
-        <v>217</v>
+        <v>207</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>208</v>
+        <v>11</v>
       </c>
       <c r="B80" t="s">
-        <v>209</v>
+        <v>222</v>
       </c>
       <c r="C80" t="s">
         <v>160</v>
@@ -4360,30 +4348,30 @@
         <v>21</v>
       </c>
       <c r="E80">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F80">
-        <v>5.6599999999999999E-4</v>
+        <v>100</v>
       </c>
       <c r="G80">
-        <v>2.0000000000000001E-4</v>
+        <v>20</v>
       </c>
       <c r="H80">
-        <v>3.2679999999999997E-4</v>
+        <v>100</v>
       </c>
       <c r="I80" t="b">
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>210</v>
+        <v>154</v>
       </c>
       <c r="K80" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>11</v>
+        <v>209</v>
       </c>
       <c r="B81" t="s">
         <v>226</v>
@@ -4395,33 +4383,33 @@
         <v>21</v>
       </c>
       <c r="E81">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F81">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="G81">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H81">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="I81" t="b">
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>154</v>
+        <v>129</v>
       </c>
       <c r="K81" t="s">
-        <v>218</v>
+        <v>149</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>213</v>
+        <v>43</v>
       </c>
       <c r="B82" t="s">
-        <v>230</v>
+        <v>216</v>
       </c>
       <c r="C82" t="s">
         <v>160</v>
@@ -4430,64 +4418,29 @@
         <v>21</v>
       </c>
       <c r="E82">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="F82">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="G82">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="H82">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="I82" t="b">
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>129</v>
+        <v>215</v>
       </c>
       <c r="K82" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A83" t="s">
-        <v>43</v>
-      </c>
-      <c r="B83" t="s">
-        <v>220</v>
-      </c>
-      <c r="C83" t="s">
-        <v>160</v>
-      </c>
-      <c r="D83" t="s">
-        <v>21</v>
-      </c>
-      <c r="E83">
-        <v>33</v>
-      </c>
-      <c r="F83">
-        <v>100</v>
-      </c>
-      <c r="G83">
-        <v>67</v>
-      </c>
-      <c r="H83">
-        <v>100</v>
-      </c>
-      <c r="I83" t="b">
-        <v>1</v>
-      </c>
-      <c r="J83" t="s">
-        <v>219</v>
-      </c>
-      <c r="K83" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K83" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K82" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated thresholds for DNA fragment size component metrics
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE95B345-A8C2-48D5-BC56-1CAEF140A09A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B4835CF-4662-47E3-A1CB-17A8A099294F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -509,12 +509,6 @@
     <t>Percentage of fragments that fall within the expected size range on gel elextrophoresis (10,000-50,000 bp)</t>
   </si>
   <si>
-    <t>Percentage of fragments that fall within the expected size range on gel elextrophoresis (100-200 bp)</t>
-  </si>
-  <si>
-    <t>Percentage of fragments that fall within the expected size range on gel elextrophoresis (490-690 bp)</t>
-  </si>
-  <si>
     <t>Distinct band at aprox 290 and sometimes 480 bp, with no smears. 1 = pass 0 = fail.</t>
   </si>
   <si>
@@ -717,6 +711,12 @@
   </si>
   <si>
     <t>Percentage of reads lost between start and end of EX pipeline</t>
+  </si>
+  <si>
+    <t>Percentage of fragments that fall within the expected size range on gel electrophoresis (80-250 bp)</t>
+  </si>
+  <si>
+    <t>Percentage of fragments that fall within the expected size range on gel elextrophoresis (450-790 bp)</t>
   </si>
 </sst>
 </file>
@@ -1639,7 +1639,7 @@
         <v>30</v>
       </c>
       <c r="B2" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="C2" t="s">
         <v>44</v>
@@ -1668,7 +1668,7 @@
         <v>31</v>
       </c>
       <c r="B3" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C3" t="s">
         <v>44</v>
@@ -1712,7 +1712,7 @@
         <v>21</v>
       </c>
       <c r="E4">
-        <v>77.2</v>
+        <v>85</v>
       </c>
       <c r="F4">
         <v>100</v>
@@ -1738,7 +1738,7 @@
         <v>40</v>
       </c>
       <c r="B5" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C5" t="s">
         <v>46</v>
@@ -1767,7 +1767,7 @@
         <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C6" t="s">
         <v>46</v>
@@ -1802,7 +1802,7 @@
         <v>41</v>
       </c>
       <c r="B7" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="C7" t="s">
         <v>46</v>
@@ -1831,7 +1831,7 @@
         <v>42</v>
       </c>
       <c r="B8" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C8" t="s">
         <v>46</v>
@@ -2006,7 +2006,7 @@
         <v>84</v>
       </c>
       <c r="B13" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C13" t="s">
         <v>49</v>
@@ -2041,7 +2041,7 @@
         <v>85</v>
       </c>
       <c r="B14" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C14" t="s">
         <v>49</v>
@@ -2076,7 +2076,7 @@
         <v>82</v>
       </c>
       <c r="B15" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C15" t="s">
         <v>49</v>
@@ -2111,7 +2111,7 @@
         <v>83</v>
       </c>
       <c r="B16" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C16" t="s">
         <v>49</v>
@@ -2213,10 +2213,10 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B19" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C19" t="s">
         <v>49</v>
@@ -2248,10 +2248,10 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B20" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C20" t="s">
         <v>49</v>
@@ -2496,7 +2496,7 @@
         <v>69</v>
       </c>
       <c r="B27" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C27" t="s">
         <v>49</v>
@@ -2531,7 +2531,7 @@
         <v>70</v>
       </c>
       <c r="B28" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C28" t="s">
         <v>49</v>
@@ -2563,10 +2563,10 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B29" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C29" t="s">
         <v>51</v>
@@ -2590,10 +2590,10 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="K29" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
@@ -2660,18 +2660,18 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="K31" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B32" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C32" t="s">
         <v>52</v>
@@ -2695,10 +2695,10 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="K32" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
@@ -2744,7 +2744,7 @@
         <v>4</v>
       </c>
       <c r="C34" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D34" t="s">
         <v>21</v>
@@ -2805,7 +2805,7 @@
         <v>23</v>
       </c>
       <c r="B36" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C36" t="s">
         <v>45</v>
@@ -2840,7 +2840,7 @@
         <v>29</v>
       </c>
       <c r="B37" t="s">
-        <v>157</v>
+        <v>225</v>
       </c>
       <c r="C37" t="s">
         <v>45</v>
@@ -2849,7 +2849,7 @@
         <v>21</v>
       </c>
       <c r="E37">
-        <v>71.3</v>
+        <v>85</v>
       </c>
       <c r="F37">
         <v>100</v>
@@ -2904,7 +2904,7 @@
         <v>33</v>
       </c>
       <c r="B39" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="C39" t="s">
         <v>45</v>
@@ -2939,7 +2939,7 @@
         <v>34</v>
       </c>
       <c r="B40" t="s">
-        <v>158</v>
+        <v>226</v>
       </c>
       <c r="C40" t="s">
         <v>45</v>
@@ -2948,13 +2948,13 @@
         <v>21</v>
       </c>
       <c r="E40">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="F40">
         <v>100</v>
       </c>
       <c r="G40">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="H40">
         <v>100</v>
@@ -2974,7 +2974,7 @@
         <v>35</v>
       </c>
       <c r="B41" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="C41" t="s">
         <v>45</v>
@@ -3079,7 +3079,7 @@
         <v>78</v>
       </c>
       <c r="B44" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C44" t="s">
         <v>48</v>
@@ -3114,7 +3114,7 @@
         <v>79</v>
       </c>
       <c r="B45" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C45" t="s">
         <v>48</v>
@@ -3149,7 +3149,7 @@
         <v>80</v>
       </c>
       <c r="B46" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C46" t="s">
         <v>48</v>
@@ -3184,7 +3184,7 @@
         <v>81</v>
       </c>
       <c r="B47" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="C47" t="s">
         <v>48</v>
@@ -3356,10 +3356,10 @@
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B52" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C52" t="s">
         <v>48</v>
@@ -3391,10 +3391,10 @@
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="B53" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C53" t="s">
         <v>48</v>
@@ -3639,7 +3639,7 @@
         <v>95</v>
       </c>
       <c r="B60" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C60" t="s">
         <v>48</v>
@@ -3674,7 +3674,7 @@
         <v>96</v>
       </c>
       <c r="B61" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C61" t="s">
         <v>48</v>
@@ -3709,7 +3709,7 @@
         <v>56</v>
       </c>
       <c r="B62" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="C62" t="s">
         <v>50</v>
@@ -3733,10 +3733,10 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="K62" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
@@ -3744,7 +3744,7 @@
         <v>104</v>
       </c>
       <c r="B63" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C63" t="s">
         <v>50</v>
@@ -3768,7 +3768,7 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="K63" t="s">
         <v>140</v>
@@ -3776,10 +3776,10 @@
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="B64" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C64" t="s">
         <v>50</v>
@@ -3803,18 +3803,18 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="K64" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B65" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C65" t="s">
         <v>50</v>
@@ -3838,18 +3838,18 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="K65" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B66" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C66" t="s">
         <v>50</v>
@@ -3873,10 +3873,10 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="K66" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
@@ -3989,7 +3989,7 @@
         <v>113</v>
       </c>
       <c r="B70" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C70" t="s">
         <v>53</v>
@@ -4021,7 +4021,7 @@
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B71" t="s">
         <v>155</v>
@@ -4126,10 +4126,10 @@
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B74" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="C74" t="s">
         <v>53</v>
@@ -4153,10 +4153,10 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="K74" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
@@ -4196,10 +4196,10 @@
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B76" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="C76" t="s">
         <v>53</v>
@@ -4226,7 +4226,7 @@
         <v>154</v>
       </c>
       <c r="K76" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
@@ -4258,18 +4258,18 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="K77" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
+        <v>208</v>
+      </c>
+      <c r="B78" t="s">
         <v>210</v>
-      </c>
-      <c r="B78" t="s">
-        <v>212</v>
       </c>
       <c r="C78" t="s">
         <v>53</v>
@@ -4293,21 +4293,21 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
+        <v>209</v>
+      </c>
+      <c r="K78" t="s">
         <v>211</v>
-      </c>
-      <c r="K78" t="s">
-        <v>213</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B79" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="C79" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D79" t="s">
         <v>21</v>
@@ -4328,10 +4328,10 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="K79" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
@@ -4339,10 +4339,10 @@
         <v>11</v>
       </c>
       <c r="B80" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="C80" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D80" t="s">
         <v>21</v>
@@ -4366,18 +4366,18 @@
         <v>154</v>
       </c>
       <c r="K80" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B81" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="C81" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D81" t="s">
         <v>21</v>
@@ -4409,10 +4409,10 @@
         <v>43</v>
       </c>
       <c r="B82" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C82" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="D82" t="s">
         <v>21</v>
@@ -4433,10 +4433,10 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
+        <v>213</v>
+      </c>
+      <c r="K82" t="s">
         <v>215</v>
-      </c>
-      <c r="K82" t="s">
-        <v>217</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added new median fragment length component metrics
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B4835CF-4662-47E3-A1CB-17A8A099294F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67A8019C-A426-48D6-BB3A-3ECB2F7F88D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metrics!$A$1:$K$82</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metrics!$A$1:$K$84</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="509" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="231">
   <si>
     <t>nn_lower</t>
   </si>
@@ -125,24 +125,15 @@
     <t>Name</t>
   </si>
   <si>
-    <t>ex_fragmented_DNA_size</t>
-  </si>
-  <si>
     <t>extracted_DNA_yield</t>
   </si>
   <si>
     <t>extracted_DNA_yield_variability</t>
   </si>
   <si>
-    <t>extracted_DNA_size</t>
-  </si>
-  <si>
     <t>ex_amplified_DNA_yield_variability</t>
   </si>
   <si>
-    <t>ex_amplified_DNA_size</t>
-  </si>
-  <si>
     <t>ex_amplified_NTC_size</t>
   </si>
   <si>
@@ -713,10 +704,31 @@
     <t>Percentage of reads lost between start and end of EX pipeline</t>
   </si>
   <si>
-    <t>Percentage of fragments that fall within the expected size range on gel electrophoresis (80-250 bp)</t>
-  </si>
-  <si>
-    <t>Percentage of fragments that fall within the expected size range on gel elextrophoresis (450-790 bp)</t>
+    <t>ex_fragmented_DNA_size_pct</t>
+  </si>
+  <si>
+    <t>ex_fragmented_DNA_size_median</t>
+  </si>
+  <si>
+    <t>Percentage of fragments that fall within the expected size range on gel (80-250 bp)</t>
+  </si>
+  <si>
+    <t>ex_amplified_DNA_size_pct</t>
+  </si>
+  <si>
+    <t>ex_amplified_DNA_size_median</t>
+  </si>
+  <si>
+    <t>Percentage of fragments that fall within the expected size range on gel (450-790 bp)</t>
+  </si>
+  <si>
+    <t>Median length of fragments on gel following fragmentation and size selection</t>
+  </si>
+  <si>
+    <t>Median length of fragments on gel following amplification</t>
+  </si>
+  <si>
+    <t>extracted_DNA_size_pct</t>
   </si>
 </sst>
 </file>
@@ -1586,7 +1598,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K82"/>
+  <dimension ref="A1:K84"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" customWidth="1"/>
@@ -1628,21 +1640,21 @@
         <v>27</v>
       </c>
       <c r="J1" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="K1" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C2" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D2" t="s">
         <v>21</v>
@@ -1657,21 +1669,21 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K2" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="C3" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D3" t="s">
         <v>22</v>
@@ -1692,21 +1704,21 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K3" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>32</v>
+        <v>230</v>
       </c>
       <c r="B4" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="C4" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D4" t="s">
         <v>21</v>
@@ -1727,21 +1739,21 @@
         <v>0</v>
       </c>
       <c r="J4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K4" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="B5" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="C5" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D5" t="s">
         <v>21</v>
@@ -1756,21 +1768,21 @@
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K5" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B6" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C6" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D6" t="s">
         <v>22</v>
@@ -1791,21 +1803,21 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K6" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B7" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="C7" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D7" t="s">
         <v>21</v>
@@ -1820,21 +1832,21 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K7" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D8" t="s">
         <v>22</v>
@@ -1855,10 +1867,10 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K8" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -1866,10 +1878,10 @@
         <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="C9" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D9" t="s">
         <v>21</v>
@@ -1890,10 +1902,10 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K9" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -1901,10 +1913,10 @@
         <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C10" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D10" t="s">
         <v>21</v>
@@ -1925,10 +1937,10 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K10" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -1936,10 +1948,10 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D11" t="s">
         <v>21</v>
@@ -1960,10 +1972,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="K11" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1971,10 +1983,10 @@
         <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="C12" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D12" t="s">
         <v>21</v>
@@ -1995,21 +2007,21 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="K12" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B13" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="C13" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D13" t="s">
         <v>21</v>
@@ -2030,21 +2042,21 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="K13" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="B14" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="C14" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D14" t="s">
         <v>21</v>
@@ -2065,21 +2077,21 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="K14" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="B15" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C15" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D15" t="s">
         <v>21</v>
@@ -2100,21 +2112,21 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="K15" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B16" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="C16" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D16" t="s">
         <v>21</v>
@@ -2135,21 +2147,21 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="K16" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="B17" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C17" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D17" t="s">
         <v>21</v>
@@ -2170,21 +2182,21 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="K17" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="B18" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C18" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D18" t="s">
         <v>21</v>
@@ -2205,21 +2217,21 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="K18" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="B19" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C19" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D19" t="s">
         <v>21</v>
@@ -2240,21 +2252,21 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="K19" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="B20" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="C20" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D20" t="s">
         <v>21</v>
@@ -2275,21 +2287,21 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="K20" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B21" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C21" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D21" t="s">
         <v>21</v>
@@ -2310,21 +2322,21 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="K21" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B22" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="C22" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D22" t="s">
         <v>21</v>
@@ -2345,21 +2357,21 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="K22" t="s">
-        <v>135</v>
+        <v>132</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B23" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C23" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D23" t="s">
         <v>21</v>
@@ -2380,21 +2392,21 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="K23" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B24" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="C24" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D24" t="s">
         <v>21</v>
@@ -2415,21 +2427,21 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="K24" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="B25" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C25" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D25" t="s">
         <v>21</v>
@@ -2450,21 +2462,21 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="K25" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="B26" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C26" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D26" t="s">
         <v>21</v>
@@ -2485,21 +2497,21 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="K26" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B27" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C27" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D27" t="s">
         <v>21</v>
@@ -2520,21 +2532,21 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="K27" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="B28" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C28" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D28" t="s">
         <v>21</v>
@@ -2555,21 +2567,21 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="K28" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B29" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="C29" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D29" t="s">
         <v>21</v>
@@ -2590,21 +2602,21 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="K29" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="B30" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C30" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D30" t="s">
         <v>21</v>
@@ -2625,21 +2637,21 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="K30" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="B31" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C31" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D31" t="s">
         <v>21</v>
@@ -2660,21 +2672,21 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="K31" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="B32" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
       <c r="C32" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D32" t="s">
         <v>21</v>
@@ -2695,21 +2707,21 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="K32" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="B33" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C33" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D33" t="s">
         <v>21</v>
@@ -2730,21 +2742,21 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="K33" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B34" t="s">
         <v>4</v>
       </c>
       <c r="C34" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="D34" t="s">
         <v>21</v>
@@ -2765,10 +2777,10 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="K34" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -2776,10 +2788,10 @@
         <v>16</v>
       </c>
       <c r="B35" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="C35" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D35" t="s">
         <v>21</v>
@@ -2794,10 +2806,10 @@
         <v>0</v>
       </c>
       <c r="J35" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K35" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -2805,10 +2817,10 @@
         <v>23</v>
       </c>
       <c r="B36" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="C36" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D36" t="s">
         <v>22</v>
@@ -2829,21 +2841,21 @@
         <v>0</v>
       </c>
       <c r="J36" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K36" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>29</v>
+        <v>222</v>
       </c>
       <c r="B37" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C37" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D37" t="s">
         <v>21</v>
@@ -2864,354 +2876,348 @@
         <v>0</v>
       </c>
       <c r="J37" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K37" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>37</v>
+        <v>223</v>
       </c>
       <c r="B38" t="s">
-        <v>38</v>
+        <v>228</v>
       </c>
       <c r="C38" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D38" t="s">
         <v>21</v>
       </c>
       <c r="E38">
-        <v>4.3</v>
-      </c>
-      <c r="F38" t="s">
-        <v>5</v>
+        <v>110</v>
+      </c>
+      <c r="F38">
+        <v>150</v>
+      </c>
+      <c r="G38">
+        <v>120</v>
+      </c>
+      <c r="H38">
+        <v>140</v>
       </c>
       <c r="I38" t="b">
         <v>0</v>
       </c>
       <c r="J38" t="s">
-        <v>54</v>
-      </c>
-      <c r="K38" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B39" t="s">
-        <v>191</v>
+        <v>35</v>
       </c>
       <c r="C39" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D39" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E39">
-        <v>0</v>
-      </c>
-      <c r="F39">
-        <v>0.4</v>
-      </c>
-      <c r="G39">
-        <v>0</v>
-      </c>
-      <c r="H39">
-        <v>0.3</v>
+        <v>4.3</v>
+      </c>
+      <c r="F39" t="s">
+        <v>5</v>
       </c>
       <c r="I39" t="b">
         <v>0</v>
       </c>
       <c r="J39" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K39" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="B40" t="s">
-        <v>226</v>
+        <v>188</v>
       </c>
       <c r="C40" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D40" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E40">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F40">
-        <v>100</v>
+        <v>0.4</v>
       </c>
       <c r="G40">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="H40">
-        <v>100</v>
+        <v>0.3</v>
       </c>
       <c r="I40" t="b">
         <v>0</v>
       </c>
       <c r="J40" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K40" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>35</v>
+        <v>225</v>
       </c>
       <c r="B41" t="s">
-        <v>157</v>
+        <v>227</v>
       </c>
       <c r="C41" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D41" t="s">
         <v>21</v>
       </c>
       <c r="E41">
-        <v>1</v>
+        <v>50</v>
       </c>
       <c r="F41">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="G41">
-        <v>1</v>
+        <v>90</v>
       </c>
       <c r="H41">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I41" t="b">
         <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K41" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>17</v>
+        <v>226</v>
       </c>
       <c r="B42" t="s">
-        <v>14</v>
+        <v>229</v>
       </c>
       <c r="C42" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D42" t="s">
         <v>21</v>
       </c>
       <c r="E42">
-        <v>544</v>
+        <v>440</v>
       </c>
       <c r="F42">
-        <v>624</v>
+        <v>740</v>
       </c>
       <c r="G42">
-        <v>564</v>
+        <v>530</v>
       </c>
       <c r="H42">
-        <v>604</v>
+        <v>650</v>
       </c>
       <c r="I42" t="b">
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>54</v>
-      </c>
-      <c r="K42" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="B43" t="s">
-        <v>15</v>
+        <v>154</v>
       </c>
       <c r="C43" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D43" t="s">
         <v>21</v>
       </c>
       <c r="E43">
-        <v>94.9</v>
+        <v>1</v>
       </c>
       <c r="F43">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="G43">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="H43">
-        <v>100</v>
+        <v>1</v>
       </c>
       <c r="I43" t="b">
         <v>0</v>
       </c>
       <c r="J43" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="K43" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>78</v>
+        <v>17</v>
       </c>
       <c r="B44" t="s">
-        <v>184</v>
+        <v>14</v>
       </c>
       <c r="C44" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D44" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="E44">
-        <v>35</v>
+        <v>544</v>
       </c>
       <c r="F44">
-        <v>40</v>
+        <v>624</v>
       </c>
       <c r="G44">
-        <v>39</v>
+        <v>564</v>
       </c>
       <c r="H44">
-        <v>40</v>
+        <v>604</v>
       </c>
       <c r="I44" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J44" t="s">
-        <v>125</v>
+        <v>51</v>
       </c>
       <c r="K44" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>79</v>
+        <v>18</v>
       </c>
       <c r="B45" t="s">
-        <v>185</v>
+        <v>15</v>
       </c>
       <c r="C45" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D45" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="E45">
-        <v>35</v>
+        <v>94.9</v>
       </c>
       <c r="F45">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="G45">
-        <v>39</v>
+        <v>100</v>
       </c>
       <c r="H45">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="I45" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J45" t="s">
-        <v>126</v>
+        <v>51</v>
       </c>
       <c r="K45" t="s">
-        <v>131</v>
+        <v>51</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="B46" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C46" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D46" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E46">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F46">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G46">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="H46">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="I46" t="b">
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="K46" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B47" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="C47" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D47" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E47">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F47">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G47">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="H47">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="I47" t="b">
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="K47" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
@@ -3219,290 +3225,290 @@
         <v>77</v>
       </c>
       <c r="B48" t="s">
-        <v>76</v>
+        <v>180</v>
       </c>
       <c r="C48" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D48" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E48">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F48">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="G48">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="H48">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="I48" t="b">
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="K48" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>86</v>
+        <v>78</v>
       </c>
       <c r="B49" t="s">
-        <v>76</v>
+        <v>180</v>
       </c>
       <c r="C49" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D49" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E49">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F49">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="G49">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="H49">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="I49" t="b">
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="K49" t="s">
-        <v>134</v>
+        <v>130</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="B50" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="C50" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D50" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E50">
-        <v>2850</v>
-      </c>
-      <c r="F50" t="s">
-        <v>5</v>
+        <v>150</v>
+      </c>
+      <c r="F50">
+        <v>150</v>
       </c>
       <c r="G50">
-        <v>3000</v>
-      </c>
-      <c r="H50" t="s">
-        <v>5</v>
+        <v>150</v>
+      </c>
+      <c r="H50">
+        <v>150</v>
       </c>
       <c r="I50" t="b">
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="K50" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B51" t="s">
-        <v>97</v>
+        <v>73</v>
       </c>
       <c r="C51" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D51" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E51">
-        <v>2850</v>
-      </c>
-      <c r="F51" t="s">
-        <v>5</v>
+        <v>150</v>
+      </c>
+      <c r="F51">
+        <v>150</v>
       </c>
       <c r="G51">
-        <v>3000</v>
-      </c>
-      <c r="H51" t="s">
-        <v>5</v>
+        <v>150</v>
+      </c>
+      <c r="H51">
+        <v>150</v>
       </c>
       <c r="I51" t="b">
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="K51" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>165</v>
+        <v>84</v>
       </c>
       <c r="B52" t="s">
-        <v>187</v>
+        <v>94</v>
       </c>
       <c r="C52" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D52" t="s">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="E52">
-        <v>30</v>
-      </c>
-      <c r="F52">
-        <v>40</v>
+        <v>2850</v>
+      </c>
+      <c r="F52" t="s">
+        <v>5</v>
       </c>
       <c r="G52">
-        <v>35</v>
-      </c>
-      <c r="H52">
-        <v>40</v>
+        <v>3000</v>
+      </c>
+      <c r="H52" t="s">
+        <v>5</v>
       </c>
       <c r="I52" t="b">
         <v>1</v>
       </c>
       <c r="J52" t="s">
+        <v>122</v>
+      </c>
+      <c r="K52" t="s">
         <v>127</v>
-      </c>
-      <c r="K52" t="s">
-        <v>132</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>166</v>
+        <v>85</v>
       </c>
       <c r="B53" t="s">
-        <v>187</v>
+        <v>94</v>
       </c>
       <c r="C53" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D53" t="s">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="E53">
-        <v>30</v>
-      </c>
-      <c r="F53">
-        <v>40</v>
+        <v>2850</v>
+      </c>
+      <c r="F53" t="s">
+        <v>5</v>
       </c>
       <c r="G53">
-        <v>35</v>
-      </c>
-      <c r="H53">
-        <v>40</v>
+        <v>3000</v>
+      </c>
+      <c r="H53" t="s">
+        <v>5</v>
       </c>
       <c r="I53" t="b">
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="K53" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>89</v>
+        <v>162</v>
       </c>
       <c r="B54" t="s">
-        <v>99</v>
+        <v>184</v>
       </c>
       <c r="C54" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D54" t="s">
         <v>21</v>
       </c>
       <c r="E54">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F54">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="G54">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H54">
-        <v>0.1</v>
+        <v>40</v>
       </c>
       <c r="I54" t="b">
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="K54" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>90</v>
+        <v>163</v>
       </c>
       <c r="B55" t="s">
-        <v>99</v>
+        <v>184</v>
       </c>
       <c r="C55" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D55" t="s">
         <v>21</v>
       </c>
       <c r="E55">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F55">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="G55">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H55">
-        <v>0.1</v>
+        <v>40</v>
       </c>
       <c r="I55" t="b">
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="K55" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B56" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C56" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D56" t="s">
         <v>21</v>
@@ -3511,33 +3517,33 @@
         <v>0</v>
       </c>
       <c r="F56">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="G56">
         <v>0</v>
       </c>
       <c r="H56">
-        <v>20</v>
+        <v>0.1</v>
       </c>
       <c r="I56" t="b">
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="K56" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B57" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C57" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D57" t="s">
         <v>21</v>
@@ -3546,33 +3552,33 @@
         <v>0</v>
       </c>
       <c r="F57">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="G57">
         <v>0</v>
       </c>
       <c r="H57">
-        <v>20</v>
+        <v>0.1</v>
       </c>
       <c r="I57" t="b">
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="K57" t="s">
-        <v>136</v>
+        <v>132</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B58" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C58" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D58" t="s">
         <v>21</v>
@@ -3581,33 +3587,33 @@
         <v>0</v>
       </c>
       <c r="F58">
+        <v>30</v>
+      </c>
+      <c r="G58">
+        <v>0</v>
+      </c>
+      <c r="H58">
         <v>20</v>
       </c>
-      <c r="G58">
-        <v>0</v>
-      </c>
-      <c r="H58">
-        <v>10</v>
-      </c>
       <c r="I58" t="b">
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="K58" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B59" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C59" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D59" t="s">
         <v>21</v>
@@ -3616,33 +3622,33 @@
         <v>0</v>
       </c>
       <c r="F59">
+        <v>30</v>
+      </c>
+      <c r="G59">
+        <v>0</v>
+      </c>
+      <c r="H59">
         <v>20</v>
       </c>
-      <c r="G59">
-        <v>0</v>
-      </c>
-      <c r="H59">
-        <v>10</v>
-      </c>
       <c r="I59" t="b">
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="K59" t="s">
-        <v>137</v>
+        <v>133</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B60" t="s">
-        <v>186</v>
+        <v>98</v>
       </c>
       <c r="C60" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D60" t="s">
         <v>21</v>
@@ -3651,33 +3657,33 @@
         <v>0</v>
       </c>
       <c r="F60">
+        <v>20</v>
+      </c>
+      <c r="G60">
+        <v>0</v>
+      </c>
+      <c r="H60">
         <v>10</v>
       </c>
-      <c r="G60">
-        <v>0</v>
-      </c>
-      <c r="H60">
-        <v>5</v>
-      </c>
       <c r="I60" t="b">
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="K60" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B61" t="s">
-        <v>186</v>
+        <v>98</v>
       </c>
       <c r="C61" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D61" t="s">
         <v>21</v>
@@ -3686,205 +3692,205 @@
         <v>0</v>
       </c>
       <c r="F61">
+        <v>20</v>
+      </c>
+      <c r="G61">
+        <v>0</v>
+      </c>
+      <c r="H61">
         <v>10</v>
       </c>
-      <c r="G61">
-        <v>0</v>
-      </c>
-      <c r="H61">
-        <v>5</v>
-      </c>
       <c r="I61" t="b">
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="K61" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>56</v>
+        <v>92</v>
       </c>
       <c r="B62" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="C62" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D62" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="E62">
         <v>0</v>
       </c>
       <c r="F62">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G62">
         <v>0</v>
       </c>
       <c r="H62">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I62" t="b">
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>174</v>
+        <v>124</v>
       </c>
       <c r="K62" t="s">
-        <v>175</v>
+        <v>135</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>104</v>
+        <v>93</v>
       </c>
       <c r="B63" t="s">
-        <v>196</v>
+        <v>183</v>
       </c>
       <c r="C63" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D63" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
       <c r="E63">
         <v>0</v>
       </c>
       <c r="F63">
-        <v>0.1</v>
+        <v>10</v>
       </c>
       <c r="G63">
         <v>0</v>
       </c>
       <c r="H63">
-        <v>0.05</v>
+        <v>5</v>
       </c>
       <c r="I63" t="b">
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>174</v>
+        <v>125</v>
       </c>
       <c r="K63" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>159</v>
+        <v>53</v>
       </c>
       <c r="B64" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="C64" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D64" t="s">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="E64">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F64">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="G64">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H64">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I64" t="b">
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="K64" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>180</v>
+        <v>101</v>
       </c>
       <c r="B65" t="s">
-        <v>169</v>
+        <v>193</v>
       </c>
       <c r="C65" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D65" t="s">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="E65">
         <v>0</v>
       </c>
       <c r="F65">
-        <v>20</v>
+        <v>0.1</v>
       </c>
       <c r="G65">
         <v>0</v>
       </c>
       <c r="H65">
-        <v>10</v>
+        <v>0.05</v>
       </c>
       <c r="I65" t="b">
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="K65" t="s">
-        <v>179</v>
+        <v>137</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>197</v>
+        <v>156</v>
       </c>
       <c r="B66" t="s">
-        <v>198</v>
+        <v>157</v>
       </c>
       <c r="C66" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D66" t="s">
         <v>21</v>
       </c>
       <c r="E66">
-        <v>70</v>
+        <v>1</v>
       </c>
       <c r="F66">
-        <v>99</v>
+        <v>40</v>
       </c>
       <c r="G66">
-        <v>85</v>
+        <v>1</v>
       </c>
       <c r="H66">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="I66" t="b">
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>199</v>
+        <v>161</v>
       </c>
       <c r="K66" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>59</v>
+        <v>177</v>
       </c>
       <c r="B67" t="s">
-        <v>71</v>
+        <v>166</v>
       </c>
       <c r="C67" t="s">
         <v>47</v>
@@ -3893,33 +3899,33 @@
         <v>21</v>
       </c>
       <c r="E67">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="F67">
-        <v>100</v>
+        <v>20</v>
       </c>
       <c r="G67">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H67">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="I67" t="b">
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>116</v>
+        <v>175</v>
       </c>
       <c r="K67" t="s">
-        <v>146</v>
+        <v>176</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>58</v>
+        <v>194</v>
       </c>
       <c r="B68" t="s">
-        <v>72</v>
+        <v>195</v>
       </c>
       <c r="C68" t="s">
         <v>47</v>
@@ -3928,71 +3934,71 @@
         <v>21</v>
       </c>
       <c r="E68">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="F68">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G68">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="H68">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I68" t="b">
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>116</v>
+        <v>196</v>
       </c>
       <c r="K68" t="s">
-        <v>148</v>
+        <v>158</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>60</v>
+        <v>56</v>
       </c>
       <c r="B69" t="s">
-        <v>105</v>
+        <v>68</v>
       </c>
       <c r="C69" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D69" t="s">
         <v>21</v>
       </c>
       <c r="E69">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="F69">
-        <v>180</v>
+        <v>100</v>
       </c>
       <c r="G69">
-        <v>140</v>
+        <v>95</v>
       </c>
       <c r="H69">
-        <v>160</v>
+        <v>100</v>
       </c>
       <c r="I69" t="b">
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="K69" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>113</v>
+        <v>55</v>
       </c>
       <c r="B70" t="s">
-        <v>170</v>
+        <v>69</v>
       </c>
       <c r="C70" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="D70" t="s">
         <v>21</v>
@@ -4001,173 +4007,173 @@
         <v>50</v>
       </c>
       <c r="F70">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="G70">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="H70">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="I70" t="b">
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>141</v>
+        <v>113</v>
       </c>
       <c r="K70" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>206</v>
+        <v>57</v>
       </c>
       <c r="B71" t="s">
-        <v>155</v>
+        <v>102</v>
       </c>
       <c r="C71" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="D71" t="s">
         <v>21</v>
       </c>
       <c r="E71">
-        <v>58.3</v>
+        <v>120</v>
       </c>
       <c r="F71">
-        <v>100</v>
+        <v>180</v>
       </c>
       <c r="G71">
-        <v>90</v>
+        <v>140</v>
       </c>
       <c r="H71">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="I71" t="b">
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>153</v>
+        <v>114</v>
       </c>
       <c r="K71" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B72" t="s">
-        <v>10</v>
+        <v>167</v>
       </c>
       <c r="C72" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D72" t="s">
         <v>21</v>
       </c>
       <c r="E72">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="F72">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="G72">
-        <v>99.5</v>
+        <v>50</v>
       </c>
       <c r="H72">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="I72" t="b">
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>145</v>
+        <v>138</v>
       </c>
       <c r="K72" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>110</v>
+        <v>203</v>
       </c>
       <c r="B73" t="s">
-        <v>109</v>
+        <v>152</v>
       </c>
       <c r="C73" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D73" t="s">
         <v>21</v>
       </c>
       <c r="E73">
-        <v>0</v>
+        <v>58.3</v>
       </c>
       <c r="F73">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="G73">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="H73">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="I73" t="b">
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="K73" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>218</v>
+        <v>108</v>
       </c>
       <c r="B74" t="s">
-        <v>222</v>
+        <v>10</v>
       </c>
       <c r="C74" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D74" t="s">
         <v>21</v>
       </c>
       <c r="E74">
-        <v>1</v>
-      </c>
-      <c r="F74" t="s">
-        <v>5</v>
+        <v>99</v>
+      </c>
+      <c r="F74">
+        <v>100</v>
       </c>
       <c r="G74">
-        <v>1</v>
-      </c>
-      <c r="H74" t="s">
-        <v>5</v>
+        <v>99.5</v>
+      </c>
+      <c r="H74">
+        <v>100</v>
       </c>
       <c r="I74" t="b">
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>216</v>
+        <v>142</v>
       </c>
       <c r="K74" t="s">
-        <v>217</v>
+        <v>140</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>12</v>
+        <v>107</v>
       </c>
       <c r="B75" t="s">
-        <v>13</v>
+        <v>106</v>
       </c>
       <c r="C75" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D75" t="s">
         <v>21</v>
@@ -4176,68 +4182,68 @@
         <v>0</v>
       </c>
       <c r="F75">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="G75">
         <v>0</v>
       </c>
       <c r="H75">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I75" t="b">
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>118</v>
+        <v>142</v>
       </c>
       <c r="K75" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="B76" t="s">
         <v>219</v>
       </c>
       <c r="C76" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D76" t="s">
         <v>21</v>
       </c>
       <c r="E76">
-        <v>14.5</v>
-      </c>
-      <c r="F76">
-        <v>100</v>
+        <v>1</v>
+      </c>
+      <c r="F76" t="s">
+        <v>5</v>
       </c>
       <c r="G76">
-        <v>26.1</v>
-      </c>
-      <c r="H76">
-        <v>100</v>
+        <v>1</v>
+      </c>
+      <c r="H76" t="s">
+        <v>5</v>
       </c>
       <c r="I76" t="b">
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>154</v>
+        <v>213</v>
       </c>
       <c r="K76" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="B77" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C77" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D77" t="s">
         <v>21</v>
@@ -4246,68 +4252,68 @@
         <v>0</v>
       </c>
       <c r="F77">
-        <v>1.2E-2</v>
+        <v>0</v>
       </c>
       <c r="G77">
-        <v>2.0000000000000001E-4</v>
+        <v>0</v>
       </c>
       <c r="H77">
-        <v>6.0000000000000001E-3</v>
+        <v>0</v>
       </c>
       <c r="I77" t="b">
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>163</v>
+        <v>115</v>
       </c>
       <c r="K77" t="s">
-        <v>162</v>
+        <v>136</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>208</v>
+        <v>220</v>
       </c>
       <c r="B78" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="C78" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D78" t="s">
         <v>21</v>
       </c>
       <c r="E78">
-        <v>69</v>
+        <v>14.5</v>
       </c>
       <c r="F78">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="G78">
-        <v>82.8</v>
+        <v>26.1</v>
       </c>
       <c r="H78">
-        <v>120</v>
+        <v>100</v>
       </c>
       <c r="I78" t="b">
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>209</v>
+        <v>151</v>
       </c>
       <c r="K78" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>202</v>
+        <v>8</v>
       </c>
       <c r="B79" t="s">
-        <v>203</v>
+        <v>9</v>
       </c>
       <c r="C79" t="s">
-        <v>158</v>
+        <v>50</v>
       </c>
       <c r="D79" t="s">
         <v>21</v>
@@ -4316,68 +4322,68 @@
         <v>0</v>
       </c>
       <c r="F79">
-        <v>5.6599999999999999E-4</v>
+        <v>1.2E-2</v>
       </c>
       <c r="G79">
         <v>2.0000000000000001E-4</v>
       </c>
       <c r="H79">
-        <v>3.2679999999999997E-4</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="I79" t="b">
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>204</v>
+        <v>160</v>
       </c>
       <c r="K79" t="s">
-        <v>205</v>
+        <v>159</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>11</v>
+        <v>205</v>
       </c>
       <c r="B80" t="s">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="C80" t="s">
-        <v>158</v>
+        <v>50</v>
       </c>
       <c r="D80" t="s">
         <v>21</v>
       </c>
       <c r="E80">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="F80">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="G80">
-        <v>20</v>
+        <v>82.8</v>
       </c>
       <c r="H80">
-        <v>100</v>
+        <v>120</v>
       </c>
       <c r="I80" t="b">
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>154</v>
+        <v>206</v>
       </c>
       <c r="K80" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="B81" t="s">
-        <v>224</v>
+        <v>200</v>
       </c>
       <c r="C81" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D81" t="s">
         <v>21</v>
@@ -4386,45 +4392,45 @@
         <v>0</v>
       </c>
       <c r="F81">
-        <v>95</v>
+        <v>5.6599999999999999E-4</v>
       </c>
       <c r="G81">
-        <v>0</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="H81">
-        <v>80</v>
+        <v>3.2679999999999997E-4</v>
       </c>
       <c r="I81" t="b">
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>129</v>
+        <v>201</v>
       </c>
       <c r="K81" t="s">
-        <v>149</v>
+        <v>202</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>43</v>
+        <v>11</v>
       </c>
       <c r="B82" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="C82" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D82" t="s">
         <v>21</v>
       </c>
       <c r="E82">
-        <v>33</v>
+        <v>4</v>
       </c>
       <c r="F82">
         <v>100</v>
       </c>
       <c r="G82">
-        <v>67</v>
+        <v>20</v>
       </c>
       <c r="H82">
         <v>100</v>
@@ -4433,14 +4439,84 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>213</v>
+        <v>151</v>
       </c>
       <c r="K82" t="s">
-        <v>215</v>
+        <v>209</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>204</v>
+      </c>
+      <c r="B83" t="s">
+        <v>221</v>
+      </c>
+      <c r="C83" t="s">
+        <v>155</v>
+      </c>
+      <c r="D83" t="s">
+        <v>21</v>
+      </c>
+      <c r="E83">
+        <v>0</v>
+      </c>
+      <c r="F83">
+        <v>95</v>
+      </c>
+      <c r="G83">
+        <v>0</v>
+      </c>
+      <c r="H83">
+        <v>80</v>
+      </c>
+      <c r="I83" t="b">
+        <v>1</v>
+      </c>
+      <c r="J83" t="s">
+        <v>126</v>
+      </c>
+      <c r="K83" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>40</v>
+      </c>
+      <c r="B84" t="s">
+        <v>211</v>
+      </c>
+      <c r="C84" t="s">
+        <v>155</v>
+      </c>
+      <c r="D84" t="s">
+        <v>21</v>
+      </c>
+      <c r="E84">
+        <v>33</v>
+      </c>
+      <c r="F84">
+        <v>100</v>
+      </c>
+      <c r="G84">
+        <v>67</v>
+      </c>
+      <c r="H84">
+        <v>100</v>
+      </c>
+      <c r="I84" t="b">
+        <v>1</v>
+      </c>
+      <c r="J84" t="s">
+        <v>210</v>
+      </c>
+      <c r="K84" t="s">
+        <v>212</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K82" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K84" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Removed rules and associated files for EX technical controls
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67A8019C-A426-48D6-BB3A-3ECB2F7F88D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12E3BF91-BC8A-4A8A-AC80-A17ACBE9432F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metrics!$A$1:$K$84</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metrics!$A$1:$K$83</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="519" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="229">
   <si>
     <t>nn_lower</t>
   </si>
@@ -134,9 +134,6 @@
     <t>ex_amplified_DNA_yield_variability</t>
   </si>
   <si>
-    <t>ex_amplified_NTC_size</t>
-  </si>
-  <si>
     <t>Quantity of DNA (ng) after enzymatic fragmentation</t>
   </si>
   <si>
@@ -498,9 +495,6 @@
   </si>
   <si>
     <t>Percentage of fragments that fall within the expected size range on gel elextrophoresis (10,000-50,000 bp)</t>
-  </si>
-  <si>
-    <t>Distinct band at aprox 290 and sometimes 480 bp, with no smears. 1 = pass 0 = fail.</t>
   </si>
   <si>
     <t>EX call somatic variants</t>
@@ -1598,7 +1592,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K84"/>
+  <dimension ref="A1:K83"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" customWidth="1"/>
@@ -1640,10 +1634,10 @@
         <v>27</v>
       </c>
       <c r="J1" t="s">
+        <v>110</v>
+      </c>
+      <c r="K1" t="s">
         <v>111</v>
-      </c>
-      <c r="K1" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
@@ -1651,10 +1645,10 @@
         <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D2" t="s">
         <v>21</v>
@@ -1669,10 +1663,10 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -1680,10 +1674,10 @@
         <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="C3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D3" t="s">
         <v>22</v>
@@ -1704,21 +1698,21 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D4" t="s">
         <v>21</v>
@@ -1739,21 +1733,21 @@
         <v>0</v>
       </c>
       <c r="J4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C5" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D5" t="s">
         <v>21</v>
@@ -1768,21 +1762,21 @@
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K5" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D6" t="s">
         <v>22</v>
@@ -1803,21 +1797,21 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B7" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D7" t="s">
         <v>21</v>
@@ -1832,21 +1826,21 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B8" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="C8" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D8" t="s">
         <v>22</v>
@@ -1867,10 +1861,10 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K8" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -1878,10 +1872,10 @@
         <v>19</v>
       </c>
       <c r="B9" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C9" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D9" t="s">
         <v>21</v>
@@ -1902,10 +1896,10 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -1913,10 +1907,10 @@
         <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D10" t="s">
         <v>21</v>
@@ -1937,10 +1931,10 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -1948,10 +1942,10 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C11" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D11" t="s">
         <v>21</v>
@@ -1972,10 +1966,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="K11" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -1983,10 +1977,10 @@
         <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C12" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D12" t="s">
         <v>21</v>
@@ -2007,21 +2001,21 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K12" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="C13" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D13" t="s">
         <v>21</v>
@@ -2042,21 +2036,21 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="K13" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D14" t="s">
         <v>21</v>
@@ -2077,21 +2071,21 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K14" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B15" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C15" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D15" t="s">
         <v>21</v>
@@ -2112,21 +2106,21 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="K15" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B16" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C16" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D16" t="s">
         <v>21</v>
@@ -2147,21 +2141,21 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K16" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C17" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D17" t="s">
         <v>21</v>
@@ -2182,21 +2176,21 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="K17" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>71</v>
+      </c>
+      <c r="B18" t="s">
         <v>72</v>
       </c>
-      <c r="B18" t="s">
-        <v>73</v>
-      </c>
       <c r="C18" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D18" t="s">
         <v>21</v>
@@ -2217,21 +2211,21 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K18" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="B19" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C19" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D19" t="s">
         <v>21</v>
@@ -2252,21 +2246,21 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K19" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B20" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C20" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D20" t="s">
         <v>21</v>
@@ -2287,21 +2281,21 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K20" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B21" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C21" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D21" t="s">
         <v>21</v>
@@ -2322,21 +2316,21 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K21" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B22" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C22" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D22" t="s">
         <v>21</v>
@@ -2357,21 +2351,21 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K22" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B23" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C23" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D23" t="s">
         <v>21</v>
@@ -2392,21 +2386,21 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K23" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B24" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C24" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D24" t="s">
         <v>21</v>
@@ -2427,21 +2421,21 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K24" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B25" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C25" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D25" t="s">
         <v>21</v>
@@ -2462,21 +2456,21 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K25" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B26" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C26" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D26" t="s">
         <v>21</v>
@@ -2497,21 +2491,21 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K26" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B27" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C27" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D27" t="s">
         <v>21</v>
@@ -2532,21 +2526,21 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K27" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B28" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C28" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D28" t="s">
         <v>21</v>
@@ -2567,21 +2561,21 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K28" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B29" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C29" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D29" t="s">
         <v>21</v>
@@ -2602,21 +2596,21 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="K29" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B30" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C30" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D30" t="s">
         <v>21</v>
@@ -2637,21 +2631,21 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="K30" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B31" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C31" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D31" t="s">
         <v>21</v>
@@ -2672,21 +2666,21 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="K31" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B32" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="C32" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D32" t="s">
         <v>21</v>
@@ -2707,21 +2701,21 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="K32" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B33" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C33" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D33" t="s">
         <v>21</v>
@@ -2742,21 +2736,21 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="K33" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B34" t="s">
         <v>4</v>
       </c>
       <c r="C34" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D34" t="s">
         <v>21</v>
@@ -2777,10 +2771,10 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
+        <v>146</v>
+      </c>
+      <c r="K34" t="s">
         <v>147</v>
-      </c>
-      <c r="K34" t="s">
-        <v>148</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
@@ -2788,10 +2782,10 @@
         <v>16</v>
       </c>
       <c r="B35" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C35" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D35" t="s">
         <v>21</v>
@@ -2806,10 +2800,10 @@
         <v>0</v>
       </c>
       <c r="J35" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K35" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
@@ -2817,10 +2811,10 @@
         <v>23</v>
       </c>
       <c r="B36" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C36" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D36" t="s">
         <v>22</v>
@@ -2841,21 +2835,21 @@
         <v>0</v>
       </c>
       <c r="J36" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K36" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>220</v>
+      </c>
+      <c r="B37" t="s">
         <v>222</v>
       </c>
-      <c r="B37" t="s">
-        <v>224</v>
-      </c>
       <c r="C37" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D37" t="s">
         <v>21</v>
@@ -2876,21 +2870,21 @@
         <v>0</v>
       </c>
       <c r="J37" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K37" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B38" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="C38" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D38" t="s">
         <v>21</v>
@@ -2911,18 +2905,18 @@
         <v>0</v>
       </c>
       <c r="J38" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
+        <v>33</v>
+      </c>
+      <c r="B39" t="s">
         <v>34</v>
       </c>
-      <c r="B39" t="s">
-        <v>35</v>
-      </c>
       <c r="C39" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D39" t="s">
         <v>21</v>
@@ -2937,10 +2931,10 @@
         <v>0</v>
       </c>
       <c r="J39" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K39" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
@@ -2948,10 +2942,10 @@
         <v>31</v>
       </c>
       <c r="B40" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C40" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D40" t="s">
         <v>22</v>
@@ -2972,21 +2966,21 @@
         <v>0</v>
       </c>
       <c r="J40" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K40" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>223</v>
+      </c>
+      <c r="B41" t="s">
         <v>225</v>
       </c>
-      <c r="B41" t="s">
-        <v>227</v>
-      </c>
       <c r="C41" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D41" t="s">
         <v>21</v>
@@ -3007,21 +3001,21 @@
         <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K41" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B42" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C42" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D42" t="s">
         <v>21</v>
@@ -3042,126 +3036,126 @@
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>32</v>
+        <v>17</v>
       </c>
       <c r="B43" t="s">
-        <v>154</v>
+        <v>14</v>
       </c>
       <c r="C43" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D43" t="s">
         <v>21</v>
       </c>
       <c r="E43">
-        <v>1</v>
+        <v>544</v>
       </c>
       <c r="F43">
-        <v>1</v>
+        <v>624</v>
       </c>
       <c r="G43">
-        <v>1</v>
+        <v>564</v>
       </c>
       <c r="H43">
-        <v>1</v>
+        <v>604</v>
       </c>
       <c r="I43" t="b">
         <v>0</v>
       </c>
       <c r="J43" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K43" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B44" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C44" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D44" t="s">
         <v>21</v>
       </c>
       <c r="E44">
-        <v>544</v>
+        <v>94.9</v>
       </c>
       <c r="F44">
-        <v>624</v>
+        <v>100</v>
       </c>
       <c r="G44">
-        <v>564</v>
+        <v>100</v>
       </c>
       <c r="H44">
-        <v>604</v>
+        <v>100</v>
       </c>
       <c r="I44" t="b">
         <v>0</v>
       </c>
       <c r="J44" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="K44" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>18</v>
+        <v>74</v>
       </c>
       <c r="B45" t="s">
-        <v>15</v>
+        <v>179</v>
       </c>
       <c r="C45" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D45" t="s">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="E45">
-        <v>94.9</v>
+        <v>35</v>
       </c>
       <c r="F45">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="G45">
-        <v>100</v>
+        <v>39</v>
       </c>
       <c r="H45">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="I45" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>51</v>
+        <v>121</v>
       </c>
       <c r="K45" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>75</v>
       </c>
       <c r="B46" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C46" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D46" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E46">
         <v>35</v>
@@ -3182,42 +3176,42 @@
         <v>122</v>
       </c>
       <c r="K46" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>76</v>
       </c>
       <c r="B47" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="C47" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D47" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E47">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="F47">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="G47">
-        <v>39</v>
+        <v>0</v>
       </c>
       <c r="H47">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="I47" t="b">
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="K47" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
@@ -3225,13 +3219,13 @@
         <v>77</v>
       </c>
       <c r="B48" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C48" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D48" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E48">
         <v>0</v>
@@ -3252,39 +3246,39 @@
         <v>122</v>
       </c>
       <c r="K48" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B49" t="s">
-        <v>180</v>
+        <v>72</v>
       </c>
       <c r="C49" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D49" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E49">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="F49">
-        <v>10</v>
+        <v>150</v>
       </c>
       <c r="G49">
-        <v>0</v>
+        <v>150</v>
       </c>
       <c r="H49">
-        <v>5</v>
+        <v>150</v>
       </c>
       <c r="I49" t="b">
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="K49" t="s">
         <v>130</v>
@@ -3292,16 +3286,16 @@
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="B50" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C50" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D50" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E50">
         <v>150</v>
@@ -3322,7 +3316,7 @@
         <v>122</v>
       </c>
       <c r="K50" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
@@ -3330,34 +3324,34 @@
         <v>83</v>
       </c>
       <c r="B51" t="s">
-        <v>73</v>
+        <v>93</v>
       </c>
       <c r="C51" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D51" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E51">
-        <v>150</v>
-      </c>
-      <c r="F51">
-        <v>150</v>
+        <v>2850</v>
+      </c>
+      <c r="F51" t="s">
+        <v>5</v>
       </c>
       <c r="G51">
-        <v>150</v>
-      </c>
-      <c r="H51">
-        <v>150</v>
+        <v>3000</v>
+      </c>
+      <c r="H51" t="s">
+        <v>5</v>
       </c>
       <c r="I51" t="b">
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="K51" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
@@ -3365,13 +3359,13 @@
         <v>84</v>
       </c>
       <c r="B52" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C52" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D52" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="E52">
         <v>2850</v>
@@ -3392,33 +3386,33 @@
         <v>122</v>
       </c>
       <c r="K52" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>85</v>
+        <v>160</v>
       </c>
       <c r="B53" t="s">
-        <v>94</v>
+        <v>182</v>
       </c>
       <c r="C53" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D53" t="s">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="E53">
-        <v>2850</v>
-      </c>
-      <c r="F53" t="s">
-        <v>5</v>
+        <v>30</v>
+      </c>
+      <c r="F53">
+        <v>40</v>
       </c>
       <c r="G53">
-        <v>3000</v>
-      </c>
-      <c r="H53" t="s">
-        <v>5</v>
+        <v>35</v>
+      </c>
+      <c r="H53">
+        <v>40</v>
       </c>
       <c r="I53" t="b">
         <v>1</v>
@@ -3427,18 +3421,18 @@
         <v>123</v>
       </c>
       <c r="K53" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B54" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C54" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D54" t="s">
         <v>21</v>
@@ -3462,42 +3456,42 @@
         <v>124</v>
       </c>
       <c r="K54" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>163</v>
+        <v>85</v>
       </c>
       <c r="B55" t="s">
-        <v>184</v>
+        <v>95</v>
       </c>
       <c r="C55" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D55" t="s">
         <v>21</v>
       </c>
       <c r="E55">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="F55">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="G55">
-        <v>35</v>
+        <v>0</v>
       </c>
       <c r="H55">
-        <v>40</v>
+        <v>0.1</v>
       </c>
       <c r="I55" t="b">
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K55" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
@@ -3505,10 +3499,10 @@
         <v>86</v>
       </c>
       <c r="B56" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C56" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D56" t="s">
         <v>21</v>
@@ -3532,7 +3526,7 @@
         <v>124</v>
       </c>
       <c r="K56" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
@@ -3543,7 +3537,7 @@
         <v>96</v>
       </c>
       <c r="C57" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D57" t="s">
         <v>21</v>
@@ -3552,19 +3546,19 @@
         <v>0</v>
       </c>
       <c r="F57">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="G57">
         <v>0</v>
       </c>
       <c r="H57">
-        <v>0.1</v>
+        <v>20</v>
       </c>
       <c r="I57" t="b">
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K57" t="s">
         <v>132</v>
@@ -3575,10 +3569,10 @@
         <v>88</v>
       </c>
       <c r="B58" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C58" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D58" t="s">
         <v>21</v>
@@ -3602,7 +3596,7 @@
         <v>124</v>
       </c>
       <c r="K58" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
@@ -3613,7 +3607,7 @@
         <v>97</v>
       </c>
       <c r="C59" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D59" t="s">
         <v>21</v>
@@ -3622,19 +3616,19 @@
         <v>0</v>
       </c>
       <c r="F59">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="G59">
         <v>0</v>
       </c>
       <c r="H59">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I59" t="b">
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K59" t="s">
         <v>133</v>
@@ -3645,10 +3639,10 @@
         <v>90</v>
       </c>
       <c r="B60" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C60" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D60" t="s">
         <v>21</v>
@@ -3672,7 +3666,7 @@
         <v>124</v>
       </c>
       <c r="K60" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
@@ -3680,10 +3674,10 @@
         <v>91</v>
       </c>
       <c r="B61" t="s">
-        <v>98</v>
+        <v>181</v>
       </c>
       <c r="C61" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D61" t="s">
         <v>21</v>
@@ -3692,19 +3686,19 @@
         <v>0</v>
       </c>
       <c r="F61">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="G61">
         <v>0</v>
       </c>
       <c r="H61">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I61" t="b">
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="K61" t="s">
         <v>134</v>
@@ -3715,10 +3709,10 @@
         <v>92</v>
       </c>
       <c r="B62" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C62" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D62" t="s">
         <v>21</v>
@@ -3742,144 +3736,144 @@
         <v>124</v>
       </c>
       <c r="K62" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>93</v>
+        <v>52</v>
       </c>
       <c r="B63" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="C63" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D63" t="s">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="E63">
         <v>0</v>
       </c>
       <c r="F63">
+        <v>25</v>
+      </c>
+      <c r="G63">
+        <v>0</v>
+      </c>
+      <c r="H63">
         <v>10</v>
       </c>
-      <c r="G63">
-        <v>0</v>
-      </c>
-      <c r="H63">
-        <v>5</v>
-      </c>
       <c r="I63" t="b">
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>125</v>
+        <v>169</v>
       </c>
       <c r="K63" t="s">
-        <v>135</v>
+        <v>170</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
+        <v>100</v>
+      </c>
+      <c r="B64" t="s">
+        <v>191</v>
+      </c>
+      <c r="C64" t="s">
+        <v>46</v>
+      </c>
+      <c r="D64" t="s">
         <v>53</v>
       </c>
-      <c r="B64" t="s">
-        <v>173</v>
-      </c>
-      <c r="C64" t="s">
-        <v>47</v>
-      </c>
-      <c r="D64" t="s">
-        <v>54</v>
-      </c>
       <c r="E64">
         <v>0</v>
       </c>
       <c r="F64">
-        <v>25</v>
+        <v>0.1</v>
       </c>
       <c r="G64">
         <v>0</v>
       </c>
       <c r="H64">
-        <v>10</v>
+        <v>0.05</v>
       </c>
       <c r="I64" t="b">
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="K64" t="s">
-        <v>172</v>
+        <v>136</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>101</v>
+        <v>154</v>
       </c>
       <c r="B65" t="s">
-        <v>193</v>
+        <v>155</v>
       </c>
       <c r="C65" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D65" t="s">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="E65">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F65">
-        <v>0.1</v>
+        <v>40</v>
       </c>
       <c r="G65">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H65">
-        <v>0.05</v>
+        <v>20</v>
       </c>
       <c r="I65" t="b">
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>171</v>
+        <v>159</v>
       </c>
       <c r="K65" t="s">
-        <v>137</v>
+        <v>172</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>156</v>
+        <v>175</v>
       </c>
       <c r="B66" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="C66" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D66" t="s">
         <v>21</v>
       </c>
       <c r="E66">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F66">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="G66">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H66">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="I66" t="b">
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>161</v>
+        <v>173</v>
       </c>
       <c r="K66" t="s">
         <v>174</v>
@@ -3887,95 +3881,95 @@
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>177</v>
+        <v>192</v>
       </c>
       <c r="B67" t="s">
-        <v>166</v>
+        <v>193</v>
       </c>
       <c r="C67" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D67" t="s">
         <v>21</v>
       </c>
       <c r="E67">
-        <v>0</v>
+        <v>70</v>
       </c>
       <c r="F67">
-        <v>20</v>
+        <v>99</v>
       </c>
       <c r="G67">
-        <v>0</v>
+        <v>85</v>
       </c>
       <c r="H67">
-        <v>10</v>
+        <v>99</v>
       </c>
       <c r="I67" t="b">
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>175</v>
+        <v>194</v>
       </c>
       <c r="K67" t="s">
-        <v>176</v>
+        <v>156</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>194</v>
+        <v>55</v>
       </c>
       <c r="B68" t="s">
-        <v>195</v>
+        <v>67</v>
       </c>
       <c r="C68" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="D68" t="s">
         <v>21</v>
       </c>
       <c r="E68">
-        <v>70</v>
+        <v>90</v>
       </c>
       <c r="F68">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G68">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="H68">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="I68" t="b">
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>196</v>
+        <v>112</v>
       </c>
       <c r="K68" t="s">
-        <v>158</v>
+        <v>142</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B69" t="s">
         <v>68</v>
       </c>
       <c r="C69" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D69" t="s">
         <v>21</v>
       </c>
       <c r="E69">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="F69">
         <v>100</v>
       </c>
       <c r="G69">
-        <v>95</v>
+        <v>75</v>
       </c>
       <c r="H69">
         <v>100</v>
@@ -3984,36 +3978,36 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="K69" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B70" t="s">
-        <v>69</v>
+        <v>101</v>
       </c>
       <c r="C70" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D70" t="s">
         <v>21</v>
       </c>
       <c r="E70">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="F70">
-        <v>100</v>
+        <v>180</v>
       </c>
       <c r="G70">
-        <v>75</v>
+        <v>140</v>
       </c>
       <c r="H70">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="I70" t="b">
         <v>1</v>
@@ -4022,100 +4016,100 @@
         <v>113</v>
       </c>
       <c r="K70" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>57</v>
+        <v>109</v>
       </c>
       <c r="B71" t="s">
-        <v>102</v>
+        <v>165</v>
       </c>
       <c r="C71" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D71" t="s">
         <v>21</v>
       </c>
       <c r="E71">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="F71">
-        <v>180</v>
+        <v>70</v>
       </c>
       <c r="G71">
-        <v>140</v>
+        <v>50</v>
       </c>
       <c r="H71">
-        <v>160</v>
+        <v>60</v>
       </c>
       <c r="I71" t="b">
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>114</v>
+        <v>137</v>
       </c>
       <c r="K71" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>110</v>
+        <v>201</v>
       </c>
       <c r="B72" t="s">
-        <v>167</v>
+        <v>151</v>
       </c>
       <c r="C72" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D72" t="s">
         <v>21</v>
       </c>
       <c r="E72">
-        <v>50</v>
+        <v>58.3</v>
       </c>
       <c r="F72">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="G72">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="H72">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="I72" t="b">
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="K72" t="s">
-        <v>139</v>
+        <v>148</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>203</v>
+        <v>107</v>
       </c>
       <c r="B73" t="s">
-        <v>152</v>
+        <v>10</v>
       </c>
       <c r="C73" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D73" t="s">
         <v>21</v>
       </c>
       <c r="E73">
-        <v>58.3</v>
+        <v>99</v>
       </c>
       <c r="F73">
         <v>100</v>
       </c>
       <c r="G73">
-        <v>90</v>
+        <v>99.5</v>
       </c>
       <c r="H73">
         <v>100</v>
@@ -4124,42 +4118,42 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="K73" t="s">
-        <v>149</v>
+        <v>139</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B74" t="s">
-        <v>10</v>
+        <v>105</v>
       </c>
       <c r="C74" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D74" t="s">
         <v>21</v>
       </c>
       <c r="E74">
-        <v>99</v>
+        <v>0</v>
       </c>
       <c r="F74">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="G74">
-        <v>99.5</v>
+        <v>0</v>
       </c>
       <c r="H74">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="I74" t="b">
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="K74" t="s">
         <v>140</v>
@@ -4167,356 +4161,321 @@
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>107</v>
+        <v>213</v>
       </c>
       <c r="B75" t="s">
-        <v>106</v>
+        <v>217</v>
       </c>
       <c r="C75" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D75" t="s">
         <v>21</v>
       </c>
       <c r="E75">
-        <v>0</v>
-      </c>
-      <c r="F75">
-        <v>15</v>
+        <v>1</v>
+      </c>
+      <c r="F75" t="s">
+        <v>5</v>
       </c>
       <c r="G75">
-        <v>0</v>
-      </c>
-      <c r="H75">
+        <v>1</v>
+      </c>
+      <c r="H75" t="s">
         <v>5</v>
       </c>
       <c r="I75" t="b">
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>142</v>
+        <v>211</v>
       </c>
       <c r="K75" t="s">
-        <v>141</v>
+        <v>212</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>215</v>
+        <v>12</v>
       </c>
       <c r="B76" t="s">
-        <v>219</v>
+        <v>13</v>
       </c>
       <c r="C76" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D76" t="s">
         <v>21</v>
       </c>
       <c r="E76">
-        <v>1</v>
-      </c>
-      <c r="F76" t="s">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="F76">
+        <v>0</v>
       </c>
       <c r="G76">
-        <v>1</v>
-      </c>
-      <c r="H76" t="s">
-        <v>5</v>
+        <v>0</v>
+      </c>
+      <c r="H76">
+        <v>0</v>
       </c>
       <c r="I76" t="b">
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>213</v>
+        <v>114</v>
       </c>
       <c r="K76" t="s">
-        <v>214</v>
+        <v>135</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>12</v>
+        <v>218</v>
       </c>
       <c r="B77" t="s">
-        <v>13</v>
+        <v>214</v>
       </c>
       <c r="C77" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D77" t="s">
         <v>21</v>
       </c>
       <c r="E77">
-        <v>0</v>
+        <v>14.5</v>
       </c>
       <c r="F77">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="G77">
-        <v>0</v>
+        <v>26.1</v>
       </c>
       <c r="H77">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="I77" t="b">
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>115</v>
+        <v>150</v>
       </c>
       <c r="K77" t="s">
-        <v>136</v>
+        <v>216</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>220</v>
+        <v>8</v>
       </c>
       <c r="B78" t="s">
-        <v>216</v>
+        <v>9</v>
       </c>
       <c r="C78" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D78" t="s">
         <v>21</v>
       </c>
       <c r="E78">
-        <v>14.5</v>
+        <v>0</v>
       </c>
       <c r="F78">
-        <v>100</v>
+        <v>1.2E-2</v>
       </c>
       <c r="G78">
-        <v>26.1</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="H78">
-        <v>100</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="I78" t="b">
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="K78" t="s">
-        <v>218</v>
+        <v>157</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>8</v>
+        <v>203</v>
       </c>
       <c r="B79" t="s">
-        <v>9</v>
+        <v>205</v>
       </c>
       <c r="C79" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D79" t="s">
         <v>21</v>
       </c>
       <c r="E79">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="F79">
-        <v>1.2E-2</v>
+        <v>120</v>
       </c>
       <c r="G79">
-        <v>2.0000000000000001E-4</v>
+        <v>82.8</v>
       </c>
       <c r="H79">
-        <v>6.0000000000000001E-3</v>
+        <v>120</v>
       </c>
       <c r="I79" t="b">
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>160</v>
+        <v>204</v>
       </c>
       <c r="K79" t="s">
-        <v>159</v>
+        <v>206</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="B80" t="s">
-        <v>207</v>
+        <v>198</v>
       </c>
       <c r="C80" t="s">
-        <v>50</v>
+        <v>153</v>
       </c>
       <c r="D80" t="s">
         <v>21</v>
       </c>
       <c r="E80">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="F80">
-        <v>120</v>
+        <v>5.6599999999999999E-4</v>
       </c>
       <c r="G80">
-        <v>82.8</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="H80">
-        <v>120</v>
+        <v>3.2679999999999997E-4</v>
       </c>
       <c r="I80" t="b">
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>206</v>
+        <v>199</v>
       </c>
       <c r="K80" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>199</v>
+        <v>11</v>
       </c>
       <c r="B81" t="s">
-        <v>200</v>
+        <v>215</v>
       </c>
       <c r="C81" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D81" t="s">
         <v>21</v>
       </c>
       <c r="E81">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F81">
-        <v>5.6599999999999999E-4</v>
+        <v>100</v>
       </c>
       <c r="G81">
-        <v>2.0000000000000001E-4</v>
+        <v>20</v>
       </c>
       <c r="H81">
-        <v>3.2679999999999997E-4</v>
+        <v>100</v>
       </c>
       <c r="I81" t="b">
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>201</v>
+        <v>150</v>
       </c>
       <c r="K81" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>11</v>
+        <v>202</v>
       </c>
       <c r="B82" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C82" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D82" t="s">
         <v>21</v>
       </c>
       <c r="E82">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F82">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="G82">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="H82">
-        <v>100</v>
+        <v>80</v>
       </c>
       <c r="I82" t="b">
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>151</v>
+        <v>125</v>
       </c>
       <c r="K82" t="s">
-        <v>209</v>
+        <v>145</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>204</v>
+        <v>39</v>
       </c>
       <c r="B83" t="s">
-        <v>221</v>
+        <v>209</v>
       </c>
       <c r="C83" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="D83" t="s">
         <v>21</v>
       </c>
       <c r="E83">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="F83">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="G83">
-        <v>0</v>
+        <v>67</v>
       </c>
       <c r="H83">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="I83" t="b">
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>126</v>
+        <v>208</v>
       </c>
       <c r="K83" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A84" t="s">
-        <v>40</v>
-      </c>
-      <c r="B84" t="s">
-        <v>211</v>
-      </c>
-      <c r="C84" t="s">
-        <v>155</v>
-      </c>
-      <c r="D84" t="s">
-        <v>21</v>
-      </c>
-      <c r="E84">
-        <v>33</v>
-      </c>
-      <c r="F84">
-        <v>100</v>
-      </c>
-      <c r="G84">
-        <v>67</v>
-      </c>
-      <c r="H84">
-        <v>100</v>
-      </c>
-      <c r="I84" t="b">
-        <v>1</v>
-      </c>
-      <c r="J84" t="s">
         <v>210</v>
       </c>
-      <c r="K84" t="s">
-        <v>212</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K84" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K83" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Changed file paths for ex pipeline to more intuative and systematic names
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12E3BF91-BC8A-4A8A-AC80-A17ACBE9432F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2962317B-631F-4C84-9951-F7925B5C5834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -374,9 +374,6 @@
     <t>value_pattern</t>
   </si>
   <si>
-    <t>_map_metrics.txt</t>
-  </si>
-  <si>
     <t>_insert_metrics.txt</t>
   </si>
   <si>
@@ -401,18 +398,6 @@
     <t>_insert_size_metrics.txt</t>
   </si>
   <si>
-    <t>_r1_fastqc_raw_metrics_summary.json</t>
-  </si>
-  <si>
-    <t>_r2_fastqc_raw_metrics_summary.json</t>
-  </si>
-  <si>
-    <t>_r1_fastqc_filter_metrics_summary.json</t>
-  </si>
-  <si>
-    <t>_r2_fastqc_filter_metrics_summary.json</t>
-  </si>
-  <si>
     <t>_total_read_loss.json</t>
   </si>
   <si>
@@ -449,9 +434,6 @@
     <t>gini_coefficient</t>
   </si>
   <si>
-    <t>_call_dsc_metrics.json</t>
-  </si>
-  <si>
     <t>reads_lost</t>
   </si>
   <si>
@@ -512,9 +494,6 @@
     <t>^duplex_disagreement_rate\s+([0-9]*\.?[0-9]+)</t>
   </si>
   <si>
-    <t>_call_codec_consensus_metrics.txt</t>
-  </si>
-  <si>
     <t>_bases_trimmed.json</t>
   </si>
   <si>
@@ -662,18 +641,12 @@
     <t>ex_dsc_high_qual_unmasked_pct.value</t>
   </si>
   <si>
-    <t>_coverage_overlap_metrics.json</t>
-  </si>
-  <si>
     <t>Percentage of all sequenced bases with 1. MS depth &gt; MS depth theshold and 2. EX duplex depth &gt; 0</t>
   </si>
   <si>
     <t>ms_depth_vs_ex_depth.pct_overlap</t>
   </si>
   <si>
-    <t>_depth_metrics.json</t>
-  </si>
-  <si>
     <t>depth_percentiles.values.50th</t>
   </si>
   <si>
@@ -723,6 +696,33 @@
   </si>
   <si>
     <t>extracted_DNA_size_pct</t>
+  </si>
+  <si>
+    <t>_fastqc_raw_metrics_summary_r1.json</t>
+  </si>
+  <si>
+    <t>_fastqc_raw_metrics_summary_r2.json</t>
+  </si>
+  <si>
+    <t>_fastqc_filter_metrics_summary_r1.json</t>
+  </si>
+  <si>
+    <t>_fastqc_filter_metrics_summary_r2.json</t>
+  </si>
+  <si>
+    <t>_alignment_metrics.txt</t>
+  </si>
+  <si>
+    <t>_call_dsc_read_loss.json</t>
+  </si>
+  <si>
+    <t>_dsc_depth_metrics.json</t>
+  </si>
+  <si>
+    <t>_call_dsc_metrics.txt</t>
+  </si>
+  <si>
+    <t>_dsc_coverage_overlap_metrics.json</t>
   </si>
 </sst>
 </file>
@@ -1593,19 +1593,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
   <dimension ref="A1:K83"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="35.140625" customWidth="1"/>
-    <col min="2" max="2" width="123.140625" customWidth="1"/>
-    <col min="3" max="4" width="35.28515625" customWidth="1"/>
+    <col min="1" max="1" width="35.1796875" customWidth="1"/>
+    <col min="2" max="2" width="123.1796875" customWidth="1"/>
+    <col min="3" max="4" width="35.26953125" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.85546875" customWidth="1"/>
-    <col min="10" max="10" width="61.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="76.85546875" customWidth="1"/>
+    <col min="9" max="9" width="12.81640625" customWidth="1"/>
+    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="76.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>28</v>
       </c>
@@ -1640,12 +1640,12 @@
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="C2" t="s">
         <v>40</v>
@@ -1669,12 +1669,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>185</v>
+        <v>178</v>
       </c>
       <c r="C3" t="s">
         <v>40</v>
@@ -1704,12 +1704,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>228</v>
+        <v>219</v>
       </c>
       <c r="B4" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="C4" t="s">
         <v>40</v>
@@ -1739,12 +1739,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="C5" t="s">
         <v>42</v>
@@ -1768,12 +1768,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="C6" t="s">
         <v>42</v>
@@ -1803,12 +1803,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>37</v>
       </c>
       <c r="B7" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="C7" t="s">
         <v>42</v>
@@ -1832,12 +1832,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>38</v>
       </c>
       <c r="B8" t="s">
-        <v>187</v>
+        <v>180</v>
       </c>
       <c r="C8" t="s">
         <v>42</v>
@@ -1867,7 +1867,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1902,7 +1902,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -1937,7 +1937,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -1966,13 +1966,13 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K11" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -2001,18 +2001,18 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="K12" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="C13" t="s">
         <v>45</v>
@@ -2036,18 +2036,18 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K13" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="C14" t="s">
         <v>45</v>
@@ -2071,18 +2071,18 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="K14" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>78</v>
       </c>
       <c r="B15" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="C15" t="s">
         <v>45</v>
@@ -2106,18 +2106,18 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K15" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>79</v>
       </c>
       <c r="B16" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="C16" t="s">
         <v>45</v>
@@ -2141,13 +2141,13 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="K16" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>70</v>
       </c>
@@ -2176,13 +2176,13 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="K17" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>71</v>
       </c>
@@ -2211,18 +2211,18 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="K18" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="B19" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="C19" t="s">
         <v>45</v>
@@ -2246,18 +2246,18 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K19" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="B20" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="C20" t="s">
         <v>45</v>
@@ -2281,13 +2281,13 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K20" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>59</v>
       </c>
@@ -2316,13 +2316,13 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K21" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>60</v>
       </c>
@@ -2351,13 +2351,13 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K22" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>61</v>
       </c>
@@ -2386,13 +2386,13 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K23" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>62</v>
       </c>
@@ -2421,13 +2421,13 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K24" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>63</v>
       </c>
@@ -2456,13 +2456,13 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K25" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>64</v>
       </c>
@@ -2491,18 +2491,18 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K26" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>65</v>
       </c>
       <c r="B27" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="C27" t="s">
         <v>45</v>
@@ -2526,18 +2526,18 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="K27" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>66</v>
       </c>
       <c r="B28" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="C28" t="s">
         <v>45</v>
@@ -2561,18 +2561,18 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="K28" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>195</v>
+        <v>188</v>
       </c>
       <c r="B29" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="C29" t="s">
         <v>47</v>
@@ -2596,13 +2596,13 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="K29" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>104</v>
       </c>
@@ -2631,13 +2631,13 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="K30" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>103</v>
       </c>
@@ -2666,18 +2666,18 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
       <c r="K31" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>183</v>
-      </c>
       <c r="B32" t="s">
-        <v>189</v>
+        <v>182</v>
       </c>
       <c r="C32" t="s">
         <v>48</v>
@@ -2701,13 +2701,13 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>184</v>
+        <v>177</v>
       </c>
       <c r="K32" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>102</v>
       </c>
@@ -2736,13 +2736,13 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="K33" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>51</v>
       </c>
@@ -2750,7 +2750,7 @@
         <v>4</v>
       </c>
       <c r="C34" t="s">
-        <v>190</v>
+        <v>183</v>
       </c>
       <c r="D34" t="s">
         <v>21</v>
@@ -2771,13 +2771,13 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="K34" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>16</v>
       </c>
@@ -2806,12 +2806,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>23</v>
       </c>
       <c r="B36" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="C36" t="s">
         <v>41</v>
@@ -2841,12 +2841,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>220</v>
+        <v>211</v>
       </c>
       <c r="B37" t="s">
-        <v>222</v>
+        <v>213</v>
       </c>
       <c r="C37" t="s">
         <v>41</v>
@@ -2876,12 +2876,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>221</v>
+        <v>212</v>
       </c>
       <c r="B38" t="s">
-        <v>226</v>
+        <v>217</v>
       </c>
       <c r="C38" t="s">
         <v>41</v>
@@ -2908,7 +2908,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>33</v>
       </c>
@@ -2937,12 +2937,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>31</v>
       </c>
       <c r="B40" t="s">
-        <v>186</v>
+        <v>179</v>
       </c>
       <c r="C40" t="s">
         <v>41</v>
@@ -2972,12 +2972,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>223</v>
+        <v>214</v>
       </c>
       <c r="B41" t="s">
-        <v>225</v>
+        <v>216</v>
       </c>
       <c r="C41" t="s">
         <v>41</v>
@@ -3007,12 +3007,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>224</v>
+        <v>215</v>
       </c>
       <c r="B42" t="s">
-        <v>227</v>
+        <v>218</v>
       </c>
       <c r="C42" t="s">
         <v>41</v>
@@ -3039,7 +3039,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>17</v>
       </c>
@@ -3074,7 +3074,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>18</v>
       </c>
@@ -3109,12 +3109,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>74</v>
       </c>
       <c r="B45" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="C45" t="s">
         <v>44</v>
@@ -3138,18 +3138,18 @@
         <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>121</v>
+        <v>220</v>
       </c>
       <c r="K45" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>75</v>
       </c>
       <c r="B46" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="C46" t="s">
         <v>44</v>
@@ -3173,18 +3173,18 @@
         <v>1</v>
       </c>
       <c r="J46" t="s">
+        <v>221</v>
+      </c>
+      <c r="K46" t="s">
         <v>122</v>
       </c>
-      <c r="K46" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>76</v>
       </c>
       <c r="B47" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="C47" t="s">
         <v>44</v>
@@ -3208,18 +3208,18 @@
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>121</v>
+        <v>220</v>
       </c>
       <c r="K47" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>77</v>
       </c>
       <c r="B48" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="C48" t="s">
         <v>44</v>
@@ -3243,13 +3243,13 @@
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>122</v>
+        <v>221</v>
       </c>
       <c r="K48" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>73</v>
       </c>
@@ -3278,13 +3278,13 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>121</v>
+        <v>220</v>
       </c>
       <c r="K49" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>82</v>
       </c>
@@ -3313,13 +3313,13 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>122</v>
+        <v>221</v>
       </c>
       <c r="K50" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>83</v>
       </c>
@@ -3348,13 +3348,13 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
+        <v>220</v>
+      </c>
+      <c r="K51" t="s">
         <v>121</v>
       </c>
-      <c r="K51" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" t="s">
         <v>84</v>
       </c>
@@ -3383,18 +3383,18 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>122</v>
+        <v>221</v>
       </c>
       <c r="K52" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>160</v>
+        <v>153</v>
       </c>
       <c r="B53" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="C53" t="s">
         <v>44</v>
@@ -3418,18 +3418,18 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
+        <v>222</v>
+      </c>
+      <c r="K53" t="s">
         <v>123</v>
       </c>
-      <c r="K53" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="B54" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
       <c r="C54" t="s">
         <v>44</v>
@@ -3453,13 +3453,13 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>124</v>
+        <v>223</v>
       </c>
       <c r="K54" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" t="s">
         <v>85</v>
       </c>
@@ -3488,13 +3488,13 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>123</v>
+        <v>222</v>
       </c>
       <c r="K55" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" t="s">
         <v>86</v>
       </c>
@@ -3523,13 +3523,13 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>124</v>
+        <v>223</v>
       </c>
       <c r="K56" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" t="s">
         <v>87</v>
       </c>
@@ -3558,13 +3558,13 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>123</v>
+        <v>222</v>
       </c>
       <c r="K57" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" t="s">
         <v>88</v>
       </c>
@@ -3593,13 +3593,13 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>124</v>
+        <v>223</v>
       </c>
       <c r="K58" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" t="s">
         <v>89</v>
       </c>
@@ -3628,13 +3628,13 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>123</v>
+        <v>222</v>
       </c>
       <c r="K59" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" t="s">
         <v>90</v>
       </c>
@@ -3663,18 +3663,18 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>124</v>
+        <v>223</v>
       </c>
       <c r="K60" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" t="s">
         <v>91</v>
       </c>
       <c r="B61" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="C61" t="s">
         <v>44</v>
@@ -3698,18 +3698,18 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>123</v>
+        <v>222</v>
       </c>
       <c r="K61" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" t="s">
         <v>92</v>
       </c>
       <c r="B62" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
       <c r="C62" t="s">
         <v>44</v>
@@ -3733,18 +3733,18 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>124</v>
+        <v>223</v>
       </c>
       <c r="K62" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" t="s">
         <v>52</v>
       </c>
       <c r="B63" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
       <c r="C63" t="s">
         <v>46</v>
@@ -3768,18 +3768,18 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="K63" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+        <v>163</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" t="s">
         <v>100</v>
       </c>
       <c r="B64" t="s">
-        <v>191</v>
+        <v>184</v>
       </c>
       <c r="C64" t="s">
         <v>46</v>
@@ -3803,18 +3803,18 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="K64" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="B65" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="C65" t="s">
         <v>46</v>
@@ -3838,18 +3838,18 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>159</v>
+        <v>152</v>
       </c>
       <c r="K65" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="B66" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
       <c r="C66" t="s">
         <v>46</v>
@@ -3873,18 +3873,18 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="K66" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+        <v>167</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>192</v>
+        <v>185</v>
       </c>
       <c r="B67" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="C67" t="s">
         <v>46</v>
@@ -3908,13 +3908,13 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
       <c r="K67" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A68" t="s">
         <v>55</v>
       </c>
@@ -3943,13 +3943,13 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>112</v>
+        <v>224</v>
       </c>
       <c r="K68" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" t="s">
         <v>54</v>
       </c>
@@ -3978,13 +3978,13 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>112</v>
+        <v>224</v>
       </c>
       <c r="K69" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+        <v>138</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" t="s">
         <v>56</v>
       </c>
@@ -4013,18 +4013,18 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="K70" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" t="s">
         <v>109</v>
       </c>
       <c r="B71" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="C71" t="s">
         <v>49</v>
@@ -4048,18 +4048,18 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>137</v>
+        <v>225</v>
       </c>
       <c r="K71" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>201</v>
+        <v>194</v>
       </c>
       <c r="B72" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="C72" t="s">
         <v>49</v>
@@ -4083,13 +4083,13 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="K72" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" t="s">
         <v>107</v>
       </c>
@@ -4118,13 +4118,13 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="K73" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" t="s">
         <v>106</v>
       </c>
@@ -4153,18 +4153,18 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="K74" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>213</v>
+        <v>204</v>
       </c>
       <c r="B75" t="s">
-        <v>217</v>
+        <v>208</v>
       </c>
       <c r="C75" t="s">
         <v>49</v>
@@ -4188,13 +4188,13 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>211</v>
+        <v>226</v>
       </c>
       <c r="K75" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A76" t="s">
         <v>12</v>
       </c>
@@ -4223,18 +4223,18 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="K76" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>218</v>
+        <v>209</v>
       </c>
       <c r="B77" t="s">
-        <v>214</v>
+        <v>205</v>
       </c>
       <c r="C77" t="s">
         <v>49</v>
@@ -4258,13 +4258,13 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="K77" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -4293,18 +4293,18 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>158</v>
+        <v>227</v>
       </c>
       <c r="K78" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>203</v>
+        <v>196</v>
       </c>
       <c r="B79" t="s">
-        <v>205</v>
+        <v>198</v>
       </c>
       <c r="C79" t="s">
         <v>49</v>
@@ -4328,21 +4328,21 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>204</v>
+        <v>197</v>
       </c>
       <c r="K79" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="B80" t="s">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="C80" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D80" t="s">
         <v>21</v>
@@ -4363,21 +4363,21 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="K80" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A81" t="s">
         <v>11</v>
       </c>
       <c r="B81" t="s">
-        <v>215</v>
+        <v>206</v>
       </c>
       <c r="C81" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D81" t="s">
         <v>21</v>
@@ -4398,21 +4398,21 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="K81" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>202</v>
+        <v>195</v>
       </c>
       <c r="B82" t="s">
-        <v>219</v>
+        <v>210</v>
       </c>
       <c r="C82" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D82" t="s">
         <v>21</v>
@@ -4433,21 +4433,21 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="K82" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A83" t="s">
         <v>39</v>
       </c>
       <c r="B83" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="C83" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="D83" t="s">
         <v>21</v>
@@ -4468,10 +4468,10 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>208</v>
+        <v>228</v>
       </c>
       <c r="K83" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
backing up work in progress
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2962317B-631F-4C84-9951-F7925B5C5834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0F2C215-BFAA-4504-916D-4717ED991F03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -374,33 +374,6 @@
     <t>value_pattern</t>
   </si>
   <si>
-    <t>_insert_metrics.txt</t>
-  </si>
-  <si>
-    <t>_softclipping_metrics.json</t>
-  </si>
-  <si>
-    <t>_r1_raw_fastqc_summary.json</t>
-  </si>
-  <si>
-    <t>_r2_raw_fastqc_summary.json</t>
-  </si>
-  <si>
-    <t>_filter_r1_fastqc_summary.json</t>
-  </si>
-  <si>
-    <t>_filter_r2_fastqc_summary.json</t>
-  </si>
-  <si>
-    <t>_alignment_stats.txt</t>
-  </si>
-  <si>
-    <t>_insert_size_metrics.txt</t>
-  </si>
-  <si>
-    <t>_total_read_loss.json</t>
-  </si>
-  <si>
     <t>total_reads</t>
   </si>
   <si>
@@ -443,9 +416,6 @@
     <t>reads_lost_to_MAPQ_filter</t>
   </si>
   <si>
-    <t>_dsc_remap_metrics.json</t>
-  </si>
-  <si>
     <t>^\d+ \+ 0 mapped \((?P&lt;percent&gt;[\d.]+)% : N/A\)$</t>
   </si>
   <si>
@@ -458,21 +428,12 @@
     <t>percent_reads_lost</t>
   </si>
   <si>
-    <t>_mask_metrics.json</t>
-  </si>
-  <si>
     <t>mask_files.combined_mask.percentage_of_ref_genome</t>
   </si>
   <si>
     <t>pct_unique_reads</t>
   </si>
   <si>
-    <t>_duplication_metrics.json</t>
-  </si>
-  <si>
-    <t>_dsc_coverage_metrics.json</t>
-  </si>
-  <si>
     <t>Percentage of reads that are unique following initial alignment</t>
   </si>
   <si>
@@ -494,9 +455,6 @@
     <t>^duplex_disagreement_rate\s+([0-9]*\.?[0-9]+)</t>
   </si>
   <si>
-    <t>_bases_trimmed.json</t>
-  </si>
-  <si>
     <t>ex_filtered_per_base_quality_r1</t>
   </si>
   <si>
@@ -524,9 +482,6 @@
     <t>Quantity of DNA (ng) required to run assay &amp; QCs (ng/uL concentration x ul sample remaining after Qubit)</t>
   </si>
   <si>
-    <t>_demux_counts_and_gini.json</t>
-  </si>
-  <si>
     <t>pct_reads_lost_demux</t>
   </si>
   <si>
@@ -536,9 +491,6 @@
     <t>percent_bases_trimmed</t>
   </si>
   <si>
-    <t>_trimmed_read_length_metrics.json</t>
-  </si>
-  <si>
     <t>percent_zero_length</t>
   </si>
   <si>
@@ -548,9 +500,6 @@
     <t>duplication_rate</t>
   </si>
   <si>
-    <t>_duplication_metrics_ms.json</t>
-  </si>
-  <si>
     <t>Percentage of flow cell tiles where mean quality score at any read position is &gt;=5 less than the global mean quality for that position</t>
   </si>
   <si>
@@ -569,9 +518,6 @@
     <t>ms_coverage_at_depth_threshold</t>
   </si>
   <si>
-    <t>_coverage_by_depth.json</t>
-  </si>
-  <si>
     <t>Variability in DNA extraction yield (normalised interquartile range)</t>
   </si>
   <si>
@@ -599,24 +545,15 @@
     <t>Percentage of reads that retained after length and quality filtering</t>
   </si>
   <si>
-    <t>_filter_metrics_ex.txt</t>
-  </si>
-  <si>
     <t>ms_reads_filtered_length_quality</t>
   </si>
   <si>
-    <t>_filter_metrics_ms.txt</t>
-  </si>
-  <si>
     <t>ex_variant_call_eligible_disagree_rate</t>
   </si>
   <si>
     <t>Watson and Crick disagreement rate among bases eligible for somatic variant calling</t>
   </si>
   <si>
-    <t>_variant_call_disagree_metrics.json</t>
-  </si>
-  <si>
     <t>observed_disagreement_rate</t>
   </si>
   <si>
@@ -629,9 +566,6 @@
     <t>ex_duplex_overlap</t>
   </si>
   <si>
-    <t>_duplex_overlap_metrics.json</t>
-  </si>
-  <si>
     <t>50th percentile for length of overlap between R1 and R2 in each duplex sequence</t>
   </si>
   <si>
@@ -698,31 +632,97 @@
     <t>extracted_DNA_size_pct</t>
   </si>
   <si>
-    <t>_fastqc_raw_metrics_summary_r1.json</t>
-  </si>
-  <si>
-    <t>_fastqc_raw_metrics_summary_r2.json</t>
-  </si>
-  <si>
-    <t>_fastqc_filter_metrics_summary_r1.json</t>
-  </si>
-  <si>
-    <t>_fastqc_filter_metrics_summary_r2.json</t>
-  </si>
-  <si>
-    <t>_alignment_metrics.txt</t>
-  </si>
-  <si>
-    <t>_call_dsc_read_loss.json</t>
-  </si>
-  <si>
-    <t>_dsc_depth_metrics.json</t>
-  </si>
-  <si>
-    <t>_call_dsc_metrics.txt</t>
-  </si>
-  <si>
-    <t>_dsc_coverage_overlap_metrics.json</t>
+    <t>EX.MET_SOFTCLIPPING</t>
+  </si>
+  <si>
+    <t>EX.MET_DSC_COVERAGE_JSON</t>
+  </si>
+  <si>
+    <t>MS.MET_FASTQC_RAW_SUMMARY_R1</t>
+  </si>
+  <si>
+    <t>MS.MET_FASTQC_RAW_SUMMARY_R2</t>
+  </si>
+  <si>
+    <t>MS.MET_FASTQC_FILTER_SUMMARY_R1</t>
+  </si>
+  <si>
+    <t>MS.MET_FASTQC_FILTER_SUMMARY_R2</t>
+  </si>
+  <si>
+    <t>MS.MET_FILTER_FASTQ</t>
+  </si>
+  <si>
+    <t>MS.MET_ALIGNMENT</t>
+  </si>
+  <si>
+    <t>MS.MET_DUPLICATION_2</t>
+  </si>
+  <si>
+    <t>MS.MET_COVERAGE_BY_DEPTH</t>
+  </si>
+  <si>
+    <t>MS.MET_INSERT_SIZE_TXT</t>
+  </si>
+  <si>
+    <t>MS.MET_MASKING</t>
+  </si>
+  <si>
+    <t>EX.MET_FASTQC_RAW_HTML_R1</t>
+  </si>
+  <si>
+    <t>EX.MET_FASTQC_RAW_HTML_R2</t>
+  </si>
+  <si>
+    <t>EX.MET_FASTQC_FILTER_SUMMARY_R1</t>
+  </si>
+  <si>
+    <t>EX.MET_FASTQC_FILTER_SUMMARY_R2</t>
+  </si>
+  <si>
+    <t>EX.MET_DEMUX_COUNTS_GINI</t>
+  </si>
+  <si>
+    <t>EX.MET_BASES_TRIMMED</t>
+  </si>
+  <si>
+    <t>EX.MET_TRIM_READ_LENGTHS</t>
+  </si>
+  <si>
+    <t>EX.MET_FILTER_FASTQ</t>
+  </si>
+  <si>
+    <t>EX.MET_ALIGNMENT</t>
+  </si>
+  <si>
+    <t>EX.MET_INSERT_SIZE_TXT</t>
+  </si>
+  <si>
+    <t>EX.MET_CALL_DSC_READ_LOSS</t>
+  </si>
+  <si>
+    <t>EX.MET_DUPLICATION</t>
+  </si>
+  <si>
+    <t>EX.MET_DSC_REMAP</t>
+  </si>
+  <si>
+    <t>EX.MET_CALL_DSC</t>
+  </si>
+  <si>
+    <t>EX.MET_DUPLEX_OVERLAP</t>
+  </si>
+  <si>
+    <t>EX.MET_VAR_CALL_DISAGREE</t>
+  </si>
+  <si>
+    <t>EX.MET_TOTAL_READ_LOSS</t>
+  </si>
+  <si>
+    <t>EX.MET_COVERAGE_OVERLAP</t>
+  </si>
+  <si>
+    <t>EX.MET_DSC_DEPTH</t>
   </si>
 </sst>
 </file>
@@ -1596,12 +1596,12 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.1796875" customWidth="1"/>
-    <col min="2" max="2" width="123.1796875" customWidth="1"/>
+    <col min="2" max="2" width="123.1796875" hidden="1" customWidth="1"/>
     <col min="3" max="4" width="35.26953125" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
     <col min="9" max="9" width="12.81640625" customWidth="1"/>
-    <col min="10" max="10" width="61.81640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="40.54296875" customWidth="1"/>
     <col min="11" max="11" width="76.81640625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1645,7 +1645,7 @@
         <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>161</v>
+        <v>147</v>
       </c>
       <c r="C2" t="s">
         <v>40</v>
@@ -1674,7 +1674,7 @@
         <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
       <c r="C3" t="s">
         <v>40</v>
@@ -1706,10 +1706,10 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
-        <v>219</v>
+        <v>197</v>
       </c>
       <c r="B4" t="s">
-        <v>146</v>
+        <v>133</v>
       </c>
       <c r="C4" t="s">
         <v>40</v>
@@ -1744,7 +1744,7 @@
         <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>160</v>
+        <v>146</v>
       </c>
       <c r="C5" t="s">
         <v>42</v>
@@ -1773,7 +1773,7 @@
         <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
       <c r="C6" t="s">
         <v>42</v>
@@ -1808,7 +1808,7 @@
         <v>37</v>
       </c>
       <c r="B7" t="s">
-        <v>159</v>
+        <v>145</v>
       </c>
       <c r="C7" t="s">
         <v>42</v>
@@ -1837,7 +1837,7 @@
         <v>38</v>
       </c>
       <c r="B8" t="s">
-        <v>180</v>
+        <v>162</v>
       </c>
       <c r="C8" t="s">
         <v>42</v>
@@ -1966,10 +1966,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>114</v>
+        <v>200</v>
       </c>
       <c r="K11" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.35">
@@ -2001,10 +2001,10 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>115</v>
+        <v>201</v>
       </c>
       <c r="K12" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
@@ -2012,7 +2012,7 @@
         <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>172</v>
+        <v>155</v>
       </c>
       <c r="C13" t="s">
         <v>45</v>
@@ -2036,10 +2036,10 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>114</v>
+        <v>200</v>
       </c>
       <c r="K13" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
@@ -2047,7 +2047,7 @@
         <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>173</v>
+        <v>156</v>
       </c>
       <c r="C14" t="s">
         <v>45</v>
@@ -2071,10 +2071,10 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>115</v>
+        <v>201</v>
       </c>
       <c r="K14" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
@@ -2082,7 +2082,7 @@
         <v>78</v>
       </c>
       <c r="B15" t="s">
-        <v>171</v>
+        <v>154</v>
       </c>
       <c r="C15" t="s">
         <v>45</v>
@@ -2106,10 +2106,10 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>114</v>
+        <v>200</v>
       </c>
       <c r="K15" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
@@ -2117,7 +2117,7 @@
         <v>79</v>
       </c>
       <c r="B16" t="s">
-        <v>171</v>
+        <v>154</v>
       </c>
       <c r="C16" t="s">
         <v>45</v>
@@ -2141,10 +2141,10 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
+        <v>201</v>
+      </c>
+      <c r="K16" t="s">
         <v>115</v>
-      </c>
-      <c r="K16" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">
@@ -2176,10 +2176,10 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>114</v>
+        <v>200</v>
       </c>
       <c r="K17" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.35">
@@ -2211,18 +2211,18 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>115</v>
+        <v>201</v>
       </c>
       <c r="K18" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="B19" t="s">
-        <v>175</v>
+        <v>158</v>
       </c>
       <c r="C19" t="s">
         <v>45</v>
@@ -2246,18 +2246,18 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>116</v>
+        <v>202</v>
       </c>
       <c r="K19" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
-        <v>156</v>
+        <v>142</v>
       </c>
       <c r="B20" t="s">
-        <v>175</v>
+        <v>158</v>
       </c>
       <c r="C20" t="s">
         <v>45</v>
@@ -2281,10 +2281,10 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>117</v>
+        <v>203</v>
       </c>
       <c r="K20" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.35">
@@ -2316,10 +2316,10 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>116</v>
+        <v>202</v>
       </c>
       <c r="K21" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.35">
@@ -2351,10 +2351,10 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
+        <v>203</v>
+      </c>
+      <c r="K22" t="s">
         <v>117</v>
-      </c>
-      <c r="K22" t="s">
-        <v>126</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.35">
@@ -2386,10 +2386,10 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>116</v>
+        <v>202</v>
       </c>
       <c r="K23" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.35">
@@ -2421,10 +2421,10 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>117</v>
+        <v>203</v>
       </c>
       <c r="K24" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.35">
@@ -2456,10 +2456,10 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>116</v>
+        <v>202</v>
       </c>
       <c r="K25" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.35">
@@ -2491,10 +2491,10 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>117</v>
+        <v>203</v>
       </c>
       <c r="K26" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.35">
@@ -2502,7 +2502,7 @@
         <v>65</v>
       </c>
       <c r="B27" t="s">
-        <v>174</v>
+        <v>157</v>
       </c>
       <c r="C27" t="s">
         <v>45</v>
@@ -2526,10 +2526,10 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>116</v>
+        <v>202</v>
       </c>
       <c r="K27" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.35">
@@ -2537,7 +2537,7 @@
         <v>66</v>
       </c>
       <c r="B28" t="s">
-        <v>174</v>
+        <v>157</v>
       </c>
       <c r="C28" t="s">
         <v>45</v>
@@ -2561,18 +2561,18 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>117</v>
+        <v>203</v>
       </c>
       <c r="K28" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
-        <v>188</v>
+        <v>169</v>
       </c>
       <c r="B29" t="s">
-        <v>186</v>
+        <v>168</v>
       </c>
       <c r="C29" t="s">
         <v>47</v>
@@ -2596,10 +2596,10 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>189</v>
+        <v>204</v>
       </c>
       <c r="K29" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.35">
@@ -2631,10 +2631,10 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>118</v>
+        <v>205</v>
       </c>
       <c r="K30" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.35">
@@ -2666,18 +2666,18 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>170</v>
+        <v>206</v>
       </c>
       <c r="K31" t="s">
-        <v>169</v>
+        <v>153</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
-        <v>176</v>
+        <v>159</v>
       </c>
       <c r="B32" t="s">
-        <v>182</v>
+        <v>164</v>
       </c>
       <c r="C32" t="s">
         <v>48</v>
@@ -2701,10 +2701,10 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>177</v>
+        <v>207</v>
       </c>
       <c r="K32" t="s">
-        <v>181</v>
+        <v>163</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.35">
@@ -2736,10 +2736,10 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>119</v>
+        <v>208</v>
       </c>
       <c r="K33" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.35">
@@ -2750,7 +2750,7 @@
         <v>4</v>
       </c>
       <c r="C34" t="s">
-        <v>183</v>
+        <v>165</v>
       </c>
       <c r="D34" t="s">
         <v>21</v>
@@ -2771,10 +2771,10 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>140</v>
+        <v>209</v>
       </c>
       <c r="K34" t="s">
-        <v>141</v>
+        <v>130</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.35">
@@ -2811,7 +2811,7 @@
         <v>23</v>
       </c>
       <c r="B36" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
       <c r="C36" t="s">
         <v>41</v>
@@ -2843,10 +2843,10 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
-        <v>211</v>
+        <v>189</v>
       </c>
       <c r="B37" t="s">
-        <v>213</v>
+        <v>191</v>
       </c>
       <c r="C37" t="s">
         <v>41</v>
@@ -2878,10 +2878,10 @@
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
-        <v>212</v>
+        <v>190</v>
       </c>
       <c r="B38" t="s">
-        <v>217</v>
+        <v>195</v>
       </c>
       <c r="C38" t="s">
         <v>41</v>
@@ -2942,7 +2942,7 @@
         <v>31</v>
       </c>
       <c r="B40" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
       <c r="C40" t="s">
         <v>41</v>
@@ -2974,10 +2974,10 @@
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
-        <v>214</v>
+        <v>192</v>
       </c>
       <c r="B41" t="s">
-        <v>216</v>
+        <v>194</v>
       </c>
       <c r="C41" t="s">
         <v>41</v>
@@ -3009,10 +3009,10 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>215</v>
+        <v>193</v>
       </c>
       <c r="B42" t="s">
-        <v>218</v>
+        <v>196</v>
       </c>
       <c r="C42" t="s">
         <v>41</v>
@@ -3114,7 +3114,7 @@
         <v>74</v>
       </c>
       <c r="B45" t="s">
-        <v>172</v>
+        <v>155</v>
       </c>
       <c r="C45" t="s">
         <v>44</v>
@@ -3138,10 +3138,10 @@
         <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="K45" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
     </row>
     <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
@@ -3149,7 +3149,7 @@
         <v>75</v>
       </c>
       <c r="B46" t="s">
-        <v>173</v>
+        <v>156</v>
       </c>
       <c r="C46" t="s">
         <v>44</v>
@@ -3173,10 +3173,10 @@
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="K46" t="s">
-        <v>122</v>
+        <v>113</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.35">
@@ -3184,7 +3184,7 @@
         <v>76</v>
       </c>
       <c r="B47" t="s">
-        <v>171</v>
+        <v>154</v>
       </c>
       <c r="C47" t="s">
         <v>44</v>
@@ -3208,10 +3208,10 @@
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="K47" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.35">
@@ -3219,7 +3219,7 @@
         <v>77</v>
       </c>
       <c r="B48" t="s">
-        <v>171</v>
+        <v>154</v>
       </c>
       <c r="C48" t="s">
         <v>44</v>
@@ -3243,10 +3243,10 @@
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="K48" t="s">
-        <v>124</v>
+        <v>115</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.35">
@@ -3278,10 +3278,10 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="K49" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.35">
@@ -3313,10 +3313,10 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="K50" t="s">
-        <v>125</v>
+        <v>116</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.35">
@@ -3348,10 +3348,10 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="K51" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.35">
@@ -3383,18 +3383,18 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>221</v>
+        <v>211</v>
       </c>
       <c r="K52" t="s">
-        <v>121</v>
+        <v>112</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="B53" t="s">
-        <v>175</v>
+        <v>158</v>
       </c>
       <c r="C53" t="s">
         <v>44</v>
@@ -3418,18 +3418,18 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="K53" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" t="s">
-        <v>154</v>
+        <v>140</v>
       </c>
       <c r="B54" t="s">
-        <v>175</v>
+        <v>158</v>
       </c>
       <c r="C54" t="s">
         <v>44</v>
@@ -3453,10 +3453,10 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="K54" t="s">
-        <v>123</v>
+        <v>114</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.35">
@@ -3488,10 +3488,10 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="K55" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.35">
@@ -3523,10 +3523,10 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="K56" t="s">
-        <v>126</v>
+        <v>117</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.35">
@@ -3558,10 +3558,10 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="K57" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.35">
@@ -3593,10 +3593,10 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="K58" t="s">
-        <v>127</v>
+        <v>118</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.35">
@@ -3628,10 +3628,10 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="K59" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.35">
@@ -3663,10 +3663,10 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="K60" t="s">
-        <v>128</v>
+        <v>119</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.35">
@@ -3674,7 +3674,7 @@
         <v>91</v>
       </c>
       <c r="B61" t="s">
-        <v>174</v>
+        <v>157</v>
       </c>
       <c r="C61" t="s">
         <v>44</v>
@@ -3698,10 +3698,10 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>222</v>
+        <v>212</v>
       </c>
       <c r="K61" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.35">
@@ -3709,7 +3709,7 @@
         <v>92</v>
       </c>
       <c r="B62" t="s">
-        <v>174</v>
+        <v>157</v>
       </c>
       <c r="C62" t="s">
         <v>44</v>
@@ -3733,10 +3733,10 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>223</v>
+        <v>213</v>
       </c>
       <c r="K62" t="s">
-        <v>129</v>
+        <v>120</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.35">
@@ -3744,7 +3744,7 @@
         <v>52</v>
       </c>
       <c r="B63" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="C63" t="s">
         <v>46</v>
@@ -3768,10 +3768,10 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>162</v>
+        <v>214</v>
       </c>
       <c r="K63" t="s">
-        <v>163</v>
+        <v>148</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.35">
@@ -3779,7 +3779,7 @@
         <v>100</v>
       </c>
       <c r="B64" t="s">
-        <v>184</v>
+        <v>166</v>
       </c>
       <c r="C64" t="s">
         <v>46</v>
@@ -3803,18 +3803,18 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>162</v>
+        <v>214</v>
       </c>
       <c r="K64" t="s">
-        <v>131</v>
+        <v>122</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" t="s">
-        <v>148</v>
+        <v>135</v>
       </c>
       <c r="B65" t="s">
-        <v>149</v>
+        <v>136</v>
       </c>
       <c r="C65" t="s">
         <v>46</v>
@@ -3838,18 +3838,18 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>152</v>
+        <v>215</v>
       </c>
       <c r="K65" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" t="s">
-        <v>168</v>
+        <v>152</v>
       </c>
       <c r="B66" t="s">
-        <v>157</v>
+        <v>143</v>
       </c>
       <c r="C66" t="s">
         <v>46</v>
@@ -3873,18 +3873,18 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>166</v>
+        <v>216</v>
       </c>
       <c r="K66" t="s">
-        <v>167</v>
+        <v>151</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" t="s">
-        <v>185</v>
+        <v>167</v>
       </c>
       <c r="B67" t="s">
-        <v>186</v>
+        <v>168</v>
       </c>
       <c r="C67" t="s">
         <v>46</v>
@@ -3908,10 +3908,10 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>187</v>
+        <v>217</v>
       </c>
       <c r="K67" t="s">
-        <v>150</v>
+        <v>137</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.35">
@@ -3943,10 +3943,10 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="K68" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.35">
@@ -3978,10 +3978,10 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="K69" t="s">
-        <v>138</v>
+        <v>128</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.35">
@@ -4013,10 +4013,10 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>112</v>
+        <v>219</v>
       </c>
       <c r="K70" t="s">
-        <v>137</v>
+        <v>127</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.35">
@@ -4024,7 +4024,7 @@
         <v>109</v>
       </c>
       <c r="B71" t="s">
-        <v>158</v>
+        <v>144</v>
       </c>
       <c r="C71" t="s">
         <v>49</v>
@@ -4048,18 +4048,18 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>225</v>
+        <v>220</v>
       </c>
       <c r="K71" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" t="s">
-        <v>194</v>
+        <v>173</v>
       </c>
       <c r="B72" t="s">
-        <v>145</v>
+        <v>132</v>
       </c>
       <c r="C72" t="s">
         <v>49</v>
@@ -4083,10 +4083,10 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>143</v>
+        <v>221</v>
       </c>
       <c r="K72" t="s">
-        <v>142</v>
+        <v>131</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.35">
@@ -4118,10 +4118,10 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>135</v>
+        <v>222</v>
       </c>
       <c r="K73" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.35">
@@ -4153,18 +4153,18 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>135</v>
+        <v>222</v>
       </c>
       <c r="K74" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" t="s">
-        <v>204</v>
+        <v>182</v>
       </c>
       <c r="B75" t="s">
-        <v>208</v>
+        <v>186</v>
       </c>
       <c r="C75" t="s">
         <v>49</v>
@@ -4188,10 +4188,10 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="K75" t="s">
-        <v>203</v>
+        <v>181</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.35">
@@ -4223,18 +4223,18 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>113</v>
+        <v>198</v>
       </c>
       <c r="K76" t="s">
-        <v>130</v>
+        <v>121</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" t="s">
-        <v>209</v>
+        <v>187</v>
       </c>
       <c r="B77" t="s">
-        <v>205</v>
+        <v>183</v>
       </c>
       <c r="C77" t="s">
         <v>49</v>
@@ -4258,10 +4258,10 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>144</v>
+        <v>199</v>
       </c>
       <c r="K77" t="s">
-        <v>207</v>
+        <v>185</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.35">
@@ -4293,18 +4293,18 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="K78" t="s">
-        <v>151</v>
+        <v>138</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A79" t="s">
-        <v>196</v>
+        <v>175</v>
       </c>
       <c r="B79" t="s">
-        <v>198</v>
+        <v>176</v>
       </c>
       <c r="C79" t="s">
         <v>49</v>
@@ -4328,21 +4328,21 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>197</v>
+        <v>224</v>
       </c>
       <c r="K79" t="s">
-        <v>199</v>
+        <v>177</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A80" t="s">
-        <v>190</v>
+        <v>170</v>
       </c>
       <c r="B80" t="s">
-        <v>191</v>
+        <v>171</v>
       </c>
       <c r="C80" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="D80" t="s">
         <v>21</v>
@@ -4363,10 +4363,10 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>192</v>
+        <v>225</v>
       </c>
       <c r="K80" t="s">
-        <v>193</v>
+        <v>172</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.35">
@@ -4374,10 +4374,10 @@
         <v>11</v>
       </c>
       <c r="B81" t="s">
-        <v>206</v>
+        <v>184</v>
       </c>
       <c r="C81" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="D81" t="s">
         <v>21</v>
@@ -4398,21 +4398,21 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>144</v>
+        <v>199</v>
       </c>
       <c r="K81" t="s">
-        <v>200</v>
+        <v>178</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A82" t="s">
-        <v>195</v>
+        <v>174</v>
       </c>
       <c r="B82" t="s">
-        <v>210</v>
+        <v>188</v>
       </c>
       <c r="C82" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="D82" t="s">
         <v>21</v>
@@ -4433,10 +4433,10 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>120</v>
+        <v>226</v>
       </c>
       <c r="K82" t="s">
-        <v>139</v>
+        <v>129</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.35">
@@ -4444,10 +4444,10 @@
         <v>39</v>
       </c>
       <c r="B83" t="s">
-        <v>201</v>
+        <v>179</v>
       </c>
       <c r="C83" t="s">
-        <v>147</v>
+        <v>134</v>
       </c>
       <c r="D83" t="s">
         <v>21</v>
@@ -4468,10 +4468,10 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="K83" t="s">
-        <v>202</v>
+        <v>180</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
1. Metrics report now uses centralised paths rather than string pattern matching 2. Improved logging for metric report script 3. Renamed metrics report script to match rule
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0F2C215-BFAA-4504-916D-4717ED991F03}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B374ED9F-FD81-4403-A650-E08553F2B987}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -668,12 +668,6 @@
     <t>MS.MET_MASKING</t>
   </si>
   <si>
-    <t>EX.MET_FASTQC_RAW_HTML_R1</t>
-  </si>
-  <si>
-    <t>EX.MET_FASTQC_RAW_HTML_R2</t>
-  </si>
-  <si>
     <t>EX.MET_FASTQC_FILTER_SUMMARY_R1</t>
   </si>
   <si>
@@ -723,6 +717,12 @@
   </si>
   <si>
     <t>EX.MET_DSC_DEPTH</t>
+  </si>
+  <si>
+    <t>EX.MET_FASTQC_RAW_SUMMARY_R1</t>
+  </si>
+  <si>
+    <t>EX.MET_FASTQC_RAW_SUMMARY_R2</t>
   </si>
 </sst>
 </file>
@@ -1596,7 +1596,7 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="35.1796875" customWidth="1"/>
-    <col min="2" max="2" width="123.1796875" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="123.1796875" customWidth="1"/>
     <col min="3" max="4" width="35.26953125" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
@@ -3138,7 +3138,7 @@
         <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>210</v>
+        <v>227</v>
       </c>
       <c r="K45" t="s">
         <v>113</v>
@@ -3173,7 +3173,7 @@
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>211</v>
+        <v>228</v>
       </c>
       <c r="K46" t="s">
         <v>113</v>
@@ -3208,7 +3208,7 @@
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>210</v>
+        <v>227</v>
       </c>
       <c r="K47" t="s">
         <v>115</v>
@@ -3243,7 +3243,7 @@
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>211</v>
+        <v>228</v>
       </c>
       <c r="K48" t="s">
         <v>115</v>
@@ -3278,7 +3278,7 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>210</v>
+        <v>227</v>
       </c>
       <c r="K49" t="s">
         <v>116</v>
@@ -3313,7 +3313,7 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>211</v>
+        <v>228</v>
       </c>
       <c r="K50" t="s">
         <v>116</v>
@@ -3348,7 +3348,7 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>210</v>
+        <v>227</v>
       </c>
       <c r="K51" t="s">
         <v>112</v>
@@ -3383,7 +3383,7 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>211</v>
+        <v>228</v>
       </c>
       <c r="K52" t="s">
         <v>112</v>
@@ -3418,7 +3418,7 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="K53" t="s">
         <v>114</v>
@@ -3453,7 +3453,7 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="K54" t="s">
         <v>114</v>
@@ -3488,7 +3488,7 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="K55" t="s">
         <v>117</v>
@@ -3523,7 +3523,7 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="K56" t="s">
         <v>117</v>
@@ -3558,7 +3558,7 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="K57" t="s">
         <v>118</v>
@@ -3593,7 +3593,7 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="K58" t="s">
         <v>118</v>
@@ -3628,7 +3628,7 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="K59" t="s">
         <v>119</v>
@@ -3663,7 +3663,7 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="K60" t="s">
         <v>119</v>
@@ -3698,7 +3698,7 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="K61" t="s">
         <v>120</v>
@@ -3733,7 +3733,7 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="K62" t="s">
         <v>120</v>
@@ -3768,7 +3768,7 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="K63" t="s">
         <v>148</v>
@@ -3803,7 +3803,7 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="K64" t="s">
         <v>122</v>
@@ -3838,7 +3838,7 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="K65" t="s">
         <v>150</v>
@@ -3873,7 +3873,7 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="K66" t="s">
         <v>151</v>
@@ -3908,7 +3908,7 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="K67" t="s">
         <v>137</v>
@@ -3943,7 +3943,7 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="K68" t="s">
         <v>126</v>
@@ -3978,7 +3978,7 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="K69" t="s">
         <v>128</v>
@@ -4013,7 +4013,7 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="K70" t="s">
         <v>127</v>
@@ -4048,7 +4048,7 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="K71" t="s">
         <v>123</v>
@@ -4083,7 +4083,7 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="K72" t="s">
         <v>131</v>
@@ -4118,7 +4118,7 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="K73" t="s">
         <v>124</v>
@@ -4153,7 +4153,7 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="K74" t="s">
         <v>125</v>
@@ -4188,7 +4188,7 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="K75" t="s">
         <v>181</v>
@@ -4293,7 +4293,7 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="K78" t="s">
         <v>138</v>
@@ -4328,7 +4328,7 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="K79" t="s">
         <v>177</v>
@@ -4363,7 +4363,7 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="K80" t="s">
         <v>172</v>
@@ -4433,7 +4433,7 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="K82" t="s">
         <v>129</v>
@@ -4468,7 +4468,7 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="K83" t="s">
         <v>180</v>

</xml_diff>

<commit_message>
Updated paths for ex trim component metrics
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl.localhost\Ubuntu-22.04\home\cam\SomaticCODEC\config\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B374ED9F-FD81-4403-A650-E08553F2B987}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E50EB6F-8989-4D16-9FE7-BCD1E3449CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="6165" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="228">
   <si>
     <t>nn_lower</t>
   </si>
@@ -488,12 +488,6 @@
     <t>Percentage of reads that are lost during demultiplexing (applicable only when all samples in lane are demuxed)</t>
   </si>
   <si>
-    <t>percent_bases_trimmed</t>
-  </si>
-  <si>
-    <t>percent_zero_length</t>
-  </si>
-  <si>
     <t>ex_zero_length_reads</t>
   </si>
   <si>
@@ -677,12 +671,6 @@
     <t>EX.MET_DEMUX_COUNTS_GINI</t>
   </si>
   <si>
-    <t>EX.MET_BASES_TRIMMED</t>
-  </si>
-  <si>
-    <t>EX.MET_TRIM_READ_LENGTHS</t>
-  </si>
-  <si>
     <t>EX.MET_FILTER_FASTQ</t>
   </si>
   <si>
@@ -723,6 +711,15 @@
   </si>
   <si>
     <t>EX.MET_FASTQC_RAW_SUMMARY_R2</t>
+  </si>
+  <si>
+    <t>EX.MET_TRIM_SUMMARY</t>
+  </si>
+  <si>
+    <t>trimmed_bases_pct.value</t>
+  </si>
+  <si>
+    <t>zero_length_pct.value</t>
   </si>
 </sst>
 </file>
@@ -1593,19 +1590,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
   <dimension ref="A1:K83"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="35.1796875" customWidth="1"/>
-    <col min="2" max="2" width="123.1796875" customWidth="1"/>
-    <col min="3" max="4" width="35.26953125" customWidth="1"/>
+    <col min="1" max="1" width="35.140625" customWidth="1"/>
+    <col min="2" max="2" width="123.140625" customWidth="1"/>
+    <col min="3" max="4" width="35.28515625" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
     <col min="8" max="8" width="9" customWidth="1"/>
-    <col min="9" max="9" width="12.81640625" customWidth="1"/>
-    <col min="10" max="10" width="40.54296875" customWidth="1"/>
-    <col min="11" max="11" width="76.81640625" customWidth="1"/>
+    <col min="9" max="9" width="12.85546875" customWidth="1"/>
+    <col min="10" max="10" width="40.5703125" customWidth="1"/>
+    <col min="11" max="11" width="76.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>28</v>
       </c>
@@ -1640,7 +1637,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>29</v>
       </c>
@@ -1669,12 +1666,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>30</v>
       </c>
       <c r="B3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="C3" t="s">
         <v>40</v>
@@ -1704,9 +1701,9 @@
         <v>50</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B4" t="s">
         <v>133</v>
@@ -1739,7 +1736,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>36</v>
       </c>
@@ -1768,12 +1765,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C6" t="s">
         <v>42</v>
@@ -1803,7 +1800,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>37</v>
       </c>
@@ -1832,12 +1829,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>38</v>
       </c>
       <c r="B8" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C8" t="s">
         <v>42</v>
@@ -1867,7 +1864,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -1902,7 +1899,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -1937,7 +1934,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>6</v>
       </c>
@@ -1966,13 +1963,13 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="K11" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -2001,18 +1998,18 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="K12" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>80</v>
       </c>
       <c r="B13" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C13" t="s">
         <v>45</v>
@@ -2036,18 +2033,18 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="K13" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C14" t="s">
         <v>45</v>
@@ -2071,18 +2068,18 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="K14" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>78</v>
       </c>
       <c r="B15" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C15" t="s">
         <v>45</v>
@@ -2106,18 +2103,18 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="K15" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>79</v>
       </c>
       <c r="B16" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C16" t="s">
         <v>45</v>
@@ -2141,13 +2138,13 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="K16" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>70</v>
       </c>
@@ -2176,13 +2173,13 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="K17" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>71</v>
       </c>
@@ -2211,18 +2208,18 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="K18" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>141</v>
       </c>
       <c r="B19" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C19" t="s">
         <v>45</v>
@@ -2246,18 +2243,18 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="K19" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>142</v>
       </c>
       <c r="B20" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C20" t="s">
         <v>45</v>
@@ -2281,13 +2278,13 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="K20" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>59</v>
       </c>
@@ -2316,13 +2313,13 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="K21" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>60</v>
       </c>
@@ -2351,13 +2348,13 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="K22" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>61</v>
       </c>
@@ -2386,13 +2383,13 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="K23" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>62</v>
       </c>
@@ -2421,13 +2418,13 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="K24" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>63</v>
       </c>
@@ -2456,13 +2453,13 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="K25" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>64</v>
       </c>
@@ -2491,18 +2488,18 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="K26" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>65</v>
       </c>
       <c r="B27" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C27" t="s">
         <v>45</v>
@@ -2526,18 +2523,18 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="K27" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>66</v>
       </c>
       <c r="B28" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C28" t="s">
         <v>45</v>
@@ -2561,18 +2558,18 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="K28" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B29" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C29" t="s">
         <v>47</v>
@@ -2596,13 +2593,13 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="K29" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>104</v>
       </c>
@@ -2631,13 +2628,13 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="K30" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>103</v>
       </c>
@@ -2666,18 +2663,18 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="K31" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="B32" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C32" t="s">
         <v>48</v>
@@ -2701,13 +2698,13 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="K32" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>102</v>
       </c>
@@ -2736,13 +2733,13 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="K33" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>51</v>
       </c>
@@ -2750,7 +2747,7 @@
         <v>4</v>
       </c>
       <c r="C34" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="D34" t="s">
         <v>21</v>
@@ -2771,13 +2768,13 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="K34" t="s">
         <v>130</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>16</v>
       </c>
@@ -2806,12 +2803,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>23</v>
       </c>
       <c r="B36" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C36" t="s">
         <v>41</v>
@@ -2841,12 +2838,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
+        <v>187</v>
+      </c>
+      <c r="B37" t="s">
         <v>189</v>
-      </c>
-      <c r="B37" t="s">
-        <v>191</v>
       </c>
       <c r="C37" t="s">
         <v>41</v>
@@ -2876,12 +2873,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B38" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C38" t="s">
         <v>41</v>
@@ -2908,7 +2905,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>33</v>
       </c>
@@ -2937,12 +2934,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>31</v>
       </c>
       <c r="B40" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="C40" t="s">
         <v>41</v>
@@ -2972,12 +2969,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
+        <v>190</v>
+      </c>
+      <c r="B41" t="s">
         <v>192</v>
-      </c>
-      <c r="B41" t="s">
-        <v>194</v>
       </c>
       <c r="C41" t="s">
         <v>41</v>
@@ -3007,12 +3004,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B42" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="C42" t="s">
         <v>41</v>
@@ -3039,7 +3036,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>17</v>
       </c>
@@ -3074,7 +3071,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>18</v>
       </c>
@@ -3109,12 +3106,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>74</v>
       </c>
       <c r="B45" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="C45" t="s">
         <v>44</v>
@@ -3138,18 +3135,18 @@
         <v>1</v>
       </c>
       <c r="J45" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="K45" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>75</v>
       </c>
       <c r="B46" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="C46" t="s">
         <v>44</v>
@@ -3173,18 +3170,18 @@
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="K46" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>76</v>
       </c>
       <c r="B47" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C47" t="s">
         <v>44</v>
@@ -3208,18 +3205,18 @@
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="K47" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>77</v>
       </c>
       <c r="B48" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="C48" t="s">
         <v>44</v>
@@ -3243,13 +3240,13 @@
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="K48" t="s">
         <v>115</v>
       </c>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>73</v>
       </c>
@@ -3278,13 +3275,13 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="K49" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>82</v>
       </c>
@@ -3313,13 +3310,13 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="K50" t="s">
         <v>116</v>
       </c>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>83</v>
       </c>
@@ -3348,13 +3345,13 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="K51" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>84</v>
       </c>
@@ -3383,18 +3380,18 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="K52" t="s">
         <v>112</v>
       </c>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>139</v>
       </c>
       <c r="B53" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C53" t="s">
         <v>44</v>
@@ -3418,18 +3415,18 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="K53" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>140</v>
       </c>
       <c r="B54" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="C54" t="s">
         <v>44</v>
@@ -3453,13 +3450,13 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="K54" t="s">
         <v>114</v>
       </c>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>85</v>
       </c>
@@ -3488,13 +3485,13 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="K55" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>86</v>
       </c>
@@ -3523,13 +3520,13 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="K56" t="s">
         <v>117</v>
       </c>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>87</v>
       </c>
@@ -3558,13 +3555,13 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="K57" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>88</v>
       </c>
@@ -3593,13 +3590,13 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="K58" t="s">
         <v>118</v>
       </c>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>89</v>
       </c>
@@ -3628,13 +3625,13 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="K59" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>90</v>
       </c>
@@ -3663,18 +3660,18 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="K60" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>91</v>
       </c>
       <c r="B61" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C61" t="s">
         <v>44</v>
@@ -3698,18 +3695,18 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="K61" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>92</v>
       </c>
       <c r="B62" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="C62" t="s">
         <v>44</v>
@@ -3733,13 +3730,13 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="K62" t="s">
         <v>120</v>
       </c>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>52</v>
       </c>
@@ -3768,18 +3765,18 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="K63" t="s">
         <v>148</v>
       </c>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>100</v>
       </c>
       <c r="B64" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C64" t="s">
         <v>46</v>
@@ -3803,13 +3800,13 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="K64" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>135</v>
       </c>
@@ -3838,15 +3835,15 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>213</v>
+        <v>225</v>
       </c>
       <c r="K65" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
         <v>150</v>
-      </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A66" t="s">
-        <v>152</v>
       </c>
       <c r="B66" t="s">
         <v>143</v>
@@ -3873,18 +3870,18 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>214</v>
+        <v>225</v>
       </c>
       <c r="K66" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="B67" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C67" t="s">
         <v>46</v>
@@ -3908,13 +3905,13 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="K67" t="s">
         <v>137</v>
       </c>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>55</v>
       </c>
@@ -3943,13 +3940,13 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="K68" t="s">
         <v>126</v>
       </c>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>54</v>
       </c>
@@ -3978,13 +3975,13 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="K69" t="s">
         <v>128</v>
       </c>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>56</v>
       </c>
@@ -4013,13 +4010,13 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="K70" t="s">
         <v>127</v>
       </c>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>109</v>
       </c>
@@ -4048,15 +4045,15 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="K71" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B72" t="s">
         <v>132</v>
@@ -4083,13 +4080,13 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="K72" t="s">
         <v>131</v>
       </c>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>107</v>
       </c>
@@ -4118,13 +4115,13 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="K73" t="s">
         <v>124</v>
       </c>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>106</v>
       </c>
@@ -4153,18 +4150,18 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="K74" t="s">
         <v>125</v>
       </c>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B75" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C75" t="s">
         <v>49</v>
@@ -4188,13 +4185,13 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="K75" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>12</v>
       </c>
@@ -4223,18 +4220,18 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="K76" t="s">
         <v>121</v>
       </c>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B77" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C77" t="s">
         <v>49</v>
@@ -4258,13 +4255,13 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="K77" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>8</v>
       </c>
@@ -4293,18 +4290,18 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="K78" t="s">
         <v>138</v>
       </c>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B79" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C79" t="s">
         <v>49</v>
@@ -4328,18 +4325,18 @@
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="K79" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B80" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="C80" t="s">
         <v>134</v>
@@ -4363,18 +4360,18 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="K80" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>11</v>
       </c>
       <c r="B81" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C81" t="s">
         <v>134</v>
@@ -4398,18 +4395,18 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="K81" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B82" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C82" t="s">
         <v>134</v>
@@ -4433,18 +4430,18 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="K82" t="s">
         <v>129</v>
       </c>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>39</v>
       </c>
       <c r="B83" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C83" t="s">
         <v>134</v>
@@ -4468,10 +4465,10 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="K83" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added component metrics for multimapping
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E50EB6F-8989-4D16-9FE7-BCD1E3449CB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62178FBC-64AB-4BE3-974E-BB7554DE6DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metrics!$A$1:$K$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metrics!$A$1:$K$86</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="238">
   <si>
     <t>nn_lower</t>
   </si>
@@ -720,6 +720,36 @@
   </si>
   <si>
     <t>zero_length_pct.value</t>
+  </si>
+  <si>
+    <t>ms_multimapped_alignment</t>
+  </si>
+  <si>
+    <t>Percentage of reads that mapped to more than one position after alignment</t>
+  </si>
+  <si>
+    <t>MS.MET_MULTIMAPPING</t>
+  </si>
+  <si>
+    <t>multimapping_pct.value</t>
+  </si>
+  <si>
+    <t>ex_multimapped_initial_alignment</t>
+  </si>
+  <si>
+    <t>EX.MET_MULTIMAPPING_RAW</t>
+  </si>
+  <si>
+    <t>ex_multimapped_dsc_realignment</t>
+  </si>
+  <si>
+    <t>Percentage of reads that mapped to more than one position, post initial alignment</t>
+  </si>
+  <si>
+    <t>Percentage of reads that mapped to more than one position, post realignment of DSC reads</t>
+  </si>
+  <si>
+    <t>EX.MET_MULTIMAPPING_DSC</t>
   </si>
 </sst>
 </file>
@@ -1589,7 +1619,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K83"/>
+  <dimension ref="A1:K86"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" customWidth="1"/>
@@ -2636,10 +2666,10 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>103</v>
+        <v>228</v>
       </c>
       <c r="B31" t="s">
-        <v>108</v>
+        <v>229</v>
       </c>
       <c r="C31" t="s">
         <v>48</v>
@@ -2651,30 +2681,30 @@
         <v>0</v>
       </c>
       <c r="F31">
-        <v>0.17</v>
+        <v>10</v>
       </c>
       <c r="G31">
         <v>0</v>
       </c>
       <c r="H31">
-        <v>0.03</v>
+        <v>5</v>
       </c>
       <c r="I31" t="b">
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>204</v>
+        <v>230</v>
       </c>
       <c r="K31" t="s">
-        <v>151</v>
+        <v>231</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>157</v>
+        <v>103</v>
       </c>
       <c r="B32" t="s">
-        <v>162</v>
+        <v>108</v>
       </c>
       <c r="C32" t="s">
         <v>48</v>
@@ -2683,33 +2713,33 @@
         <v>21</v>
       </c>
       <c r="E32">
-        <v>21.75</v>
+        <v>0</v>
       </c>
       <c r="F32">
-        <v>100</v>
+        <v>0.17</v>
       </c>
       <c r="G32">
-        <v>26.1</v>
+        <v>0</v>
       </c>
       <c r="H32">
-        <v>100</v>
+        <v>0.03</v>
       </c>
       <c r="I32" t="b">
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="K32" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>102</v>
+        <v>157</v>
       </c>
       <c r="B33" t="s">
-        <v>69</v>
+        <v>162</v>
       </c>
       <c r="C33" t="s">
         <v>48</v>
@@ -2718,115 +2748,115 @@
         <v>21</v>
       </c>
       <c r="E33">
-        <v>125</v>
+        <v>21.75</v>
       </c>
       <c r="F33">
-        <v>175</v>
+        <v>100</v>
       </c>
       <c r="G33">
-        <v>140</v>
+        <v>26.1</v>
       </c>
       <c r="H33">
-        <v>160</v>
+        <v>100</v>
       </c>
       <c r="I33" t="b">
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="K33" t="s">
-        <v>127</v>
+        <v>161</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>51</v>
+        <v>102</v>
       </c>
       <c r="B34" t="s">
-        <v>4</v>
+        <v>69</v>
       </c>
       <c r="C34" t="s">
-        <v>163</v>
+        <v>48</v>
       </c>
       <c r="D34" t="s">
         <v>21</v>
       </c>
       <c r="E34">
-        <v>70</v>
+        <v>125</v>
       </c>
       <c r="F34">
-        <v>90</v>
+        <v>175</v>
       </c>
       <c r="G34">
-        <v>70</v>
+        <v>140</v>
       </c>
       <c r="H34">
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="I34" t="b">
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K34" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="B35" t="s">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="C35" t="s">
-        <v>41</v>
+        <v>163</v>
       </c>
       <c r="D35" t="s">
         <v>21</v>
       </c>
       <c r="E35">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F35">
-        <v>1000</v>
+        <v>90</v>
+      </c>
+      <c r="G35">
+        <v>70</v>
+      </c>
+      <c r="H35">
+        <v>80</v>
       </c>
       <c r="I35" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>50</v>
+        <v>207</v>
       </c>
       <c r="K35" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B36" t="s">
-        <v>159</v>
+        <v>32</v>
       </c>
       <c r="C36" t="s">
         <v>41</v>
       </c>
       <c r="D36" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E36">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F36">
-        <v>0.3</v>
-      </c>
-      <c r="G36">
-        <v>0</v>
-      </c>
-      <c r="H36">
-        <v>0.2</v>
+        <v>1000</v>
       </c>
       <c r="I36" t="b">
         <v>0</v>
@@ -2840,28 +2870,28 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>187</v>
+        <v>23</v>
       </c>
       <c r="B37" t="s">
-        <v>189</v>
+        <v>159</v>
       </c>
       <c r="C37" t="s">
         <v>41</v>
       </c>
       <c r="D37" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E37">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="F37">
-        <v>100</v>
+        <v>0.3</v>
       </c>
       <c r="G37">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H37">
-        <v>100</v>
+        <v>0.2</v>
       </c>
       <c r="I37" t="b">
         <v>0</v>
@@ -2875,10 +2905,10 @@
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B38" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="C38" t="s">
         <v>41</v>
@@ -2887,16 +2917,16 @@
         <v>21</v>
       </c>
       <c r="E38">
-        <v>110</v>
+        <v>85</v>
       </c>
       <c r="F38">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="G38">
-        <v>120</v>
+        <v>95</v>
       </c>
       <c r="H38">
-        <v>140</v>
+        <v>100</v>
       </c>
       <c r="I38" t="b">
         <v>0</v>
@@ -2904,13 +2934,16 @@
       <c r="J38" t="s">
         <v>50</v>
       </c>
+      <c r="K38" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>33</v>
+        <v>188</v>
       </c>
       <c r="B39" t="s">
-        <v>34</v>
+        <v>193</v>
       </c>
       <c r="C39" t="s">
         <v>41</v>
@@ -2919,10 +2952,16 @@
         <v>21</v>
       </c>
       <c r="E39">
-        <v>4.3</v>
-      </c>
-      <c r="F39" t="s">
-        <v>5</v>
+        <v>110</v>
+      </c>
+      <c r="F39">
+        <v>150</v>
+      </c>
+      <c r="G39">
+        <v>120</v>
+      </c>
+      <c r="H39">
+        <v>140</v>
       </c>
       <c r="I39" t="b">
         <v>0</v>
@@ -2930,34 +2969,25 @@
       <c r="J39" t="s">
         <v>50</v>
       </c>
-      <c r="K39" t="s">
-        <v>50</v>
-      </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B40" t="s">
-        <v>159</v>
+        <v>34</v>
       </c>
       <c r="C40" t="s">
         <v>41</v>
       </c>
       <c r="D40" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E40">
-        <v>0</v>
-      </c>
-      <c r="F40">
-        <v>0.4</v>
-      </c>
-      <c r="G40">
-        <v>0</v>
-      </c>
-      <c r="H40">
-        <v>0.3</v>
+        <v>4.3</v>
+      </c>
+      <c r="F40" t="s">
+        <v>5</v>
       </c>
       <c r="I40" t="b">
         <v>0</v>
@@ -2971,28 +3001,28 @@
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>190</v>
+        <v>31</v>
       </c>
       <c r="B41" t="s">
-        <v>192</v>
+        <v>159</v>
       </c>
       <c r="C41" t="s">
         <v>41</v>
       </c>
       <c r="D41" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E41">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F41">
-        <v>100</v>
+        <v>0.4</v>
       </c>
       <c r="G41">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="H41">
-        <v>100</v>
+        <v>0.3</v>
       </c>
       <c r="I41" t="b">
         <v>0</v>
@@ -3006,10 +3036,10 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B42" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C42" t="s">
         <v>41</v>
@@ -3018,16 +3048,16 @@
         <v>21</v>
       </c>
       <c r="E42">
-        <v>440</v>
+        <v>50</v>
       </c>
       <c r="F42">
-        <v>740</v>
+        <v>100</v>
       </c>
       <c r="G42">
-        <v>530</v>
+        <v>90</v>
       </c>
       <c r="H42">
-        <v>650</v>
+        <v>100</v>
       </c>
       <c r="I42" t="b">
         <v>0</v>
@@ -3035,13 +3065,16 @@
       <c r="J42" t="s">
         <v>50</v>
       </c>
+      <c r="K42" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>17</v>
+        <v>191</v>
       </c>
       <c r="B43" t="s">
-        <v>14</v>
+        <v>194</v>
       </c>
       <c r="C43" t="s">
         <v>41</v>
@@ -3050,16 +3083,16 @@
         <v>21</v>
       </c>
       <c r="E43">
-        <v>544</v>
+        <v>440</v>
       </c>
       <c r="F43">
-        <v>624</v>
+        <v>740</v>
       </c>
       <c r="G43">
-        <v>564</v>
+        <v>530</v>
       </c>
       <c r="H43">
-        <v>604</v>
+        <v>650</v>
       </c>
       <c r="I43" t="b">
         <v>0</v>
@@ -3067,16 +3100,13 @@
       <c r="J43" t="s">
         <v>50</v>
       </c>
-      <c r="K43" t="s">
-        <v>50</v>
-      </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B44" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C44" t="s">
         <v>41</v>
@@ -3085,16 +3115,16 @@
         <v>21</v>
       </c>
       <c r="E44">
-        <v>94.9</v>
+        <v>544</v>
       </c>
       <c r="F44">
-        <v>100</v>
+        <v>624</v>
       </c>
       <c r="G44">
-        <v>100</v>
+        <v>564</v>
       </c>
       <c r="H44">
-        <v>100</v>
+        <v>604</v>
       </c>
       <c r="I44" t="b">
         <v>0</v>
@@ -3108,45 +3138,45 @@
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
+        <v>18</v>
+      </c>
+      <c r="B45" t="s">
+        <v>15</v>
+      </c>
+      <c r="C45" t="s">
+        <v>41</v>
+      </c>
+      <c r="D45" t="s">
+        <v>21</v>
+      </c>
+      <c r="E45">
+        <v>94.9</v>
+      </c>
+      <c r="F45">
+        <v>100</v>
+      </c>
+      <c r="G45">
+        <v>100</v>
+      </c>
+      <c r="H45">
+        <v>100</v>
+      </c>
+      <c r="I45" t="b">
+        <v>0</v>
+      </c>
+      <c r="J45" t="s">
+        <v>50</v>
+      </c>
+      <c r="K45" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
         <v>74</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B46" t="s">
         <v>153</v>
-      </c>
-      <c r="C45" t="s">
-        <v>44</v>
-      </c>
-      <c r="D45" t="s">
-        <v>53</v>
-      </c>
-      <c r="E45">
-        <v>35</v>
-      </c>
-      <c r="F45">
-        <v>40</v>
-      </c>
-      <c r="G45">
-        <v>39</v>
-      </c>
-      <c r="H45">
-        <v>40</v>
-      </c>
-      <c r="I45" t="b">
-        <v>1</v>
-      </c>
-      <c r="J45" t="s">
-        <v>223</v>
-      </c>
-      <c r="K45" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>75</v>
-      </c>
-      <c r="B46" t="s">
-        <v>154</v>
       </c>
       <c r="C46" t="s">
         <v>44</v>
@@ -3170,18 +3200,18 @@
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="K46" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B47" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C47" t="s">
         <v>44</v>
@@ -3190,30 +3220,30 @@
         <v>53</v>
       </c>
       <c r="E47">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F47">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G47">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="H47">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="I47" t="b">
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K47" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="48" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B48" t="s">
         <v>152</v>
@@ -3240,7 +3270,7 @@
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="K48" t="s">
         <v>115</v>
@@ -3248,10 +3278,10 @@
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B49" t="s">
-        <v>72</v>
+        <v>152</v>
       </c>
       <c r="C49" t="s">
         <v>44</v>
@@ -3260,30 +3290,30 @@
         <v>53</v>
       </c>
       <c r="E49">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F49">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="G49">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="H49">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="I49" t="b">
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K49" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="B50" t="s">
         <v>72</v>
@@ -3310,7 +3340,7 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="K50" t="s">
         <v>116</v>
@@ -3318,10 +3348,10 @@
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B51" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="C51" t="s">
         <v>44</v>
@@ -3330,30 +3360,30 @@
         <v>53</v>
       </c>
       <c r="E51">
-        <v>2850</v>
-      </c>
-      <c r="F51" t="s">
-        <v>5</v>
+        <v>150</v>
+      </c>
+      <c r="F51">
+        <v>150</v>
       </c>
       <c r="G51">
-        <v>3000</v>
-      </c>
-      <c r="H51" t="s">
-        <v>5</v>
+        <v>150</v>
+      </c>
+      <c r="H51">
+        <v>150</v>
       </c>
       <c r="I51" t="b">
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="K51" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B52" t="s">
         <v>93</v>
@@ -3380,7 +3410,7 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="K52" t="s">
         <v>112</v>
@@ -3388,42 +3418,42 @@
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>139</v>
+        <v>84</v>
       </c>
       <c r="B53" t="s">
-        <v>156</v>
+        <v>93</v>
       </c>
       <c r="C53" t="s">
         <v>44</v>
       </c>
       <c r="D53" t="s">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="E53">
-        <v>30</v>
-      </c>
-      <c r="F53">
-        <v>40</v>
+        <v>2850</v>
+      </c>
+      <c r="F53" t="s">
+        <v>5</v>
       </c>
       <c r="G53">
-        <v>35</v>
-      </c>
-      <c r="H53">
-        <v>40</v>
+        <v>3000</v>
+      </c>
+      <c r="H53" t="s">
+        <v>5</v>
       </c>
       <c r="I53" t="b">
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>208</v>
+        <v>224</v>
       </c>
       <c r="K53" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B54" t="s">
         <v>156</v>
@@ -3450,7 +3480,7 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="K54" t="s">
         <v>114</v>
@@ -3458,10 +3488,10 @@
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>85</v>
+        <v>140</v>
       </c>
       <c r="B55" t="s">
-        <v>95</v>
+        <v>156</v>
       </c>
       <c r="C55" t="s">
         <v>44</v>
@@ -3470,30 +3500,30 @@
         <v>21</v>
       </c>
       <c r="E55">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F55">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="G55">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H55">
-        <v>0.1</v>
+        <v>40</v>
       </c>
       <c r="I55" t="b">
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K55" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B56" t="s">
         <v>95</v>
@@ -3520,7 +3550,7 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="K56" t="s">
         <v>117</v>
@@ -3528,10 +3558,10 @@
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B57" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C57" t="s">
         <v>44</v>
@@ -3543,27 +3573,27 @@
         <v>0</v>
       </c>
       <c r="F57">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="G57">
         <v>0</v>
       </c>
       <c r="H57">
-        <v>20</v>
+        <v>0.1</v>
       </c>
       <c r="I57" t="b">
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K57" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B58" t="s">
         <v>96</v>
@@ -3590,7 +3620,7 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="K58" t="s">
         <v>118</v>
@@ -3598,10 +3628,10 @@
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B59" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C59" t="s">
         <v>44</v>
@@ -3613,27 +3643,27 @@
         <v>0</v>
       </c>
       <c r="F59">
+        <v>30</v>
+      </c>
+      <c r="G59">
+        <v>0</v>
+      </c>
+      <c r="H59">
         <v>20</v>
       </c>
-      <c r="G59">
-        <v>0</v>
-      </c>
-      <c r="H59">
-        <v>10</v>
-      </c>
       <c r="I59" t="b">
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K59" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B60" t="s">
         <v>97</v>
@@ -3660,7 +3690,7 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="K60" t="s">
         <v>119</v>
@@ -3668,10 +3698,10 @@
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B61" t="s">
-        <v>155</v>
+        <v>97</v>
       </c>
       <c r="C61" t="s">
         <v>44</v>
@@ -3683,27 +3713,27 @@
         <v>0</v>
       </c>
       <c r="F61">
+        <v>20</v>
+      </c>
+      <c r="G61">
+        <v>0</v>
+      </c>
+      <c r="H61">
         <v>10</v>
       </c>
-      <c r="G61">
-        <v>0</v>
-      </c>
-      <c r="H61">
-        <v>5</v>
-      </c>
       <c r="I61" t="b">
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="K61" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B62" t="s">
         <v>155</v>
@@ -3730,7 +3760,7 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="K62" t="s">
         <v>120</v>
@@ -3738,45 +3768,45 @@
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>52</v>
+        <v>92</v>
       </c>
       <c r="B63" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="C63" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D63" t="s">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="E63">
         <v>0</v>
       </c>
       <c r="F63">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G63">
         <v>0</v>
       </c>
       <c r="H63">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I63" t="b">
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="K63" t="s">
-        <v>148</v>
+        <v>120</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>100</v>
+        <v>52</v>
       </c>
       <c r="B64" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="C64" t="s">
         <v>46</v>
@@ -3788,13 +3818,13 @@
         <v>0</v>
       </c>
       <c r="F64">
-        <v>0.1</v>
+        <v>25</v>
       </c>
       <c r="G64">
         <v>0</v>
       </c>
       <c r="H64">
-        <v>0.05</v>
+        <v>10</v>
       </c>
       <c r="I64" t="b">
         <v>1</v>
@@ -3803,50 +3833,50 @@
         <v>210</v>
       </c>
       <c r="K64" t="s">
-        <v>122</v>
+        <v>148</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>135</v>
+        <v>100</v>
       </c>
       <c r="B65" t="s">
-        <v>136</v>
+        <v>164</v>
       </c>
       <c r="C65" t="s">
         <v>46</v>
       </c>
       <c r="D65" t="s">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="E65">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F65">
-        <v>40</v>
+        <v>0.1</v>
       </c>
       <c r="G65">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H65">
-        <v>20</v>
+        <v>0.05</v>
       </c>
       <c r="I65" t="b">
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>225</v>
+        <v>210</v>
       </c>
       <c r="K65" t="s">
-        <v>226</v>
+        <v>122</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="B66" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="C66" t="s">
         <v>46</v>
@@ -3855,16 +3885,16 @@
         <v>21</v>
       </c>
       <c r="E66">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F66">
+        <v>40</v>
+      </c>
+      <c r="G66">
+        <v>1</v>
+      </c>
+      <c r="H66">
         <v>20</v>
-      </c>
-      <c r="G66">
-        <v>0</v>
-      </c>
-      <c r="H66">
-        <v>10</v>
       </c>
       <c r="I66" t="b">
         <v>1</v>
@@ -3873,15 +3903,15 @@
         <v>225</v>
       </c>
       <c r="K66" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="B67" t="s">
-        <v>166</v>
+        <v>143</v>
       </c>
       <c r="C67" t="s">
         <v>46</v>
@@ -3890,68 +3920,68 @@
         <v>21</v>
       </c>
       <c r="E67">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="F67">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="G67">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="H67">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="I67" t="b">
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>211</v>
+        <v>225</v>
       </c>
       <c r="K67" t="s">
-        <v>137</v>
+        <v>227</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>55</v>
+        <v>165</v>
       </c>
       <c r="B68" t="s">
-        <v>67</v>
+        <v>166</v>
       </c>
       <c r="C68" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D68" t="s">
         <v>21</v>
       </c>
       <c r="E68">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="F68">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G68">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="H68">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I68" t="b">
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="K68" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B69" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C69" t="s">
         <v>43</v>
@@ -3960,13 +3990,13 @@
         <v>21</v>
       </c>
       <c r="E69">
-        <v>50</v>
+        <v>90</v>
       </c>
       <c r="F69">
         <v>100</v>
       </c>
       <c r="G69">
-        <v>75</v>
+        <v>95</v>
       </c>
       <c r="H69">
         <v>100</v>
@@ -3978,15 +4008,15 @@
         <v>212</v>
       </c>
       <c r="K69" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>56</v>
+        <v>232</v>
       </c>
       <c r="B70" t="s">
-        <v>101</v>
+        <v>235</v>
       </c>
       <c r="C70" t="s">
         <v>43</v>
@@ -3995,36 +4025,36 @@
         <v>21</v>
       </c>
       <c r="E70">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="F70">
-        <v>180</v>
+        <v>10</v>
       </c>
       <c r="G70">
-        <v>140</v>
+        <v>0</v>
       </c>
       <c r="H70">
-        <v>160</v>
+        <v>5</v>
       </c>
       <c r="I70" t="b">
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>213</v>
+        <v>233</v>
       </c>
       <c r="K70" t="s">
-        <v>127</v>
+        <v>231</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>109</v>
+        <v>54</v>
       </c>
       <c r="B71" t="s">
-        <v>144</v>
+        <v>68</v>
       </c>
       <c r="C71" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="D71" t="s">
         <v>21</v>
@@ -4033,65 +4063,65 @@
         <v>50</v>
       </c>
       <c r="F71">
-        <v>70</v>
+        <v>100</v>
       </c>
       <c r="G71">
-        <v>50</v>
+        <v>75</v>
       </c>
       <c r="H71">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="I71" t="b">
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="K71" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>171</v>
+        <v>56</v>
       </c>
       <c r="B72" t="s">
-        <v>132</v>
+        <v>101</v>
       </c>
       <c r="C72" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="D72" t="s">
         <v>21</v>
       </c>
       <c r="E72">
-        <v>58.3</v>
+        <v>120</v>
       </c>
       <c r="F72">
-        <v>100</v>
+        <v>180</v>
       </c>
       <c r="G72">
-        <v>90</v>
+        <v>140</v>
       </c>
       <c r="H72">
-        <v>100</v>
+        <v>160</v>
       </c>
       <c r="I72" t="b">
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="K72" t="s">
-        <v>131</v>
+        <v>127</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B73" t="s">
-        <v>10</v>
+        <v>144</v>
       </c>
       <c r="C73" t="s">
         <v>49</v>
@@ -4100,33 +4130,33 @@
         <v>21</v>
       </c>
       <c r="E73">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="F73">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="G73">
-        <v>99.5</v>
+        <v>50</v>
       </c>
       <c r="H73">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="I73" t="b">
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="K73" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>106</v>
+        <v>171</v>
       </c>
       <c r="B74" t="s">
-        <v>105</v>
+        <v>132</v>
       </c>
       <c r="C74" t="s">
         <v>49</v>
@@ -4135,33 +4165,33 @@
         <v>21</v>
       </c>
       <c r="E74">
-        <v>0</v>
+        <v>58.3</v>
       </c>
       <c r="F74">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="G74">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="H74">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="I74" t="b">
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="K74" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>180</v>
+        <v>107</v>
       </c>
       <c r="B75" t="s">
-        <v>184</v>
+        <v>10</v>
       </c>
       <c r="C75" t="s">
         <v>49</v>
@@ -4170,33 +4200,33 @@
         <v>21</v>
       </c>
       <c r="E75">
-        <v>1</v>
-      </c>
-      <c r="F75" t="s">
-        <v>5</v>
+        <v>99</v>
+      </c>
+      <c r="F75">
+        <v>100</v>
       </c>
       <c r="G75">
-        <v>1</v>
-      </c>
-      <c r="H75" t="s">
-        <v>5</v>
+        <v>99.5</v>
+      </c>
+      <c r="H75">
+        <v>100</v>
       </c>
       <c r="I75" t="b">
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="K75" t="s">
-        <v>179</v>
+        <v>124</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>12</v>
+        <v>234</v>
       </c>
       <c r="B76" t="s">
-        <v>13</v>
+        <v>236</v>
       </c>
       <c r="C76" t="s">
         <v>49</v>
@@ -4208,30 +4238,30 @@
         <v>0</v>
       </c>
       <c r="F76">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="G76">
         <v>0</v>
       </c>
       <c r="H76">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I76" t="b">
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>196</v>
+        <v>237</v>
       </c>
       <c r="K76" t="s">
-        <v>121</v>
+        <v>231</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>185</v>
+        <v>106</v>
       </c>
       <c r="B77" t="s">
-        <v>181</v>
+        <v>105</v>
       </c>
       <c r="C77" t="s">
         <v>49</v>
@@ -4240,33 +4270,33 @@
         <v>21</v>
       </c>
       <c r="E77">
-        <v>14.5</v>
+        <v>0</v>
       </c>
       <c r="F77">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="G77">
-        <v>26.1</v>
+        <v>0</v>
       </c>
       <c r="H77">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="I77" t="b">
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>197</v>
+        <v>216</v>
       </c>
       <c r="K77" t="s">
-        <v>183</v>
+        <v>125</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>8</v>
+        <v>180</v>
       </c>
       <c r="B78" t="s">
-        <v>9</v>
+        <v>184</v>
       </c>
       <c r="C78" t="s">
         <v>49</v>
@@ -4275,33 +4305,33 @@
         <v>21</v>
       </c>
       <c r="E78">
-        <v>0</v>
-      </c>
-      <c r="F78">
-        <v>1.2E-2</v>
+        <v>1</v>
+      </c>
+      <c r="F78" t="s">
+        <v>5</v>
       </c>
       <c r="G78">
-        <v>2.0000000000000001E-4</v>
-      </c>
-      <c r="H78">
-        <v>6.0000000000000001E-3</v>
+        <v>1</v>
+      </c>
+      <c r="H78" t="s">
+        <v>5</v>
       </c>
       <c r="I78" t="b">
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="K78" t="s">
-        <v>138</v>
+        <v>179</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>173</v>
+        <v>12</v>
       </c>
       <c r="B79" t="s">
-        <v>174</v>
+        <v>13</v>
       </c>
       <c r="C79" t="s">
         <v>49</v>
@@ -4310,138 +4340,138 @@
         <v>21</v>
       </c>
       <c r="E79">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="F79">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="G79">
-        <v>82.8</v>
+        <v>0</v>
       </c>
       <c r="H79">
-        <v>120</v>
+        <v>0</v>
       </c>
       <c r="I79" t="b">
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>218</v>
+        <v>196</v>
       </c>
       <c r="K79" t="s">
-        <v>175</v>
+        <v>121</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>168</v>
+        <v>185</v>
       </c>
       <c r="B80" t="s">
-        <v>169</v>
+        <v>181</v>
       </c>
       <c r="C80" t="s">
-        <v>134</v>
+        <v>49</v>
       </c>
       <c r="D80" t="s">
         <v>21</v>
       </c>
       <c r="E80">
-        <v>0</v>
+        <v>14.5</v>
       </c>
       <c r="F80">
-        <v>5.6599999999999999E-4</v>
+        <v>100</v>
       </c>
       <c r="G80">
-        <v>2.0000000000000001E-4</v>
+        <v>26.1</v>
       </c>
       <c r="H80">
-        <v>3.2679999999999997E-4</v>
+        <v>100</v>
       </c>
       <c r="I80" t="b">
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>219</v>
+        <v>197</v>
       </c>
       <c r="K80" t="s">
-        <v>170</v>
+        <v>183</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B81" t="s">
-        <v>182</v>
+        <v>9</v>
       </c>
       <c r="C81" t="s">
-        <v>134</v>
+        <v>49</v>
       </c>
       <c r="D81" t="s">
         <v>21</v>
       </c>
       <c r="E81">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F81">
-        <v>100</v>
+        <v>1.2E-2</v>
       </c>
       <c r="G81">
-        <v>20</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="H81">
-        <v>100</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="I81" t="b">
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>197</v>
+        <v>217</v>
       </c>
       <c r="K81" t="s">
-        <v>176</v>
+        <v>138</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B82" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="C82" t="s">
-        <v>134</v>
+        <v>49</v>
       </c>
       <c r="D82" t="s">
         <v>21</v>
       </c>
       <c r="E82">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="F82">
-        <v>95</v>
+        <v>120</v>
       </c>
       <c r="G82">
-        <v>0</v>
+        <v>82.8</v>
       </c>
       <c r="H82">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="I82" t="b">
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="K82" t="s">
-        <v>129</v>
+        <v>175</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>39</v>
+        <v>168</v>
       </c>
       <c r="B83" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
       <c r="C83" t="s">
         <v>134</v>
@@ -4450,29 +4480,134 @@
         <v>21</v>
       </c>
       <c r="E83">
+        <v>0</v>
+      </c>
+      <c r="F83">
+        <v>5.6599999999999999E-4</v>
+      </c>
+      <c r="G83">
+        <v>2.0000000000000001E-4</v>
+      </c>
+      <c r="H83">
+        <v>3.2679999999999997E-4</v>
+      </c>
+      <c r="I83" t="b">
+        <v>1</v>
+      </c>
+      <c r="J83" t="s">
+        <v>219</v>
+      </c>
+      <c r="K83" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>11</v>
+      </c>
+      <c r="B84" t="s">
+        <v>182</v>
+      </c>
+      <c r="C84" t="s">
+        <v>134</v>
+      </c>
+      <c r="D84" t="s">
+        <v>21</v>
+      </c>
+      <c r="E84">
+        <v>4</v>
+      </c>
+      <c r="F84">
+        <v>100</v>
+      </c>
+      <c r="G84">
+        <v>20</v>
+      </c>
+      <c r="H84">
+        <v>100</v>
+      </c>
+      <c r="I84" t="b">
+        <v>1</v>
+      </c>
+      <c r="J84" t="s">
+        <v>197</v>
+      </c>
+      <c r="K84" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>172</v>
+      </c>
+      <c r="B85" t="s">
+        <v>186</v>
+      </c>
+      <c r="C85" t="s">
+        <v>134</v>
+      </c>
+      <c r="D85" t="s">
+        <v>21</v>
+      </c>
+      <c r="E85">
+        <v>0</v>
+      </c>
+      <c r="F85">
+        <v>95</v>
+      </c>
+      <c r="G85">
+        <v>0</v>
+      </c>
+      <c r="H85">
+        <v>80</v>
+      </c>
+      <c r="I85" t="b">
+        <v>1</v>
+      </c>
+      <c r="J85" t="s">
+        <v>220</v>
+      </c>
+      <c r="K85" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>39</v>
+      </c>
+      <c r="B86" t="s">
+        <v>177</v>
+      </c>
+      <c r="C86" t="s">
+        <v>134</v>
+      </c>
+      <c r="D86" t="s">
+        <v>21</v>
+      </c>
+      <c r="E86">
         <v>33</v>
       </c>
-      <c r="F83">
+      <c r="F86">
         <v>100</v>
       </c>
-      <c r="G83">
+      <c r="G86">
         <v>67</v>
       </c>
-      <c r="H83">
+      <c r="H86">
         <v>100</v>
       </c>
-      <c r="I83" t="b">
-        <v>1</v>
-      </c>
-      <c r="J83" t="s">
+      <c r="I86" t="b">
+        <v>1</v>
+      </c>
+      <c r="J86" t="s">
         <v>221</v>
       </c>
-      <c r="K83" t="s">
+      <c r="K86" t="s">
         <v>178</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K83" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K86" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Reconciled ms file names with ex file names
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62178FBC-64AB-4BE3-974E-BB7554DE6DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{417A84A5-F8E8-4FB1-AF0F-0BFD0541899C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -650,12 +650,6 @@
     <t>MS.MET_ALIGNMENT</t>
   </si>
   <si>
-    <t>MS.MET_DUPLICATION_2</t>
-  </si>
-  <si>
-    <t>MS.MET_COVERAGE_BY_DEPTH</t>
-  </si>
-  <si>
     <t>MS.MET_INSERT_SIZE_TXT</t>
   </si>
   <si>
@@ -750,6 +744,12 @@
   </si>
   <si>
     <t>EX.MET_MULTIMAPPING_DSC</t>
+  </si>
+  <si>
+    <t>MS.MET_DUPLICATION</t>
+  </si>
+  <si>
+    <t>MS.MET_COVERAGE</t>
   </si>
 </sst>
 </file>
@@ -2666,10 +2666,10 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B31" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="C31" t="s">
         <v>48</v>
@@ -2693,10 +2693,10 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="K31" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
@@ -2728,7 +2728,7 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>204</v>
+        <v>236</v>
       </c>
       <c r="K32" t="s">
         <v>151</v>
@@ -2763,7 +2763,7 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>205</v>
+        <v>237</v>
       </c>
       <c r="K33" t="s">
         <v>161</v>
@@ -2798,7 +2798,7 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="K34" t="s">
         <v>127</v>
@@ -2833,7 +2833,7 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="K35" t="s">
         <v>130</v>
@@ -3200,7 +3200,7 @@
         <v>1</v>
       </c>
       <c r="J46" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="K46" t="s">
         <v>113</v>
@@ -3235,7 +3235,7 @@
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="K47" t="s">
         <v>113</v>
@@ -3270,7 +3270,7 @@
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="K48" t="s">
         <v>115</v>
@@ -3305,7 +3305,7 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="K49" t="s">
         <v>115</v>
@@ -3340,7 +3340,7 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="K50" t="s">
         <v>116</v>
@@ -3375,7 +3375,7 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="K51" t="s">
         <v>116</v>
@@ -3410,7 +3410,7 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="K52" t="s">
         <v>112</v>
@@ -3445,7 +3445,7 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="K53" t="s">
         <v>112</v>
@@ -3480,7 +3480,7 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="K54" t="s">
         <v>114</v>
@@ -3515,7 +3515,7 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="K55" t="s">
         <v>114</v>
@@ -3550,7 +3550,7 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="K56" t="s">
         <v>117</v>
@@ -3585,7 +3585,7 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="K57" t="s">
         <v>117</v>
@@ -3620,7 +3620,7 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="K58" t="s">
         <v>118</v>
@@ -3655,7 +3655,7 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="K59" t="s">
         <v>118</v>
@@ -3690,7 +3690,7 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="K60" t="s">
         <v>119</v>
@@ -3725,7 +3725,7 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="K61" t="s">
         <v>119</v>
@@ -3760,7 +3760,7 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="K62" t="s">
         <v>120</v>
@@ -3795,7 +3795,7 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="K63" t="s">
         <v>120</v>
@@ -3830,7 +3830,7 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="K64" t="s">
         <v>148</v>
@@ -3865,7 +3865,7 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="K65" t="s">
         <v>122</v>
@@ -3900,10 +3900,10 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="K66" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
@@ -3935,10 +3935,10 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
+        <v>223</v>
+      </c>
+      <c r="K67" t="s">
         <v>225</v>
-      </c>
-      <c r="K67" t="s">
-        <v>227</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
@@ -3970,7 +3970,7 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="K68" t="s">
         <v>137</v>
@@ -4005,7 +4005,7 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="K69" t="s">
         <v>126</v>
@@ -4013,10 +4013,10 @@
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B70" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="C70" t="s">
         <v>43</v>
@@ -4040,10 +4040,10 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="K70" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
@@ -4075,7 +4075,7 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="K71" t="s">
         <v>128</v>
@@ -4110,7 +4110,7 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="K72" t="s">
         <v>127</v>
@@ -4145,7 +4145,7 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="K73" t="s">
         <v>123</v>
@@ -4180,7 +4180,7 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="K74" t="s">
         <v>131</v>
@@ -4215,7 +4215,7 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="K75" t="s">
         <v>124</v>
@@ -4223,10 +4223,10 @@
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
+        <v>232</v>
+      </c>
+      <c r="B76" t="s">
         <v>234</v>
-      </c>
-      <c r="B76" t="s">
-        <v>236</v>
       </c>
       <c r="C76" t="s">
         <v>49</v>
@@ -4250,10 +4250,10 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="K76" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
@@ -4285,7 +4285,7 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="K77" t="s">
         <v>125</v>
@@ -4320,7 +4320,7 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="K78" t="s">
         <v>179</v>
@@ -4425,7 +4425,7 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="K81" t="s">
         <v>138</v>
@@ -4460,7 +4460,7 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="K82" t="s">
         <v>175</v>
@@ -4495,7 +4495,7 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="K83" t="s">
         <v>170</v>
@@ -4565,7 +4565,7 @@
         <v>1</v>
       </c>
       <c r="J85" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="K85" t="s">
         <v>129</v>
@@ -4600,7 +4600,7 @@
         <v>1</v>
       </c>
       <c r="J86" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="K86" t="s">
         <v>178</v>

</xml_diff>

<commit_message>
Added component metric for germline risk rate
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{417A84A5-F8E8-4FB1-AF0F-0BFD0541899C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11A660C4-EFF6-41E2-B92C-92494E17E231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23148" yWindow="7404" windowWidth="23256" windowHeight="13896" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
   <sheets>
     <sheet name="Metrics" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metrics!$A$1:$K$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Metrics!$A$1:$K$87</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="531" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="242">
   <si>
     <t>nn_lower</t>
   </si>
@@ -750,6 +750,18 @@
   </si>
   <si>
     <t>MS.MET_COVERAGE</t>
+  </si>
+  <si>
+    <t>ms_germline_risk_rate</t>
+  </si>
+  <si>
+    <t>Rate of germline risk positions among callable bases (depth &gt;= min_depth)</t>
+  </si>
+  <si>
+    <t>MS.MET_GERM_RISK_RATE</t>
+  </si>
+  <si>
+    <t>germline_risk_rate.value</t>
   </si>
 </sst>
 </file>
@@ -1619,7 +1631,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}">
-  <dimension ref="A1:K86"/>
+  <dimension ref="A1:K87"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" customWidth="1"/>
@@ -2806,10 +2818,10 @@
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>51</v>
+        <v>238</v>
       </c>
       <c r="B35" t="s">
-        <v>4</v>
+        <v>239</v>
       </c>
       <c r="C35" t="s">
         <v>163</v>
@@ -2818,80 +2830,80 @@
         <v>21</v>
       </c>
       <c r="E35">
-        <v>70</v>
+        <v>2.5000000000000001E-3</v>
       </c>
       <c r="F35">
-        <v>90</v>
+        <v>5.4999999999999997E-3</v>
       </c>
       <c r="G35">
-        <v>70</v>
+        <v>3.5000000000000001E-3</v>
       </c>
       <c r="H35">
-        <v>80</v>
+        <v>4.4999999999999997E-3</v>
       </c>
       <c r="I35" t="b">
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>205</v>
+        <v>240</v>
       </c>
       <c r="K35" t="s">
-        <v>130</v>
+        <v>241</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>16</v>
+        <v>51</v>
       </c>
       <c r="B36" t="s">
-        <v>32</v>
+        <v>4</v>
       </c>
       <c r="C36" t="s">
-        <v>41</v>
+        <v>163</v>
       </c>
       <c r="D36" t="s">
         <v>21</v>
       </c>
       <c r="E36">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="F36">
-        <v>1000</v>
+        <v>90</v>
+      </c>
+      <c r="G36">
+        <v>70</v>
+      </c>
+      <c r="H36">
+        <v>80</v>
       </c>
       <c r="I36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>50</v>
+        <v>205</v>
       </c>
       <c r="K36" t="s">
-        <v>50</v>
+        <v>130</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="B37" t="s">
-        <v>159</v>
+        <v>32</v>
       </c>
       <c r="C37" t="s">
         <v>41</v>
       </c>
       <c r="D37" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E37">
-        <v>0</v>
+        <v>75</v>
       </c>
       <c r="F37">
-        <v>0.3</v>
-      </c>
-      <c r="G37">
-        <v>0</v>
-      </c>
-      <c r="H37">
-        <v>0.2</v>
+        <v>1000</v>
       </c>
       <c r="I37" t="b">
         <v>0</v>
@@ -2905,28 +2917,28 @@
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>187</v>
+        <v>23</v>
       </c>
       <c r="B38" t="s">
-        <v>189</v>
+        <v>159</v>
       </c>
       <c r="C38" t="s">
         <v>41</v>
       </c>
       <c r="D38" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E38">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="F38">
-        <v>100</v>
+        <v>0.3</v>
       </c>
       <c r="G38">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="H38">
-        <v>100</v>
+        <v>0.2</v>
       </c>
       <c r="I38" t="b">
         <v>0</v>
@@ -2940,10 +2952,10 @@
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B39" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="C39" t="s">
         <v>41</v>
@@ -2952,16 +2964,16 @@
         <v>21</v>
       </c>
       <c r="E39">
-        <v>110</v>
+        <v>85</v>
       </c>
       <c r="F39">
-        <v>150</v>
+        <v>100</v>
       </c>
       <c r="G39">
-        <v>120</v>
+        <v>95</v>
       </c>
       <c r="H39">
-        <v>140</v>
+        <v>100</v>
       </c>
       <c r="I39" t="b">
         <v>0</v>
@@ -2969,13 +2981,16 @@
       <c r="J39" t="s">
         <v>50</v>
       </c>
+      <c r="K39" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>33</v>
+        <v>188</v>
       </c>
       <c r="B40" t="s">
-        <v>34</v>
+        <v>193</v>
       </c>
       <c r="C40" t="s">
         <v>41</v>
@@ -2984,10 +2999,16 @@
         <v>21</v>
       </c>
       <c r="E40">
-        <v>4.3</v>
-      </c>
-      <c r="F40" t="s">
-        <v>5</v>
+        <v>110</v>
+      </c>
+      <c r="F40">
+        <v>150</v>
+      </c>
+      <c r="G40">
+        <v>120</v>
+      </c>
+      <c r="H40">
+        <v>140</v>
       </c>
       <c r="I40" t="b">
         <v>0</v>
@@ -3001,28 +3022,22 @@
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B41" t="s">
-        <v>159</v>
+        <v>34</v>
       </c>
       <c r="C41" t="s">
         <v>41</v>
       </c>
       <c r="D41" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E41">
-        <v>0</v>
-      </c>
-      <c r="F41">
-        <v>0.4</v>
-      </c>
-      <c r="G41">
-        <v>0</v>
-      </c>
-      <c r="H41">
-        <v>0.3</v>
+        <v>4.3</v>
+      </c>
+      <c r="F41" t="s">
+        <v>5</v>
       </c>
       <c r="I41" t="b">
         <v>0</v>
@@ -3036,28 +3051,28 @@
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>190</v>
+        <v>31</v>
       </c>
       <c r="B42" t="s">
-        <v>192</v>
+        <v>159</v>
       </c>
       <c r="C42" t="s">
         <v>41</v>
       </c>
       <c r="D42" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E42">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F42">
-        <v>100</v>
+        <v>0.4</v>
       </c>
       <c r="G42">
-        <v>90</v>
+        <v>0</v>
       </c>
       <c r="H42">
-        <v>100</v>
+        <v>0.3</v>
       </c>
       <c r="I42" t="b">
         <v>0</v>
@@ -3071,10 +3086,10 @@
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B43" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C43" t="s">
         <v>41</v>
@@ -3083,16 +3098,16 @@
         <v>21</v>
       </c>
       <c r="E43">
-        <v>440</v>
+        <v>50</v>
       </c>
       <c r="F43">
-        <v>740</v>
+        <v>100</v>
       </c>
       <c r="G43">
-        <v>530</v>
+        <v>90</v>
       </c>
       <c r="H43">
-        <v>650</v>
+        <v>100</v>
       </c>
       <c r="I43" t="b">
         <v>0</v>
@@ -3100,13 +3115,16 @@
       <c r="J43" t="s">
         <v>50</v>
       </c>
+      <c r="K43" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>17</v>
+        <v>191</v>
       </c>
       <c r="B44" t="s">
-        <v>14</v>
+        <v>194</v>
       </c>
       <c r="C44" t="s">
         <v>41</v>
@@ -3115,16 +3133,16 @@
         <v>21</v>
       </c>
       <c r="E44">
-        <v>544</v>
+        <v>440</v>
       </c>
       <c r="F44">
-        <v>624</v>
+        <v>740</v>
       </c>
       <c r="G44">
-        <v>564</v>
+        <v>530</v>
       </c>
       <c r="H44">
-        <v>604</v>
+        <v>650</v>
       </c>
       <c r="I44" t="b">
         <v>0</v>
@@ -3138,10 +3156,10 @@
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B45" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C45" t="s">
         <v>41</v>
@@ -3150,16 +3168,16 @@
         <v>21</v>
       </c>
       <c r="E45">
-        <v>94.9</v>
+        <v>544</v>
       </c>
       <c r="F45">
-        <v>100</v>
+        <v>624</v>
       </c>
       <c r="G45">
-        <v>100</v>
+        <v>564</v>
       </c>
       <c r="H45">
-        <v>100</v>
+        <v>604</v>
       </c>
       <c r="I45" t="b">
         <v>0</v>
@@ -3173,45 +3191,45 @@
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
+        <v>18</v>
+      </c>
+      <c r="B46" t="s">
+        <v>15</v>
+      </c>
+      <c r="C46" t="s">
+        <v>41</v>
+      </c>
+      <c r="D46" t="s">
+        <v>21</v>
+      </c>
+      <c r="E46">
+        <v>94.9</v>
+      </c>
+      <c r="F46">
+        <v>100</v>
+      </c>
+      <c r="G46">
+        <v>100</v>
+      </c>
+      <c r="H46">
+        <v>100</v>
+      </c>
+      <c r="I46" t="b">
+        <v>0</v>
+      </c>
+      <c r="J46" t="s">
+        <v>50</v>
+      </c>
+      <c r="K46" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
         <v>74</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B47" t="s">
         <v>153</v>
-      </c>
-      <c r="C46" t="s">
-        <v>44</v>
-      </c>
-      <c r="D46" t="s">
-        <v>53</v>
-      </c>
-      <c r="E46">
-        <v>35</v>
-      </c>
-      <c r="F46">
-        <v>40</v>
-      </c>
-      <c r="G46">
-        <v>39</v>
-      </c>
-      <c r="H46">
-        <v>40</v>
-      </c>
-      <c r="I46" t="b">
-        <v>1</v>
-      </c>
-      <c r="J46" t="s">
-        <v>221</v>
-      </c>
-      <c r="K46" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>75</v>
-      </c>
-      <c r="B47" t="s">
-        <v>154</v>
       </c>
       <c r="C47" t="s">
         <v>44</v>
@@ -3235,18 +3253,18 @@
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="K47" t="s">
         <v>113</v>
       </c>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B48" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C48" t="s">
         <v>44</v>
@@ -3255,30 +3273,30 @@
         <v>53</v>
       </c>
       <c r="E48">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="F48">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="G48">
-        <v>0</v>
+        <v>39</v>
       </c>
       <c r="H48">
-        <v>5</v>
+        <v>40</v>
       </c>
       <c r="I48" t="b">
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="K48" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B49" t="s">
         <v>152</v>
@@ -3305,7 +3323,7 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="K49" t="s">
         <v>115</v>
@@ -3313,10 +3331,10 @@
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="B50" t="s">
-        <v>72</v>
+        <v>152</v>
       </c>
       <c r="C50" t="s">
         <v>44</v>
@@ -3325,30 +3343,30 @@
         <v>53</v>
       </c>
       <c r="E50">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="F50">
-        <v>150</v>
+        <v>10</v>
       </c>
       <c r="G50">
-        <v>150</v>
+        <v>0</v>
       </c>
       <c r="H50">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="I50" t="b">
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="K50" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="B51" t="s">
         <v>72</v>
@@ -3375,7 +3393,7 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="K51" t="s">
         <v>116</v>
@@ -3383,10 +3401,10 @@
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B52" t="s">
-        <v>93</v>
+        <v>72</v>
       </c>
       <c r="C52" t="s">
         <v>44</v>
@@ -3395,30 +3413,30 @@
         <v>53</v>
       </c>
       <c r="E52">
-        <v>2850</v>
-      </c>
-      <c r="F52" t="s">
-        <v>5</v>
+        <v>150</v>
+      </c>
+      <c r="F52">
+        <v>150</v>
       </c>
       <c r="G52">
-        <v>3000</v>
-      </c>
-      <c r="H52" t="s">
-        <v>5</v>
+        <v>150</v>
+      </c>
+      <c r="H52">
+        <v>150</v>
       </c>
       <c r="I52" t="b">
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="K52" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B53" t="s">
         <v>93</v>
@@ -3445,7 +3463,7 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="K53" t="s">
         <v>112</v>
@@ -3453,42 +3471,42 @@
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>139</v>
+        <v>84</v>
       </c>
       <c r="B54" t="s">
-        <v>156</v>
+        <v>93</v>
       </c>
       <c r="C54" t="s">
         <v>44</v>
       </c>
       <c r="D54" t="s">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="E54">
-        <v>30</v>
-      </c>
-      <c r="F54">
-        <v>40</v>
+        <v>2850</v>
+      </c>
+      <c r="F54" t="s">
+        <v>5</v>
       </c>
       <c r="G54">
-        <v>35</v>
-      </c>
-      <c r="H54">
-        <v>40</v>
+        <v>3000</v>
+      </c>
+      <c r="H54" t="s">
+        <v>5</v>
       </c>
       <c r="I54" t="b">
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>206</v>
+        <v>222</v>
       </c>
       <c r="K54" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B55" t="s">
         <v>156</v>
@@ -3515,7 +3533,7 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K55" t="s">
         <v>114</v>
@@ -3523,10 +3541,10 @@
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>85</v>
+        <v>140</v>
       </c>
       <c r="B56" t="s">
-        <v>95</v>
+        <v>156</v>
       </c>
       <c r="C56" t="s">
         <v>44</v>
@@ -3535,30 +3553,30 @@
         <v>21</v>
       </c>
       <c r="E56">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="F56">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="G56">
-        <v>0</v>
+        <v>35</v>
       </c>
       <c r="H56">
-        <v>0.1</v>
+        <v>40</v>
       </c>
       <c r="I56" t="b">
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="K56" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B57" t="s">
         <v>95</v>
@@ -3585,7 +3603,7 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K57" t="s">
         <v>117</v>
@@ -3593,10 +3611,10 @@
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B58" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C58" t="s">
         <v>44</v>
@@ -3608,27 +3626,27 @@
         <v>0</v>
       </c>
       <c r="F58">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="G58">
         <v>0</v>
       </c>
       <c r="H58">
-        <v>20</v>
+        <v>0.1</v>
       </c>
       <c r="I58" t="b">
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="K58" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B59" t="s">
         <v>96</v>
@@ -3655,7 +3673,7 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K59" t="s">
         <v>118</v>
@@ -3663,10 +3681,10 @@
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B60" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C60" t="s">
         <v>44</v>
@@ -3678,27 +3696,27 @@
         <v>0</v>
       </c>
       <c r="F60">
+        <v>30</v>
+      </c>
+      <c r="G60">
+        <v>0</v>
+      </c>
+      <c r="H60">
         <v>20</v>
       </c>
-      <c r="G60">
-        <v>0</v>
-      </c>
-      <c r="H60">
-        <v>10</v>
-      </c>
       <c r="I60" t="b">
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="K60" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B61" t="s">
         <v>97</v>
@@ -3725,7 +3743,7 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K61" t="s">
         <v>119</v>
@@ -3733,10 +3751,10 @@
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B62" t="s">
-        <v>155</v>
+        <v>97</v>
       </c>
       <c r="C62" t="s">
         <v>44</v>
@@ -3748,27 +3766,27 @@
         <v>0</v>
       </c>
       <c r="F62">
+        <v>20</v>
+      </c>
+      <c r="G62">
+        <v>0</v>
+      </c>
+      <c r="H62">
         <v>10</v>
       </c>
-      <c r="G62">
-        <v>0</v>
-      </c>
-      <c r="H62">
-        <v>5</v>
-      </c>
       <c r="I62" t="b">
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="K62" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B63" t="s">
         <v>155</v>
@@ -3795,7 +3813,7 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="K63" t="s">
         <v>120</v>
@@ -3803,45 +3821,45 @@
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>52</v>
+        <v>92</v>
       </c>
       <c r="B64" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="C64" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D64" t="s">
-        <v>53</v>
+        <v>21</v>
       </c>
       <c r="E64">
         <v>0</v>
       </c>
       <c r="F64">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="G64">
         <v>0</v>
       </c>
       <c r="H64">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="I64" t="b">
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="K64" t="s">
-        <v>148</v>
+        <v>120</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>100</v>
+        <v>52</v>
       </c>
       <c r="B65" t="s">
-        <v>164</v>
+        <v>149</v>
       </c>
       <c r="C65" t="s">
         <v>46</v>
@@ -3853,13 +3871,13 @@
         <v>0</v>
       </c>
       <c r="F65">
-        <v>0.1</v>
+        <v>25</v>
       </c>
       <c r="G65">
         <v>0</v>
       </c>
       <c r="H65">
-        <v>0.05</v>
+        <v>10</v>
       </c>
       <c r="I65" t="b">
         <v>1</v>
@@ -3868,50 +3886,50 @@
         <v>208</v>
       </c>
       <c r="K65" t="s">
-        <v>122</v>
+        <v>148</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>135</v>
+        <v>100</v>
       </c>
       <c r="B66" t="s">
-        <v>136</v>
+        <v>164</v>
       </c>
       <c r="C66" t="s">
         <v>46</v>
       </c>
       <c r="D66" t="s">
-        <v>21</v>
+        <v>53</v>
       </c>
       <c r="E66">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F66">
-        <v>40</v>
+        <v>0.1</v>
       </c>
       <c r="G66">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H66">
-        <v>20</v>
+        <v>0.05</v>
       </c>
       <c r="I66" t="b">
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>223</v>
+        <v>208</v>
       </c>
       <c r="K66" t="s">
-        <v>224</v>
+        <v>122</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>150</v>
+        <v>135</v>
       </c>
       <c r="B67" t="s">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="C67" t="s">
         <v>46</v>
@@ -3920,16 +3938,16 @@
         <v>21</v>
       </c>
       <c r="E67">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F67">
+        <v>40</v>
+      </c>
+      <c r="G67">
+        <v>1</v>
+      </c>
+      <c r="H67">
         <v>20</v>
-      </c>
-      <c r="G67">
-        <v>0</v>
-      </c>
-      <c r="H67">
-        <v>10</v>
       </c>
       <c r="I67" t="b">
         <v>1</v>
@@ -3938,15 +3956,15 @@
         <v>223</v>
       </c>
       <c r="K67" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>165</v>
+        <v>150</v>
       </c>
       <c r="B68" t="s">
-        <v>166</v>
+        <v>143</v>
       </c>
       <c r="C68" t="s">
         <v>46</v>
@@ -3955,68 +3973,68 @@
         <v>21</v>
       </c>
       <c r="E68">
-        <v>70</v>
+        <v>0</v>
       </c>
       <c r="F68">
-        <v>99</v>
+        <v>20</v>
       </c>
       <c r="G68">
-        <v>85</v>
+        <v>0</v>
       </c>
       <c r="H68">
-        <v>99</v>
+        <v>10</v>
       </c>
       <c r="I68" t="b">
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>209</v>
+        <v>223</v>
       </c>
       <c r="K68" t="s">
-        <v>137</v>
+        <v>225</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>55</v>
+        <v>165</v>
       </c>
       <c r="B69" t="s">
-        <v>67</v>
+        <v>166</v>
       </c>
       <c r="C69" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D69" t="s">
         <v>21</v>
       </c>
       <c r="E69">
-        <v>90</v>
+        <v>70</v>
       </c>
       <c r="F69">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G69">
-        <v>95</v>
+        <v>85</v>
       </c>
       <c r="H69">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="I69" t="b">
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="K69" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>230</v>
+        <v>55</v>
       </c>
       <c r="B70" t="s">
-        <v>233</v>
+        <v>67</v>
       </c>
       <c r="C70" t="s">
         <v>43</v>
@@ -4025,33 +4043,33 @@
         <v>21</v>
       </c>
       <c r="E70">
-        <v>0</v>
+        <v>90</v>
       </c>
       <c r="F70">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="G70">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="H70">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="I70" t="b">
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>231</v>
+        <v>210</v>
       </c>
       <c r="K70" t="s">
-        <v>229</v>
+        <v>126</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>54</v>
+        <v>230</v>
       </c>
       <c r="B71" t="s">
-        <v>68</v>
+        <v>233</v>
       </c>
       <c r="C71" t="s">
         <v>43</v>
@@ -4060,33 +4078,33 @@
         <v>21</v>
       </c>
       <c r="E71">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="F71">
-        <v>100</v>
+        <v>10</v>
       </c>
       <c r="G71">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="H71">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="I71" t="b">
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="K71" t="s">
-        <v>128</v>
+        <v>229</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="B72" t="s">
-        <v>101</v>
+        <v>68</v>
       </c>
       <c r="C72" t="s">
         <v>43</v>
@@ -4095,68 +4113,68 @@
         <v>21</v>
       </c>
       <c r="E72">
-        <v>120</v>
+        <v>50</v>
       </c>
       <c r="F72">
-        <v>180</v>
+        <v>100</v>
       </c>
       <c r="G72">
-        <v>140</v>
+        <v>75</v>
       </c>
       <c r="H72">
-        <v>160</v>
+        <v>100</v>
       </c>
       <c r="I72" t="b">
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="K72" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>109</v>
+        <v>56</v>
       </c>
       <c r="B73" t="s">
-        <v>144</v>
+        <v>101</v>
       </c>
       <c r="C73" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="D73" t="s">
         <v>21</v>
       </c>
       <c r="E73">
-        <v>50</v>
+        <v>120</v>
       </c>
       <c r="F73">
-        <v>70</v>
+        <v>180</v>
       </c>
       <c r="G73">
-        <v>50</v>
+        <v>140</v>
       </c>
       <c r="H73">
-        <v>60</v>
+        <v>160</v>
       </c>
       <c r="I73" t="b">
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="K73" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>171</v>
+        <v>109</v>
       </c>
       <c r="B74" t="s">
-        <v>132</v>
+        <v>144</v>
       </c>
       <c r="C74" t="s">
         <v>49</v>
@@ -4165,33 +4183,33 @@
         <v>21</v>
       </c>
       <c r="E74">
-        <v>58.3</v>
+        <v>50</v>
       </c>
       <c r="F74">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="G74">
-        <v>90</v>
+        <v>50</v>
       </c>
       <c r="H74">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="I74" t="b">
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="K74" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>107</v>
+        <v>171</v>
       </c>
       <c r="B75" t="s">
-        <v>10</v>
+        <v>132</v>
       </c>
       <c r="C75" t="s">
         <v>49</v>
@@ -4200,13 +4218,13 @@
         <v>21</v>
       </c>
       <c r="E75">
-        <v>99</v>
+        <v>58.3</v>
       </c>
       <c r="F75">
         <v>100</v>
       </c>
       <c r="G75">
-        <v>99.5</v>
+        <v>90</v>
       </c>
       <c r="H75">
         <v>100</v>
@@ -4215,18 +4233,18 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="K75" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>232</v>
+        <v>107</v>
       </c>
       <c r="B76" t="s">
-        <v>234</v>
+        <v>10</v>
       </c>
       <c r="C76" t="s">
         <v>49</v>
@@ -4235,33 +4253,33 @@
         <v>21</v>
       </c>
       <c r="E76">
-        <v>0</v>
+        <v>99</v>
       </c>
       <c r="F76">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="G76">
-        <v>0</v>
+        <v>99.5</v>
       </c>
       <c r="H76">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="I76" t="b">
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>235</v>
+        <v>214</v>
       </c>
       <c r="K76" t="s">
-        <v>229</v>
+        <v>124</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>106</v>
+        <v>232</v>
       </c>
       <c r="B77" t="s">
-        <v>105</v>
+        <v>234</v>
       </c>
       <c r="C77" t="s">
         <v>49</v>
@@ -4273,7 +4291,7 @@
         <v>0</v>
       </c>
       <c r="F77">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="G77">
         <v>0</v>
@@ -4285,18 +4303,18 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>214</v>
+        <v>235</v>
       </c>
       <c r="K77" t="s">
-        <v>125</v>
+        <v>229</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>180</v>
+        <v>106</v>
       </c>
       <c r="B78" t="s">
-        <v>184</v>
+        <v>105</v>
       </c>
       <c r="C78" t="s">
         <v>49</v>
@@ -4305,33 +4323,33 @@
         <v>21</v>
       </c>
       <c r="E78">
-        <v>1</v>
-      </c>
-      <c r="F78" t="s">
+        <v>0</v>
+      </c>
+      <c r="F78">
+        <v>15</v>
+      </c>
+      <c r="G78">
+        <v>0</v>
+      </c>
+      <c r="H78">
         <v>5</v>
       </c>
-      <c r="G78">
-        <v>1</v>
-      </c>
-      <c r="H78" t="s">
-        <v>5</v>
-      </c>
       <c r="I78" t="b">
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
       <c r="K78" t="s">
-        <v>179</v>
+        <v>125</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>12</v>
+        <v>180</v>
       </c>
       <c r="B79" t="s">
-        <v>13</v>
+        <v>184</v>
       </c>
       <c r="C79" t="s">
         <v>49</v>
@@ -4340,33 +4358,33 @@
         <v>21</v>
       </c>
       <c r="E79">
-        <v>0</v>
-      </c>
-      <c r="F79">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="F79" t="s">
+        <v>5</v>
       </c>
       <c r="G79">
-        <v>0</v>
-      </c>
-      <c r="H79">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="H79" t="s">
+        <v>5</v>
       </c>
       <c r="I79" t="b">
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>196</v>
+        <v>220</v>
       </c>
       <c r="K79" t="s">
-        <v>121</v>
+        <v>179</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>185</v>
+        <v>12</v>
       </c>
       <c r="B80" t="s">
-        <v>181</v>
+        <v>13</v>
       </c>
       <c r="C80" t="s">
         <v>49</v>
@@ -4375,33 +4393,33 @@
         <v>21</v>
       </c>
       <c r="E80">
-        <v>14.5</v>
+        <v>0</v>
       </c>
       <c r="F80">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="G80">
-        <v>26.1</v>
+        <v>0</v>
       </c>
       <c r="H80">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="I80" t="b">
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="K80" t="s">
-        <v>183</v>
+        <v>121</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>8</v>
+        <v>185</v>
       </c>
       <c r="B81" t="s">
-        <v>9</v>
+        <v>181</v>
       </c>
       <c r="C81" t="s">
         <v>49</v>
@@ -4410,33 +4428,33 @@
         <v>21</v>
       </c>
       <c r="E81">
-        <v>0</v>
+        <v>14.5</v>
       </c>
       <c r="F81">
-        <v>1.2E-2</v>
+        <v>100</v>
       </c>
       <c r="G81">
-        <v>2.0000000000000001E-4</v>
+        <v>26.1</v>
       </c>
       <c r="H81">
-        <v>6.0000000000000001E-3</v>
+        <v>100</v>
       </c>
       <c r="I81" t="b">
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>215</v>
+        <v>197</v>
       </c>
       <c r="K81" t="s">
-        <v>138</v>
+        <v>183</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>173</v>
+        <v>8</v>
       </c>
       <c r="B82" t="s">
-        <v>174</v>
+        <v>9</v>
       </c>
       <c r="C82" t="s">
         <v>49</v>
@@ -4445,68 +4463,68 @@
         <v>21</v>
       </c>
       <c r="E82">
-        <v>69</v>
+        <v>0</v>
       </c>
       <c r="F82">
-        <v>120</v>
+        <v>1.2E-2</v>
       </c>
       <c r="G82">
-        <v>82.8</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="H82">
-        <v>120</v>
+        <v>6.0000000000000001E-3</v>
       </c>
       <c r="I82" t="b">
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="K82" t="s">
-        <v>175</v>
+        <v>138</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="B83" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="C83" t="s">
-        <v>134</v>
+        <v>49</v>
       </c>
       <c r="D83" t="s">
         <v>21</v>
       </c>
       <c r="E83">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="F83">
-        <v>5.6599999999999999E-4</v>
+        <v>120</v>
       </c>
       <c r="G83">
-        <v>2.0000000000000001E-4</v>
+        <v>82.8</v>
       </c>
       <c r="H83">
-        <v>3.2679999999999997E-4</v>
+        <v>120</v>
       </c>
       <c r="I83" t="b">
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="K83" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>11</v>
+        <v>168</v>
       </c>
       <c r="B84" t="s">
-        <v>182</v>
+        <v>169</v>
       </c>
       <c r="C84" t="s">
         <v>134</v>
@@ -4515,33 +4533,33 @@
         <v>21</v>
       </c>
       <c r="E84">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F84">
-        <v>100</v>
+        <v>5.6599999999999999E-4</v>
       </c>
       <c r="G84">
-        <v>20</v>
+        <v>2.0000000000000001E-4</v>
       </c>
       <c r="H84">
-        <v>100</v>
+        <v>3.2679999999999997E-4</v>
       </c>
       <c r="I84" t="b">
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>197</v>
+        <v>217</v>
       </c>
       <c r="K84" t="s">
-        <v>176</v>
+        <v>170</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>172</v>
+        <v>11</v>
       </c>
       <c r="B85" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="C85" t="s">
         <v>134</v>
@@ -4550,33 +4568,33 @@
         <v>21</v>
       </c>
       <c r="E85">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="F85">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="G85">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="H85">
-        <v>80</v>
+        <v>100</v>
       </c>
       <c r="I85" t="b">
         <v>1</v>
       </c>
       <c r="J85" t="s">
-        <v>218</v>
+        <v>197</v>
       </c>
       <c r="K85" t="s">
-        <v>129</v>
+        <v>176</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>39</v>
+        <v>172</v>
       </c>
       <c r="B86" t="s">
-        <v>177</v>
+        <v>186</v>
       </c>
       <c r="C86" t="s">
         <v>134</v>
@@ -4585,29 +4603,64 @@
         <v>21</v>
       </c>
       <c r="E86">
+        <v>0</v>
+      </c>
+      <c r="F86">
+        <v>95</v>
+      </c>
+      <c r="G86">
+        <v>0</v>
+      </c>
+      <c r="H86">
+        <v>80</v>
+      </c>
+      <c r="I86" t="b">
+        <v>1</v>
+      </c>
+      <c r="J86" t="s">
+        <v>218</v>
+      </c>
+      <c r="K86" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>39</v>
+      </c>
+      <c r="B87" t="s">
+        <v>177</v>
+      </c>
+      <c r="C87" t="s">
+        <v>134</v>
+      </c>
+      <c r="D87" t="s">
+        <v>21</v>
+      </c>
+      <c r="E87">
         <v>33</v>
       </c>
-      <c r="F86">
+      <c r="F87">
         <v>100</v>
       </c>
-      <c r="G86">
+      <c r="G87">
         <v>67</v>
       </c>
-      <c r="H86">
+      <c r="H87">
         <v>100</v>
       </c>
-      <c r="I86" t="b">
-        <v>1</v>
-      </c>
-      <c r="J86" t="s">
+      <c r="I87" t="b">
+        <v>1</v>
+      </c>
+      <c r="J87" t="s">
         <v>219</v>
       </c>
-      <c r="K86" t="s">
+      <c r="K87" t="s">
         <v>178</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K86" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
+  <autoFilter ref="A1:K87" xr:uid="{1962EE11-078F-475B-B93E-E7A708AD4D14}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Changed nn lower threshold for ex_unique_reads_initial_alignment from 58.3 to 50
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{11A660C4-EFF6-41E2-B92C-92494E17E231}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D75D5834-BA2D-4142-B00D-413FF420AB3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -4218,7 +4218,7 @@
         <v>21</v>
       </c>
       <c r="E75">
-        <v>58.3</v>
+        <v>50</v>
       </c>
       <c r="F75">
         <v>100</v>

</xml_diff>

<commit_message>
Updated formatting of docs
</commit_message>
<xml_diff>
--- a/config/component_level_metrics.xlsx
+++ b/config/component_level_metrics.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\wsl$\Ubuntu\home\joshj\SomaticCODEC\config\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D75D5834-BA2D-4142-B00D-413FF420AB3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E84F1C7-829C-4635-8F84-514149D87B86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{B4BEDC58-0418-40BE-BDF6-0FEFABA94EA8}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="241">
   <si>
     <t>nn_lower</t>
   </si>
@@ -68,9 +68,6 @@
     <t>Rate at which Watson and Crick complementary bases disagree (total R1R2 disagreements divided by total duplex bases for each sample)</t>
   </si>
   <si>
-    <t>Percentage of reads which successfully aligned during DSC realignment</t>
-  </si>
-  <si>
     <t>ex_variant_call_eligible</t>
   </si>
   <si>
@@ -80,12 +77,6 @@
     <t>Number of soft clipped bases for 90th percentile most softclipped reads</t>
   </si>
   <si>
-    <t>Mean length of the largest peak</t>
-  </si>
-  <si>
-    <t>Integrated area of the largest peak</t>
-  </si>
-  <si>
     <t>ex_fragmented_DNA_yield</t>
   </si>
   <si>
@@ -245,9 +236,6 @@
     <t>Percentage of reads properly paired, post initial alignment</t>
   </si>
   <si>
-    <t>Median insert size (start of R1 to end of R2) as determined during alignment (bp)</t>
-  </si>
-  <si>
     <t>ms_raw_read_length_r1</t>
   </si>
   <si>
@@ -317,12 +305,6 @@
     <t>ex_filtered_per_base_N_content_r2</t>
   </si>
   <si>
-    <t>Total raw reads obtained from standard Illumina sequencing by AGRF (x million reads, 3B lane)</t>
-  </si>
-  <si>
-    <t>Total raw reads obtained from standard Illumina sequencing by AGRF (x million reads, 4 samples in 1B lane)</t>
-  </si>
-  <si>
     <t>Percentage of total filtered sequences made up by any one identical sequence</t>
   </si>
   <si>
@@ -335,9 +317,6 @@
     <t>Percentage of filtered sequences made up by any one identical sequence</t>
   </si>
   <si>
-    <t>Percentage of reads successfully mapped to the reference genome, post alignment</t>
-  </si>
-  <si>
     <t>ex_lane_demux_read_gini</t>
   </si>
   <si>
@@ -353,9 +332,6 @@
     <t>ms_mapped_alignment</t>
   </si>
   <si>
-    <t>Percentage of reads lost to MAPQ filter</t>
-  </si>
-  <si>
     <t>ex_reads_filtered_MAPQ</t>
   </si>
   <si>
@@ -437,9 +413,6 @@
     <t>Percentage of reads that are unique following initial alignment</t>
   </si>
   <si>
-    <t>Percentage of fragments that fall within the expected size range on gel elextrophoresis (10,000-50,000 bp)</t>
-  </si>
-  <si>
     <t>EX call somatic variants</t>
   </si>
   <si>
@@ -467,21 +440,6 @@
     <t>ms_filtered_per_base_quality_r2</t>
   </si>
   <si>
-    <t>Reads with a length of zero after trimming (e.g. blank ligation)</t>
-  </si>
-  <si>
-    <t>Percentage of reads lost from creation of DSC</t>
-  </si>
-  <si>
-    <t>Quantity of DNA (ng) after adaptor ligation (ng/uL concentration x ul sample remaining after Qubit)</t>
-  </si>
-  <si>
-    <t>Quantity of DNA (ng) after enzymatic fragmentation (ng/uL concentration x ul sample remaining after Qubit)</t>
-  </si>
-  <si>
-    <t>Quantity of DNA (ng) required to run assay &amp; QCs (ng/uL concentration x ul sample remaining after Qubit)</t>
-  </si>
-  <si>
     <t>pct_reads_lost_demux</t>
   </si>
   <si>
@@ -506,9 +464,6 @@
     <t>Maximum percentage of bases recorded as N at any one position in filtered reads</t>
   </si>
   <si>
-    <t>Minimum IQR lower quartile for base quality at any position in reads (Phred score)</t>
-  </si>
-  <si>
     <t>ms_coverage_at_depth_threshold</t>
   </si>
   <si>
@@ -524,15 +479,9 @@
     <t>pct_coverage_min_depth</t>
   </si>
   <si>
-    <t>Percentage of genome with depth &gt;= minimum MS depth value defined in config</t>
-  </si>
-  <si>
     <t>MS mask regions</t>
   </si>
   <si>
-    <t>Gini coefficient for inequality between ex_samples</t>
-  </si>
-  <si>
     <t>ex_reads_filtered_length_quality</t>
   </si>
   <si>
@@ -569,9 +518,6 @@
     <t>ex_dsc_high_qual_unmasked_pct.value</t>
   </si>
   <si>
-    <t>Percentage of all sequenced bases with 1. MS depth &gt; MS depth theshold and 2. EX duplex depth &gt; 0</t>
-  </si>
-  <si>
     <t>ms_depth_vs_ex_depth.pct_overlap</t>
   </si>
   <si>
@@ -581,18 +527,9 @@
     <t>ex_median_duplex_depth</t>
   </si>
   <si>
-    <t>Percentage of genome with duplex depth &gt; 0 and QUAL &gt; min_base_quality</t>
-  </si>
-  <si>
-    <t>Percentage of genome eligible for variant calling (duplex depth &gt; 0, QUAL &gt; min_base_quality, unmasked)</t>
-  </si>
-  <si>
     <t>ex_dsc_high_qual_pct.value</t>
   </si>
   <si>
-    <t>Median duplex depth for positions that are eligible for variant calling</t>
-  </si>
-  <si>
     <t>ex_high_qual_coverage</t>
   </si>
   <si>
@@ -719,9 +656,6 @@
     <t>ms_multimapped_alignment</t>
   </si>
   <si>
-    <t>Percentage of reads that mapped to more than one position after alignment</t>
-  </si>
-  <si>
     <t>MS.MET_MULTIMAPPING</t>
   </si>
   <si>
@@ -755,13 +689,76 @@
     <t>ms_germline_risk_rate</t>
   </si>
   <si>
-    <t>Rate of germline risk positions among callable bases (depth &gt;= min_depth)</t>
-  </si>
-  <si>
     <t>MS.MET_GERM_RISK_RATE</t>
   </si>
   <si>
     <t>germline_risk_rate.value</t>
+  </si>
+  <si>
+    <t>Percentage of fragments that fall within the expected size range on gel elextrophoresis (&gt;=10,000 bp)</t>
+  </si>
+  <si>
+    <t>Quantity of DNA (ng) required to run assay &amp; QC (ng/uL concentration x uL sample)</t>
+  </si>
+  <si>
+    <t>Quantity of DNA (ng) after enzymatic fragmentation (ng/uL concentration x uL sample)</t>
+  </si>
+  <si>
+    <t>Quantity of DNA (ng) after adaptor ligation (ng/uL concentration x uL sample)</t>
+  </si>
+  <si>
+    <t>Total raw reads obtained from standard Illumina sequencing (6 samples in 3B lane of NovaSeqX)</t>
+  </si>
+  <si>
+    <t>Minimum of IQR lower quartiles for base quality at any position in reads (Phred score)</t>
+  </si>
+  <si>
+    <t>Percentage of reads retained after length and quality filtering</t>
+  </si>
+  <si>
+    <t>Percentage of reads successfully mapped to the reference genome</t>
+  </si>
+  <si>
+    <t>Percentage of reads that mapped to more than one position</t>
+  </si>
+  <si>
+    <t>Percentage of genome with depth &gt;= min_depth value defined in config</t>
+  </si>
+  <si>
+    <t>Median insert size (start of R1 to end of R2) as determined by alignment (bp)</t>
+  </si>
+  <si>
+    <t>Rate of germline risk positions among callable bases</t>
+  </si>
+  <si>
+    <t>Total raw reads obtained from standard Illumina sequencing (1x 3B lane of NovaSeqX)</t>
+  </si>
+  <si>
+    <t>Gini coefficient for inequality in the number of reads demuxed to each ex_sample</t>
+  </si>
+  <si>
+    <t>Reads with a length of zero after trimming (e.g. blank ligations)</t>
+  </si>
+  <si>
+    <t>Percentage of reads lost during duplex consensus calling</t>
+  </si>
+  <si>
+    <t>Percentage of reads successfully mapped to reference genome, post realignment of DSC reads</t>
+  </si>
+  <si>
+    <t>Percentage of reads lost to MAPQ filter, post realignment of DSC reads</t>
+  </si>
+  <si>
+    <t>Median duplex depth of positions that are eligible for variant calling</t>
+  </si>
+  <si>
+    <t>Percentage of genome with duplex depth &gt; 0 and QUAL &gt;= min_base_quality</t>
+  </si>
+  <si>
+    <t>Percentage of genome eligible for variant calling (duplex depth &gt; 0, QUAL &gt;= min_base_quality, unmasked)</t>
+  </si>
+  <si>
+    <t>Percentage of all sequenced bases with MS depth &gt;= min_depth threshold AND EX duplex depth &gt; 0</t>
   </si>
 </sst>
 </file>
@@ -1245,8 +1242,9 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1646,16 +1644,16 @@
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="B1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D1" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E1" t="s">
         <v>0</v>
@@ -1670,27 +1668,27 @@
         <v>3</v>
       </c>
       <c r="I1" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="J1" t="s">
-        <v>110</v>
+        <v>102</v>
       </c>
       <c r="K1" t="s">
-        <v>111</v>
+        <v>103</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>147</v>
+        <v>220</v>
       </c>
       <c r="C2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D2" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E2">
         <v>2500</v>
@@ -1702,24 +1700,24 @@
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K2" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="B3" t="s">
-        <v>158</v>
+        <v>143</v>
       </c>
       <c r="C3" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -1737,24 +1735,24 @@
         <v>0</v>
       </c>
       <c r="J3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K3" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>195</v>
+        <v>174</v>
       </c>
       <c r="B4" t="s">
-        <v>133</v>
+        <v>219</v>
       </c>
       <c r="C4" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D4" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E4">
         <v>85</v>
@@ -1772,24 +1770,24 @@
         <v>0</v>
       </c>
       <c r="J4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K4" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>146</v>
+        <v>221</v>
       </c>
       <c r="C5" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D5" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E5">
         <v>86.2</v>
@@ -1801,24 +1799,24 @@
         <v>0</v>
       </c>
       <c r="J5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K5" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="B6" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="C6" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D6" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -1836,24 +1834,24 @@
         <v>0</v>
       </c>
       <c r="J6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K6" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>145</v>
+        <v>222</v>
       </c>
       <c r="C7" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D7" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E7">
         <v>45</v>
@@ -1865,24 +1863,24 @@
         <v>0</v>
       </c>
       <c r="J7" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K7" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
       <c r="C8" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D8" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -1900,24 +1898,24 @@
         <v>0</v>
       </c>
       <c r="J8" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K8" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C9" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D9" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E9">
         <v>280</v>
@@ -1935,24 +1933,24 @@
         <v>0</v>
       </c>
       <c r="J9" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K9" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="C10" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D10" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E10">
         <v>87.9</v>
@@ -1970,10 +1968,10 @@
         <v>0</v>
       </c>
       <c r="J10" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K10" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.25">
@@ -1981,22 +1979,22 @@
         <v>6</v>
       </c>
       <c r="B11" t="s">
-        <v>94</v>
+        <v>223</v>
       </c>
       <c r="C11" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D11" t="s">
-        <v>21</v>
-      </c>
-      <c r="E11">
-        <v>200</v>
+        <v>18</v>
+      </c>
+      <c r="E11" s="1">
+        <v>400000000</v>
       </c>
       <c r="F11" t="s">
         <v>5</v>
       </c>
-      <c r="G11">
-        <v>300</v>
+      <c r="G11" s="1">
+        <v>500000000</v>
       </c>
       <c r="H11" t="s">
         <v>5</v>
@@ -2005,10 +2003,10 @@
         <v>1</v>
       </c>
       <c r="J11" t="s">
-        <v>198</v>
+        <v>177</v>
       </c>
       <c r="K11" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -2016,22 +2014,22 @@
         <v>7</v>
       </c>
       <c r="B12" t="s">
-        <v>94</v>
+        <v>223</v>
       </c>
       <c r="C12" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D12" t="s">
-        <v>21</v>
-      </c>
-      <c r="E12">
-        <v>200</v>
+        <v>18</v>
+      </c>
+      <c r="E12" s="1">
+        <v>400000000</v>
       </c>
       <c r="F12" t="s">
         <v>5</v>
       </c>
-      <c r="G12">
-        <v>300</v>
+      <c r="G12" s="1">
+        <v>500000000</v>
       </c>
       <c r="H12" t="s">
         <v>5</v>
@@ -2040,24 +2038,24 @@
         <v>1</v>
       </c>
       <c r="J12" t="s">
-        <v>199</v>
+        <v>178</v>
       </c>
       <c r="K12" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="B13" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="C13" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D13" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E13">
         <v>35</v>
@@ -2075,24 +2073,24 @@
         <v>1</v>
       </c>
       <c r="J13" t="s">
-        <v>198</v>
+        <v>177</v>
       </c>
       <c r="K13" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="B14" t="s">
-        <v>154</v>
+        <v>140</v>
       </c>
       <c r="C14" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D14" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E14">
         <v>35</v>
@@ -2110,24 +2108,24 @@
         <v>1</v>
       </c>
       <c r="J14" t="s">
-        <v>199</v>
+        <v>178</v>
       </c>
       <c r="K14" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="B15" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="C15" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D15" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -2145,24 +2143,24 @@
         <v>1</v>
       </c>
       <c r="J15" t="s">
-        <v>198</v>
+        <v>177</v>
       </c>
       <c r="K15" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="B16" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="C16" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D16" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -2180,24 +2178,24 @@
         <v>1</v>
       </c>
       <c r="J16" t="s">
-        <v>199</v>
+        <v>178</v>
       </c>
       <c r="K16" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="B17" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C17" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D17" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E17">
         <v>150</v>
@@ -2215,24 +2213,24 @@
         <v>1</v>
       </c>
       <c r="J17" t="s">
-        <v>198</v>
+        <v>177</v>
       </c>
       <c r="K17" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>71</v>
+        <v>67</v>
       </c>
       <c r="B18" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C18" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D18" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E18">
         <v>150</v>
@@ -2250,24 +2248,24 @@
         <v>1</v>
       </c>
       <c r="J18" t="s">
-        <v>199</v>
+        <v>178</v>
       </c>
       <c r="K18" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="B19" t="s">
-        <v>156</v>
+        <v>224</v>
       </c>
       <c r="C19" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D19" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E19">
         <v>30</v>
@@ -2285,24 +2283,24 @@
         <v>1</v>
       </c>
       <c r="J19" t="s">
-        <v>200</v>
+        <v>179</v>
       </c>
       <c r="K19" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="B20" t="s">
-        <v>156</v>
+        <v>224</v>
       </c>
       <c r="C20" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D20" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E20">
         <v>30</v>
@@ -2320,24 +2318,24 @@
         <v>1</v>
       </c>
       <c r="J20" t="s">
-        <v>201</v>
+        <v>180</v>
       </c>
       <c r="K20" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="B21" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="C21" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D21" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -2355,24 +2353,24 @@
         <v>1</v>
       </c>
       <c r="J21" t="s">
-        <v>200</v>
+        <v>179</v>
       </c>
       <c r="K21" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="B22" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
       <c r="C22" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D22" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -2390,24 +2388,24 @@
         <v>1</v>
       </c>
       <c r="J22" t="s">
-        <v>201</v>
+        <v>180</v>
       </c>
       <c r="K22" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="B23" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C23" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D23" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -2425,24 +2423,24 @@
         <v>1</v>
       </c>
       <c r="J23" t="s">
-        <v>200</v>
+        <v>179</v>
       </c>
       <c r="K23" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="B24" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C24" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D24" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -2460,24 +2458,24 @@
         <v>1</v>
       </c>
       <c r="J24" t="s">
-        <v>201</v>
+        <v>180</v>
       </c>
       <c r="K24" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="B25" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="C25" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D25" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -2495,24 +2493,24 @@
         <v>1</v>
       </c>
       <c r="J25" t="s">
-        <v>200</v>
+        <v>179</v>
       </c>
       <c r="K25" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="B26" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="C26" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D26" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E26">
         <v>0</v>
@@ -2530,24 +2528,24 @@
         <v>1</v>
       </c>
       <c r="J26" t="s">
-        <v>201</v>
+        <v>180</v>
       </c>
       <c r="K26" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B27" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="C27" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D27" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -2565,24 +2563,24 @@
         <v>1</v>
       </c>
       <c r="J27" t="s">
-        <v>200</v>
+        <v>179</v>
       </c>
       <c r="K27" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="B28" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="C28" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D28" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -2600,24 +2598,24 @@
         <v>1</v>
       </c>
       <c r="J28" t="s">
-        <v>201</v>
+        <v>180</v>
       </c>
       <c r="K28" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>167</v>
+        <v>150</v>
       </c>
       <c r="B29" t="s">
-        <v>166</v>
+        <v>225</v>
       </c>
       <c r="C29" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="D29" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E29">
         <v>70</v>
@@ -2635,24 +2633,24 @@
         <v>1</v>
       </c>
       <c r="J29" t="s">
-        <v>202</v>
+        <v>181</v>
       </c>
       <c r="K29" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="B30" t="s">
-        <v>99</v>
+        <v>226</v>
       </c>
       <c r="C30" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D30" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E30">
         <v>90</v>
@@ -2670,24 +2668,24 @@
         <v>1</v>
       </c>
       <c r="J30" t="s">
-        <v>203</v>
+        <v>182</v>
       </c>
       <c r="K30" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>226</v>
+        <v>205</v>
       </c>
       <c r="B31" t="s">
         <v>227</v>
       </c>
       <c r="C31" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D31" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -2705,24 +2703,24 @@
         <v>1</v>
       </c>
       <c r="J31" t="s">
-        <v>228</v>
+        <v>206</v>
       </c>
       <c r="K31" t="s">
-        <v>229</v>
+        <v>207</v>
       </c>
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="B32" t="s">
-        <v>108</v>
+        <v>100</v>
       </c>
       <c r="C32" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D32" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E32">
         <v>0</v>
@@ -2740,24 +2738,24 @@
         <v>1</v>
       </c>
       <c r="J32" t="s">
-        <v>236</v>
+        <v>214</v>
       </c>
       <c r="K32" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>157</v>
+        <v>142</v>
       </c>
       <c r="B33" t="s">
-        <v>162</v>
+        <v>228</v>
       </c>
       <c r="C33" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D33" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E33">
         <v>21.75</v>
@@ -2775,24 +2773,24 @@
         <v>1</v>
       </c>
       <c r="J33" t="s">
-        <v>237</v>
+        <v>215</v>
       </c>
       <c r="K33" t="s">
-        <v>161</v>
+        <v>146</v>
       </c>
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>102</v>
+        <v>95</v>
       </c>
       <c r="B34" t="s">
-        <v>69</v>
+        <v>229</v>
       </c>
       <c r="C34" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D34" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E34">
         <v>125</v>
@@ -2810,24 +2808,24 @@
         <v>1</v>
       </c>
       <c r="J34" t="s">
-        <v>204</v>
+        <v>183</v>
       </c>
       <c r="K34" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>238</v>
+        <v>216</v>
       </c>
       <c r="B35" t="s">
-        <v>239</v>
+        <v>230</v>
       </c>
       <c r="C35" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
       <c r="D35" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E35">
         <v>2.5000000000000001E-3</v>
@@ -2845,24 +2843,24 @@
         <v>1</v>
       </c>
       <c r="J35" t="s">
-        <v>240</v>
+        <v>217</v>
       </c>
       <c r="K35" t="s">
-        <v>241</v>
+        <v>218</v>
       </c>
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B36" t="s">
         <v>4</v>
       </c>
       <c r="C36" t="s">
-        <v>163</v>
+        <v>147</v>
       </c>
       <c r="D36" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E36">
         <v>70</v>
@@ -2880,24 +2878,24 @@
         <v>1</v>
       </c>
       <c r="J36" t="s">
-        <v>205</v>
+        <v>184</v>
       </c>
       <c r="K36" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B37" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C37" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D37" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E37">
         <v>75</v>
@@ -2909,24 +2907,24 @@
         <v>0</v>
       </c>
       <c r="J37" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K37" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="38" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B38" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="C38" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D38" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E38">
         <v>0</v>
@@ -2944,24 +2942,24 @@
         <v>0</v>
       </c>
       <c r="J38" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K38" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="39" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>187</v>
+        <v>166</v>
       </c>
       <c r="B39" t="s">
-        <v>189</v>
+        <v>168</v>
       </c>
       <c r="C39" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D39" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E39">
         <v>85</v>
@@ -2979,24 +2977,24 @@
         <v>0</v>
       </c>
       <c r="J39" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K39" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="40" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>188</v>
+        <v>167</v>
       </c>
       <c r="B40" t="s">
-        <v>193</v>
+        <v>172</v>
       </c>
       <c r="C40" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D40" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E40">
         <v>110</v>
@@ -3014,24 +3012,24 @@
         <v>0</v>
       </c>
       <c r="J40" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K40" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="41" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="B41" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="C41" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D41" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E41">
         <v>4.3</v>
@@ -3043,24 +3041,24 @@
         <v>0</v>
       </c>
       <c r="J41" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K41" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="42" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="B42" t="s">
-        <v>159</v>
+        <v>144</v>
       </c>
       <c r="C42" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D42" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E42">
         <v>0</v>
@@ -3078,24 +3076,24 @@
         <v>0</v>
       </c>
       <c r="J42" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K42" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="43" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>190</v>
+        <v>169</v>
       </c>
       <c r="B43" t="s">
-        <v>192</v>
+        <v>171</v>
       </c>
       <c r="C43" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D43" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E43">
         <v>50</v>
@@ -3113,24 +3111,24 @@
         <v>0</v>
       </c>
       <c r="J43" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K43" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="44" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>191</v>
+        <v>170</v>
       </c>
       <c r="B44" t="s">
-        <v>194</v>
+        <v>173</v>
       </c>
       <c r="C44" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D44" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E44">
         <v>440</v>
@@ -3148,24 +3146,24 @@
         <v>0</v>
       </c>
       <c r="J44" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K44" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="45" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="B45" t="s">
-        <v>14</v>
+        <v>54</v>
       </c>
       <c r="C45" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D45" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E45">
         <v>544</v>
@@ -3183,24 +3181,24 @@
         <v>0</v>
       </c>
       <c r="J45" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K45" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="46" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B46" t="s">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="C46" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D46" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E46">
         <v>94.9</v>
@@ -3218,24 +3216,24 @@
         <v>0</v>
       </c>
       <c r="J46" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="K46" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
     </row>
     <row r="47" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>74</v>
+        <v>70</v>
       </c>
       <c r="B47" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="C47" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D47" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E47">
         <v>35</v>
@@ -3253,24 +3251,24 @@
         <v>1</v>
       </c>
       <c r="J47" t="s">
-        <v>221</v>
+        <v>200</v>
       </c>
       <c r="K47" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
     </row>
     <row r="48" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="B48" t="s">
-        <v>154</v>
+        <v>140</v>
       </c>
       <c r="C48" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D48" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E48">
         <v>35</v>
@@ -3288,24 +3286,24 @@
         <v>1</v>
       </c>
       <c r="J48" t="s">
-        <v>222</v>
+        <v>201</v>
       </c>
       <c r="K48" t="s">
-        <v>113</v>
+        <v>105</v>
       </c>
     </row>
     <row r="49" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="B49" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="C49" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D49" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E49">
         <v>0</v>
@@ -3323,24 +3321,24 @@
         <v>1</v>
       </c>
       <c r="J49" t="s">
-        <v>221</v>
+        <v>200</v>
       </c>
       <c r="K49" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>77</v>
+        <v>73</v>
       </c>
       <c r="B50" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="C50" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D50" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E50">
         <v>0</v>
@@ -3358,24 +3356,24 @@
         <v>1</v>
       </c>
       <c r="J50" t="s">
-        <v>222</v>
+        <v>201</v>
       </c>
       <c r="K50" t="s">
-        <v>115</v>
+        <v>107</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>73</v>
+        <v>69</v>
       </c>
       <c r="B51" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C51" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D51" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E51">
         <v>150</v>
@@ -3393,24 +3391,24 @@
         <v>1</v>
       </c>
       <c r="J51" t="s">
-        <v>221</v>
+        <v>200</v>
       </c>
       <c r="K51" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="B52" t="s">
-        <v>72</v>
+        <v>68</v>
       </c>
       <c r="C52" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D52" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E52">
         <v>150</v>
@@ -3428,33 +3426,33 @@
         <v>1</v>
       </c>
       <c r="J52" t="s">
-        <v>222</v>
+        <v>201</v>
       </c>
       <c r="K52" t="s">
-        <v>116</v>
+        <v>108</v>
       </c>
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="B53" t="s">
-        <v>93</v>
+        <v>231</v>
       </c>
       <c r="C53" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D53" t="s">
-        <v>53</v>
-      </c>
-      <c r="E53">
-        <v>2850</v>
+        <v>50</v>
+      </c>
+      <c r="E53" s="1">
+        <v>2850000000</v>
       </c>
       <c r="F53" t="s">
         <v>5</v>
       </c>
-      <c r="G53">
-        <v>3000</v>
+      <c r="G53" s="1">
+        <v>3000000000</v>
       </c>
       <c r="H53" t="s">
         <v>5</v>
@@ -3463,33 +3461,33 @@
         <v>1</v>
       </c>
       <c r="J53" t="s">
-        <v>221</v>
+        <v>200</v>
       </c>
       <c r="K53" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="B54" t="s">
-        <v>93</v>
+        <v>231</v>
       </c>
       <c r="C54" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D54" t="s">
-        <v>53</v>
-      </c>
-      <c r="E54">
-        <v>2850</v>
+        <v>50</v>
+      </c>
+      <c r="E54" s="1">
+        <v>2850000000</v>
       </c>
       <c r="F54" t="s">
         <v>5</v>
       </c>
-      <c r="G54">
-        <v>3000</v>
+      <c r="G54" s="1">
+        <v>3000000000</v>
       </c>
       <c r="H54" t="s">
         <v>5</v>
@@ -3498,24 +3496,24 @@
         <v>1</v>
       </c>
       <c r="J54" t="s">
-        <v>222</v>
+        <v>201</v>
       </c>
       <c r="K54" t="s">
-        <v>112</v>
+        <v>104</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="B55" t="s">
-        <v>156</v>
+        <v>224</v>
       </c>
       <c r="C55" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D55" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E55">
         <v>30</v>
@@ -3533,24 +3531,24 @@
         <v>1</v>
       </c>
       <c r="J55" t="s">
-        <v>206</v>
+        <v>185</v>
       </c>
       <c r="K55" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="B56" t="s">
-        <v>156</v>
+        <v>224</v>
       </c>
       <c r="C56" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D56" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E56">
         <v>30</v>
@@ -3568,24 +3566,24 @@
         <v>1</v>
       </c>
       <c r="J56" t="s">
-        <v>207</v>
+        <v>186</v>
       </c>
       <c r="K56" t="s">
-        <v>114</v>
+        <v>106</v>
       </c>
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="B57" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="C57" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D57" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E57">
         <v>0</v>
@@ -3603,24 +3601,24 @@
         <v>1</v>
       </c>
       <c r="J57" t="s">
-        <v>206</v>
+        <v>185</v>
       </c>
       <c r="K57" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>86</v>
+        <v>82</v>
       </c>
       <c r="B58" t="s">
-        <v>95</v>
+        <v>89</v>
       </c>
       <c r="C58" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D58" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E58">
         <v>0</v>
@@ -3638,24 +3636,24 @@
         <v>1</v>
       </c>
       <c r="J58" t="s">
-        <v>207</v>
+        <v>186</v>
       </c>
       <c r="K58" t="s">
-        <v>117</v>
+        <v>109</v>
       </c>
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>87</v>
+        <v>83</v>
       </c>
       <c r="B59" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C59" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D59" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E59">
         <v>0</v>
@@ -3673,24 +3671,24 @@
         <v>1</v>
       </c>
       <c r="J59" t="s">
-        <v>206</v>
+        <v>185</v>
       </c>
       <c r="K59" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>88</v>
+        <v>84</v>
       </c>
       <c r="B60" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="C60" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D60" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E60">
         <v>0</v>
@@ -3708,24 +3706,24 @@
         <v>1</v>
       </c>
       <c r="J60" t="s">
-        <v>207</v>
+        <v>186</v>
       </c>
       <c r="K60" t="s">
-        <v>118</v>
+        <v>110</v>
       </c>
     </row>
     <row r="61" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>89</v>
+        <v>85</v>
       </c>
       <c r="B61" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="C61" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D61" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E61">
         <v>0</v>
@@ -3743,24 +3741,24 @@
         <v>1</v>
       </c>
       <c r="J61" t="s">
-        <v>206</v>
+        <v>185</v>
       </c>
       <c r="K61" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
     </row>
     <row r="62" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="B62" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="C62" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D62" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E62">
         <v>0</v>
@@ -3778,24 +3776,24 @@
         <v>1</v>
       </c>
       <c r="J62" t="s">
-        <v>207</v>
+        <v>186</v>
       </c>
       <c r="K62" t="s">
-        <v>119</v>
+        <v>111</v>
       </c>
     </row>
     <row r="63" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="B63" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="C63" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D63" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E63">
         <v>0</v>
@@ -3813,24 +3811,24 @@
         <v>1</v>
       </c>
       <c r="J63" t="s">
-        <v>206</v>
+        <v>185</v>
       </c>
       <c r="K63" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
     </row>
     <row r="64" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="B64" t="s">
-        <v>155</v>
+        <v>141</v>
       </c>
       <c r="C64" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D64" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E64">
         <v>0</v>
@@ -3848,24 +3846,24 @@
         <v>1</v>
       </c>
       <c r="J64" t="s">
-        <v>207</v>
+        <v>186</v>
       </c>
       <c r="K64" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
     </row>
     <row r="65" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="B65" t="s">
-        <v>149</v>
+        <v>135</v>
       </c>
       <c r="C65" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D65" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E65">
         <v>0</v>
@@ -3883,24 +3881,24 @@
         <v>1</v>
       </c>
       <c r="J65" t="s">
-        <v>208</v>
+        <v>187</v>
       </c>
       <c r="K65" t="s">
-        <v>148</v>
+        <v>134</v>
       </c>
     </row>
     <row r="66" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
-        <v>100</v>
+        <v>93</v>
       </c>
       <c r="B66" t="s">
-        <v>164</v>
+        <v>232</v>
       </c>
       <c r="C66" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D66" t="s">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E66">
         <v>0</v>
@@ -3918,24 +3916,24 @@
         <v>1</v>
       </c>
       <c r="J66" t="s">
-        <v>208</v>
+        <v>187</v>
       </c>
       <c r="K66" t="s">
-        <v>122</v>
+        <v>114</v>
       </c>
     </row>
     <row r="67" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="B67" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="C67" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D67" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E67">
         <v>1</v>
@@ -3953,24 +3951,24 @@
         <v>1</v>
       </c>
       <c r="J67" t="s">
-        <v>223</v>
+        <v>202</v>
       </c>
       <c r="K67" t="s">
-        <v>224</v>
+        <v>203</v>
       </c>
     </row>
     <row r="68" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="B68" t="s">
-        <v>143</v>
+        <v>233</v>
       </c>
       <c r="C68" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D68" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E68">
         <v>0</v>
@@ -3988,24 +3986,24 @@
         <v>1</v>
       </c>
       <c r="J68" t="s">
-        <v>223</v>
+        <v>202</v>
       </c>
       <c r="K68" t="s">
-        <v>225</v>
+        <v>204</v>
       </c>
     </row>
     <row r="69" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
-        <v>165</v>
+        <v>148</v>
       </c>
       <c r="B69" t="s">
-        <v>166</v>
+        <v>149</v>
       </c>
       <c r="C69" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D69" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E69">
         <v>70</v>
@@ -4023,24 +4021,24 @@
         <v>1</v>
       </c>
       <c r="J69" t="s">
-        <v>209</v>
+        <v>188</v>
       </c>
       <c r="K69" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
     </row>
     <row r="70" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="B70" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C70" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D70" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E70">
         <v>90</v>
@@ -4058,24 +4056,24 @@
         <v>1</v>
       </c>
       <c r="J70" t="s">
-        <v>210</v>
+        <v>189</v>
       </c>
       <c r="K70" t="s">
-        <v>126</v>
+        <v>118</v>
       </c>
     </row>
     <row r="71" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
-        <v>230</v>
+        <v>208</v>
       </c>
       <c r="B71" t="s">
-        <v>233</v>
+        <v>211</v>
       </c>
       <c r="C71" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D71" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E71">
         <v>0</v>
@@ -4093,24 +4091,24 @@
         <v>1</v>
       </c>
       <c r="J71" t="s">
-        <v>231</v>
+        <v>209</v>
       </c>
       <c r="K71" t="s">
-        <v>229</v>
+        <v>207</v>
       </c>
     </row>
     <row r="72" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="B72" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C72" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D72" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E72">
         <v>50</v>
@@ -4128,24 +4126,24 @@
         <v>1</v>
       </c>
       <c r="J72" t="s">
-        <v>210</v>
+        <v>189</v>
       </c>
       <c r="K72" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="B73" t="s">
-        <v>101</v>
+        <v>94</v>
       </c>
       <c r="C73" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D73" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E73">
         <v>120</v>
@@ -4163,24 +4161,24 @@
         <v>1</v>
       </c>
       <c r="J73" t="s">
-        <v>211</v>
+        <v>190</v>
       </c>
       <c r="K73" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>109</v>
+        <v>101</v>
       </c>
       <c r="B74" t="s">
-        <v>144</v>
+        <v>234</v>
       </c>
       <c r="C74" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D74" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E74">
         <v>50</v>
@@ -4198,24 +4196,24 @@
         <v>1</v>
       </c>
       <c r="J74" t="s">
-        <v>212</v>
+        <v>191</v>
       </c>
       <c r="K74" t="s">
-        <v>123</v>
+        <v>115</v>
       </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>171</v>
+        <v>154</v>
       </c>
       <c r="B75" t="s">
-        <v>132</v>
+        <v>124</v>
       </c>
       <c r="C75" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D75" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E75">
         <v>50</v>
@@ -4233,24 +4231,24 @@
         <v>1</v>
       </c>
       <c r="J75" t="s">
-        <v>213</v>
+        <v>192</v>
       </c>
       <c r="K75" t="s">
-        <v>131</v>
+        <v>123</v>
       </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>107</v>
+        <v>99</v>
       </c>
       <c r="B76" t="s">
-        <v>10</v>
+        <v>235</v>
       </c>
       <c r="C76" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D76" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E76">
         <v>99</v>
@@ -4268,24 +4266,24 @@
         <v>1</v>
       </c>
       <c r="J76" t="s">
-        <v>214</v>
+        <v>193</v>
       </c>
       <c r="K76" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>232</v>
+        <v>210</v>
       </c>
       <c r="B77" t="s">
-        <v>234</v>
+        <v>212</v>
       </c>
       <c r="C77" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D77" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E77">
         <v>0</v>
@@ -4303,24 +4301,24 @@
         <v>1</v>
       </c>
       <c r="J77" t="s">
-        <v>235</v>
+        <v>213</v>
       </c>
       <c r="K77" t="s">
-        <v>229</v>
+        <v>207</v>
       </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="B78" t="s">
-        <v>105</v>
+        <v>236</v>
       </c>
       <c r="C78" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D78" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E78">
         <v>0</v>
@@ -4338,24 +4336,24 @@
         <v>1</v>
       </c>
       <c r="J78" t="s">
-        <v>214</v>
+        <v>193</v>
       </c>
       <c r="K78" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>180</v>
+        <v>162</v>
       </c>
       <c r="B79" t="s">
-        <v>184</v>
+        <v>237</v>
       </c>
       <c r="C79" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D79" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E79">
         <v>1</v>
@@ -4363,34 +4361,28 @@
       <c r="F79" t="s">
         <v>5</v>
       </c>
-      <c r="G79">
-        <v>1</v>
-      </c>
-      <c r="H79" t="s">
-        <v>5</v>
-      </c>
       <c r="I79" t="b">
         <v>1</v>
       </c>
       <c r="J79" t="s">
-        <v>220</v>
+        <v>199</v>
       </c>
       <c r="K79" t="s">
-        <v>179</v>
+        <v>161</v>
       </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
+        <v>11</v>
+      </c>
+      <c r="B80" t="s">
         <v>12</v>
       </c>
-      <c r="B80" t="s">
-        <v>13</v>
-      </c>
       <c r="C80" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D80" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E80">
         <v>0</v>
@@ -4408,24 +4400,24 @@
         <v>1</v>
       </c>
       <c r="J80" t="s">
-        <v>196</v>
+        <v>175</v>
       </c>
       <c r="K80" t="s">
-        <v>121</v>
+        <v>113</v>
       </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>185</v>
+        <v>164</v>
       </c>
       <c r="B81" t="s">
-        <v>181</v>
+        <v>238</v>
       </c>
       <c r="C81" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D81" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E81">
         <v>14.5</v>
@@ -4443,10 +4435,10 @@
         <v>1</v>
       </c>
       <c r="J81" t="s">
-        <v>197</v>
+        <v>176</v>
       </c>
       <c r="K81" t="s">
-        <v>183</v>
+        <v>163</v>
       </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
@@ -4457,10 +4449,10 @@
         <v>9</v>
       </c>
       <c r="C82" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D82" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E82">
         <v>0</v>
@@ -4478,24 +4470,24 @@
         <v>1</v>
       </c>
       <c r="J82" t="s">
-        <v>215</v>
+        <v>194</v>
       </c>
       <c r="K82" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>173</v>
+        <v>156</v>
       </c>
       <c r="B83" t="s">
-        <v>174</v>
+        <v>157</v>
       </c>
       <c r="C83" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D83" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E83">
         <v>69</v>
@@ -4513,24 +4505,24 @@
         <v>1</v>
       </c>
       <c r="J83" t="s">
-        <v>216</v>
+        <v>195</v>
       </c>
       <c r="K83" t="s">
-        <v>175</v>
+        <v>158</v>
       </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>168</v>
+        <v>151</v>
       </c>
       <c r="B84" t="s">
-        <v>169</v>
+        <v>152</v>
       </c>
       <c r="C84" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="D84" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E84">
         <v>0</v>
@@ -4548,24 +4540,24 @@
         <v>1</v>
       </c>
       <c r="J84" t="s">
-        <v>217</v>
+        <v>196</v>
       </c>
       <c r="K84" t="s">
-        <v>170</v>
+        <v>153</v>
       </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B85" t="s">
-        <v>182</v>
+        <v>239</v>
       </c>
       <c r="C85" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="D85" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E85">
         <v>4</v>
@@ -4583,24 +4575,24 @@
         <v>1</v>
       </c>
       <c r="J85" t="s">
-        <v>197</v>
+        <v>176</v>
       </c>
       <c r="K85" t="s">
-        <v>176</v>
+        <v>159</v>
       </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>172</v>
+        <v>155</v>
       </c>
       <c r="B86" t="s">
-        <v>186</v>
+        <v>165</v>
       </c>
       <c r="C86" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="D86" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E86">
         <v>0</v>
@@ -4618,24 +4610,24 @@
         <v>1</v>
       </c>
       <c r="J86" t="s">
-        <v>218</v>
+        <v>197</v>
       </c>
       <c r="K86" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B87" t="s">
-        <v>177</v>
+        <v>240</v>
       </c>
       <c r="C87" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="D87" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="E87">
         <v>33</v>
@@ -4653,10 +4645,10 @@
         <v>1</v>
       </c>
       <c r="J87" t="s">
-        <v>219</v>
+        <v>198</v>
       </c>
       <c r="K87" t="s">
-        <v>178</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>

</xml_diff>